<commit_message>
chore: daily job scan 2026-05-05
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -771,12 +771,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PineGap.ai</t>
+          <t>Kobie</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -785,26 +785,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>85</v>
-      </c>
       <c r="H5" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years meets the 2-year minimum). The resume matches many key terms but lacks explicit AI/ML and product vision language, which is the main keyword gap.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>AI product roadmap, AI/ML concepts, product vision, OKRs, A/B testing, NPS improvement, MAU growth, Snowflake</t>
+          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -822,7 +820,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -839,17 +837,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Kobie</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
@@ -858,19 +856,19 @@
         <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
+          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -888,7 +886,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -905,38 +903,38 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>Soho Square Solutions</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -954,7 +952,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -971,17 +969,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Simplilearn</t>
+          <t>AppBroda</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Growth)</t>
+          <t>Product Manager (UAGenuis)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -990,19 +988,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement and title level, yielding a solid ATS score due to strong keyword overlap, but the candidate's domain (enterprise SaaS, travel tech) only partially aligns with the growth-focused education platform role, lowering the fit score; the biggest keyword gap is the lack of explicit Go-To-Market experience.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (travel tech, enterprise SaaS) does not align well with the AdTech/creative automation focus, lowering the fit score; the most important missing keyword is a specific ad platform such as "Meta Ads".</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Go-To-Market strategy, market research, NPS, CSAT, A/B testing, OKRs, pricing optimization, content management, sales enablement, user segmentation</t>
+          <t>Meta Ads, TikTok Ads, Unity Ads, A/B testing, creative automation, performance marketing, north-star metrics, GTM readiness</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1020,7 +1018,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1037,38 +1035,40 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
+          <t>Opkey</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager -Workday</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>69</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding a solid ATS score due to many matching keywords, but lacks Workday‑specific terms, lowering the fit score because the candidate's domain experience is not aligned with HR/Workday products.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+          <t>Workday, HCM, Payroll, Benefits, Integrations, OKRs, RICE prioritization, UAT planning, defect triage</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1103,12 +1103,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Opkey</t>
+          <t>CARD91</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Workday</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1118,25 +1118,25 @@
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding a solid ATS score due to many matching keywords, but lacks Workday‑specific terms, lowering the fit score because the candidate's domain experience is not aligned with HR/Workday products.</t>
+          <t>The candidate meets the 4-year experience requirement and title alignment, yielding a solid ATS score, but lacks fintech/payment-specific keywords and domain experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Workday, HCM, Payroll, Benefits, Integrations, OKRs, RICE prioritization, UAT planning, defect triage</t>
+          <t>API products, RBI regulations, prepaid, UPI, payment issuance, FinTech, banking, go-to-market strategy, sales collaboration</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1171,12 +1171,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AppBroda</t>
+          <t>Wing Assistant</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (UAGenuis)</t>
+          <t>Product Manager, AI Solutions</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1187,22 +1187,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (travel tech, enterprise SaaS) does not align well with the AdTech/creative automation focus, lowering the fit score; the most important missing keyword is a specific ad platform such as "Meta Ads".</t>
+          <t>Hard rules pass (4 years experience matches no higher minimum). The resume contains many core keywords but misses several JD-specific tools and activities, lowering the ATS score; the strongest gap is the lack of mentioned video/Canva and playbook creation tools. The candidate's GenAI and SaaS experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads, TikTok Ads, Unity Ads, A/B testing, creative automation, performance marketing, north-star metrics, GTM readiness</t>
+          <t>Canva, Asana, Notion, Airtable, HubSpot, product video creation, playbook building, customer interview shadowing, retention metrics analysis, C-level stakeholder communication</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1237,12 +1237,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CARD91</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Technical Product Manager (m/f/d) for API Management @ BTP Integration Suite</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1251,26 +1251,24 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title alignment, yielding a solid ATS score, but lacks fintech/payment-specific keywords and domain experience, lowering the fit score.</t>
+          <t>The resume meets the experience requirement and passes all hard rules, but lacks several API‑specific keywords and direct API management experience, which lowers the fit score; the biggest keyword gap is the absence of "API Management".</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>API products, RBI regulations, prepaid, UPI, payment issuance, FinTech, banking, go-to-market strategy, sales collaboration</t>
+          <t>API Management, Kubernetes, Machine Learning based anomaly detection, Multi‑cloud (AWS, GCP, Azure), API marketplace, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1288,7 +1286,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1305,12 +1303,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Wing Assistant</t>
+          <t>IGEL Technology</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AI Solutions</t>
+          <t>Product Manager (m/f/d) - Bangalore</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1321,22 +1319,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no higher minimum). The resume contains many core keywords but misses several JD-specific tools and activities, lowering the ATS score; the strongest gap is the lack of mentioned video/Canva and playbook creation tools. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Canva, Asana, Notion, Airtable, HubSpot, product video creation, playbook building, customer interview shadowing, retention metrics analysis, C-level stakeholder communication</t>
+          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1371,38 +1369,40 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Avnet</t>
+          <t>GHX India</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Assistant Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and aligns on years, location, and title, yielding a solid ATS score, but the candidate's SaaS/GenAI background mismatches the electronics distribution domain, lowering the fit score; the most notable keyword gap is the lack of explicit "Excel"/"SLA" experience.</t>
+          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Excel, SLA, customer service, global stakeholder communication, quality assurance, inventory management, NPI, EOL</t>
+          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1437,38 +1437,40 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>IGEL Technology</t>
+          <t>ve.ai - the intent company</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (m/f/d) - Bangalore</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F15" s="2" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
+          <t>The candidate meets the 4-year experience requirement and title level, yielding strong keyword overlap and domain relevance; the main keyword gap is lack of explicit OKR or A/B testing experience.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Jobs-to-be-Done, NPS improvement</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1482,7 +1484,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1503,7 +1505,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GHX India</t>
+          <t>GHX</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1521,22 +1523,22 @@
         <v>1</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
+          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
+          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1571,12 +1573,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ve.ai - the intent company</t>
+          <t>Raphus Solutions</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1585,26 +1587,24 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title level, yielding strong keyword overlap and domain relevance; the main keyword gap is lack of explicit OKR or A/B testing experience.</t>
+          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Jobs-to-be-Done, NPS improvement</t>
+          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1639,12 +1639,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GHX</t>
+          <t>Eltropy</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager – AI &amp; Analytics</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1654,25 +1654,25 @@
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F18" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H18" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>77</v>
-      </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
+          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1707,38 +1707,38 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Raphus Solutions</t>
+          <t>Mastercard</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Technical Product Owner</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords (Jira, Agile, SQL, Power BI, stakeholder management) but lacks payment‑security specific terms, lowering the fit score.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
+          <t>Secure SDLC, Payment processing, Compliance, Risk management, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1752,11 +1752,11 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -1773,40 +1773,38 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Eltropy</t>
+          <t>TransPerfect</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI &amp; Analytics</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>70</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but misses several integration-specific terms, yielding a moderate ATS score. The candidate's strong GenAI and SaaS experience aligns well with the role, though domain specifics like CMS/e‑commerce integration are lacking.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+          <t>API evaluation, GraphQL, CMS integration, Statement of Work (SOW) preparation, vendor management, test strategy review, UI/UX design participation, continuous upgrade planning</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1820,7 +1818,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
@@ -1833,138 +1831,6 @@
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Associate Technical Product Owner</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords (Jira, Agile, SQL, Power BI, stakeholder management) but lacks payment‑security specific terms, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Secure SDLC, Payment processing, Compliance, Risk management, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>TransPerfect</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Manager</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but misses several integration-specific terms, yielding a moderate ATS score. The candidate's strong GenAI and SaaS experience aligns well with the role, though domain specifics like CMS/e‑commerce integration are lacking.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>API evaluation, GraphQL, CMS integration, Statement of Work (SOW) preparation, vendor management, test strategy review, UI/UX design participation, continuous upgrade planning</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>2026-05-05</t>
         </is>
@@ -1991,8 +1857,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2110,38 +1974,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager, Private Cloud Domain</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks retail‑specific terms like inventory visibility and OOS, leading to a moderate ATS score and a slightly lower fit due to domain mismatch.</t>
+          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>inventory visibility, out-of-stock, supply chain, merchandising, personalization, OKRs, A/B testing</t>
+          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2176,38 +2040,38 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>eGov Foundation</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Digital Health (Public Health)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
+          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks retail‑specific terms like inventory visibility and OOS, leading to a moderate ATS score and a slightly lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
+          <t>inventory visibility, out-of-stock, supply chain, merchandising, personalization, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2225,7 +2089,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -2242,12 +2106,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>First Advantage</t>
+          <t>eGov Foundation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Data Analytics- Remote</t>
+          <t>Product Manager - Digital Health (Public Health)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2258,22 +2122,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>51</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and location, so hard rules do not penalize; however, keyword density for data‑analytics specific terms is moderate, leading to a modest ATS score, while the candidate's SaaS and GenAI background gives a decent fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Snowflake, Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2308,38 +2172,38 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Aptita</t>
+          <t>First Advantage</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Data Analytics- Remote</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, but lacks many JD‑specific keywords (e.g., Confluence, API, microservices), resulting in a low ATS score; the candidate’s SaaS and enterprise background is relevant but the banking/financial domain is a mismatch.</t>
+          <t>The resume meets the 4-year experience requirement and location, so hard rules do not penalize; however, keyword density for data‑analytics specific terms is moderate, leading to a modest ATS score, while the candidate's SaaS and GenAI background gives a decent fit.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Confluence, API, microservices, CI/CD, financial compliance</t>
+          <t>Snowflake, Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2357,7 +2221,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -2374,38 +2238,38 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Autodesk</t>
+          <t>Aptita</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Web Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'messaging platform'.</t>
+          <t>The resume meets the 4‑year experience requirement and location, but lacks many JD‑specific keywords (e.g., Confluence, API, microservices), resulting in a low ATS score; the candidate’s SaaS and enterprise background is relevant but the banking/financial domain is a mismatch.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>messaging platform, multi-channel delivery, governance, personalization, API integration, campaign configuration, analytics, preference management</t>
+          <t>Confluence, API, microservices, CI/CD, financial compliance</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2423,7 +2287,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -2638,12 +2502,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Altimate AI</t>
+          <t>Hire Feed</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Remote)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2700,40 +2564,36 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Altimate AI</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, LLM/ML Domain</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2745,7 +2605,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -2771,7 +2631,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Observability Domain</t>
+          <t>Technical Product Manager, LLM/ML Domain</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2785,19 +2645,19 @@
         <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
+          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2832,12 +2692,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
+          <t>Technical Product Manager, Observability Domain</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2848,22 +2708,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
+          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
+          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2881,7 +2741,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -2898,12 +2758,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Zemoso Technologies</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Branch Operations Product</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2914,20 +2774,24 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as "branch banking operations" and "product success metrics".</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>branch banking operations, product success metrics, OKRs, A/B testing, risk posture</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2960,12 +2824,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Payments</t>
+          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2974,24 +2838,26 @@
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3007,7 +2873,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -3024,12 +2890,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Hire Feed</t>
+          <t>Zemoso Technologies</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Remote)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3086,12 +2952,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Transformation</t>
+          <t>Product Owner – Payments</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3100,7 +2966,9 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
       </c>
@@ -3148,40 +3016,36 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Private Cloud Domain</t>
+          <t>Product Owner - Transformation</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3193,7 +3057,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-06
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -628,7 +628,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -696,19 +696,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>North Hires</t>
+          <t>PineGap.ai</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner (Immediate Joiners)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -718,25 +718,25 @@
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches the associate level, yielding solid ATS and fit scores; the most notable keyword gap is the absence of explicit OKR/RICE prioritization terminology.</t>
+          <t>Hard rules are satisfied (4 years meets the 2-year minimum). The resume matches many key terms but lacks explicit AI/ML and product vision language, which is the main keyword gap.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, Snowflake</t>
+          <t>AI product roadmap, AI/ML concepts, product vision, OKRs, A/B testing, NPS improvement, MAU growth, Snowflake</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -830,24 +830,24 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
@@ -856,19 +856,19 @@
         <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; it contains many JD keywords but lacks ecommerce‑specific terms, lowering the fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>ecommerce, API documentation, A/B testing, OKRs, NPS improvement, data pipeline, SQL reporting</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -896,45 +896,45 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
+          <t>ALLEN Digital</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+          <t>The resume meets the hard rules with 4+ years experience and appropriate title; it contains many JD keywords but lacks education‑tech specific terms, lowering the fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, MAU growth, PLG, Jobs-to-be-Done</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,34 +952,34 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AppBroda</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (UAGenuis)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -988,19 +988,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (travel tech, enterprise SaaS) does not align well with the AdTech/creative automation focus, lowering the fit score; the most important missing keyword is a specific ad platform such as "Meta Ads".</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads, TikTok Ads, Unity Ads, A/B testing, creative automation, performance marketing, north-star metrics, GTM readiness</t>
+          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1028,47 +1028,45 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Opkey</t>
+          <t>Simplilearn</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Workday</t>
+          <t>Product Manager (Growth)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding a solid ATS score due to many matching keywords, but lacks Workday‑specific terms, lowering the fit score because the candidate's domain experience is not aligned with HR/Workday products.</t>
+          <t>The resume meets the experience requirement and title level, yielding a solid ATS score due to strong keyword overlap, but the candidate's domain (enterprise SaaS, travel tech) only partially aligns with the growth-focused education platform role, lowering the fit score; the biggest keyword gap is the lack of explicit Go-To-Market experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Workday, HCM, Payroll, Benefits, Integrations, OKRs, RICE prioritization, UAT planning, defect triage</t>
+          <t>Go-To-Market strategy, market research, NPS, CSAT, A/B testing, OKRs, pricing optimization, content management, sales enablement, user segmentation</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1096,19 +1094,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>CARD91</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1117,26 +1115,24 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title alignment, yielding a solid ATS score, but lacks fintech/payment-specific keywords and domain experience, lowering the fit score.</t>
+          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>API products, RBI regulations, prepaid, UPI, payment issuance, FinTech, banking, go-to-market strategy, sales collaboration</t>
+          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1154,29 +1150,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Wing Assistant</t>
+          <t>Opkey</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AI Solutions</t>
+          <t>Product Manager -Workday</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1185,24 +1181,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F11" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no higher minimum). The resume contains many core keywords but misses several JD-specific tools and activities, lowering the ATS score; the strongest gap is the lack of mentioned video/Canva and playbook creation tools. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding a solid ATS score due to many matching keywords, but lacks Workday‑specific terms, lowering the fit score because the candidate's domain experience is not aligned with HR/Workday products.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Canva, Asana, Notion, Airtable, HubSpot, product video creation, playbook building, customer interview shadowing, retention metrics analysis, C-level stakeholder communication</t>
+          <t>Workday, HCM, Payroll, Benefits, Integrations, OKRs, RICE prioritization, UAT planning, defect triage</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1220,7 +1218,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1230,19 +1228,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>CARD91</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (m/f/d) for API Management @ BTP Integration Suite</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1251,24 +1249,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement and passes all hard rules, but lacks several API‑specific keywords and direct API management experience, which lowers the fit score; the biggest keyword gap is the absence of "API Management".</t>
+          <t>The candidate meets the 4-year experience requirement and title alignment, yielding a solid ATS score, but lacks fintech/payment-specific keywords and domain experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>API Management, Kubernetes, Machine Learning based anomaly detection, Multi‑cloud (AWS, GCP, Azure), API marketplace, OKRs, RICE prioritization, NPS improvement</t>
+          <t>API products, RBI regulations, prepaid, UPI, payment issuance, FinTech, banking, go-to-market strategy, sales collaboration</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1296,19 +1296,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>IGEL Technology</t>
+          <t>Wing Assistant</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (m/f/d) - Bangalore</t>
+          <t>Product Manager, AI Solutions</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1319,22 +1319,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
+          <t>Hard rules pass (4 years experience matches no higher minimum). The resume contains many core keywords but misses several JD-specific tools and activities, lowering the ATS score; the strongest gap is the lack of mentioned video/Canva and playbook creation tools. The candidate's GenAI and SaaS experience aligns well with the role.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
+          <t>Canva, Asana, Notion, Airtable, HubSpot, product video creation, playbook building, customer interview shadowing, retention metrics analysis, C-level stakeholder communication</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1362,65 +1362,63 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GHX India</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Technical Product Manager (m/f/d) for API Management @ BTP Integration Suite</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the experience requirement and passes all hard rules, but lacks several API‑specific keywords and direct API management experience, which lowers the fit score; the biggest keyword gap is the absence of "API Management".</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>API Management, Kubernetes, Machine Learning based anomaly detection, Multi‑cloud (AWS, GCP, Azure), API marketplace, OKRs, RICE prioritization, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1430,47 +1428,45 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ve.ai - the intent company</t>
+          <t>IGEL Technology</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager (m/f/d) - Bangalore</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title level, yielding strong keyword overlap and domain relevance; the main keyword gap is lack of explicit OKR or A/B testing experience.</t>
+          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, Jobs-to-be-Done, NPS improvement</t>
+          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1484,7 +1480,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1498,14 +1494,14 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GHX</t>
+          <t>GHX India</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1523,22 +1519,22 @@
         <v>1</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
+          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
+          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1566,19 +1562,19 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Raphus Solutions</t>
+          <t>ve.ai - the intent company</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1587,24 +1583,26 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F17" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
+          <t>The candidate meets the 4-year experience requirement and title level, yielding strong keyword overlap and domain relevance; the main keyword gap is lack of explicit OKR or A/B testing experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, Jobs-to-be-Done, NPS improvement</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1632,19 +1630,19 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Eltropy</t>
+          <t>GHX</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI &amp; Analytics</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1654,25 +1652,25 @@
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1700,45 +1698,45 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Mastercard</t>
+          <t>Raphus Solutions</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Associate Technical Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords (Jira, Agile, SQL, Power BI, stakeholder management) but lacks payment‑security specific terms, lowering the fit score.</t>
+          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Secure SDLC, Payment processing, Compliance, Risk management, OKRs, A/B testing</t>
+          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1752,11 +1750,11 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -1766,73 +1764,207 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TransPerfect</t>
+          <t>Eltropy</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager – AI &amp; Analytics</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F20" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>70</v>
       </c>
       <c r="H20" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Associate Technical Product Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains many JD keywords (Jira, Agile, SQL, Power BI, stakeholder management) but lacks payment‑security specific terms, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Secure SDLC, Payment processing, Compliance, Risk management, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TransPerfect</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H22" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Hard rules are satisfied; the resume contains many relevant keywords but misses several integration-specific terms, yielding a moderate ATS score. The candidate's strong GenAI and SaaS experience aligns well with the role, though domain specifics like CMS/e‑commerce integration are lacking.</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>API evaluation, GraphQL, CMS integration, Statement of Work (SOW) preparation, vendor management, test strategy review, UI/UX design participation, continuous upgrade planning</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -1857,6 +1989,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1868,7 +2002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1979,7 +2113,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Private Cloud Domain</t>
+          <t>Technical Product Manager, LLM/ML Domain</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1990,22 +2124,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
+          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2033,45 +2167,45 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager, Observability Domain</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks retail‑specific terms like inventory visibility and OOS, leading to a moderate ATS score and a slightly lower fit due to domain mismatch.</t>
+          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>inventory visibility, out-of-stock, supply chain, merchandising, personalization, OKRs, A/B testing</t>
+          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2099,7 +2233,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2299,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2365,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -2297,19 +2431,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PHINIA</t>
+          <t>Tazapay</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Finance Application Product Owner and RPA</t>
+          <t>Product Manager – Risk &amp; Compliance Platform</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2318,24 +2452,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is low because key finance and SAP/RPA keywords are missing; the biggest gap is the lack of any SAP or UiPath experience. Fit score reflects domain mismatch but strong GenAI and SaaS background.</t>
+          <t>Hard rules are satisfied (4 years experience matches requirement). ATS score is low due to missing core fintech and risk compliance keywords, while the fit score is limited by domain mismatch despite strong GenAI and SaaS experience.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>UiPath, RPA, SAP S/4HANA, SAP BTP, Finance application, P2P/AP, O2C/AR, Master Data management</t>
+          <t>KYC, KYB, AML, transaction monitoring, sanctions screening, risk decisioning, low-code/no-code workflow automation, false positives, turnaround time, risk rules and alerts</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2358,24 +2494,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tredence Inc.</t>
+          <t>Autodesk</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Web Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2386,22 +2522,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rule triggered because the JD requires 7-12 years of experience while the candidate has only 4 years, forcing both scores below 30; the resume also lacks explicit mention of 'question expansion' and 'hypothesis testing' keywords.</t>
+          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'messaging platform'.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>question expansion, hypothesis generation, data sufficiency, LLM-based agents, A/B testing</t>
+          <t>messaging platform, multi-channel delivery, governance, personalization, API integration, campaign configuration, analytics, preference management</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2429,19 +2565,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Tredence Inc.</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Partners</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2462,12 +2598,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several partner‑facing keywords.</t>
+          <t>Hard rule triggered because the JD requires 7-12 years of experience while the candidate has only 4 years, forcing both scores below 30; the resume also lacks explicit mention of 'question expansion' and 'hypothesis testing' keywords.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>partner onboarding, B2B2C platform, partner ecosystem, sales collaboration, financial services / FinTech, OKRs</t>
+          <t>question expansion, hypothesis generation, data sufficiency, LLM-based agents, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2485,7 +2621,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -2495,19 +2631,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Hire Feed</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Remote)</t>
+          <t>Product Manager - Partners</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2518,20 +2654,24 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several partner‑facing keywords.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>partner onboarding, B2B2C platform, partner ecosystem, sales collaboration, financial services / FinTech, OKRs</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2557,7 +2697,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -2619,7 +2759,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2771,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, LLM/ML Domain</t>
+          <t>Technical Product Manager, Private Cloud Domain</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2642,22 +2782,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>55</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>65</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>59</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
+          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
+          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2685,19 +2825,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Observability Domain</t>
+          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2708,22 +2848,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
+          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2741,7 +2881,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -2751,7 +2891,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -2817,19 +2957,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Zemoso Technologies</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2840,24 +2980,20 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2873,7 +3009,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -2883,19 +3019,19 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Zemoso Technologies</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner – Payments</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -2904,7 +3040,9 @@
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F16" s="2" t="n">
         <v>0</v>
       </c>
@@ -2945,19 +3083,19 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Payments</t>
+          <t>Product Owner - Transformation</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2966,9 +3104,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
         <v>0</v>
       </c>
@@ -3009,43 +3145,47 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Knorr- Bremse Systems for Commercial  Vehicles India Pvt. Ltd. Pune</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Transformation</t>
+          <t>Regional Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
+          <t>Hard rules pass; the resume contains some product management keywords but lacks many JD-specific terms, leading to a modest ATS score and a lower fit due to domain mismatch.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Product roadmap, R&amp;D footprint, Make/Buy analysis, Budget planning, P&amp;L management, Risk management, M&amp;A</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3057,11 +3197,11 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -3071,45 +3211,45 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Knorr- Bremse Systems for Commercial  Vehicles India Pvt. Ltd. Pune</t>
+          <t>Siemens Energy</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Regional Product Manager</t>
+          <t>API Expert &amp; Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains some product management keywords but lacks many JD-specific terms, leading to a modest ATS score and a lower fit due to domain mismatch.</t>
+          <t>Hard rules are satisfied, but the resume lacks core API and integration keywords and does not mention the required location, resulting in a low ATS score; the biggest gap is the absence of API design and governance terminology.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Product roadmap, R&amp;D footprint, Make/Buy analysis, Budget planning, P&amp;L management, Risk management, M&amp;A</t>
+          <t>OpenAPI, API contract design, API governance, CI/CD, SAP ERP integration, Salesforce integration, KPI dashboard, SLAs/SLIs/SLOs</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3127,7 +3267,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -3137,19 +3277,19 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Siemens Energy</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>API Expert &amp; Product Manager</t>
+          <t>IT PRODUCT OWNER - SD BILLING (SAP S/4HANA) - VOIS</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3160,22 +3300,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G20" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>32</v>
-      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks core API and integration keywords and does not mention the required location, resulting in a low ATS score; the biggest gap is the absence of API design and governance terminology.</t>
+          <t>Hard rules pass, but the resume lacks SAP billing keywords and domain experience, resulting in low ATS and fit scores; the most critical missing keyword is 'SAP SD Billing'.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>OpenAPI, API contract design, API governance, CI/CD, SAP ERP integration, Salesforce integration, KPI dashboard, SLAs/SLIs/SLOs</t>
+          <t>SAP SD, S/4HANA, fit‑gap analysis, UAT, intercompany billing, SAP methodology, billing governance</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3193,7 +3333,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -3203,7 +3343,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3269,28 +3409,30 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>AGDATA, LP</t>
+          <t>Live Connections</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>AI ML Product Owner - BFSI</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F22" s="2" t="n">
         <v>25</v>
       </c>
@@ -3302,12 +3444,12 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The JD title includes 'Senior' which triggers hard rule 3, forcing both scores below 30 regardless of experience or keyword match; the resume lacks key senior‑level product ownership language.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit AI/ML and financial services terminology.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Snowflake, Data platform roadmap, NPS improvement, Marketplace dynamics, Cross‑functional data team collaboration</t>
+          <t>AI/ML model evaluation, AWS cloud platform, Financial services / Asset Management, Product Owner certification (CSPO/CPO), Metrics definition and data‑driven decision making</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3330,48 +3472,52 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>AGDATA, LP</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>VP- Custody Tax Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>The JD title includes 'Senior' which triggers hard rule 3, forcing both scores below 30 regardless of experience or keyword match; the resume lacks key senior‑level product ownership language.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, Snowflake, Data platform roadmap, NPS improvement, Marketplace dynamics, Cross‑functional data team collaboration</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3397,7 +3543,69 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Citi</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>VP- Custody Tax Product Manager</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
         </is>
       </c>
     </row>
@@ -3425,6 +3633,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-08
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cube</t>
+          <t>Rang De</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>88</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1‑year minimum and title matches exactly, yielding a high ATS score; the biggest keyword gap is the lack of explicit marketing‑tech terms like SEO or A/B testing.</t>
+          <t>The resume meets the 2‑year minimum and matches the Associate Product Manager title, yielding a strong ATS score; however, the candidate lacks fintech‑specific experience, lowering the fit score, and the JD’s keyword "user research" is missing.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>SEO, A/B testing, Mixpanel, Snowflake, OKRs, RICE prioritization, NPS improvement, product roadmap, growth team collaboration</t>
+          <t>user research, PMF surveys, design sprint, A/B testing, analytics platform, Excel, NPS improvement, OKRs</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,24 +618,24 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rang De</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -649,26 +649,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>81</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and matches the Associate Product Manager title, yielding a strong ATS score; however, the candidate lacks fintech‑specific experience, lowering the fit score, and the JD’s keyword "user research" is missing.</t>
+          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>user research, PMF surveys, design sprint, A/B testing, analytics platform, Excel, NPS improvement, OKRs</t>
+          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -686,7 +684,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -696,14 +694,14 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Greenway Health</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -719,22 +717,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>85</v>
+        <v>64</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
+          <t>The resume meets all hard rules and contains many JD keywords, yielding a high ATS score; however, the candidate's experience is in SaaS and travel tech rather than healthcare, creating a domain mismatch that lowers the fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
+          <t>healthcare regulations, ambulatory care workflows, EMR/EHR integration, HIPAA compliance, clinical user interface design, patient engagement metrics, digital health market research</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -757,24 +755,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Kapture CX</t>
+          <t>Ascendion</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner/ Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,26 +781,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and title match, yielding strong keyword overlap; the biggest gap is the lack of explicit market research/competitor analysis terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement). ATS score is solid due to strong keyword overlap and relevant title, but missing workshop and release‑plan terms. Fit score reflects good SaaS and GenAI experience but limited direct product‑owner domain exposure.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>market research, competitor analysis, roadmap development, OKRs, A/B testing, Mixpanel, NPS improvement, user adoption metrics</t>
+          <t>workshops, release planning, OKRs, product vision, customer interviews</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -820,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ascendion</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner/ Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -853,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement). ATS score is solid due to strong keyword overlap and relevant title, but missing workshop and release‑plan terms. Fit score reflects good SaaS and GenAI experience but limited direct product‑owner domain exposure.</t>
+          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>workshops, release planning, OKRs, product vision, customer interviews</t>
+          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,34 +882,34 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -922,19 +918,19 @@
         <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; it contains many JD keywords but lacks ecommerce‑specific terms, lowering the fit.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>ecommerce, API documentation, A/B testing, OKRs, NPS improvement, data pipeline, SQL reporting</t>
+          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,7 +948,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -962,7 +958,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1014,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1028,45 +1024,47 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Personalization &amp; Data Platforms</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1084,34 +1082,34 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Infineon Technologies</t>
+          <t>BeBetta</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Manager - Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1127,12 +1125,12 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's SaaS/GenAI focus does not align well with the hardware web product domain, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and matches the Associate Product Manager title, yielding a solid ATS score, but the candidate's domain (B2B/B2C SaaS, travel and enterprise tools) does not align with BeBetta's gaming focus, lowering the fit score; the biggest keyword gap is the lack of analytics tools like Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CX reports, roadmap planning, backlog grooming, Evaluation Board Finder</t>
+          <t>Mixpanel, A/B testing, NPS improvement, DAU/MAU growth, gaming industry experience, sports domain knowledge, Google Analytics, Data Studio</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1155,19 +1153,19 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Nexus Venture Partners</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1181,24 +1179,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>69</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, but lacks fintech-specific experience, lowering the overall fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
+          <t>RBI guidelines, underwriting rules, conversion KPI, CAC, risk management, credit product, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1216,29 +1216,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AppBroda</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (UAGenuis)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1249,22 +1249,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>69</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (travel tech, enterprise SaaS) does not align well with the AdTech/creative automation focus, lowering the fit score; the most important missing keyword is a specific ad platform such as "Meta Ads".</t>
+          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Meta Ads, TikTok Ads, Unity Ads, A/B testing, creative automation, performance marketing, north-star metrics, GTM readiness</t>
+          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1282,57 +1282,55 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CARD91</t>
+          <t>Infineon Technologies</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Manager - Product Owner</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and title alignment, yielding a solid ATS score, but lacks fintech/payment-specific keywords and domain experience, lowering the fit score.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's SaaS/GenAI focus does not align well with the hardware web product domain, lowering the fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>API products, RBI regulations, prepaid, UPI, payment issuance, FinTech, banking, go-to-market strategy, sales collaboration</t>
+          <t>A/B testing, CX reports, roadmap planning, backlog grooming, Evaluation Board Finder</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1350,29 +1348,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Wing Assistant</t>
+          <t>Opkey</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AI Solutions</t>
+          <t>Product Manager -Workday</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1381,24 +1379,26 @@
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F14" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H14" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no higher minimum). The resume contains many core keywords but misses several JD-specific tools and activities, lowering the ATS score; the strongest gap is the lack of mentioned video/Canva and playbook creation tools. The candidate's GenAI and SaaS experience aligns well with the role.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding a solid ATS score due to many matching keywords, but lacks Workday‑specific terms, lowering the fit score because the candidate's domain experience is not aligned with HR/Workday products.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Canva, Asana, Notion, Airtable, HubSpot, product video creation, playbook building, customer interview shadowing, retention metrics analysis, C-level stakeholder communication</t>
+          <t>Workday, HCM, Payroll, Benefits, Integrations, OKRs, RICE prioritization, UAT planning, defect triage</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1426,45 +1426,45 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Golden Opportunities</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
+          <t>Product Manager, Amazon Business India</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
+          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
+          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1482,29 +1482,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>IGEL Technology</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (m/f/d) - Bangalore</t>
+          <t>Technical Product Manager (m/f/d) for API Management @ BTP Integration Suite</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1515,22 +1515,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
+          <t>The resume meets the experience requirement and passes all hard rules, but lacks several API‑specific keywords and direct API management experience, which lowers the fit score; the biggest keyword gap is the absence of "API Management".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
+          <t>API Management, Kubernetes, Machine Learning based anomaly detection, Multi‑cloud (AWS, GCP, Azure), API marketplace, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1558,65 +1558,63 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GHX India</t>
+          <t>IGEL Technology</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager (m/f/d) - Bangalore</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -1626,14 +1624,14 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AIxCompass</t>
+          <t>Raphus Solutions</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1652,19 +1650,19 @@
         <v>75</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score; the biggest gap is the lack of explicit 'roadmap development' and 'market research' terminology.</t>
+          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>roadmap development, market research, competitive analysis, customer feedback, OKRs, A/B testing</t>
+          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1682,29 +1680,29 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Raphus Solutions</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>FBS Customer Experience Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1715,22 +1713,22 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many core keywords but misses several JD-specific tools and metrics, leading to a solid but not top ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a good fit score.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
+          <t>Mixpanel, Qualtrics, Fullstory, CSAT, FCR, predictive analytics, real-time dashboards, AI-driven insights, KPI monitoring</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1748,29 +1746,29 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GHX</t>
+          <t>Hitachi Digital Services</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager-63827</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1779,26 +1777,24 @@
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
+          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1816,57 +1812,55 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Eltropy</t>
+          <t>ParentPay Group</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI &amp; Analytics</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1880,59 +1874,61 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services</t>
+          <t>Omnibound AI</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-63827</t>
+          <t>Martech Product manager</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F22" s="2" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+          <t>The resume meets the 2‑year minimum and title level, so hard rules pass; it contains many JD keywords but lacks direct marketing experience, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+          <t>marketing automation, ABM, SEO, paid campaigns, digital marketing workflows, KPIs for marketing, US‑based team collaboration, LLMs, co‑pilot technologies</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1946,7 +1942,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -1955,24 +1951,24 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group</t>
+          <t>EXL</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Manager-Product Development-Technology/Digital Product Owner</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1983,22 +1979,22 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2016,7 +2012,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -2026,205 +2022,7 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Associate Technical Product Owner</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords (Jira, Agile, SQL, Power BI, stakeholder management) but lacks payment‑security specific terms, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Secure SDLC, Payment processing, Compliance, Risk management, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>VOIS</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>TECHNOLOGY PRODUCT OWNER - MARKETPLACE VOIS</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords and relevant tools, giving a solid ATS score, but lacks marketplace‑specific terminology and some listed methodologies, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Marketplace platform, Two-sided marketplace, OKRs, Lean Portfolio Management, Technical debt, Data privacy, Vendor management</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>EXL</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Manager-Product Development-Technology/Digital Product Owner</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -2252,9 +2050,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2266,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2372,12 +2167,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rang De</t>
+          <t>Kapture CX</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Growth</t>
+          <t>Technical Product Manager – Applied AI (Voice)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2388,22 +2183,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and has no senior‑level title conflict, so hard rules pass; however, it lacks many growth‑specific tools and terminology from the JD, lowering the ATS score, while its SaaS and product lifecycle experience gives a moderate job‑fit score.</t>
+          <t>The candidate meets the 4-year experience requirement and the title is not senior, so hard rules pass; however the resume lacks key voice AI terms like LLM, STT/TTS, reducing the ATS keyword match.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>WebEngage, MoEngage, Clevertap, WhatsApp conversational journeys, A/B testing, cohort analysis, growth dashboards, marketing automation, retention metrics</t>
+          <t>LLM, STT, TTS, voice bot, conversation quality, benchmarking, latency, cost optimization</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2421,7 +2216,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -2431,19 +2226,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kapture CX</t>
+          <t>Motorola Solutions</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager – Applied AI (Voice)</t>
+          <t>Planview - Technical Product Owner</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2454,22 +2249,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title is not senior, so hard rules pass; however the resume lacks key voice AI terms like LLM, STT/TTS, reducing the ATS keyword match.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume matches many general product management keywords but lacks several JD‑specific tools and processes, lowering the ATS score; the strongest gap is the absence of Planview/Projectplace/Agileplace terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>LLM, STT, TTS, voice bot, conversation quality, benchmarking, latency, cost optimization</t>
+          <t>Planview, Projectplace, Agileplace, ERP integration, CRM integration, SIT/UAT planning, Cutover planning, functional documentation, automation use cases, dashboard creation</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2492,24 +2287,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Nielsen</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Observability Domain</t>
+          <t>Product Manager (Client Facing Product Development)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2520,22 +2315,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>The resume meets the 4-year experience requirement and location, but lacks many JD-specific keywords and direct sports‑media domain experience, resulting in a modest ATS score and a moderate job‑fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
+          <t>customer interviews, surveys, A/B testing, OKRs, RICE prioritization, Mixpanel, Snowflake, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2553,29 +2348,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Snapmint</t>
+          <t>PW (PhysicsWallah)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2584,24 +2379,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3-5 year experience requirement, so no hard rule penalty; however, the resume lacks many payment-specific keywords, lowering the ATS score. The biggest keyword gap is the absence of any UPI or payments terminology.</t>
+          <t>Hard rules pass (4 years meets the 2‑year minimum). ATS score is low because key JD terms like A/B testing, DAU/MAU, and engagement metrics are missing; fit score is moderate due to domain mismatch despite solid SaaS experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>UPI, payments ecosystem, PSP integration, NPCI regulations, financial compliance, A/B testing, growth metrics (MAU, retention), OKRs</t>
+          <t>A/B testing, DAU, MAU, engagement metrics, retention, habit formation, growth team collaboration, user behavior analysis</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2619,7 +2416,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -2629,45 +2426,45 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>eGov Foundation</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Digital Health (Public Health)</t>
+          <t>Acceptance Risk - Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of explicit API design/architecture terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
+          <t>API specifications, solution architecture, merchant integration, transaction processing, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2685,29 +2482,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Nielsen</t>
+          <t>PHINIA</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Client Facing Product Development)</t>
+          <t>Finance Application Product Owner and RPA</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2718,22 +2515,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and location, but lacks many JD-specific keywords and direct sports‑media domain experience, resulting in a modest ATS score and a moderate job‑fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is low because key finance and SAP/RPA keywords are missing; the biggest gap is the lack of any SAP or UiPath experience. Fit score reflects domain mismatch but strong GenAI and SaaS background.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>customer interviews, surveys, A/B testing, OKRs, RICE prioritization, Mixpanel, Snowflake, NPS improvement, MAU growth</t>
+          <t>UiPath, RPA, SAP S/4HANA, SAP BTP, Finance application, P2P/AP, O2C/AR, Master Data management</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2751,29 +2548,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PERSOL APAC</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Vice President - Product Manager - Managed Solution</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2784,22 +2581,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and passes all hard rules, but it lacks many JD‑specific keywords and domain experience, resulting in a moderate ATS score and low job‑fit score; the biggest gap is the absence of Adobe Analytics/Marketing Automation terminology.</t>
+          <t>The JD requires 10+ years of product management experience, which exceeds the candidate's 4 years, triggering hard rule 2; therefore both scores are forced below 30. The resume also lacks key AI/ML governance terms such as MLOps and risk compliance.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Adobe Campaign Classic, marketing automation, campaign orchestration, mobile push notifications, tagging/data‑collection, NPS improvement</t>
+          <t>MLOps, risk management, executive storytelling, OKRs, LLMs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2822,24 +2619,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PW (PhysicsWallah)</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-2</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2848,26 +2645,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2‑year minimum). ATS score is low because key JD terms like A/B testing, DAU/MAU, and engagement metrics are missing; fit score is moderate due to domain mismatch despite solid SaaS experience.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "Kanban" and "support operations".</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, DAU, MAU, engagement metrics, retention, habit formation, growth team collaboration, user behavior analysis</t>
+          <t>Kanban, support operations, defect resolution, production support, release planning, test scenarios, application performance monitoring</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2885,7 +2680,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -2895,19 +2690,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PHINIA</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Finance Application Product Owner and RPA</t>
+          <t>Product Manager - Payments</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2918,22 +2713,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is low because key finance and SAP/RPA keywords are missing; the biggest gap is the lack of any SAP or UiPath experience. Fit score reflects domain mismatch but strong GenAI and SaaS background.</t>
+          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>UiPath, RPA, SAP S/4HANA, SAP BTP, Finance application, P2P/AP, O2C/AR, Master Data management</t>
+          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2951,57 +2746,53 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>American Express Global Business Travel</t>
+          <t>Altimate AI</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like "WordPress" and "API integrations".</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>WordPress, API integrations, content management system, website performance monitoring, vendor management</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3017,55 +2808,55 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Ashika Group</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Product Manager - Stock Broking</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
+          <t>Hard rules pass (4 years experience matches no &gt;4 requirement). ATS score is moderate due to decent keyword overlap but missing finance-specific terms and location mismatch; the biggest keyword gap is lack of financial analysis experience.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
+          <t>Financial analysis, Strategic planning, Product lifecycle management, Presentation skills, Market research, Finance industry experience, Data visualization tools (e.g., Tableau)</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3079,7 +2870,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -3088,50 +2879,50 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Technical Product Manager, Observability Domain</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "Kanban" and "support operations".</t>
+          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Kanban, support operations, defect resolution, production support, release planning, test scenarios, application performance monitoring</t>
+          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3145,57 +2936,61 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Altimate AI</t>
+          <t>Recykal.com</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - AI &amp; Innovation</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
+          <t>Hard rules are satisfied (4 years experience matches the 2-3 year requirement). The resume misses several JD-specific terms like A/B testing and rapid prototyping, lowering the ATS score, while the candidate's GenAI and SaaS experience strongly aligns with the role.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, rapid prototyping, low-code/no-code, vibe coding, experiment design</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3207,33 +3002,33 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Recykal.com</t>
+          <t>Keyloop</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI &amp; Innovation</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3244,22 +3039,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H15" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches the 2-3 year requirement). The resume misses several JD-specific terms like A/B testing and rapid prototyping, lowering the ATS score, while the candidate's GenAI and SaaS experience strongly aligns with the role.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, rapid prototyping, low-code/no-code, vibe coding, experiment design</t>
+          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3282,24 +3077,24 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TALENTMATE</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - APAC Onboarding And KYC</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3310,22 +3105,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement, but the resume lacks many core KYC/FinTech keywords, lowering both ATS and fit scores; the biggest gap is missing KYC and AML terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>KYC, AML compliance, identity verification, fincrime risk mitigation, regulatory requirements, FinTech, customer onboarding metrics</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3348,24 +3143,24 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Zemoso Technologies</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3376,20 +3171,24 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3405,17 +3204,17 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3278,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -3541,47 +3340,43 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Zemoso Technologies</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Private Cloud Domain</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3593,21 +3388,21 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
           <t>2026-05-05</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -3673,19 +3468,19 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner- Technology</t>
+          <t>Technical Product Manager, Private Cloud Domain</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3696,22 +3491,22 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G22" s="2" t="n">
-        <v>48</v>
-      </c>
       <c r="H22" s="2" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword presence (Jira, Agile, SQL, Power BI, GenAI) but missing key CLM-specific terms and location mismatch. The biggest keyword gap is the absence of KYC/regulatory language.</t>
+          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>KYC, Regulatory compliance, Risk management, API design, UAT, Change adoption</t>
+          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3729,29 +3524,29 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Knorr- Bremse Systems for Commercial  Vehicles India Pvt. Ltd. Pune</t>
+          <t>Mindtickle</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Regional Product Manager</t>
+          <t>Technical Product Owner- II (Engineering Manager - DevOps Team)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3760,24 +3555,26 @@
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F23" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains some product management keywords but lacks many JD-specific terms, leading to a modest ATS score and a lower fit due to domain mismatch.</t>
+          <t>The resume meets the 2‑year minimum and seniority rules, but lacks many DevOps/SRE specific terms, lowering the ATS score; the biggest keyword gap is the absence of observability and pipeline tooling experience.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Product roadmap, R&amp;D footprint, Make/Buy analysis, Budget planning, P&amp;L management, Risk management, M&amp;A</t>
+          <t>observability, CI/CD pipelines, cost governance, incident response, SRE, Loki, on‑call rotation, platform security</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -3795,55 +3592,55 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>Hempel A/S</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>IT PRODUCT OWNER - SD BILLING (SAP S/4HANA) - VOIS</t>
+          <t>Finance Product Owner, PtP</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP billing keywords and domain experience, resulting in low ATS and fit scores; the most critical missing keyword is 'SAP SD Billing'.</t>
+          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>SAP SD, S/4HANA, fit‑gap analysis, UAT, intercompany billing, SAP methodology, billing governance</t>
+          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -3861,17 +3658,17 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3726,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -3939,47 +3736,45 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>JK Treel</t>
+          <t>Virtusa</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Entry-Level Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>26</v>
-      </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The candidate exceeds the 0–2 year experience range and lacks automotive/IOT keywords, resulting in low ATS and fit scores; the biggest gap is missing domain-specific terms like TPMS and IoT.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>TPMS, Android Auto, Apple CarPlay, IoT, Bluetooth, OEM interaction, mobile app coordination, product testing, automotive innovation</t>
+          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -3997,7 +3792,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -4007,24 +3802,24 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>EPAM Systems</t>
+          <t>AGDATA, LP</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Finance</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -4033,19 +3828,19 @@
         <v>25</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10-15 years of experience, which exceeds the candidate's 4 years, triggering the hard rule that forces both scores below 30; the resume also lacks key terms like OKRs and finance domain keywords.</t>
+          <t>The JD title includes 'Senior' which triggers hard rule 3, forcing both scores below 30 regardless of experience or keyword match; the resume lacks key senior‑level product ownership language.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>OKRs, Finance domain expertise, Data Science, Event‑based architecture, Snowflake or similar data warehouse</t>
+          <t>OKRs, A/B testing, Snowflake, Data platform roadmap, NPS improvement, Marketplace dynamics, Cross‑functional data team collaboration</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4063,7 +3858,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
@@ -4073,19 +3868,19 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>VP- Custody Tax Product Manager</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -4096,24 +3891,20 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -4129,55 +3920,57 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TransUnion</t>
+          <t>Azuga, Inc.</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, IPI - Global Fraud Solutions</t>
+          <t>Product Manager – Connected Hardware &amp; Telematics (HW / FW / IoT)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bagalur, Karnataka, India</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F29" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of IT experience; the candidate has only 4 years, triggering hard rule 4, so both scores are forced below 30. The biggest keyword gap is the lack of explicit fraud‑related experience.</t>
+          <t>The candidate meets the 3‑year minimum experience, but the resume lacks most hardware/IoT keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of telematics and firmware terminology.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>fraud prevention, Scaled Agile Framework (SAFe), Product Owner certification, financial services, risk analytics</t>
+          <t>OBD‑II, J1939, CAN protocol, OTA firmware upgrade, BLE beacon, LTE Cat M1, FCC certification, telematics vendor management</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -4191,149 +3984,21 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>AGDATA, LP</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>The JD title includes 'Senior' which triggers hard rule 3, forcing both scores below 30 regardless of experience or keyword match; the resume lacks key senior‑level product ownership language.</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, A/B testing, Snowflake, Data platform roadmap, NPS improvement, Marketplace dynamics, Cross‑functional data team collaboration</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Citi</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>VP- Custody Tax Product Manager</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4367,8 +4032,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-09
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rang De</t>
+          <t>Sharpsell.ai</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,26 +581,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and matches the Associate Product Manager title, yielding a strong ATS score; however, the candidate lacks fintech‑specific experience, lowering the fit score, and the JD’s keyword "user research" is missing.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains most JD keywords and tools, yielding a high ATS score, but lacks several specific experimentation and metric terms.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>user research, PMF surveys, design sprint, A/B testing, analytics platform, Excel, NPS improvement, OKRs</t>
+          <t>A/B testing, OKRs, RICE prioritization, Mixpanel, NPS improvement, customer retention metrics</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,29 +616,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,24 +647,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
+          <t>The resume meets the 2-year minimum and aligns with the Product Manager I title, yielding strong ATS keyword coverage; the biggest gap is the lack of specific analytics and growth‑hacking tools mentioned in the JD.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
+          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, NPS improvement, MAU growth, Snowflake, RICE prioritization</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Greenway Health</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,24 +715,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F4" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets all hard rules and contains many JD keywords, yielding a high ATS score; however, the candidate's experience is in SaaS and travel tech rather than healthcare, creating a domain mismatch that lowers the fit score.</t>
+          <t>The resume meets the 3‑year minimum and matches the Bangalore location, so hard rules do not penalize; keyword density is strong with many JD terms present, but a few core analytics tools are missing.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, ambulatory care workflows, EMR/EHR integration, HIPAA compliance, clinical user interface design, patient engagement metrics, digital health market research</t>
+          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, conversion funnel analysis</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -755,24 +757,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Ascendion</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Owner/ Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,22 +785,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement). ATS score is solid due to strong keyword overlap and relevant title, but missing workshop and release‑plan terms. Fit score reflects good SaaS and GenAI experience but limited direct product‑owner domain exposure.</t>
+          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>workshops, release planning, OKRs, product vision, customer interviews</t>
+          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,7 +818,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -826,19 +828,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Greenway Health</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +851,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
+          <t>The resume meets all hard rules and contains many JD keywords, yielding a high ATS score; however, the candidate's experience is in SaaS and travel tech rather than healthcare, creating a domain mismatch that lowers the fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
+          <t>healthcare regulations, ambulatory care workflows, EMR/EHR integration, HIPAA compliance, clinical user interface design, patient engagement metrics, digital health market research</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,7 +884,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -892,45 +894,45 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>Pocket FM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>62</v>
-      </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The resume meets the experience requirement (4 years vs 1-2 years needed) and title alignment, yielding a solid ATS score; the most important keyword gap is the lack of explicit mention of subscription and loyalty program experience.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>Subscription, Loyalty Programs, Pricing strategy, Offers, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,29 +950,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dezerv</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Data</t>
+          <t>Product Manager, Amazon Now</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -984,19 +986,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but lacks finance‑specific tools and frameworks; the biggest gap is finance‑domain terminology.</t>
+          <t>The resume meets the 3+ year requirement and the location, so hard rules pass; it contains many JD keywords (SQL, Agile, stakeholder management) but lacks VBA and explicit cost/benefit analysis terms, leading to a solid ATS score but only moderate overall fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Snowflake, OKRs, RICE prioritization, NPS improvement, MAU growth, two‑sided marketplace</t>
+          <t>VBA, cost/benefit analysis, business case development, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,29 +1016,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Personalization &amp; Data Platforms</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,26 +1047,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H9" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
+          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
+          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1092,19 +1092,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BeBetta</t>
+          <t>Dezerv</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager - Data</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1118,19 +1118,19 @@
         <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and matches the Associate Product Manager title, yielding a solid ATS score, but the candidate's domain (B2B/B2C SaaS, travel and enterprise tools) does not align with BeBetta's gaming focus, lowering the fit score; the biggest keyword gap is the lack of analytics tools like Mixpanel or A/B testing.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but lacks finance‑specific tools and frameworks; the biggest gap is finance‑domain terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, NPS improvement, DAU/MAU growth, gaming industry experience, sports domain knowledge, Google Analytics, Data Studio</t>
+          <t>A/B testing, Mixpanel, Snowflake, OKRs, RICE prioritization, NPS improvement, MAU growth, two‑sided marketplace</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,29 +1148,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Nexus Venture Partners</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Personalization &amp; Data Platforms</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1180,25 +1180,25 @@
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, but lacks fintech-specific experience, lowering the overall fit.</t>
+          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>RBI guidelines, underwriting rules, conversion KPI, CAC, risk management, credit product, A/B testing</t>
+          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1226,24 +1226,24 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Groww</t>
+          <t>Ecolab</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Owner – eQMS</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -1252,19 +1252,19 @@
         <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>69</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the candidate meets the 4‑year experience threshold and title level. ATS score is moderate due to strong keyword overlap but missing fintech‑specific terms. Fit score is good thanks to solid SaaS and GenAI experience, though domain mismatch with fintech lowers it slightly.</t>
+          <t>The resume meets the 4‑year experience requirement and the title level, so hard rules do not penalize the scores; however, key JD terms like Azure DevOps, DevSecOps, and PI Planning are missing, lowering the ATS keyword density. The strongest gap is the lack of explicit Azure DevOps/DevSecOps experience.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Fintech, A/B testing, OKRs, NPS improvement, MAU growth, Marketplace dynamics</t>
+          <t>Azure DevOps, DevSecOps, PI Planning, Definition of Ready, Definition of Done, Agile Release Train, enhancement tracking, bug tracking</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1287,12 +1287,12 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -1358,19 +1358,19 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Opkey</t>
+          <t>BeBetta</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Workday</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1379,9 +1379,7 @@
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
         <v>78</v>
       </c>
@@ -1393,12 +1391,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding a solid ATS score due to many matching keywords, but lacks Workday‑specific terms, lowering the fit score because the candidate's domain experience is not aligned with HR/Workday products.</t>
+          <t>The resume meets the 4‑year experience requirement and matches the Associate Product Manager title, yielding a solid ATS score, but the candidate's domain (B2B/B2C SaaS, travel and enterprise tools) does not align with BeBetta's gaming focus, lowering the fit score; the biggest keyword gap is the lack of analytics tools like Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Workday, HCM, Payroll, Benefits, Integrations, OKRs, RICE prioritization, UAT planning, defect triage</t>
+          <t>Mixpanel, A/B testing, NPS improvement, DAU/MAU growth, gaming industry experience, sports domain knowledge, Google Analytics, Data Studio</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1416,17 +1414,17 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1480,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1492,19 +1490,19 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Bread Financial India</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (m/f/d) for API Management @ BTP Integration Suite</t>
+          <t>Product Owner 2 - Marketing</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1525,12 +1523,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement and passes all hard rules, but lacks several API‑specific keywords and direct API management experience, which lowers the fit score; the biggest keyword gap is the absence of "API Management".</t>
+          <t>The resume meets the 2+ year requirement and title level, so hard rules pass; however, it lacks several JD-specific tools and marketing analytics terms, lowering the ATS score, and the candidate's domain experience (travel tech, FMCG, renewable) only loosely aligns with a marketing product role in financial services.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>API Management, Kubernetes, Machine Learning based anomaly detection, Multi‑cloud (AWS, GCP, Azure), API marketplace, OKRs, RICE prioritization, NPS improvement</t>
+          <t>Adobe Tag Manager, Adobe Experience Platform, digital attribution, analytics platform, tagging</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,29 +1546,29 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>IGEL Technology</t>
+          <t>Zeta</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (m/f/d) - Bangalore</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1579,24 +1577,26 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F17" s="2" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>61</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches no explicit higher minimum). ATS score is moderate due to missing many JD-specific tech keywords, while the fit score reflects decent domain alignment but limited cloud/DaaS experience.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) so hard rules do not penalize; however, the resume only partially matches the banking‑focused keywords and tools, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>DaaS, cloud service architecture, Linux, virtualization, device management, security, UI/UX design, OKRs</t>
+          <t>core banking, cloud-native, OKRs, A/B testing, NPS improvement, Snowflake, marketplace dynamics</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1614,55 +1614,55 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Raphus Solutions</t>
+          <t>66degrees</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and aligns well with the Product Manager title, yielding strong ATS and fit scores; the most important keyword gap is the absence of OKRs/A/B testing terminology.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks many JD-specific keywords such as cloud architecture and build‑vs‑buy analysis, lowering the ATS score; the strongest gap is the missing "cloud" and "architecture" terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Metrics tracking, Roadmap planning, User segmentation</t>
+          <t>cloud architecture, build vs buy analysis, product roadmap planning, OKRs, A/B testing, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1676,33 +1676,33 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>FBS Customer Experience Product Manager</t>
+          <t>Product Owner — General</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1711,24 +1711,26 @@
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F19" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core keywords but misses several JD-specific tools and metrics, leading to a solid but not top ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a good fit score.</t>
+          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Qualtrics, Fullstory, CSAT, FCR, predictive analytics, real-time dashboards, AI-driven insights, KPI monitoring</t>
+          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1751,24 +1753,24 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services</t>
+          <t>Merck Life Science</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-63827</t>
+          <t>Global Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1779,22 +1781,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1812,55 +1814,55 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>FBS Customer Experience Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+          <t>Hard rules are satisfied; the resume contains many core keywords but misses several JD-specific tools and metrics, leading to a solid but not top ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a good fit score.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+          <t>Mixpanel, Qualtrics, Fullstory, CSAT, FCR, predictive analytics, real-time dashboards, AI-driven insights, KPI monitoring</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1874,61 +1876,61 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Omnibound AI</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Martech Product manager</t>
+          <t>Product Owner (Tax)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title level, so hard rules pass; it contains many JD keywords but lacks direct marketing experience, which lowers the fit score.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>marketing automation, ABM, SEO, paid campaigns, digital marketing workflows, KPIs for marketing, US‑based team collaboration, LLMs, co‑pilot technologies</t>
+          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1942,7 +1944,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -1951,78 +1953,410 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EXL</t>
+          <t>Hitachi Digital Services</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Manager-Product Development-Technology/Digital Product Owner</t>
+          <t>Product Manager-63827</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Cornerstone OnDemand</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager | Pune</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Cornerstone OnDemand</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Omnibound AI</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Martech Product manager</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H27" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 2‑year minimum and title level, so hard rules pass; it contains many JD keywords but lacks direct marketing experience, which lowers the fit score.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>marketing automation, ABM, SEO, paid campaigns, digital marketing workflows, KPIs for marketing, US‑based team collaboration, LLMs, co‑pilot technologies</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>EXL</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Manager-Product Development-Technology/Digital Product Owner</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G28" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -2050,6 +2384,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2061,7 +2400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2167,12 +2506,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kapture CX</t>
+          <t>Endava</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager – Applied AI (Voice)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2183,22 +2522,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>58</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title is not senior, so hard rules pass; however the resume lacks key voice AI terms like LLM, STT/TTS, reducing the ATS keyword match.</t>
+          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>LLM, STT, TTS, voice bot, conversation quality, benchmarking, latency, cost optimization</t>
+          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2216,17 +2555,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2621,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -2292,19 +2631,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Nielsen</t>
+          <t>Nexus Point</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Client Facing Product Development)</t>
+          <t>Product Manager - Shopping Experience and Growth (CX)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2315,22 +2654,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="G4" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>49</v>
-      </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and location, but lacks many JD-specific keywords and direct sports‑media domain experience, resulting in a modest ATS score and a moderate job‑fit score.</t>
+          <t>The resume meets the 3+ years requirement and location, but lacks many e‑commerce specific keywords, lowering the ATS score; the biggest gap is the absence of terms like dynamic pricing and checkout optimization.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>customer interviews, surveys, A/B testing, OKRs, RICE prioritization, Mixpanel, Snowflake, NPS improvement, MAU growth</t>
+          <t>dynamic pricing, discount frameworks, A/B testing, GMV growth, conversion rate optimization, personalization, checkout flow, EMI integration, BNPL, marketplace dynamics</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2348,29 +2687,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PW (PhysicsWallah)</t>
+          <t>Snapmint</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-2</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2379,26 +2718,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="G5" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>40</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2‑year minimum). ATS score is low because key JD terms like A/B testing, DAU/MAU, and engagement metrics are missing; fit score is moderate due to domain mismatch despite solid SaaS experience.</t>
+          <t>The candidate meets the 3-5 year experience requirement, so no hard rule penalty; however, the resume lacks many payment-specific keywords, lowering the ATS score. The biggest keyword gap is the absence of any UPI or payments terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, DAU, MAU, engagement metrics, retention, habit formation, growth team collaboration, user behavior analysis</t>
+          <t>UPI, payments ecosystem, PSP integration, NPCI regulations, financial compliance, A/B testing, growth metrics (MAU, retention), OKRs</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2416,7 +2753,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -2426,45 +2763,47 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>Blackhawk Network India</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Acceptance Risk - Product Manager</t>
+          <t>Product Manager (Technology)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of explicit API design/architecture terminology.</t>
+          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks many API‑ and fintech‑specific terms required by the JD, lowering both scores. The biggest keyword gap is the absence of any mention of APIs.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>API specifications, solution architecture, merchant integration, transaction processing, OKRs, A/B testing, Snowflake</t>
+          <t>API, Fintech, Payments, Developer onboarding, Integration documentation, API adoption metrics, Roadmap management, Compliance</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2487,24 +2826,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PHINIA</t>
+          <t>Tata Communications</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Finance Application Product Owner and RPA</t>
+          <t>Product Manager (Deputy General Manager)- SMS</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2515,22 +2854,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is low because key finance and SAP/RPA keywords are missing; the biggest gap is the lack of any SAP or UiPath experience. Fit score reflects domain mismatch but strong GenAI and SaaS background.</t>
+          <t>Hard rules are satisfied; the resume contains many core product keywords but lacks telecom-specific terms, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>UiPath, RPA, SAP S/4HANA, SAP BTP, Finance application, P2P/AP, O2C/AR, Master Data management</t>
+          <t>SMS routing, A2P messaging, CPaaS platform, pricing models, vendor management, telecom regulations, delivery latency optimization</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2548,29 +2887,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Nielsen</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Vice President - Product Manager - Managed Solution</t>
+          <t>Product Manager (Client Facing Product Development)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2581,22 +2920,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of product management experience, which exceeds the candidate's 4 years, triggering hard rule 2; therefore both scores are forced below 30. The resume also lacks key AI/ML governance terms such as MLOps and risk compliance.</t>
+          <t>The resume meets the 4-year experience requirement and location, but lacks many JD-specific keywords and direct sports‑media domain experience, resulting in a modest ATS score and a moderate job‑fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>MLOps, risk management, executive storytelling, OKRs, LLMs</t>
+          <t>customer interviews, surveys, A/B testing, OKRs, RICE prioritization, Mixpanel, Snowflake, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2614,29 +2953,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>PERSOL APAC</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2647,22 +2986,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "Kanban" and "support operations".</t>
+          <t>The resume meets the 4‑year experience requirement and passes all hard rules, but it lacks many JD‑specific keywords and domain experience, resulting in a moderate ATS score and low job‑fit score; the biggest gap is the absence of Adobe Analytics/Marketing Automation terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Kanban, support operations, defect resolution, production support, release planning, test scenarios, application performance monitoring</t>
+          <t>Adobe Analytics, Adobe Campaign Classic, marketing automation, campaign orchestration, mobile push notifications, tagging/data‑collection, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2680,7 +3019,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -2690,19 +3029,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Arctic Wolf</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Product Manager – AI SOC Automation</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2713,22 +3052,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
+          <t>Hard rules pass (4 years experience matches no higher minimum). ATS score is low due to limited overlap with SOC and security‑focused keywords; the biggest gap is missing SOC/AI‑agent terminology. Fit score reflects domain mismatch despite strong GenAI and SaaS experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
+          <t>SOC operations, security operations, AI agent, Mixture-of-Experts, detection engineering, incident response, automation workflow, KPI measurement, MDR service</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2746,53 +3085,57 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Altimate AI</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Acceptance Risk - Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of explicit API design/architecture terminology.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>API specifications, solution architecture, merchant integration, transaction processing, OKRs, A/B testing, Snowflake</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -2808,55 +3151,55 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Ashika Group</t>
+          <t>MKS Inc.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Stock Broking</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no &gt;4 requirement). ATS score is moderate due to decent keyword overlap but missing finance-specific terms and location mismatch; the biggest keyword gap is lack of financial analysis experience.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'pricing strategy'.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Financial analysis, Strategic planning, Product lifecycle management, Presentation skills, Market research, Finance industry experience, Data visualization tools (e.g., Tableau)</t>
+          <t>pricing strategy, market research, competitive analysis, product positioning, key account management, decoratives &amp; plating on plastics</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2870,7 +3213,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -2879,50 +3222,50 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Observability Domain</t>
+          <t>Product Manager - Employee Platforms</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as "risk management" and "compliance".</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
+          <t>risk management, compliance, privacy, OKRs, A/B testing, market research</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2936,59 +3279,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Recykal.com</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI &amp; Innovation</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bangalore Rural, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches the 2-3 year requirement). The resume misses several JD-specific terms like A/B testing and rapid prototyping, lowering the ATS score, while the candidate's GenAI and SaaS experience strongly aligns with the role.</t>
+          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key Salesforce and data‑migration keywords.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, rapid prototyping, low-code/no-code, vibe coding, experiment design</t>
+          <t>Salesforce Apex, Lightning components, Sales Cloud, Data migration, Data quality, Integrations, System architecture, GitHub Copilot</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3002,59 +3345,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Keyloop</t>
+          <t>Teradata</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (IC), Agentic AI</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The JD requires 5+ years of AI/ML product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key AI/ML terms.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
+          <t>LLMs, foundation models, inference pipelines, multi‑modal AI, Snowflake, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3068,7 +3411,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -3077,12 +3420,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -3094,33 +3437,33 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
+          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3134,7 +3477,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -3143,29 +3486,29 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Product Manager - Payments</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -3181,12 +3524,12 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3200,121 +3543,127 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Payments</t>
+          <t>Vice President - Product Manager - Managed Solution</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 10+ years of product management experience, which exceeds the candidate's 4 years, triggering hard rule 2; therefore both scores are forced below 30. The resume also lacks key AI/ML governance terms such as MLOps and risk compliance.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>MLOps, risk management, executive storytelling, OKRs, LLMs</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Ashika Group</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Transformation</t>
+          <t>Product Manager - Stock Broking</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
+          <t>Hard rules pass (4 years experience matches no &gt;4 requirement). ATS score is moderate due to decent keyword overlap but missing finance-specific terms and location mismatch; the biggest keyword gap is lack of financial analysis experience.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Financial analysis, Strategic planning, Product lifecycle management, Presentation skills, Market research, Finance industry experience, Data visualization tools (e.g., Tableau)</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3326,33 +3675,33 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Zemoso Technologies</t>
+          <t>Recykal.com</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - AI &amp; Innovation</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3363,20 +3712,24 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr"/>
+          <t>Hard rules are satisfied (4 years experience matches the 2-3 year requirement). The resume misses several JD-specific terms like A/B testing and rapid prototyping, lowering the ATS score, while the candidate's GenAI and SaaS experience strongly aligns with the role.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, rapid prototyping, low-code/no-code, vibe coding, experiment design</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3392,55 +3745,55 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, LLM/ML Domain</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3454,59 +3807,59 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Keyloop</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Private Cloud Domain</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
+          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3520,61 +3873,59 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Mindtickle</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner- II (Engineering Manager - DevOps Team)</t>
+          <t>Product Manager (Materials Program)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and seniority rules, but lacks many DevOps/SRE specific terms, lowering the ATS score; the biggest keyword gap is the absence of observability and pipeline tooling experience.</t>
+          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>observability, CI/CD pipelines, cost governance, incident response, SRE, Loki, on‑call rotation, platform security</t>
+          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -3588,7 +3939,7 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
@@ -3597,50 +3948,50 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Hempel A/S</t>
+          <t>TALENTMATE</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Finance Product Owner, PtP</t>
+          <t>Product Manager - APAC Onboarding And KYC</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>30</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
+          <t>The candidate meets the 3+ years requirement, but the resume lacks many core KYC/FinTech keywords, lowering both ATS and fit scores; the biggest gap is missing KYC and AML terminology.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
+          <t>KYC, AML compliance, identity verification, fincrime risk mitigation, regulatory requirements, FinTech, customer onboarding metrics</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -3654,7 +4005,7 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -3663,52 +4014,50 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Mindtickle</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner - II (Devops)</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum but lacks DevOps/SRE keywords and location alignment, resulting in a low ATS match; the biggest gap is missing core DevOps terminology.</t>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>DevOps, SRE, CI/CD pipelines, observability, Loki, cost governance, incident response, on-call rotation, automation, platform security</t>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -3722,7 +4071,7 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
@@ -3731,52 +4080,48 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>Zemoso Technologies</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3788,59 +4133,59 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>AGDATA, LP</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The JD title includes 'Senior' which triggers hard rule 3, forcing both scores below 30 regardless of experience or keyword match; the resume lacks key senior‑level product ownership language.</t>
+          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Snowflake, Data platform roadmap, NPS improvement, Marketplace dynamics, Cross‑functional data team collaboration</t>
+          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -3858,53 +4203,59 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Mindtickle</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>VP- Custody Tax Product Manager</t>
+          <t>Technical Product Owner- II (Engineering Manager - DevOps Team)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr"/>
+          <t>The resume meets the 2‑year minimum and seniority rules, but lacks many DevOps/SRE specific terms, lowering the ATS score; the biggest keyword gap is the absence of observability and pipeline tooling experience.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>observability, CI/CD pipelines, cost governance, incident response, SRE, Loki, on‑call rotation, platform security</t>
+        </is>
+      </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3920,57 +4271,55 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Azuga, Inc.</t>
+          <t>bp</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – Connected Hardware &amp; Telematics (HW / FW / IoT)</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Bagalur, Karnataka, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum experience, but the resume lacks most hardware/IoT keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of telematics and firmware terminology.</t>
+          <t>The resume meets the 4‑year experience requirement, so hard rules do not penalize the scores; however, key developer‑platform keywords and location match are missing, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate fit.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>OBD‑II, J1939, CAN protocol, OTA firmware upgrade, BLE beacon, LTE Cat M1, FCC certification, telematics vendor management</t>
+          <t>API design, SDK development, Developer Experience (DX), Observability, DevOps/SRE, Technical documentation, Service contracts</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -3984,21 +4333,419 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Citi</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Payments Product Owner - Direct Debit- Vice President</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied, but the candidate's associate-level title and lack of payment-specific experience reduce both scores; the biggest keyword gap is the absence of payment scheme terms like Direct Debit, NACH, and UPI AutoPay.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Direct Debit, NACH, UPI AutoPay, SEPA, payment scheme regulatory analysis, mandate management, compliance, payment product roadmap</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Hempel A/S</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Finance Product Owner, PtP</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Mindtickle</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Owner - II (Devops)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 2‑year minimum but lacks DevOps/SRE keywords and location alignment, resulting in a low ATS match; the biggest gap is missing core DevOps terminology.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>DevOps, SRE, CI/CD pipelines, observability, Loki, cost governance, incident response, on-call rotation, automation, platform security</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>GlobalLogic</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Owner IRC291187</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Hard rule triggered: candidate has only 4 years experience while JD requires 6-8 years, so both scores are forced below 30; the resume also lacks key data platform terms.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Data Lake, ETL, Data Warehouse, Snowflake, BI tool (Tableau), Data governance, metadata standards, API integration, advanced analytics</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Virtusa</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TransUnion</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner, IPI - Global Fraud Solutions</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 7+ years of IT experience; the candidate has only 4 years, triggering hard rule 4, so both scores are forced below 30. The biggest keyword gap is the lack of explicit fraud‑related experience.</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>fraud prevention, Scaled Agile Framework (SAFe), Product Owner certification, financial services, risk analytics</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -4032,6 +4779,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-10
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -648,25 +648,25 @@
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>85</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-year minimum and aligns with the Product Manager I title, yielding strong ATS keyword coverage; the biggest gap is the lack of specific analytics and growth‑hacking tools mentioned in the JD.</t>
+          <t>The resume meets the 3‑year minimum and matches the Bangalore location, so hard rules do not penalize; keyword density is strong with many JD terms present, but a few core analytics tools are missing.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, NPS improvement, MAU growth, Snowflake, RICE prioritization</t>
+          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, conversion funnel analysis</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -694,19 +694,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>Greenway Health</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,26 +715,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and matches the Bangalore location, so hard rules do not penalize; keyword density is strong with many JD terms present, but a few core analytics tools are missing.</t>
+          <t>The resume meets all hard rules and contains many JD keywords, yielding a high ATS score; however, the candidate's experience is in SaaS and travel tech rather than healthcare, creating a domain mismatch that lowers the fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, conversion funnel analysis</t>
+          <t>healthcare regulations, ambulatory care workflows, EMR/EHR integration, HIPAA compliance, clinical user interface design, patient engagement metrics, digital health market research</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -788,19 +786,19 @@
         <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
+          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
+          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,24 +816,24 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Greenway Health</t>
+          <t>Pocket FM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -851,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets all hard rules and contains many JD keywords, yielding a high ATS score; however, the candidate's experience is in SaaS and travel tech rather than healthcare, creating a domain mismatch that lowers the fit score.</t>
+          <t>The resume meets the experience requirement (4 years vs 1-2 years needed) and title alignment, yielding a solid ATS score; the most important keyword gap is the lack of explicit mention of subscription and loyalty program experience.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, ambulatory care workflows, EMR/EHR integration, HIPAA compliance, clinical user interface design, patient engagement metrics, digital health market research</t>
+          <t>Subscription, Loyalty Programs, Pricing strategy, Offers, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -884,29 +882,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Pocket FM</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -917,22 +915,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years vs 1-2 years needed) and title alignment, yielding a solid ATS score; the most important keyword gap is the lack of explicit mention of subscription and loyalty program experience.</t>
+          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Subscription, Loyalty Programs, Pricing strategy, Offers, A/B testing, OKRs, NPS improvement</t>
+          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,29 +948,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Simplilearn</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Now</t>
+          <t>Product Manager (Growth)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -986,19 +984,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ year requirement and the location, so hard rules pass; it contains many JD keywords (SQL, Agile, stakeholder management) but lacks VBA and explicit cost/benefit analysis terms, leading to a solid ATS score but only moderate overall fit due to domain mismatch.</t>
+          <t>The resume meets the experience requirement and title level, yielding a solid ATS score due to strong keyword overlap, but the candidate's domain (enterprise SaaS, travel tech) only partially aligns with the growth-focused education platform role, lowering the fit score; the biggest keyword gap is the lack of explicit Go-To-Market experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>VBA, cost/benefit analysis, business case development, OKRs, A/B testing, NPS improvement</t>
+          <t>Go-To-Market strategy, market research, NPS, CSAT, A/B testing, OKRs, pricing optimization, content management, sales enablement, user segmentation</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1016,29 +1014,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Personalization &amp; Data Platforms</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1047,24 +1045,26 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
+          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
+          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1092,19 +1092,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dezerv</t>
+          <t>Auric AI Labs</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Data</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1118,19 +1118,19 @@
         <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but lacks finance‑specific tools and frameworks; the biggest gap is finance‑domain terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with AI‑vision defense, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Snowflake, OKRs, RICE prioritization, NPS improvement, MAU growth, two‑sided marketplace</t>
+          <t>AI-powered vision, image ingestion, quality review, MVP definition, roadmap planning, OKRs, RICE prioritization, A/B testing, analyst journey mapping</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,29 +1148,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>BeBetta</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Personalization &amp; Data Platforms</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1179,26 +1179,24 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
+          <t>The resume meets the 4‑year experience requirement and matches the Associate Product Manager title, yielding a solid ATS score, but the candidate's domain (B2B/B2C SaaS, travel and enterprise tools) does not align with BeBetta's gaming focus, lowering the fit score; the biggest keyword gap is the lack of analytics tools like Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
+          <t>Mixpanel, A/B testing, NPS improvement, DAU/MAU growth, gaming industry experience, sports domain knowledge, Google Analytics, Data Studio</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1226,45 +1224,45 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Ecolab</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner – eQMS</t>
+          <t>Product Manager AI</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>69</v>
-      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title level, so hard rules do not penalize the scores; however, key JD terms like Azure DevOps, DevSecOps, and PI Planning are missing, lowering the ATS keyword density. The strongest gap is the lack of explicit Azure DevOps/DevSecOps experience.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps, DevSecOps, PI Planning, Definition of Ready, Definition of Done, Agile Release Train, enhancement tracking, bug tracking</t>
+          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1282,55 +1280,55 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Infineon Technologies</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Manager - Product Owner</t>
+          <t>Product Manager, Amazon Business India</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G13" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H13" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's SaaS/GenAI focus does not align well with the hardware web product domain, lowering the fit score.</t>
+          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CX reports, roadmap planning, backlog grooming, Evaluation Board Finder</t>
+          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,29 +1346,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BeBetta</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager -Growth</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1381,22 +1379,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and matches the Associate Product Manager title, yielding a solid ATS score, but the candidate's domain (B2B/B2C SaaS, travel and enterprise tools) does not align with BeBetta's gaming focus, lowering the fit score; the biggest keyword gap is the lack of analytics tools like Mixpanel or A/B testing.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, stakeholder management, SaaS, data‑driven) but lacks growth‑specific terms, lowering the ATS score. The biggest keyword gap is the absence of explicit growth‑experiment language such as "A/B testing".</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, NPS improvement, DAU/MAU growth, gaming industry experience, sports domain knowledge, Google Analytics, Data Studio</t>
+          <t>A/B testing, Mixpanel, Snowflake, OKRs, Referral program, Loyalty program, Personalized notifications, Cohort analysis</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1419,24 +1417,24 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Finkraft</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Business India</t>
+          <t>Product Manager — Travel &amp; Hospitality Tech</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1445,24 +1443,26 @@
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F15" s="2" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however the resume lacks several JD‑specific terms (e.g., GST, PMS, GDS, OTA, ecosystem mapping), lowering the ATS keyword density.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
+          <t>GST invoicing, PMS (Property Management System), GDS, OTA, TMC, Concur integration, ecosystem mapping</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1480,34 +1480,34 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Bread Financial India</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner 2 - Marketing</t>
+          <t>Product Manager II, Policy &amp; Governance (Hybrid, Bangalore)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1523,12 +1523,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and title level, so hard rules pass; however, it lacks several JD-specific tools and marketing analytics terms, lowering the ATS score, and the candidate's domain experience (travel tech, FMCG, renewable) only loosely aligns with a marketing product role in financial services.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks core policy/governance terms, lowering the ATS score; the candidate's domain is SaaS and GenAI rather than enterprise governance, creating the biggest fit gap.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Adobe Tag Manager, Adobe Experience Platform, digital attribution, analytics platform, tagging</t>
+          <t>policy enforcement, governance, GDPR, CCPA, legal compliance, security, pricing strategy, monetization</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1546,29 +1546,29 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Zeta</t>
+          <t>Bread Financial India</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Owner 2 - Marketing</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1577,26 +1577,24 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) so hard rules do not penalize; however, the resume only partially matches the banking‑focused keywords and tools, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>The resume meets the 2+ year requirement and title level, so hard rules pass; however, it lacks several JD-specific tools and marketing analytics terms, lowering the ATS score, and the candidate's domain experience (travel tech, FMCG, renewable) only loosely aligns with a marketing product role in financial services.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>core banking, cloud-native, OKRs, A/B testing, NPS improvement, Snowflake, marketplace dynamics</t>
+          <t>Adobe Tag Manager, Adobe Experience Platform, digital attribution, analytics platform, tagging</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1614,7 +1612,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -1624,19 +1622,19 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>66degrees</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Data Product Manager - Marketplace</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1645,24 +1643,26 @@
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>70</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks many JD-specific keywords such as cloud architecture and build‑vs‑buy analysis, lowering the ATS score; the strongest gap is the missing "cloud" and "architecture" terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and the title does not violate seniority rules, but the resume lacks many JD‑specific keywords such as API gateway and real‑time governance, resulting in a moderate ATS score; however, strong travel‑tech and GenAI experience make the candidate a good domain fit.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>cloud architecture, build vs buy analysis, product roadmap planning, OKRs, A/B testing, Snowflake, NPS improvement</t>
+          <t>API gateway, real-time data processing, governed data, traveller profile, personalization, Marketplace dynamics, A/B testing</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1680,57 +1680,57 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Zeta</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Owner — General</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) so hard rules do not penalize; however, the resume only partially matches the banking‑focused keywords and tools, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
+          <t>core banking, cloud-native, OKRs, A/B testing, NPS improvement, Snowflake, marketplace dynamics</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1744,11 +1744,11 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -1758,19 +1758,19 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Merck Life Science</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Global Product Manager</t>
+          <t>Product Owner — General</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1779,24 +1779,26 @@
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F20" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
+          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
+          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1814,7 +1816,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -1824,19 +1826,19 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>Merck Life Science</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>FBS Customer Experience Product Manager</t>
+          <t>Global Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1850,19 +1852,19 @@
         <v>68</v>
       </c>
       <c r="G21" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H21" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core keywords but misses several JD-specific tools and metrics, leading to a solid but not top ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a good fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Qualtrics, Fullstory, CSAT, FCR, predictive analytics, real-time dashboards, AI-driven insights, KPI monitoring</t>
+          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1880,29 +1882,29 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Capgemini</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (Tax)</t>
+          <t>FBS Customer Experience Product Manager</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1911,26 +1913,24 @@
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many core keywords but misses several JD-specific tools and metrics, leading to a solid but not top ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a good fit score.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
+          <t>Mixpanel, Qualtrics, Fullstory, CSAT, FCR, predictive analytics, real-time dashboards, AI-driven insights, KPI monitoring</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1948,29 +1948,29 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-63827</t>
+          <t>Product Owner (Tax)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1979,24 +1979,26 @@
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F23" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2014,17 +2016,17 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2082,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2090,7 +2092,7 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2148,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -2156,7 +2158,7 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2214,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -2222,7 +2224,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -2290,73 +2292,7 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>EXL</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Manager-Product Development-Technology/Digital Product Owner</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H28" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2324,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2400,7 +2335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2555,7 +2490,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -2565,19 +2500,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Motorola Solutions</t>
+          <t>Finkraft</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Planview - Technical Product Owner</t>
+          <t>Product Manager — GST &amp; Tax Tech</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2588,22 +2523,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H3" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume matches many general product management keywords but lacks several JD‑specific tools and processes, lowering the ATS score; the strongest gap is the absence of Planview/Projectplace/Agileplace terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to limited GST/tax keyword overlap; the biggest gap is missing GST-specific terms. Fit score reflects decent SaaS and GenAI experience but weak domain alignment with GST/Tax tech.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Planview, Projectplace, Agileplace, ERP integration, CRM integration, SIT/UAT planning, Cutover planning, functional documentation, automation use cases, dashboard creation</t>
+          <t>GST reconciliation, ITC matching, e-invoicing, API integration, knowledge base, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2621,29 +2556,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Nexus Point</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Shopping Experience and Growth (CX)</t>
+          <t>Product Manager , Amazon Now</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2654,22 +2589,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ years requirement and location, but lacks many e‑commerce specific keywords, lowering the ATS score; the biggest gap is the absence of terms like dynamic pricing and checkout optimization.</t>
+          <t>The candidate meets the 3+ years requirement and location, but the resume lacks several JD-specific keywords, lowering the ATS score; the biggest gap is missing terms like VBA and cost/benefit analysis.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>dynamic pricing, discount frameworks, A/B testing, GMV growth, conversion rate optimization, personalization, checkout flow, EMI integration, BNPL, marketplace dynamics</t>
+          <t>VBA, cost/benefit analysis, business case development, global launch, scalable processes, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2687,29 +2622,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Snapmint</t>
+          <t>Tata Communications</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Deputy General Manager)- SMS</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2720,22 +2655,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3-5 year experience requirement, so no hard rule penalty; however, the resume lacks many payment-specific keywords, lowering the ATS score. The biggest keyword gap is the absence of any UPI or payments terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many core product keywords but lacks telecom-specific terms, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>UPI, payments ecosystem, PSP integration, NPCI regulations, financial compliance, A/B testing, growth metrics (MAU, retention), OKRs</t>
+          <t>SMS routing, A2P messaging, CPaaS platform, pricing models, vendor management, telecom regulations, delivery latency optimization</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2753,29 +2688,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Blackhawk Network India</t>
+          <t>First Advantage</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Technology)</t>
+          <t>Product Owner, Data Analytics- Remote</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2784,26 +2719,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks many API‑ and fintech‑specific terms required by the JD, lowering both scores. The biggest keyword gap is the absence of any mention of APIs.</t>
+          <t>The resume meets the 4-year experience requirement and location, so hard rules do not penalize; however, keyword density for data‑analytics specific terms is moderate, leading to a modest ATS score, while the candidate's SaaS and GenAI background gives a decent fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>API, Fintech, Payments, Developer onboarding, Integration documentation, API adoption metrics, Roadmap management, Compliance</t>
+          <t>Snowflake, Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2826,24 +2759,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tata Communications</t>
+          <t>Greenway Health</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Deputy General Manager)- SMS</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2854,22 +2787,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H7" s="2" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product keywords but lacks telecom-specific terms, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is low due to missing key workflow and automation terms, while fit score reflects good SaaS and GenAI experience but limited healthcare domain relevance.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>SMS routing, A2P messaging, CPaaS platform, pricing models, vendor management, telecom regulations, delivery latency optimization</t>
+          <t>workflow automation, API integration, roadmap definition, backlog management, UAT, success metrics</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2887,55 +2820,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Nielsen</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Client Facing Product Development)</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>49</v>
-      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and location, but lacks many JD-specific keywords and direct sports‑media domain experience, resulting in a modest ATS score and a moderate job‑fit score.</t>
+          <t>The resume contains many generic product management keywords but lacks the specific PKI, certificate lifecycle, and cybersecurity terms required by the JD, resulting in a modest ATS score; domain mismatch drives a low fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>customer interviews, surveys, A/B testing, OKRs, RICE prioritization, Mixpanel, Snowflake, NPS improvement, MAU growth</t>
+          <t>PKI, certificate lifecycle, SCEP/EST APIs, TPM integration, cybersecurity, secure SDLC, regulatory compliance, PKIaaS, device identity</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2953,55 +2886,55 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PERSOL APAC</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Product Manager - Roundel (Ad Tech)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and passes all hard rules, but it lacks many JD‑specific keywords and domain experience, resulting in a moderate ATS score and low job‑fit score; the biggest gap is the absence of Adobe Analytics/Marketing Automation terminology.</t>
+          <t>The resume meets the 4‑year experience requirement, but it lacks many ad‑tech specific keywords and domain experience, resulting in a modest ATS score and a lower job‑fit score; the biggest gap is missing ad‑serving and observability terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Adobe Analytics, Adobe Campaign Classic, marketing automation, campaign orchestration, mobile push notifications, tagging/data‑collection, NPS improvement</t>
+          <t>ad serving, event tracking, observability, low‑latency, billing, anomaly detection</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -3019,29 +2952,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Arctic Wolf</t>
+          <t>Unified GlobalTech (I) Pvt Ltd</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI SOC Automation</t>
+          <t>Product Manager- Interconnect</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3052,22 +2985,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no higher minimum). ATS score is low due to limited overlap with SOC and security‑focused keywords; the biggest gap is missing SOC/AI‑agent terminology. Fit score reflects domain mismatch despite strong GenAI and SaaS experience.</t>
+          <t>Hard rules pass (4 years experience, no &gt;4 year requirement). ATS score is low because the resume contains few of the sales‑ and OEM‑focused keywords from the JD. The biggest keyword gap is the lack of OEM/quote/inventory management terms.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SOC operations, security operations, AI agent, Mixture-of-Experts, detection engineering, incident response, automation workflow, KPI measurement, MDR service</t>
+          <t>OEM relationship management, quote management, inventory management, GP% improvement, field application engineer training, sales enablement, industrial components, margin handling</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3090,50 +3023,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>MKS Inc.</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Acceptance Risk - Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of explicit API design/architecture terminology.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'pricing strategy'.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>API specifications, solution architecture, merchant integration, transaction processing, OKRs, A/B testing, Snowflake</t>
+          <t>pricing strategy, market research, competitive analysis, product positioning, key account management, decoratives &amp; plating on plastics</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3151,34 +3084,34 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MKS Inc.</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Employee Platforms</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -3194,12 +3127,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'pricing strategy'.</t>
+          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as "risk management" and "compliance".</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, market research, competitive analysis, product positioning, key account management, decoratives &amp; plating on plastics</t>
+          <t>risk management, compliance, privacy, OKRs, A/B testing, market research</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3217,7 +3150,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -3227,24 +3160,24 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Employee Platforms</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Rural, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -3253,19 +3186,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as "risk management" and "compliance".</t>
+          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key Salesforce and data‑migration keywords.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>risk management, compliance, privacy, OKRs, A/B testing, market research</t>
+          <t>Salesforce Apex, Lightning components, Sales Cloud, Data migration, Data quality, Integrations, System architecture, GitHub Copilot</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3283,7 +3216,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -3293,24 +3226,24 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Rural, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -3326,12 +3259,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key Salesforce and data‑migration keywords.</t>
+          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Salesforce Apex, Lightning components, Sales Cloud, Data migration, Data quality, Integrations, System architecture, GitHub Copilot</t>
+          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3349,7 +3282,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -3359,7 +3292,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3348,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -3425,24 +3358,24 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Virtusa</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Vice President</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -3458,12 +3391,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
+          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3481,55 +3414,55 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Ashika Group</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Product Manager - Stock Broking</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Kolkata, West Bengal, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
+          <t>Hard rules pass (4 years experience matches no &gt;4 requirement). ATS score is moderate due to decent keyword overlap but missing finance-specific terms and location mismatch; the biggest keyword gap is lack of financial analysis experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
+          <t>Financial analysis, Strategic planning, Product lifecycle management, Presentation skills, Market research, Finance industry experience, Data visualization tools (e.g., Tableau)</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3543,59 +3476,59 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Keyloop</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Vice President - Product Manager - Managed Solution</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of product management experience, which exceeds the candidate's 4 years, triggering hard rule 2; therefore both scores are forced below 30. The resume also lacks key AI/ML governance terms such as MLOps and risk compliance.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>MLOps, risk management, executive storytelling, OKRs, LLMs</t>
+          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3609,59 +3542,59 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Ashika Group</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Stock Broking</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>45</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no &gt;4 requirement). ATS score is moderate due to decent keyword overlap but missing finance-specific terms and location mismatch; the biggest keyword gap is lack of financial analysis experience.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Financial analysis, Strategic planning, Product lifecycle management, Presentation skills, Market research, Finance industry experience, Data visualization tools (e.g., Tableau)</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3675,33 +3608,33 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Recykal.com</t>
+          <t>Sanofi</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - AI &amp; Innovation</t>
+          <t>Digital R&amp;D Lab Equipment Automation Jr. Product Owner</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3712,22 +3645,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G20" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G20" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H20" s="2" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches the 2-3 year requirement). The resume misses several JD-specific terms like A/B testing and rapid prototyping, lowering the ATS score, while the candidate's GenAI and SaaS experience strongly aligns with the role.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on Agile, Jira, SQL, GenAI but missing many lab‑specific terms; fit score is lower because the candidate's SaaS/GenAI background does not align closely with R&amp;D lab equipment automation.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, rapid prototyping, low-code/no-code, vibe coding, experiment design</t>
+          <t>lab automation, R&amp;D workflow orchestration, instrument integration, data capture for AI research, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3745,17 +3678,17 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3700,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Reference Standards)</t>
+          <t>Product Manager (Materials Program)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3778,22 +3711,22 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>45</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
+          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
+          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3811,7 +3744,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -3821,19 +3754,19 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Keyloop</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3844,22 +3777,22 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3887,19 +3820,19 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>Zemoso Technologies</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Materials Program)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3910,24 +3843,20 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3943,55 +3872,57 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TALENTMATE</t>
+          <t>Mindtickle</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - APAC Onboarding And KYC</t>
+          <t>Technical Product Owner- II (Engineering Manager - DevOps Team)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F24" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G24" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>30</v>
-      </c>
       <c r="H24" s="2" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement, but the resume lacks many core KYC/FinTech keywords, lowering both ATS and fit scores; the biggest gap is missing KYC and AML terminology.</t>
+          <t>The resume meets the 2‑year minimum and seniority rules, but lacks many DevOps/SRE specific terms, lowering the ATS score; the biggest keyword gap is the absence of observability and pipeline tooling experience.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>KYC, AML compliance, identity verification, fincrime risk mitigation, regulatory requirements, FinTech, customer onboarding metrics</t>
+          <t>observability, CI/CD pipelines, cost governance, incident response, SRE, Loki, on‑call rotation, platform security</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -4005,59 +3936,59 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Xplor Technologies</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Product Owner, Billing &amp; Settlement</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -4071,57 +4002,61 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Zemoso Technologies</t>
+          <t>bp</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
+          <t>The resume meets the 4‑year experience requirement, so hard rules do not penalize the scores; however, key developer‑platform keywords and location match are missing, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate fit.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>API design, SDK development, Developer Experience (DX), Observability, DevOps/SRE, Technical documentation, Service contracts</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -4133,33 +4068,33 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Payments Product Owner - Direct Debit- Vice President</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -4170,22 +4105,22 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
+          <t>Hard rules are satisfied, but the candidate's associate-level title and lack of payment-specific experience reduce both scores; the biggest keyword gap is the absence of payment scheme terms like Direct Debit, NACH, and UPI AutoPay.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
+          <t>Direct Debit, NACH, UPI AutoPay, SEPA, payment scheme regulatory analysis, mandate management, compliance, payment product roadmap</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4203,7 +4138,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
@@ -4213,47 +4148,45 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Mindtickle</t>
+          <t>Nasdaq</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner- II (Engineering Manager - DevOps Team)</t>
+          <t>Product Manager Specialist</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and seniority rules, but lacks many DevOps/SRE specific terms, lowering the ATS score; the biggest keyword gap is the absence of observability and pipeline tooling experience.</t>
+          <t>The resume meets the 4-year experience requirement, but lacks many domain-specific keywords and regulatory expertise required for the Nasdaq role, resulting in low ATS and fit scores; the biggest gap is the absence of regulatory reporting and Chartered Accountant credentials.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>observability, CI/CD pipelines, cost governance, incident response, SRE, Loki, on‑call rotation, platform security</t>
+          <t>Chartered Accountant, Regulatory reporting, Basel, Financial statements, Functional Specification Document, ControllerView, AxiomSL, Banking products, APAC regulatory frameworks</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -4271,55 +4204,55 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>bp</t>
+          <t>Hempel A/S</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Finance Product Owner, PtP</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, so hard rules do not penalize the scores; however, key developer‑platform keywords and location match are missing, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate fit.</t>
+          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>API design, SDK development, Developer Experience (DX), Observability, DevOps/SRE, Technical documentation, Service contracts</t>
+          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -4337,29 +4270,29 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Sibros</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Payments Product Owner - Direct Debit- Vice President</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -4370,22 +4303,22 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="3" t="inlineStr"/>
       <c r="F30" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the candidate's associate-level title and lack of payment-specific experience reduce both scores; the biggest keyword gap is the absence of payment scheme terms like Direct Debit, NACH, and UPI AutoPay.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Direct Debit, NACH, UPI AutoPay, SEPA, payment scheme regulatory analysis, mandate management, compliance, payment product roadmap</t>
+          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -4408,24 +4341,24 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Hempel A/S</t>
+          <t>GlobalLogic</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Finance Product Owner, PtP</t>
+          <t>Technical Product Owner IRC291187</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -4436,22 +4369,22 @@
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="2" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
+          <t>Hard rule triggered: candidate has only 4 years experience while JD requires 6-8 years, so both scores are forced below 30; the resume also lacks key data platform terms.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
+          <t>Data Lake, ETL, Data Warehouse, Snowflake, BI tool (Tableau), Data governance, metadata standards, API integration, advanced analytics</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -4474,278 +4407,12 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Mindtickle</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Owner - II (Devops)</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 2‑year minimum but lacks DevOps/SRE keywords and location alignment, resulting in a low ATS match; the biggest gap is missing core DevOps terminology.</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>DevOps, SRE, CI/CD pipelines, observability, Loki, cost governance, incident response, on-call rotation, automation, platform security</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>GlobalLogic</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Owner IRC291187</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G33" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H33" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>Hard rule triggered: candidate has only 4 years experience while JD requires 6-8 years, so both scores are forced below 30; the resume also lacks key data platform terms.</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Data Lake, ETL, Data Warehouse, Snowflake, BI tool (Tableau), Data governance, metadata standards, API integration, advanced analytics</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Virtusa</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H34" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>TransUnion</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner, IPI - Global Fraud Solutions</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G35" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H35" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 7+ years of IT experience; the candidate has only 4 years, triggering hard rule 4, so both scores are forced below 30. The biggest keyword gap is the lack of explicit fraud‑related experience.</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>fraud prevention, Scaled Agile Framework (SAFe), Product Owner certification, financial services, risk analytics</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L35" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P35" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -4781,10 +4448,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-11
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Momentum</t>
+          <t>Libra AI</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,26 +647,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and matches the Bangalore location, so hard rules do not penalize; keyword density is strong with many JD terms present, but a few core analytics tools are missing.</t>
+          <t>The resume meets the 1‑2 year experience requirement and matches the associate product manager title, yielding a strong ATS score; the most notable keyword gap is the lack of explicit mention of pixel‑perfect UI/UX and user interview experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, conversion funnel analysis</t>
+          <t>pixel-perfect UI/UX, user interviews, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Greenway Health</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,22 +715,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets all hard rules and contains many JD keywords, yielding a high ATS score; however, the candidate's experience is in SaaS and travel tech rather than healthcare, creating a domain mismatch that lowers the fit score.</t>
+          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, ambulatory care workflows, EMR/EHR integration, HIPAA compliance, clinical user interface design, patient engagement metrics, digital health market research</t>
+          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +748,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -793,12 +791,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules with 4 years experience and appropriate seniority; it contains many JD keywords but lacks e‑commerce marketplace specifics, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; it contains many JD keywords but lacks ecommerce‑specific terms, lowering the fit.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Jobs-to-be-Done, Marketplace dynamics, Two-sided platform, NPS improvement, MAU growth</t>
+          <t>ecommerce, API documentation, A/B testing, OKRs, NPS improvement, data pipeline, SQL reporting</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +814,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pocket FM</t>
+          <t>Simplilearn</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager (Growth)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +847,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years vs 1-2 years needed) and title alignment, yielding a solid ATS score; the most important keyword gap is the lack of explicit mention of subscription and loyalty program experience.</t>
+          <t>The resume meets the experience requirement and title level, yielding a solid ATS score due to strong keyword overlap, but the candidate's domain (enterprise SaaS, travel tech) only partially aligns with the growth-focused education platform role, lowering the fit score; the biggest keyword gap is the lack of explicit Go-To-Market experience.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Subscription, Loyalty Programs, Pricing strategy, Offers, A/B testing, OKRs, NPS improvement</t>
+          <t>Go-To-Market strategy, market research, NPS, CSAT, A/B testing, OKRs, pricing optimization, content management, sales enablement, user segmentation</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -887,50 +885,50 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Candescent</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>SW product Manager III</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). It scores well on ATS keywords and title alignment but lacks several banking‑specific terms, lowering the fit.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
+          <t>release planning, product roadmap, backlog grooming, digital banking, cloud‑based solutions, NPS improvement, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,29 +946,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Simplilearn</t>
+          <t>Auric AI Labs</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Growth)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -984,19 +982,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement and title level, yielding a solid ATS score due to strong keyword overlap, but the candidate's domain (enterprise SaaS, travel tech) only partially aligns with the growth-focused education platform role, lowering the fit score; the biggest keyword gap is the lack of explicit Go-To-Market experience.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with AI‑vision defense, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Go-To-Market strategy, market research, NPS, CSAT, A/B testing, OKRs, pricing optimization, content management, sales enablement, user segmentation</t>
+          <t>AI-powered vision, image ingestion, quality review, MVP definition, roadmap planning, OKRs, RICE prioritization, A/B testing, analyst journey mapping</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,29 +1012,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Personalization &amp; Data Platforms</t>
+          <t>Product Manager AI</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,26 +1043,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
+          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,29 +1078,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Auric AI Labs</t>
+          <t>Finkraft</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager — Travel &amp; Hospitality Tech</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1113,24 +1109,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;4 year requirement) and contains many JD keywords, but the candidate's domain (GenAI SaaS and travel tech) only loosely aligns with AI‑vision defense, creating a moderate fit gap.</t>
+          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however the resume lacks several JD‑specific terms (e.g., GST, PMS, GDS, OTA, ecosystem mapping), lowering the ATS keyword density.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>AI-powered vision, image ingestion, quality review, MVP definition, roadmap planning, OKRs, RICE prioritization, A/B testing, analyst journey mapping</t>
+          <t>GST invoicing, PMS (Property Management System), GDS, OTA, TMC, Concur integration, ecosystem mapping</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,7 +1146,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1158,19 +1156,19 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BeBetta</t>
+          <t>Bread Financial India</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner 2 - Marketing</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1181,22 +1179,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and matches the Associate Product Manager title, yielding a solid ATS score, but the candidate's domain (B2B/B2C SaaS, travel and enterprise tools) does not align with BeBetta's gaming focus, lowering the fit score; the biggest keyword gap is the lack of analytics tools like Mixpanel or A/B testing.</t>
+          <t>The resume meets the 2+ year requirement and title level, so hard rules pass; however, it lacks several JD-specific tools and marketing analytics terms, lowering the ATS score, and the candidate's domain experience (travel tech, FMCG, renewable) only loosely aligns with a marketing product role in financial services.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, NPS improvement, DAU/MAU growth, gaming industry experience, sports domain knowledge, Google Analytics, Data Studio</t>
+          <t>Adobe Tag Manager, Adobe Experience Platform, digital attribution, analytics platform, tagging</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,29 +1212,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager AI</t>
+          <t>Data Product Manager - Marketplace</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1245,24 +1243,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and the title does not violate seniority rules, but the resume lacks many JD‑specific keywords such as API gateway and real‑time governance, resulting in a moderate ATS score; however, strong travel‑tech and GenAI experience make the candidate a good domain fit.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
+          <t>API gateway, real-time data processing, governed data, traveller profile, personalization, Marketplace dynamics, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1290,45 +1290,47 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Business India</t>
+          <t>Product Owner — General</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="G13" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H13" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
+          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
+          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1342,59 +1344,61 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Growth</t>
+          <t>Product Owner, B2B Experience</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, stakeholder management, SaaS, data‑driven) but lacks growth‑specific terms, lowering the ATS score. The biggest keyword gap is the absence of explicit growth‑experiment language such as "A/B testing".</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; the main gap is lack of fintech‑specific terminology.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Snowflake, OKRs, Referral program, Loyalty program, Personalized notifications, Cohort analysis</t>
+          <t>Fintech, Electronic Bill Presentment and Payment (EBPP), AutoPay, paperless adoption, billing process management, AI-driven workflows, self‑serve capabilities, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1408,61 +1412,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Finkraft</t>
+          <t>ICIMS</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager — Travel &amp; Hospitality Tech</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and title level, so hard rules do not penalize the scores; however the resume lacks several JD‑specific terms (e.g., GST, PMS, GDS, OTA, ecosystem mapping), lowering the ATS keyword density.</t>
+          <t>The resume meets the hard rules and contains many JD keywords, but lacks several product‑launch and measurement terms; the biggest gap is missing explicit release‑management/GTM experience.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>GST invoicing, PMS (Property Management System), GDS, OTA, TMC, Concur integration, ecosystem mapping</t>
+          <t>release management, go-to-market (GTM) strategy, customer beta program, NPS improvement, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1476,38 +1478,38 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Merck Life Science</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II, Policy &amp; Governance (Hybrid, Bangalore)</t>
+          <t>Global Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1516,19 +1518,19 @@
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks core policy/governance terms, lowering the ATS score; the candidate's domain is SaaS and GenAI rather than enterprise governance, creating the biggest fit gap.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>policy enforcement, governance, GDPR, CCPA, legal compliance, security, pricing strategy, monetization</t>
+          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1542,7 +1544,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1551,50 +1553,50 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Bread Financial India</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner 2 - Marketing</t>
+          <t>Product Owner (AI)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G17" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H17" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and title level, so hard rules pass; however, it lacks several JD-specific tools and marketing analytics terms, lowering the ATS score, and the candidate's domain experience (travel tech, FMCG, renewable) only loosely aligns with a marketing product role in financial services.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks fintech‑specific terminology and some AI delivery keywords.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Adobe Tag Manager, Adobe Experience Platform, digital attribution, analytics platform, tagging</t>
+          <t>telemetry, observability, evaluation strategy, offline/online testing, A/B testing, OKRs, risk/dependency reviews, rollout plan, Mixpanel</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1608,38 +1610,38 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Data Product Manager - Marketplace</t>
+          <t>Product Owner (Tax)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -1647,22 +1649,22 @@
         <v>3</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and the title does not violate seniority rules, but the resume lacks many JD‑specific keywords such as API gateway and real‑time governance, resulting in a moderate ATS score; however, strong travel‑tech and GenAI experience make the candidate a good domain fit.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>API gateway, real-time data processing, governed data, traveller profile, personalization, Marketplace dynamics, A/B testing</t>
+          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1676,7 +1678,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -1685,120 +1687,116 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Zeta</t>
+          <t>Sanofi</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Digital Product Owner – Portfolio &amp; Clinical AI Workflows</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains many core product and technical keywords but lacks several domain‑specific terms from the JD, leading to a moderate ATS score and a lower fit score due to mismatch with clinical/portfolio AI workflow focus.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>clinical workflow, portfolio strategy, AI/ML model operationalization, auditability, traceability, regulatory compliance, success metrics, pilot launch</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F19" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) so hard rules do not penalize; however, the resume only partially matches the banking‑focused keywords and tools, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>core banking, cloud-native, OKRs, A/B testing, NPS improvement, Snowflake, marketplace dynamics</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Owner — General</t>
+          <t>Associate Product Manager | Pune</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
+          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1812,7 +1810,7 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
@@ -1826,45 +1824,45 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Merck Life Science</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Global Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
+          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
+          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1878,7 +1876,7 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
@@ -1892,45 +1890,45 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Capgemini</t>
+          <t>ParentPay Group</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>FBS Customer Experience Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G22" s="2" t="n">
-        <v>72</v>
-      </c>
       <c r="H22" s="2" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core keywords but misses several JD-specific tools and metrics, leading to a solid but not top ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a good fit score.</t>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Qualtrics, Fullstory, CSAT, FCR, predictive analytics, real-time dashboards, AI-driven insights, KPI monitoring</t>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1944,61 +1942,59 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>PerkinElmer</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (Tax)</t>
+          <t>Software Product Manager (GTM Strategy)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) giving a strong ATS score, but lacks domain-specific scientific software experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
+          <t>go-to-market strategy, customer migration, adoption metrics, NPS improvement, OKRs</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2012,33 +2008,33 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager | Pune</t>
+          <t>TECHNOLOGY PRODUCT OWNER - MARKETPLACE VOIS</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2049,22 +2045,22 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords and relevant tools, giving a solid ATS score, but lacks marketplace‑specific terminology and some listed methodologies, lowering the fit score.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
+          <t>Marketplace platform, Two-sided marketplace, OKRs, Lean Portfolio Management, Technical debt, Data privacy, Vendor management</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2082,217 +2078,17 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Cornerstone OnDemand</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>ParentPay Group</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Omnibound AI</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Martech Product manager</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 2‑year minimum and title level, so hard rules pass; it contains many JD keywords but lacks direct marketing experience, which lowers the fit score.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>marketing automation, ABM, SEO, paid campaigns, digital marketing workflows, KPIs for marketing, US‑based team collaboration, LLMs, co‑pilot technologies</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -2321,9 +2117,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2335,7 +2128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2500,19 +2293,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Finkraft</t>
+          <t>Blackhawk Network India</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager — GST &amp; Tax Tech</t>
+          <t>Product Manager (Technology)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2521,24 +2314,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to limited GST/tax keyword overlap; the biggest gap is missing GST-specific terms. Fit score reflects decent SaaS and GenAI experience but weak domain alignment with GST/Tax tech.</t>
+          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks many API‑ and fintech‑specific terms required by the JD, lowering both scores. The biggest keyword gap is the absence of any mention of APIs.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>GST reconciliation, ITC matching, e-invoicing, API integration, knowledge base, OKRs, RICE prioritization</t>
+          <t>API, Fintech, Payments, Developer onboarding, Integration documentation, API adoption metrics, Roadmap management, Compliance</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2556,17 +2351,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -2632,7 +2427,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -2698,19 +2493,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>First Advantage</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Data Analytics- Remote</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2721,22 +2516,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and location, so hard rules do not penalize; however, keyword density for data‑analytics specific terms is moderate, leading to a modest ATS score, while the candidate's SaaS and GenAI background gives a decent fit.</t>
+          <t>Hard rules are satisfied (4 years experience meets the &gt;3 years requirement). The resume matches many general product management keywords but lacks telecom‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of 3GPP/HLR/SS7 related terms.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Snowflake, Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>3GPP, HLR, HSS, UDM, SS7, DIAMETER, cloud, http2, 5G, cost‑benefit analysis</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2754,55 +2549,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Greenway Health</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is low due to missing key workflow and automation terms, while fit score reflects good SaaS and GenAI experience but limited healthcare domain relevance.</t>
+          <t>The resume contains many generic product management keywords but lacks the specific PKI, certificate lifecycle, and cybersecurity terms required by the JD, resulting in a modest ATS score; domain mismatch drives a low fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>workflow automation, API integration, roadmap definition, backlog management, UAT, success metrics</t>
+          <t>PKI, certificate lifecycle, SCEP/EST APIs, TPM integration, cybersecurity, secure SDLC, regulatory compliance, PKIaaS, device identity</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2820,7 +2615,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -2830,45 +2625,45 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Owner - Data Analytics (AI/ML)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many generic product management keywords but lacks the specific PKI, certificate lifecycle, and cybersecurity terms required by the JD, resulting in a modest ATS score; domain mismatch drives a low fit score.</t>
+          <t>The candidate meets the 4-year experience requirement, so no hard rule penalty applies; however, the resume lacks many core JD keywords (e.g., Snowflake, Databricks, Python, Git, ETL) resulting in a modest ATS score and limited domain alignment.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>PKI, certificate lifecycle, SCEP/EST APIs, TPM integration, cybersecurity, secure SDLC, regulatory compliance, PKIaaS, device identity</t>
+          <t>Snowflake, Databricks, Python, Git, ETL/ELT processes, Qlik / Tableau, Data pipelines</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2886,29 +2681,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Provation</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Roundel (Ad Tech)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2919,22 +2714,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, but it lacks many ad‑tech specific keywords and domain experience, resulting in a modest ATS score and a lower job‑fit score; the biggest gap is missing ad‑serving and observability terminology.</t>
+          <t>The JD requires 7+ years of product experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'HIPAA'.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>ad serving, event tracking, observability, low‑latency, billing, anomaly detection</t>
+          <t>HIPAA, HL7, FHIR, Certified Scrum Product Owner, healthcare SaaS, regulatory compliance, user research, analytics tools</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2952,29 +2747,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Unified GlobalTech (I) Pvt Ltd</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Interconnect</t>
+          <t>Product Manager - HashiCorp Boundary</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2985,22 +2780,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no &gt;4 year requirement). ATS score is low because the resume contains few of the sales‑ and OEM‑focused keywords from the JD. The biggest keyword gap is the lack of OEM/quote/inventory management terms.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'Privileged Access Management'.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OEM relationship management, quote management, inventory management, GP% improvement, field application engineer training, sales enablement, industrial components, margin handling</t>
+          <t>Privileged Access Management, session recording, secrets management, PKI, threat monitoring</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3018,24 +2813,24 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>MKS Inc.</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -3045,28 +2840,28 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru South, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'pricing strategy'.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, market research, competitive analysis, product positioning, key account management, decoratives &amp; plating on plastics</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3084,29 +2879,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Mashreq</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Employee Platforms</t>
+          <t>SM Proxy Product Owner_Agile Squad Mgmt Reporting.Corporate Affairs-Head</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3127,12 +2922,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as "risk management" and "compliance".</t>
+          <t>Hard rule triggered: the job title includes 'Head', so both scores must be below 30 regardless of experience or keyword overlap. The most important missing keyword is 'report automation'.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>risk management, compliance, privacy, OKRs, A/B testing, market research</t>
+          <t>report automation, management reporting, finance stakeholder management, profitability reporting, SQL reporting, data workflow orchestration</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3150,24 +2945,24 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HCLTech</t>
+          <t>MKS Inc.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -3177,7 +2972,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Rural, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -3186,19 +2981,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key Salesforce and data‑migration keywords.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important missing keyword is 'pricing strategy'.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Salesforce Apex, Lightning components, Sales Cloud, Data migration, Data quality, Integrations, System architecture, GitHub Copilot</t>
+          <t>pricing strategy, market research, competitive analysis, product positioning, key account management, decoratives &amp; plating on plastics</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3226,7 +3021,7 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3033,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Vice President</t>
+          <t>Product Manager - Employee Platforms</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3252,19 +3047,19 @@
         <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
+          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as "risk management" and "compliance".</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
+          <t>risk management, compliance, privacy, OKRs, A/B testing, market research</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3292,19 +3087,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Teradata</t>
+          <t>Kenvue</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (IC), Agentic AI</t>
+          <t>Associate Product Owner</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3318,19 +3113,19 @@
         <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of AI/ML product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key AI/ML terms.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'Definition of Done'.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>LLMs, foundation models, inference pipelines, multi‑modal AI, Snowflake, OKRs</t>
+          <t>Definition of Done, Non-functional requirements, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3348,34 +3143,34 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bangalore Rural, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -3391,12 +3186,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
+          <t>The candidate has only 4 years of experience while the JD requires 9+ years, triggering a hard rule that forces both scores below 30; the resume also lacks key Salesforce and data‑migration keywords.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
+          <t>Salesforce Apex, Lightning components, Sales Cloud, Data migration, Data quality, Integrations, System architecture, GitHub Copilot</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3414,55 +3209,55 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Ashika Group</t>
+          <t>Teradata</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Stock Broking</t>
+          <t>Product Manager (IC), Agentic AI</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Kolkata, West Bengal, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no &gt;4 requirement). ATS score is moderate due to decent keyword overlap but missing finance-specific terms and location mismatch; the biggest keyword gap is lack of financial analysis experience.</t>
+          <t>The JD requires 5+ years of AI/ML product experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key AI/ML terms.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Financial analysis, Strategic planning, Product lifecycle management, Presentation skills, Market research, Finance industry experience, Data visualization tools (e.g., Tableau)</t>
+          <t>LLMs, foundation models, inference pipelines, multi‑modal AI, Snowflake, OKRs</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3476,59 +3271,59 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Keyloop</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
+          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3542,21 +3337,21 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -3622,19 +3417,19 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Sanofi</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Digital R&amp;D Lab Equipment Automation Jr. Product Owner</t>
+          <t>Product Manager (Materials Program)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3655,12 +3450,12 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on Agile, Jira, SQL, GenAI but missing many lab‑specific terms; fit score is lower because the candidate's SaaS/GenAI background does not align closely with R&amp;D lab equipment automation.</t>
+          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>lab automation, R&amp;D workflow orchestration, instrument integration, data capture for AI research, OKRs, A/B testing, Snowflake</t>
+          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3683,24 +3478,24 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Materials Program)</t>
+          <t>Product Owner – Payments</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3709,26 +3504,24 @@
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F21" s="2" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
-        </is>
-      </c>
+          <t>scoring failed after 3 attempts</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3744,55 +3537,55 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>American Bureau of Shipping (ABS)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Freedom Product Owner (PO)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is moderate due to limited keyword overlap with the Freedom product domain; the biggest gap is missing stage‑gate and impact assessment terminology.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>stage‑gate process, impact assessment, training material, customer satisfaction, MyFreedom portal</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3806,57 +3599,61 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Zemoso Technologies</t>
+          <t>Xplor Technologies</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Billing &amp; Settlement</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -3868,33 +3665,33 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Mindtickle</t>
+          <t>bp</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner- II (Engineering Manager - DevOps Team)</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3903,26 +3700,24 @@
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and seniority rules, but lacks many DevOps/SRE specific terms, lowering the ATS score; the biggest keyword gap is the absence of observability and pipeline tooling experience.</t>
+          <t>The resume meets the 4‑year experience requirement, so hard rules do not penalize the scores; however, key developer‑platform keywords and location match are missing, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate fit.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>observability, CI/CD pipelines, cost governance, incident response, SRE, Loki, on‑call rotation, platform security</t>
+          <t>API design, SDK development, Developer Experience (DX), Observability, DevOps/SRE, Technical documentation, Service contracts</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -3940,29 +3735,29 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Xplor Technologies</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Billing &amp; Settlement</t>
+          <t>Payments Product Owner - Direct Debit- Vice President</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3973,22 +3768,22 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
+          <t>Hard rules are satisfied, but the candidate's associate-level title and lack of payment-specific experience reduce both scores; the biggest keyword gap is the absence of payment scheme terms like Direct Debit, NACH, and UPI AutoPay.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
+          <t>Direct Debit, NACH, UPI AutoPay, SEPA, payment scheme regulatory analysis, mandate management, compliance, payment product roadmap</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -4006,55 +3801,55 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>bp</t>
+          <t>Nasdaq</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager Specialist</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement, so hard rules do not penalize the scores; however, key developer‑platform keywords and location match are missing, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate fit.</t>
+          <t>The resume meets the 4-year experience requirement, but lacks many domain-specific keywords and regulatory expertise required for the Nasdaq role, resulting in low ATS and fit scores; the biggest gap is the absence of regulatory reporting and Chartered Accountant credentials.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>API design, SDK development, Developer Experience (DX), Observability, DevOps/SRE, Technical documentation, Service contracts</t>
+          <t>Chartered Accountant, Regulatory reporting, Basel, Financial statements, Functional Specification Document, ControllerView, AxiomSL, Banking products, APAC regulatory frameworks</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -4072,29 +3867,29 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Payments Product Owner - Direct Debit- Vice President</t>
+          <t>IT Product Manager - SAP IBP - VOIS</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -4105,22 +3900,22 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the candidate's associate-level title and lack of payment-specific experience reduce both scores; the biggest keyword gap is the absence of payment scheme terms like Direct Debit, NACH, and UPI AutoPay.</t>
+          <t>The resume lacks core SAP IBP and supply‑chain terminology required by the JD, resulting in a low ATS match; the candidate's SaaS/GenAI background does not align well with the SAP planning domain, leading to a modest fit score.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Direct Debit, NACH, UPI AutoPay, SEPA, payment scheme regulatory analysis, mandate management, compliance, payment product roadmap</t>
+          <t>SAP IBP, supply chain planning, release management, data cleansing, governance, security compliance, demand planning</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4138,29 +3933,29 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Nasdaq</t>
+          <t>Sibros</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Product Manager Specialist</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -4171,22 +3966,22 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement, but lacks many domain-specific keywords and regulatory expertise required for the Nasdaq role, resulting in low ATS and fit scores; the biggest gap is the absence of regulatory reporting and Chartered Accountant credentials.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Chartered Accountant, Regulatory reporting, Basel, Financial statements, Functional Specification Document, ControllerView, AxiomSL, Banking products, APAC regulatory frameworks</t>
+          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -4204,7 +3999,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -4214,205 +4009,7 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Hempel A/S</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Finance Product Owner, PtP</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N29" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Sibros</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>GlobalLogic</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Owner IRC291187</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>Hard rule triggered: candidate has only 4 years experience while JD requires 6-8 years, so both scores are forced below 30; the resume also lacks key data platform terms.</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Data Lake, ETL, Data Warehouse, Snowflake, BI tool (Tableau), Data governance, metadata standards, API integration, advanced analytics</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
@@ -4445,9 +4042,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-14
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -628,19 +628,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Samaaro</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,24 +649,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
+          <t>The resume meets the 2-year minimum and contains most core JD keywords, yielding a strong ATS score; the main gap is lack of event‑marketing specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
+          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, CRM integration, analytics dashboards, PLG</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,24 +691,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager — Website Builder</t>
+          <t>Product Manager - Platform</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,24 +717,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; however, the candidate lacks direct website‑builder and AI‑native product experience, lowering the fit score.</t>
+          <t>The resume meets the 2‑year minimum and contains most of the key JD terms, yielding a strong ATS score; the main keyword gap is the lack of explicit OKRs/metrics language.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>AI-native product vision, drag-and-drop builder, templates and themes, SEO / AEO, LLM prototyping, full‑stack builder mindset, customer backward thinking, OKRs</t>
+          <t>OKRs, A/B testing, Snowflake, Mixpanel, risk management, payment platform experience, workflow automation frameworks</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -755,24 +759,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Reo.Dev</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,22 +787,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3-5 year experience requirement, and the resume contains many JD keywords, but lacks explicit self‑serve B2B and growth/retention metrics, which lowers the fit.</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>self‑serve, growth metrics, retention, OKRs, A/B testing</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,7 +820,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -826,19 +830,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Cube</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager — Website Builder</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +853,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and contains many relevant keywords, but lacks several JD-specific terms such as product roadmap and A/B testing, lowering the ATS score slightly; the strongest keyword gap is the missing "product roadmap" phrase.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; however, the candidate lacks direct website‑builder and AI‑native product experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, A/B testing, OKRs, user research, NPS improvement</t>
+          <t>AI-native product vision, drag-and-drop builder, templates and themes, SEO / AEO, LLM prototyping, full‑stack builder mindset, customer backward thinking, OKRs</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,7 +886,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -892,19 +896,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Recruiterflow</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Full Stack Builder</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -918,19 +922,19 @@
         <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>75</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks recruiting‑specific domain experience, lowering the fit score.</t>
+          <t>The resume meets the experience and title requirements and contains many JD keywords, yielding a solid ATS score; the main gap is lack of fintech‑specific tools and frameworks.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, product marketing collaboration, customer success partnership, sales alignment, OKRs, A/B testing, Mixpanel, NPS improvement</t>
+          <t>A/B testing, OKRs, Mixpanel, Snowflake, PLG, Jobs-to-be-Done</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -953,29 +957,29 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ShareChat</t>
+          <t>Reo.Dev</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -984,19 +988,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title alignment, yielding a strong ATS score, but the candidate's domain (B2B/enterprise SaaS) differs from ShareChat's consumer social media focus, lowering the fit score; the most notable missing keyword is 'North Star metric'.</t>
+          <t>The candidate meets the 3-5 year experience requirement, and the resume contains many JD keywords, but lacks explicit self‑serve B2B and growth/retention metrics, which lowers the fit.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, Snowflake, OKRs, North Star metric, Python, User research, MAU growth</t>
+          <t>self‑serve, growth metrics, retention, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,7 +1018,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1024,19 +1028,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II — No-Code Products</t>
+          <t>Loop Health - Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,24 +1049,26 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4+ years requirement and aligns on title level, yielding a strong ATS match, but lacks direct payments/no‑code experience, lowering the fit score; the biggest keyword gap is the absence of any payment‑product terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title level, so hard rules do not penalize; strong keyword overlap but missing several AI‑specific terms lowers ATS score slightly.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Payment Links, Payment Pages, agentic AI, A/B testing, OKRs, NPS improvement, Mixpanel, go-to-market plan, customer empathy interviews</t>
+          <t>LLM, AI‑first product, agentic workflows, model performance benchmarks, evaluation frameworks, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1080,40 +1086,38 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dezerv</t>
+          <t>ShareChat</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
         <v>78</v>
       </c>
@@ -1125,12 +1129,12 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title level, yielding a solid ATS match thanks to many overlapping keywords; however, the candidate's experience is in SaaS and enterprise tools rather than wealth‑management fintech, creating a domain gap.</t>
+          <t>The resume meets the 4‑year experience requirement and title alignment, yielding a strong ATS score, but the candidate's domain (B2B/enterprise SaaS) differs from ShareChat's consumer social media focus, lowering the fit score; the most notable missing keyword is 'North Star metric'.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>wealth management, investment portfolio, A/B testing, OKRs, NPS improvement, Snowflake, Mixpanel</t>
+          <t>Mixpanel, A/B testing, Snowflake, OKRs, North Star metric, Python, User research, MAU growth</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,29 +1152,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager II — No-Code Products</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1181,22 +1185,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many core keywords, but lacks several JD-specific terms such as payments and compliance, leading to a moderate ATS score; the candidate's SaaS and travel‑tech background aligns reasonably well with the events platform domain.</t>
+          <t>The resume meets the 4+ years requirement and aligns on title level, yielding a strong ATS match, but lacks direct payments/no‑code experience, lowering the fit score; the biggest keyword gap is the absence of any payment‑product terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>payments, risk compliance, regulatory requirements, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>Payment Links, Payment Pages, agentic AI, A/B testing, OKRs, NPS improvement, Mixpanel, go-to-market plan, customer empathy interviews</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,7 +1218,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1224,19 +1228,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Meesho</t>
+          <t>Dezerv</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1245,24 +1249,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F12" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
+          <t>The resume meets the 3‑year minimum and title level, yielding a solid ATS match thanks to many overlapping keywords; however, the candidate's experience is in SaaS and enterprise tools rather than wealth‑management fintech, creating a domain gap.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
+          <t>wealth management, investment portfolio, A/B testing, OKRs, NPS improvement, Snowflake, Mixpanel</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1285,24 +1291,24 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Wisemonk</t>
+          <t>InCred Financial Services</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Tier-1 Colleges Only)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1315,22 +1321,22 @@
         <v>4</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks direct HR/recruitment domain experience, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score, but lacks direct lending workflow experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>HR tech, recruitment workflow, assessment platform, agentic sourcing, OKRs, A/B testing, NPS improvement</t>
+          <t>lending workflow, origination, underwriting, vendor integration, API specifications, PRFAQ, US client stakeholder calls, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,29 +1354,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Breathe ESG</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Vice President) - Access Administration</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1379,26 +1385,24 @@
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1‑year minimum and aligns on title and location, yielding a strong ATS score, but lacks ESG and carbon‑accounting experience, lowering the fit score; the biggest keyword gap is specific carbon accounting terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no &gt;4 year requirement, no senior title), and contains many JD keywords, but the seniority gap (Associate vs VP) lowers the ATS title score; the biggest keyword gap is lack of explicit user research/journey mapping experience.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>carbon accounting, GHG Protocol, Scope 1/2/3, OKRs, A/B testing, Mixpanel, NPS improvement</t>
+          <t>user research, journey mapping, market analysis, product backlog, OKRs, risk management, transaction thresholds, segregation of duties</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1421,24 +1425,24 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1452,19 +1456,19 @@
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, but lacks several domain‑specific terms and data‑governance experience, leading to moderate ATS and fit scores.</t>
+          <t>The resume meets the 4-year experience requirement and contains many core keywords, but lacks several JD-specific terms such as payments and compliance, leading to a moderate ATS score; the candidate's SaaS and travel‑tech background aligns reasonably well with the events platform domain.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>data governance, AI/Agentic AI implementation, roadmap refinement, OKRs, risk and compliance</t>
+          <t>payments, risk compliance, regulatory requirements, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1482,7 +1486,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1492,45 +1496,45 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Zynga</t>
+          <t>Caterpillar Inc.</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords but lacks gaming‑specific terms, lowering the ATS score. The biggest gap is the absence of mobile gaming and player‑centric metrics.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS, travel, FMCG) does not align closely with Caterpillar's mining technology focus, lowering the fit score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>mobile gaming, A/B testing, user acquisition, KPIs, OKRs, Mixpanel, player engagement metrics, live ops</t>
+          <t>OKRs, RICE prioritization, A/B testing, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,29 +1552,29 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Easyship</t>
+          <t>Wisemonk</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (API)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1580,25 +1584,25 @@
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (4 years) and title rules, so hard rules do not penalize the scores. ATS keywords like Jira, SQL, Agile, B2B SaaS and stakeholder management are present, but core API‑product terms are missing, lowering the ATS score. The biggest fit gap is the lack of explicit API and developer‑platform experience.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks direct HR/recruitment domain experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>API, developer platform, usage analytics, ROI assessment, integration speed, developer satisfaction, OKRs, A/B testing, partner integration</t>
+          <t>HR tech, recruitment workflow, assessment platform, agentic sourcing, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1616,7 +1620,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -1626,19 +1630,19 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Decathlon</t>
+          <t>Breathe ESG</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1647,24 +1651,26 @@
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience rule and location, and contains many JD keywords, but lacks several retail‑specific terms, lowering the ATS density; the biggest keyword gap is the absence of "Omni‑experience" related language.</t>
+          <t>The resume meets the 1‑year minimum and aligns on title and location, yielding a strong ATS score, but lacks ESG and carbon‑accounting experience, lowering the fit score; the biggest keyword gap is specific carbon accounting terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Omni‑experience, phygital, circularity, AI‑augmented innovation, store‑to‑digital synchronicity, OKRs, A/B testing, NPS improvement</t>
+          <t>carbon accounting, GHG Protocol, Scope 1/2/3, OKRs, A/B testing, Mixpanel, NPS improvement</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1682,72 +1688,70 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Decathlon</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, B2B Experience</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4-year experience rule and location, and contains many JD keywords, but lacks several retail‑specific terms, lowering the ATS density; the biggest keyword gap is the absence of "Omni‑experience" related language.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Omni‑experience, phygital, circularity, AI‑augmented innovation, store‑to‑digital synchronicity, OKRs, A/B testing, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; the main gap is lack of fintech‑specific terminology.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Fintech, Electronic Bill Presentment and Payment (EBPP), AutoPay, paperless adoption, billing process management, AI-driven workflows, self‑serve capabilities, OKRs, RICE prioritization, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
           <t>2026-05-11</t>
@@ -1755,50 +1759,50 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
+          <t>Zynga</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager 2</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a strong ATS score, but lacks several domain-specific terms and finance reporting experience, lowering the fit score.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords but lacks gaming‑specific terms, lowering the ATS score. The biggest gap is the absence of mobile gaming and player‑centric metrics.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>OKRs, roadmap planning, governed data solutions, enterprise reporting standards, Snowflake, A/B testing, NPS improvement, financial services domain</t>
+          <t>mobile gaming, A/B testing, user acquisition, KPIs, OKRs, Mixpanel, player engagement metrics, live ops</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1812,11 +1816,11 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -1826,45 +1830,45 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (AI)</t>
+          <t>Product Manager - Agile Release Train</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks fintech‑specific terminology and some AI delivery keywords.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords but the title is a step below the target and the domain (medical imaging) does not align with the candidate's SaaS/GenAI background, creating the biggest gap.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>telemetry, observability, evaluation strategy, offline/online testing, A/B testing, OKRs, risk/dependency reviews, rollout plan, Mixpanel</t>
+          <t>angiography, clinical workflow, intervention room, regulatory compliance, Change Control Board, risk management, product roadmap, solution manager</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1878,28 +1882,28 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>NxtWave</t>
+          <t>S&amp;P Global</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1915,22 +1919,22 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G22" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H22" s="2" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords and meets the 3+ years requirement, but lacks several edtech‑specific terms and location match, lowering the ATS score. The biggest keyword gap is the absence of analytics and testing tools like Mixpanel and A/B testing.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a strong ATS score, but lacks several domain-specific terms and finance reporting experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, cohort analysis, SEO/content strategy, pedagogy</t>
+          <t>OKRs, roadmap planning, governed data solutions, enterprise reporting standards, Snowflake, A/B testing, NPS improvement, financial services domain</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1948,7 +1952,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -1958,19 +1962,19 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Sanofi</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner – Portfolio &amp; Clinical AI Workflows</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1984,19 +1988,19 @@
         <v>68</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product and technical keywords but lacks several domain‑specific terms from the JD, leading to a moderate ATS score and a lower fit score due to mismatch with clinical/portfolio AI workflow focus.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, but lacks several domain‑specific terms and data‑governance experience, leading to moderate ATS and fit scores.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>clinical workflow, portfolio strategy, AI/ML model operationalization, auditability, traceability, regulatory compliance, success metrics, pilot launch</t>
+          <t>data governance, AI/Agentic AI implementation, roadmap refinement, OKRs, risk and compliance</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2014,55 +2018,55 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>NxtWave</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Tech Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and relevant experience, meeting the hard rules; the main gap is lack of explicit KYC/regulatory terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords and meets the 3+ years requirement, but lacks several edtech‑specific terms and location match, lowering the ATS score. The biggest keyword gap is the absence of analytics and testing tools like Mixpanel and A/B testing.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>KYC, Regulatory compliance, Workflow automation, Risk management, API design</t>
+          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, cohort analysis, SEO/content strategy, pedagogy</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2076,11 +2080,11 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2090,19 +2094,19 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Tech Product Owner</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2113,22 +2117,22 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>82</v>
       </c>
-      <c r="G25" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H25" s="2" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+          <t>The resume contains many JD keywords and relevant experience, meeting the hard rules; the main gap is lack of explicit KYC/regulatory terminology.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+          <t>KYC, Regulatory compliance, Workflow automation, Risk management, API design</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2146,55 +2150,57 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>Uplers</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>VACE Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F26" s="2" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience meets implicit requirement). Resume contains many JD keywords but lacks finance‑specific terms, yielding a solid ATS score and moderate job fit.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches, so hard rules are satisfied; the resume lacks explicit mentions of PRD, Claude/ChatGPT, roadmap and OKR terminology, which is the biggest keyword gap.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
+          <t>PRD, Claude, ChatGPT, roadmap, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2212,29 +2218,29 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>ParentPay Group</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>CYBER PRODUCT MANAGER - VOIS</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2245,22 +2251,22 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is high due to strong keyword overlap (Jira, Agile, SQL, Power BI, GenAI, RAG, stakeholder management). The biggest gap is lack of cyber‑security and compliance terminology.</t>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Cyber Security, Baseline Security Requirements, Compliance, Privacy, Risk Management, Automated workflows, Roadmap development, CHRM, Trust by Design</t>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2283,50 +2289,52 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Allianz Technology</t>
+          <t>Omnibound AI</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Agile Product Owner_D2741</t>
+          <t>Martech Product manager</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F28" s="2" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
+          <t>The resume meets the 2‑year minimum and title level, so hard rules pass; it contains many JD keywords but lacks direct marketing experience, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
+          <t>marketing automation, ABM, SEO, paid campaigns, digital marketing workflows, KPIs for marketing, US‑based team collaboration, LLMs, co‑pilot technologies</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2349,24 +2357,24 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Zinnia</t>
+          <t>VOIS</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Compliance Workflow Automation</t>
+          <t>TECHNOLOGY PRODUCT OWNER - MARKETPLACE VOIS</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2377,22 +2385,22 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to strong keyword overlap but title mismatch; fit score is lower because domain experience in compliance workflow is limited.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords and relevant tools, giving a solid ATS score, but lacks marketplace‑specific terminology and some listed methodologies, lowering the fit score.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Compliance workflow, Regulatory process redesign, ERP integration, PeopleSoft, Subpoena handling, DOI complaints, Audit workflow automation</t>
+          <t>Marketplace platform, Two-sided marketplace, OKRs, Lean Portfolio Management, Technical debt, Data privacy, Vendor management</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2410,17 +2418,347 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Capco</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>VACE Product Manager</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience meets implicit requirement). Resume contains many JD keywords but lacks finance‑specific terms, yielding a solid ATS score and moderate job fit.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, RICE prioritization, A/B testing, Mixpanel, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>VOIS</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>CYBER PRODUCT MANAGER - VOIS</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is high due to strong keyword overlap (Jira, Agile, SQL, Power BI, GenAI, RAG, stakeholder management). The biggest gap is lack of cyber‑security and compliance terminology.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Cyber Security, Baseline Security Requirements, Compliance, Privacy, Risk Management, Automated workflows, Roadmap development, CHRM, Trust by Design</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group - India</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and the title is comparable, yielding a decent ATS score, but it lacks many education‑specific keywords and domain experience, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>product backlog, product vision, education market, UK education sector, storytelling, technical liaison, OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Allianz Technology</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Agile Product Owner_D2741</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="P29" s="2" t="inlineStr">
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Zinnia</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager II - Compliance Workflow Automation</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to strong keyword overlap but title mismatch; fit score is lower because domain experience in compliance workflow is limited.</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Compliance workflow, Regulatory process redesign, ERP integration, PeopleSoft, Subpoena handling, DOI complaints, Audit workflow automation</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -2454,6 +2792,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2465,7 +2808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2571,38 +2914,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Norstella</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several domain‑specific terms such as life‑sciences and LLMs, lowering the ATS score; the biggest gap is the missing life‑sciences/pharma experience.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap but missing several core JD terms; the biggest gap is the lack of CRM and customer service operations keywords.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>LLM, life sciences, pharmaceutical, data mastering, product marketing, commercial strategy, OKRs, market research (pharma focus), AI‑driven workflow</t>
+          <t>CRM platform, customer service operations, regulatory compliance, product roadmap, testing and implementation plans, product backlog prioritization, OKRs</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2620,29 +2963,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Endava</t>
+          <t>8club</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2656,19 +2999,19 @@
         <v>68</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
+          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however the resume lacks several core JD keywords and the domain (consumer social/event app) does not align with the candidate's B2B/enterprise SaaS background, leading to a moderate ATS score and lower fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
+          <t>Mixpanel, Amplitude, A/B testing, Notion, Dovetail, Claude, user research interviews, retention metrics, engagement metrics, growth loops</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2686,55 +3029,55 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Kapture CX</t>
+          <t>Norstella</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager – Applied AI (Voice)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>58</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title is not senior, so hard rules pass; however the resume lacks key voice AI terms like LLM, STT/TTS, reducing the ATS keyword match.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several domain‑specific terms such as life‑sciences and LLMs, lowering the ATS score; the biggest gap is the missing life‑sciences/pharma experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>LLM, STT, TTS, voice bot, conversation quality, benchmarking, latency, cost optimization</t>
+          <t>LLM, life sciences, pharmaceutical, data mastering, product marketing, commercial strategy, OKRs, market research (pharma focus), AI‑driven workflow</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2752,29 +3095,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Blackhawk Network India</t>
+          <t>Endava</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Technology)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2783,26 +3126,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>53</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks many API‑ and fintech‑specific terms required by the JD, lowering both scores. The biggest keyword gap is the absence of any mention of APIs.</t>
+          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>API, Fintech, Payments, Developer onboarding, Integration documentation, API adoption metrics, Roadmap management, Compliance</t>
+          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2820,7 +3161,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -2830,19 +3171,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>Motorola Solutions</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- App &amp; Web Products</t>
+          <t>Planview - Technical Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2853,22 +3194,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>60</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title is appropriate, but it lacks several JD‑specific tools and metrics, lowering the ATS keyword density; the biggest gap is the absence of analytics tools like Mixpanel or Google Analytics.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume matches many general product management keywords but lacks several JD‑specific tools and processes, lowering the ATS score; the strongest gap is the absence of Planview/Projectplace/Agileplace terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Google Analytics, Firebase, Confluence, A/B testing, OKRs, NPS improvement, MAU growth, competitor research</t>
+          <t>Planview, Projectplace, Agileplace, ERP integration, CRM integration, SIT/UAT planning, Cutover planning, functional documentation, automation use cases, dashboard creation</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2886,29 +3227,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>2070 Health</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II — Website Builder (Full-Stack Builder Role)</t>
+          <t>Product Manager- App &amp; Web Products</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2919,22 +3260,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>51</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience rule, but the candidate's domain (travel tech, FMCG, renewable energy) does not align closely with Razorpay's fintech/payment focus, leading to a modest fit score; the most important keyword gap is the lack of fintech/payment‑specific terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and the title is appropriate, but it lacks several JD‑specific tools and metrics, lowering the ATS keyword density; the biggest gap is the absence of analytics tools like Mixpanel or Google Analytics.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Payments, Fintech, A/B testing, OKRs, Metrics-driven growth, NPS improvement, Risk intelligence, Marketplace dynamics</t>
+          <t>Mixpanel, Google Analytics, Firebase, Confluence, A/B testing, OKRs, NPS improvement, MAU growth, competitor research</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2952,7 +3293,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -2962,19 +3303,19 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>UL Solutions</t>
+          <t>First Advantage</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner HRSD ServiceNow</t>
+          <t>Product Owner, Data Analytics- Remote</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2985,22 +3326,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is low due to missing core HR ServiceNow keywords, while fit score reflects decent product skills but weak domain alignment.</t>
+          <t>The resume meets the 4-year experience requirement and location, so hard rules do not penalize; however, keyword density for data‑analytics specific terms is moderate, leading to a modest ATS score, while the candidate's SaaS and GenAI background gives a decent fit.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, HR knowledge management, taxonomy, adoption strategy, risk evaluation, OKRs, analytics, portal governance, NPS improvement</t>
+          <t>Snowflake, Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -3018,55 +3359,55 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Standard Chartered India</t>
+          <t>Nykaa</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Entity Management Product Owner - CLM-T (Singapore, India)</t>
+          <t>Product Manager II - Personalisation</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume matches many core keywords (Jira, Agile, stakeholder management, GenAI, RAG, SQL, Power BI) but lacks specific CLM and compliance terminology, lowering the ATS score; the biggest gap is the absence of CLM/Compliance keywords.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>CLM, Compliance, Financial Crime, OKRs, Product vision, Roadmap, Legal stakeholder engagement</t>
+          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -3084,55 +3425,57 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Nykaa</t>
+          <t>Testsigma</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Personalisation</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
+          <t>Hard rules pass (4 years experience meets the 4-year minimum). ATS score is low due to missing many JD-specific tools and terms; the biggest keyword gap is the lack of GitHub/Confluence/Mixpanel mentions. Fit score reflects decent domain overlap (SaaS, GenAI) but limited testing‑automation experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
+          <t>GitHub, Confluence, Linear, Mixpanel, AI autonomous testing, coverage and traceability, release readiness score, dashboard for VP Engineering, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3155,50 +3498,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Aptita</t>
+          <t>Philips</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager MR Software</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, but lacks many JD‑specific keywords (e.g., Confluence, API, microservices), resulting in a low ATS score; the candidate’s SaaS and enterprise background is relevant but the banking/financial domain is a mismatch.</t>
+          <t>Hard rules are satisfied; the resume lacks many JD-specific terms, leading to a low ATS score, while the candidate's SaaS and enterprise experience gives a moderate job fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Confluence, API, microservices, CI/CD, financial compliance</t>
+          <t>PDLM, value proposition, go-to-market, regulatory compliance, installed base growth, clinical claims, roadmap</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3221,24 +3564,24 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Commvault</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Digital Channels Detection</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3249,22 +3592,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, but lacks key virtualization keywords and seniority alignment, resulting in modest ATS and fit scores; the biggest gap is missing virtualization platform experience.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the absence of "market research" and related discovery terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>VMware vSphere, VMware Cloud Foundation, Nutanix AHV, Microsoft Hyper‑V, OpenStack, VM snapshot mechanisms, Change Block Tracking (CBT), storage integration, high availability</t>
+          <t>market research, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3287,24 +3630,24 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>zenda</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Onboarding Infra</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3313,24 +3656,26 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no &gt;4 year requirement). ATS score is low due to limited overlap with fintech onboarding keywords; the biggest gap is missing KYC/authentication terminology. Fit score is moderate because the candidate has strong SaaS and GenAI experience but limited direct fintech onboarding exposure.</t>
+          <t>Hard rule triggered because the JD requires 5+ years of experience, but the candidate has only 4 years, so both scores are forced below 30; the resume also lacks several key JD terms such as A/B testing and OKRs.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>KYC, authentication, risk management, zero-touch onboarding, agentic AI, platform scalability, uptime, OKRs</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, mobile-first, user engagement metrics, PLG, two-sided marketplace</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3348,34 +3693,34 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Alegeus</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Data Platform</t>
+          <t>Product Manager - Employee Platforms</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -3391,12 +3736,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires &gt;7 years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks core data platform keywords such as "data ingestion" and "data APIs".</t>
+          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. Additionally, key terms like "product strategy" and "risk posture" are missing.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>data platform, data ingestion, data transformation, AI enablement, data APIs, Snowflake, OKRs, A/B testing, NPS improvement, MAU growth</t>
+          <t>product strategy, risk posture, compliance, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3414,34 +3759,34 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>NTT DATA North America</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Microsoft Dynamics CRM &amp; Field Service</t>
+          <t>Product Manager, Risk &amp; Compliance</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -3457,12 +3802,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any mention of Microsoft Dynamics CRM or Field Service.</t>
+          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key risk‑and‑compliance terminology.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Dynamics CRM, Dynamics 365 Field Service, Azure DevOps, Waterfall methodology, customer service operations</t>
+          <t>KYC, KYB, risk-based verification, adaptive verification, API design, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3480,29 +3825,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GlobalLogic</t>
+          <t>EvoluteIQ</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner/Manager with Aviation domain knowledge IRC294109</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3523,12 +3868,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD demands 10+ years in aviation product ownership, but the candidate has only 4 years, triggering the hard‑rule cutoff so both scores stay below 30; the resume also lacks key aviation domain terms.</t>
+          <t>The JD requires at least 10+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "AI/ML roadmap".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Crew Planning, Flight Operations, Navigational Data, Release Backlog, OKRs</t>
+          <t>AI/ML roadmap, post‑release assessment, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3551,50 +3896,50 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Zenwork, Inc</t>
+          <t>GlobalLogic</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner/Manager with Aviation domain knowledge IRC294109</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on SaaS and Agile tools but missing core payments/AP‑AR terms. The biggest fit gap is the lack of payments and AP/AR experience.</t>
+          <t>The JD demands 10+ years in aviation product ownership, but the candidate has only 4 years, triggering the hard‑rule cutoff so both scores stay below 30; the resume also lacks key aviation domain terms.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>payments, AP/AR, API, tax automation, compliance, product roadmap, OKRs, U.S. market, payments platform</t>
+          <t>Crew Planning, Flight Operations, Navigational Data, Release Backlog, OKRs</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3608,33 +3953,33 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Zenwork, Inc</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Global - Benefits Product Manager- SAP SuccessFactors Employee Central Benefits</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3645,22 +3990,22 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks core HR and SAP SuccessFactors terminology, resulting in modest keyword coverage and a weak domain fit; the biggest gap is missing Benefits and SAP-specific keywords.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on SaaS and Agile tools but missing core payments/AP‑AR terms. The biggest fit gap is the lack of payments and AP/AR experience.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>SAP SuccessFactors, Employee Central Benefits, Benefits configuration, Vendor integration, NPS improvement, Adoption KPIs, HR technology, Total Rewards</t>
+          <t>payments, AP/AR, API, tax automation, compliance, product roadmap, OKRs, U.S. market, payments platform</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3678,29 +4023,29 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ValGenesis</t>
+          <t>State Street</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Manufacturing Execution &amp; Batch Lifecycle</t>
+          <t>Financing Solutions Product Owner, Assistant Vice President</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3714,19 +4059,19 @@
         <v>25</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The JD demands 5+ years of manufacturing execution experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is lack of any mention of electronic batch records or regulated manufacturing terminology.</t>
+          <t>The JD explicitly seeks 10+ years of experience, far exceeding the candidate's 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key finance‑product terms.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>electronic batch records, FDA 21 CFR Part 11, MES, batch release workflow, regulatory intelligence</t>
+          <t>Equity Swaps, Agency Lending, Prime Services, Regulatory compliance, Risk management, Benefit realization, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3744,17 +4089,17 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -3766,7 +4111,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3780,19 +4125,19 @@
         <v>25</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as 'product strategy' and 'key success metrics'.</t>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the resume also lacks key technical terms like 'Spring Boot', 'GraphQL', and 'OpenTelemetry'.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>Spring Boot, GraphQL, OpenTelemetry, SLI/SLO, OAuth2, REST (OpenAPI), observability, error budgets</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3810,29 +4155,29 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Storable</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Account Opening</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3853,12 +4198,12 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core JD keywords such as "product strategy" and "AI native features".</t>
+          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit CRM experience.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, discovery, roadmap, key success metrics, risk posture, reliability, AI native features, AI tools, NPS improvement</t>
+          <t>CRM, card payment processing, OKRs, A/B testing, customer behavior metrics</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3881,24 +4226,24 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Thermo Fisher Scientific</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>AI &amp; Automation Product Owner</t>
+          <t>Product Manager (Vice President) - Global Customer Platform</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3919,12 +4264,12 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of AI/Automation product ownership, but the candidate has only 4 years total experience, triggering a hard rule that caps both scores below 30; the resume also lacks key AI/ML terminology such as 'model deployment' or 'ROI analysis'.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit "product strategy" language.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>AI/ML model deployment, ROI/business case development, OKRs, A/B testing, process automation</t>
+          <t>product strategy, product vision, market research, product backlog, key success metrics, operational management, change readiness</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3947,24 +4292,24 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Payments</t>
+          <t>Data &amp; AI Product Owner – Finance &amp; Commercial</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3973,24 +4318,26 @@
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>scoring failed after 3 attempts</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>The JD requires 5+ years of product ownership experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key finance‑AI terminology.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>financial planning &amp; forecasting, budgeting, pricing optimization, revenue management, variance analysis</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Linkedin</t>
@@ -4006,55 +4353,55 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>dsm-firmenich</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Vice President, POM Product Owner</t>
+          <t>Manager D&amp;T Data+AI Product Manager - Sustainability</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience and no senior title requirement). ATS score is moderate due to missing key finance and custody terminology; the biggest keyword gap is the lack of institutional banking/custody language.</t>
+          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key sustainability and data‑governance terminology.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>institutional banking, custody platform, regulatory compliance, roadmap, release planning, risk management, OKRs</t>
+          <t>data governance, sustainability reporting, CSRD, EcoVadis, CDP, data catalog, AI/ML product lifecycle</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -4068,59 +4415,59 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>VOIS</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>IT Product Manager - SAP IBP - VOIS</t>
+          <t>Product Manager - Payments</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core SAP IBP and supply‑chain terminology required by the JD, resulting in a low ATS match; the candidate's SaaS/GenAI background does not align well with the SAP planning domain, leading to a modest fit score.</t>
+          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as 'product strategy' and 'key success metrics'.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>SAP IBP, supply chain planning, release management, data cleansing, governance, security compliance, demand planning</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -4134,38 +4481,38 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Account Opening</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -4174,19 +4521,19 @@
         <v>25</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years of experience while the JD requires 10+ years (and explicitly mentions 5+ years), triggering hard rules that force both scores below 30; the resume also lacks key risk‑management terminology.</t>
+          <t>The JD explicitly requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core JD keywords such as "product strategy" and "AI native features".</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>CCAR, DFAST, retail credit risk, PD, LGD, EAD, risk modelling, SAFe 6.0 certification</t>
+          <t>product strategy, product vision, discovery, roadmap, key success metrics, risk posture, reliability, AI native features, AI tools, NPS improvement</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -4200,11 +4547,11 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -4214,30 +4561,28 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Live Connections</t>
+          <t>Thermo Fisher Scientific</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>AI ML Product Owner - BFSI</t>
+          <t>AI &amp; Automation Product Owner</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
         <v>25</v>
       </c>
@@ -4249,12 +4594,12 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit AI/ML and financial services terminology.</t>
+          <t>The JD requires 5+ years of AI/Automation product ownership, but the candidate has only 4 years total experience, triggering a hard rule that caps both scores below 30; the resume also lacks key AI/ML terminology such as 'model deployment' or 'ROI analysis'.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>AI/ML model evaluation, AWS cloud platform, Financial services / Asset Management, Product Owner certification (CSPO/CPO), Metrics definition and data‑driven decision making</t>
+          <t>AI/ML model deployment, ROI/business case development, OKRs, A/B testing, process automation</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4268,21 +4613,219 @@
         </is>
       </c>
       <c r="M27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Qualys</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement), but it lacks many cybersecurity-specific keywords and domain experience, resulting in moderate ATS and low job fit scores; the biggest gap is missing risk and security terminology.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>ServiceNow, CMDB, CSPM, vulnerability management, risk prioritization, cloud security, risk insights, remediation workflows, threat intelligence, compliance</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N27" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Citi</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Vice President - Product Manager</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 10+ years of experience and the title includes VP, both exceeding the candidate's 4 years, triggering hard rules that force both scores below 30; the resume also lacks key investor‑services and AI/ML terminology.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Investor Services, Middle Office, Fund Accounting, Custody, Data and Client Platforms (DCP), design thinking, user persona development, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Virtusa</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>The candidate has only 4 years of experience while the JD requires 10+ years (and explicitly mentions 5+ years), triggering hard rules that force both scores below 30; the resume also lacks key risk‑management terminology.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>CCAR, DFAST, retail credit risk, PD, LGD, EAD, risk modelling, SAFe 6.0 certification</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -4314,6 +4857,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-16
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cube</t>
+          <t>Pine Labs</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>AI Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1‑year minimum and title matches exactly, yielding a high ATS score; the biggest keyword gap is the lack of explicit marketing‑tech terms like SEO or A/B testing.</t>
+          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Manager role, yielding strong ATS keyword coverage; the biggest gap is the lack of explicit mention of rapid AI prototyping frameworks like LLMs or A/B testing.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>SEO, A/B testing, Mixpanel, Snowflake, OKRs, RICE prioritization, NPS improvement, product roadmap, growth team collaboration</t>
+          <t>LLMs, A/B testing, OKRs, RICE prioritization, experiment tracking, customer NPS improvement, Mixpanel, agent-based AI</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,17 +618,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -830,19 +830,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Curefit</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager — Website Builder</t>
+          <t>Product Manager 2 - Operations Excellence</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -853,22 +853,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>77</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; however, the candidate lacks direct website‑builder and AI‑native product experience, lowering the fit score.</t>
+          <t>The resume hits most JD keywords and meets location and experience criteria, yielding a high ATS score; however, the candidate lacks direct IoT and fitness‑center operations experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>AI-native product vision, drag-and-drop builder, templates and themes, SEO / AEO, LLM prototyping, full‑stack builder mindset, customer backward thinking, OKRs</t>
+          <t>IoT, vision-tech, real-time visibility, workflow automation, user research, OKRs, metrics, CCTV</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,29 +886,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Full Stack Builder</t>
+          <t>Associate Product Manager II</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -922,19 +922,19 @@
         <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>75</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience and title requirements and contains many JD keywords, yielding a solid ATS score; the main gap is lack of fintech‑specific tools and frameworks.</t>
+          <t>The resume meets the 2-5 year requirement and title level, yielding a solid ATS match, but lacks several finance‑specific product keywords and metrics.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, Snowflake, PLG, Jobs-to-be-Done</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, MAU growth, Jobs-to-be-Done</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,29 +952,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Reo.Dev</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner - ATLAS Program (SAP Global Cloud Operations)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -988,19 +988,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>75</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3-5 year experience requirement, and the resume contains many JD keywords, but lacks explicit self‑serve B2B and growth/retention metrics, which lowers the fit.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; the main gap is missing specific process frameworks like OKRs and RICE.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>self‑serve, growth metrics, retention, OKRs, A/B testing</t>
+          <t>OKRs, RICE prioritization, A/B testing, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,24 +1018,24 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cube</t>
+          <t>Reo.Dev</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and contains many relevant keywords, but lacks several JD-specific terms such as product roadmap and A/B testing, lowering the ATS score slightly; the strongest keyword gap is the missing "product roadmap" phrase.</t>
+          <t>The candidate meets the 3-5 year experience requirement, and the resume contains many JD keywords, but lacks explicit self‑serve B2B and growth/retention metrics, which lowers the fit.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, A/B testing, OKRs, user research, NPS improvement</t>
+          <t>self‑serve, growth metrics, retention, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -1162,24 +1162,24 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>DIAGEO India</t>
+          <t>ShareChat</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Data Product Manager - Commercial</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1195,12 +1195,12 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains most core keywords and matches location and education, yielding a strong ATS score, but lacks several data‑product specific terms and direct experience, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and title alignment, yielding a strong ATS score, but the candidate's domain (B2B/enterprise SaaS) differs from ShareChat's consumer social media focus, lowering the fit score; the most notable missing keyword is 'North Star metric'.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Data product strategy, Data governance, Snowflake, A/B testing, OKRs, NPS improvement, Customer segmentation</t>
+          <t>Mixpanel, A/B testing, Snowflake, OKRs, North Star metric, Python, User research, MAU growth</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1218,29 +1218,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>WeRize</t>
+          <t>DIAGEO India</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Data Product Manager - Commercial</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1249,9 +1249,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
         <v>78</v>
       </c>
@@ -1263,12 +1261,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3-year minimum (has 4 years) and title seniority is acceptable, yielding a strong keyword match; the biggest gap is lack of fintech/financial‑product experience.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains most core keywords and matches location and education, yielding a strong ATS score, but lacks several data‑product specific terms and direct experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, MAU growth, financial product roadmap, unsecured consumer credit, social distribution platform, customer acquisition cost (CAC) reduction</t>
+          <t>Data product strategy, Data governance, Snowflake, A/B testing, OKRs, NPS improvement, Customer segmentation</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1286,7 +1284,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1296,19 +1294,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ShareChat</t>
+          <t>Candescent</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>SW product Manager III</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1322,19 +1320,19 @@
         <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title alignment, yielding a strong ATS score, but the candidate's domain (B2B/enterprise SaaS) differs from ShareChat's consumer social media focus, lowering the fit score; the most notable missing keyword is 'North Star metric'.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). It scores well on ATS keywords and title alignment but lacks several banking‑specific terms, lowering the fit.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, Snowflake, OKRs, North Star metric, Python, User research, MAU growth</t>
+          <t>release planning, product roadmap, backlog grooming, digital banking, cloud‑based solutions, NPS improvement, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1352,29 +1350,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>DIAGEO India</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II — No-Code Products</t>
+          <t>Technical Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1385,22 +1383,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="H14" s="2" t="n">
-        <v>73</v>
-      </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4+ years requirement and aligns on title level, yielding a strong ATS match, but lacks direct payments/no‑code experience, lowering the fit score; the biggest keyword gap is the absence of any payment‑product terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several data‑asset specific terms from the JD, lowering the ATS score; the strongest keyword gap is data governance.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Payment Links, Payment Pages, agentic AI, A/B testing, OKRs, NPS improvement, Mixpanel, go-to-market plan, customer empathy interviews</t>
+          <t>Data governance, Data quality, Data catalog, Snowflake, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1418,29 +1416,29 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Unacademy</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Vice President) - Access Administration</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1449,24 +1447,26 @@
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F15" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no &gt;4 year requirement, no senior title), and contains many JD keywords, but the seniority gap (Associate vs VP) lowers the ATS title score; the biggest keyword gap is lack of explicit user research/journey mapping experience.</t>
+          <t>The candidate meets the 2‑year minimum (has 4 years) so hard rules pass; the resume contains many JD keywords but lacks core B2C test‑prep specifics, lowering the fit score. The biggest keyword gap is the absence of A/B testing/experiment metrics.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>user research, journey mapping, market analysis, product backlog, OKRs, risk management, transaction thresholds, segregation of duties</t>
+          <t>A/B testing, Mixpanel, OKRs, NPS improvement, MAU growth, Retention metrics, Product roadmap</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1489,24 +1489,24 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Siemens Healthineers</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Agile Release Train</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1517,22 +1517,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many core keywords, but lacks several JD-specific terms such as payments and compliance, leading to a moderate ATS score; the candidate's SaaS and travel‑tech background aligns reasonably well with the events platform domain.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords but the title is a step below the target and the domain (medical imaging) does not align with the candidate's SaaS/GenAI background, creating the biggest gap.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>payments, risk compliance, regulatory requirements, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>angiography, clinical workflow, intervention room, regulatory compliance, Change Control Board, risk management, product roadmap, solution manager</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1550,24 +1550,24 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Wisemonk</t>
+          <t>ve.ai - the intent company</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1577,30 +1577,28 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks direct HR/recruitment domain experience, lowering the fit score.</t>
+          <t>Hard rules are satisfied; the resume contains most required keywords and strong GenAI/SaaS experience, but lacks explicit mention of product roadmaps and machine learning.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>HR tech, recruitment workflow, assessment platform, agentic sourcing, OKRs, A/B testing, NPS improvement</t>
+          <t>product roadmap, machine learning, AI strategy, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1614,59 +1612,61 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DIAGEO India</t>
+          <t>TriNet</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several data‑asset specific terms from the JD, lowering the ATS score; the strongest keyword gap is data governance.</t>
+          <t>The resume meets the 2‑year minimum and title alignment, yielding a strong ATS match; the biggest gap is lack of HR‑specific terminology like OKRs and A/B testing.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Data governance, Data quality, Data catalog, Snowflake, OKRs, A/B testing, NPS improvement</t>
+          <t>OKRs, A/B testing, NPS improvement, user feedback loops, product roadmap planning</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1680,11 +1680,11 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -1694,47 +1694,45 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Unacademy</t>
+          <t>Accurate Background</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (has 4 years) so hard rules pass; the resume contains many JD keywords but lacks core B2C test‑prep specifics, lowering the fit score. The biggest keyword gap is the absence of A/B testing/experiment metrics.</t>
+          <t>The resume contains most required keywords and meets the experience level, yielding a strong ATS score; however, the candidate's domain (travel tech, renewable energy, FMCG) only partially aligns with background screening, lowering the fit score.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, OKRs, NPS improvement, MAU growth, Retention metrics, Product roadmap</t>
+          <t>OKRs, A/B testing, Mixpanel, NPS improvement, go-to-market, release notes, customer-facing collateral</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1748,33 +1746,33 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ve.ai - the intent company</t>
+          <t>Soho Square Solutions</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1785,22 +1783,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains most required keywords and strong GenAI/SaaS experience, but lacks explicit mention of product roadmaps and machine learning.</t>
+          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, machine learning, AI strategy, OKRs, A/B testing</t>
+          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1823,12 +1821,12 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1838,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1849,26 +1847,24 @@
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, yielding a strong ATS match; the biggest gap is lack of HR‑specific terminology like OKRs and A/B testing.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, user feedback loops, product roadmap planning</t>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1891,50 +1887,50 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BIG4</t>
+          <t>bp</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst\Product Owner (4-7 years Early joiner Preferred)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many relevant keywords, but lacks several JD-specific terms and does not clearly indicate Hyderabad location, lowering the ATS score; the strongest keyword gap is the absence of "Roadmap" and related planning terms.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score; the biggest gap is the lack of explicit platform‑release and vendor management terminology.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Roadmap, Risk Management, Incident Management, User Acceptance Testing (UAT), Customer Centricity, Release Notes, OKRs</t>
+          <t>global platform, release readiness, vendor management, operational processes, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1948,11 +1944,11 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -1962,45 +1958,45 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Tech Product Owner</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, but lacks several domain‑specific terms and data‑governance experience, leading to moderate ATS and fit scores.</t>
+          <t>The resume contains many JD keywords and relevant experience, meeting the hard rules; the main gap is lack of explicit KYC/regulatory terminology.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>data governance, AI/Agentic AI implementation, roadmap refinement, OKRs, risk and compliance</t>
+          <t>KYC, Regulatory compliance, Workflow automation, Risk management, API design</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2014,59 +2010,61 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>NxtWave</t>
+          <t>Uplers</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F24" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many JD keywords and meets the 3+ years requirement, but lacks several edtech‑specific terms and location match, lowering the ATS score. The biggest keyword gap is the absence of analytics and testing tools like Mixpanel and A/B testing.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches, so hard rules are satisfied; the resume lacks explicit mentions of PRD, Claude/ChatGPT, roadmap and OKR terminology, which is the biggest keyword gap.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, Jobs-to-be-Done, RICE prioritization, NPS improvement, MAU growth, cohort analysis, SEO/content strategy, pedagogy</t>
+          <t>PRD, Claude, ChatGPT, roadmap, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2080,7 +2078,7 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
@@ -2089,24 +2087,24 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>bp</t>
+          <t>ParentPay Group</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2117,22 +2115,22 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score; the biggest gap is the lack of explicit platform‑release and vendor management terminology.</t>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>global platform, release readiness, vendor management, operational processes, OKRs, A/B testing, NPS improvement</t>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2150,29 +2148,29 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Abacus Insights</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Tech Product Owner</t>
+          <t>Product Owner, AI Solutions</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2183,22 +2181,22 @@
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and relevant experience, meeting the hard rules; the main gap is lack of explicit KYC/regulatory terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It scores high on ATS due to strong keyword overlap (Jira, Agile, GenAI, RAG, stakeholder management, SQL, Power BI, etc.). Fit is moderate because the candidate lacks direct healthcare/payments domain experience.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>KYC, Regulatory compliance, Workflow automation, Risk management, API design</t>
+          <t>payment integrity, healthcare data, unstructured data solutions, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2216,57 +2214,55 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Uplers</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>LEA Product Manager</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title matches, so hard rules are satisfied; the resume lacks explicit mentions of PRD, Claude/ChatGPT, roadmap and OKR terminology, which is the biggest keyword gap.</t>
+          <t>The resume contains many JD keywords and meets the experience level, so ATS score is high; however the candidate lacks direct experience in GenAI visualization and conversational analytics for financial services, lowering the fit score.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>PRD, Claude, ChatGPT, roadmap, OKRs, A/B testing, Mixpanel</t>
+          <t>visualization, conversational analytics, business intelligence (BI), A/B testing, OKRs, Snowflake, user adoption metrics, NPS improvement</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2284,29 +2280,29 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Abacus Insights</t>
+          <t>Qualys</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, AI Solutions</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2320,19 +2316,19 @@
         <v>82</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It scores high on ATS due to strong keyword overlap (Jira, Agile, GenAI, RAG, stakeholder management, SQL, Power BI, etc.). Fit is moderate because the candidate lacks direct healthcare/payments domain experience.</t>
+          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>payment integrity, healthcare data, unstructured data solutions, OKRs, A/B testing, Snowflake</t>
+          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2350,7 +2346,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -2360,19 +2356,19 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2383,22 +2379,22 @@
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap (Jira, SQL, Agile, stakeholder management) but missing key JD terms like OKRs and ROI. Fit score is lower because the candidate's domain (SaaS, travel, renewable energy) does not directly align with HSBC's banking digital products.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+          <t>OKRs, ROI, market research, user research, product backlog</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2416,281 +2412,17 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Capco</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>LEA Product Manager</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains many JD keywords and meets the experience level, so ATS score is high; however the candidate lacks direct experience in GenAI visualization and conversational analytics for financial services, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>visualization, conversational analytics, business intelligence (BI), A/B testing, OKRs, Snowflake, user adoption metrics, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Qualys</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H31" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Allianz Technology</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Agile Product Owner_D2741</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H32" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Zinnia</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager II - Compliance Workflow Automation</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G33" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="H33" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to strong keyword overlap but title mismatch; fit score is lower because domain experience in compliance workflow is limited.</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Compliance workflow, Regulatory process redesign, ERP integration, PeopleSoft, Subpoena handling, DOI complaints, Audit workflow automation</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -2724,10 +2456,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2904,19 +2632,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Kapture CX</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Vice President</t>
+          <t>Technical Product Manager – Applied AI (Voice)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2927,22 +2655,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap but missing several core JD terms; the biggest gap is the lack of CRM and customer service operations keywords.</t>
+          <t>The candidate meets the 4-year experience requirement and the title is not senior, so hard rules pass; however the resume lacks key voice AI terms like LLM, STT/TTS, reducing the ATS keyword match.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>CRM platform, customer service operations, regulatory compliance, product roadmap, testing and implementation plans, product backlog prioritization, OKRs</t>
+          <t>LLM, STT, TTS, voice bot, conversation quality, benchmarking, latency, cost optimization</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2960,24 +2688,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Norstella</t>
+          <t>Flexera</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2987,28 +2715,28 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>44</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several domain‑specific terms such as life‑sciences and LLMs, lowering the ATS score; the biggest gap is the missing life‑sciences/pharma experience.</t>
+          <t>The candidate meets the 3+ years requirement and the title is close enough, so hard rules do not penalize; however, the resume lacks many container‑cloud and FinOps keywords, lowering the ATS match and overall fit.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>LLM, life sciences, pharmaceutical, data mastering, product marketing, commercial strategy, OKRs, market research (pharma focus), AI‑driven workflow</t>
+          <t>containers, cloud computing, FinOps, cost optimization, hybrid IT, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -3026,29 +2754,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Blackhawk Network India</t>
+          <t>Scouto AI</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Technology)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -3057,26 +2785,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>53</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum and has no senior title, so hard rules pass; however the resume lacks many API‑ and fintech‑specific terms required by the JD, lowering both scores. The biggest keyword gap is the absence of any mention of APIs.</t>
+          <t>The candidate meets the 4-year experience requirement, so hard rules do not penalize the scores; however, key JD terms like go-to-market, product launch, KPI definition, and competitive analysis are missing, lowering the ATS score. The strongest keyword gap is the lack of any go-to-market or launch experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>API, Fintech, Payments, Developer onboarding, Integration documentation, API adoption metrics, Roadmap management, Compliance</t>
+          <t>go-to-market strategy, product launch, KPI definition, competitive analysis, OKRs, A/B testing, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -3094,29 +2820,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GLOBELANCE</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Acquisition &amp; Monetisation)</t>
+          <t>Product Manager - Inventory Purchasing and Positioning</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -3137,12 +2863,12 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes hard rules, but the senior title and lack of direct acquisition/monetization keywords lower both scores; the most important missing keyword is 'A/B testing'.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap on Agile, Jira, stakeholder management but missing core inventory and supply‑chain terms. Fit score is lower because the candidate's SaaS/GenAI background does not align closely with Target's inventory purchasing and positioning domain.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, User acquisition, Monetization strategy, ARPU, Retention metrics, OKRs, Jobs-to-be-Done</t>
+          <t>inventory management, capacity planning, supply chain analytics, data science collaboration, A/B testing, OKRs, Snowflake, Mixpanel, algorithmic decision‑making</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -3165,50 +2891,50 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2070 Health</t>
+          <t>GLOBELANCE</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- App &amp; Web Products</t>
+          <t>Product Manager (Acquisition &amp; Monetisation)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru South, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>45</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>51</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title is appropriate, but it lacks several JD‑specific tools and metrics, lowering the ATS keyword density; the biggest gap is the absence of analytics tools like Mixpanel or Google Analytics.</t>
+          <t>The resume meets the 4-year experience requirement and passes hard rules, but the senior title and lack of direct acquisition/monetization keywords lower both scores; the most important missing keyword is 'A/B testing'.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, Google Analytics, Firebase, Confluence, A/B testing, OKRs, NPS improvement, MAU growth, competitor research</t>
+          <t>A/B testing, Mixpanel, User acquisition, Monetization strategy, ARPU, Retention metrics, OKRs, Jobs-to-be-Done</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -3226,17 +2952,17 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -3302,19 +3028,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Testsigma</t>
+          <t>Ingram Micro</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Assistant Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -3324,25 +3050,25 @@
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>40</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience meets the 4-year minimum). ATS score is low due to missing many JD-specific tools and terms; the biggest keyword gap is the lack of GitHub/Confluence/Mixpanel mentions. Fit score reflects decent domain overlap (SaaS, GenAI) but limited testing‑automation experience.</t>
+          <t>The resume meets the 1‑year minimum but lacks many vendor‑focused keywords, lowering the ATS score; the biggest gap is the absence of vendor management/contract negotiation terms.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>GitHub, Confluence, Linear, Mixpanel, AI autonomous testing, coverage and traceability, release readiness score, dashboard for VP Engineering, OKRs</t>
+          <t>vendor management, contract negotiation, invoice reconciliation, marketing training, lifecycle solutions, cloud solutions, commerce platforms</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -3360,29 +3086,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Rakuten Symphony</t>
+          <t>Testsigma</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Telco-Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3391,24 +3117,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules passed; ATS score is low due to limited overlap with telco‑specific keywords and a lower senior title, while the fit score reflects good GenAI experience but a domain mismatch with telecom/network optimization.</t>
+          <t>Hard rules pass (4 years experience meets the 4-year minimum). ATS score is low due to missing many JD-specific tools and terms; the biggest keyword gap is the lack of GitHub/Confluence/Mixpanel mentions. Fit score reflects decent domain overlap (SaaS, GenAI) but limited testing‑automation experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Geospatial Visualization, Agentic AI, RAN/NTN network optimization, Cloud-native platform, OKRs, A/B testing</t>
+          <t>GitHub, Confluence, Linear, Mixpanel, AI autonomous testing, coverage and traceability, release readiness score, dashboard for VP Engineering, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3426,29 +3154,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro</t>
+          <t>Rakuten Symphony</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - inverters &amp; Converters</t>
+          <t>Telco-Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3459,22 +3187,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume passes the hard rules but contains few power‑electronics keywords and limited domain relevance, resulting in low ATS and fit scores; the biggest gap is the absence of core product terms like AC‑DC converters.</t>
+          <t>Hard rules passed; ATS score is low due to limited overlap with telco‑specific keywords and a lower senior title, while the fit score reflects good GenAI experience but a domain mismatch with telecom/network optimization.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>AC‑DC converters, DC‑DC converters, EV chargers, inverters, energy storage systems, market sizing, competitive benchmarking, product roadmap</t>
+          <t>Geospatial Visualization, Agentic AI, RAN/NTN network optimization, Cloud-native platform, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3492,7 +3220,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -3502,19 +3230,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>JFrog</t>
+          <t>Larsen &amp; Toubro</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager - inverters &amp; Converters</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3525,22 +3253,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rule triggered because the JD requires &gt;4 years (12+ years) of experience, so both scores are forced below 30; the resume also lacks senior‑level keywords.</t>
+          <t>The resume passes the hard rules but contains few power‑electronics keywords and limited domain relevance, resulting in low ATS and fit scores; the biggest gap is the absence of core product terms like AC‑DC converters.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Snowflake, Mixpanel, customer NPS, PLG, two‑sided platform</t>
+          <t>AC‑DC converters, DC‑DC converters, EV chargers, inverters, energy storage systems, market sizing, competitive benchmarking, product roadmap</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3558,7 +3286,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -3568,14 +3296,14 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>nVent</t>
+          <t>Emergent</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -3601,12 +3329,12 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "voice of the customer" and "product line strategy".</t>
+          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key conversion and monetization terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>voice of the customer (VOC), product line strategy, roadmap implementation, value proposition, networking and data center infrastructure</t>
+          <t>A/B testing, conversion funnel, LTV, churn reduction, growth experimentation, OKRs, Mixpanel, PLG, customer insight loop, pricing strategy</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3629,24 +3357,24 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>EvoluteIQ</t>
+          <t>Guidewire Software</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager, Release Engineering</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3667,12 +3395,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires at least 10+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "AI/ML roadmap".</t>
+          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key release‑engineering terminology such as "CI/CD", "DevOps", and "release velocity".</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>AI/ML roadmap, post‑release assessment, OKRs, A/B testing, Snowflake</t>
+          <t>CI/CD, DevOps, release velocity, KPIs, cloud hosting</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3690,24 +3418,24 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>zenda</t>
+          <t>nVent</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -3721,9 +3449,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
         <v>25</v>
       </c>
@@ -3735,12 +3461,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rule triggered because the JD requires 5+ years of experience, but the candidate has only 4 years, so both scores are forced below 30; the resume also lacks several key JD terms such as A/B testing and OKRs.</t>
+          <t>The JD requires 5+ years of experience but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "voice of the customer" and "product line strategy".</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, NPS improvement, mobile-first, user engagement metrics, PLG, two-sided marketplace</t>
+          <t>voice of the customer (VOC), product line strategy, roadmap implementation, value proposition, networking and data center infrastructure</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3758,29 +3484,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Stripe</t>
+          <t>EvoluteIQ</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Risk &amp; Compliance</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3801,12 +3527,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key risk‑and‑compliance terminology.</t>
+          <t>The JD requires at least 10+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "AI/ML roadmap".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>KYC, KYB, risk-based verification, adaptive verification, API design, OKRs, A/B testing, NPS improvement</t>
+          <t>AI/ML roadmap, post‑release assessment, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3824,7 +3550,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -3834,7 +3560,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3616,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -3900,19 +3626,19 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Endava</t>
+          <t>Penguin Ai</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product owner - Payment Integrity</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3923,22 +3649,22 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
+          <t>Hard rules pass; the resume contains many generic product management keywords but lacks healthcare‑payment integrity specific terms, leading to moderate ATS score and lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
+          <t>payment integrity, claims workflow, denials management, operational automation, AI/ML integration, roadmap planning, prior authorization</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3956,29 +3682,29 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Outamation</t>
+          <t>Mushroom Solutions</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager/Product Owner – Compliance &amp; Data Privacy Solutions</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3989,22 +3715,22 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title seniority rules, but lacks many healthcare‑specific keywords, lowering the ATS score; the biggest gap is missing HIPAA/HL7/FHIR terminology.</t>
+          <t>The candidate meets the 3+ years requirement, so hard rules do not penalize the scores; however, the resume lacks many compliance‑specific keywords and domain experience, leading to a modest ATS score and a lower job‑fit score.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>HIPAA, HL7, FHIR, claims processing, prior authorization, EDI 837/835, UI/UX design system, product demos, onboarding workshops</t>
+          <t>FDA 21 CFR Part 11, GDPR, HIPAA, Data Protection Impact Assessment (DPIA), PHI (Protected Health Information), Regulatory compliance, Consent management, Security controls</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -4022,7 +3748,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -4032,19 +3758,19 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Mushroom Solutions</t>
+          <t>UBS</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager/Product Owner – Compliance &amp; Data Privacy Solutions</t>
+          <t>Product Manager, Americas Securities settlements &amp; Confirmations</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -4055,22 +3781,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement, so hard rules do not penalize the scores; however, the resume lacks many compliance‑specific keywords and domain experience, leading to a modest ATS score and a lower job‑fit score.</t>
+          <t>Hard rules are satisfied (4 years experience matches the unspecified minimum). ATS score is low due to missing many finance‑specific keywords and limited title alignment; the biggest keyword gap is the lack of any securities‑settlements or DTCC terminology.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>FDA 21 CFR Part 11, GDPR, HIPAA, Data Protection Impact Assessment (DPIA), PHI (Protected Health Information), Regulatory compliance, Consent management, Security controls</t>
+          <t>Securities settlements, DTCC, OKRs, UX testing, production stability, performance monitoring, financial regulatory compliance, risk management</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -4088,7 +3814,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -4098,19 +3824,19 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Americas Securities settlements &amp; Confirmations</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -4124,19 +3850,19 @@
         <v>28</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches the unspecified minimum). ATS score is low due to missing many finance‑specific keywords and limited title alignment; the biggest keyword gap is the lack of any securities‑settlements or DTCC terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Securities settlements, DTCC, OKRs, UX testing, production stability, performance monitoring, financial regulatory compliance, risk management</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -4159,12 +3885,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -4176,7 +3902,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Product Manager (Vice President) - Global Customer Platform</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -4220,17 +3946,17 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -4242,7 +3968,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Account Opening</t>
+          <t>Product Manager - Payments</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -4256,19 +3982,19 @@
         <v>25</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as 'product strategy' and 'market research'.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>product strategy, market research, product backlog, key success metrics, AI native features, scalability</t>
+          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -4286,7 +4012,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -4296,19 +4022,19 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ValGenesis</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Manufacturing Execution &amp; Batch Lifecycle</t>
+          <t>Vice President - Product Manager - Machine Learning &amp; Intelligent Operations</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -4329,12 +4055,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The JD demands 5+ years of manufacturing execution experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is lack of any mention of electronic batch records or regulated manufacturing terminology.</t>
+          <t>The JD explicitly requires 6+ years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'machine learning'.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>electronic batch records, FDA 21 CFR Part 11, MES, batch release workflow, regulatory intelligence</t>
+          <t>machine learning, model governance, risk and compliance, AI strategy, product roadmap, customer contact reduction</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -4352,29 +4078,29 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Giggso</t>
+          <t>Talent Corner HR Services Pvt Ltd</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -4388,19 +4114,19 @@
         <v>25</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key data‑governance terminology.</t>
+          <t>The JD requires 5+ years of product design experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any hardware or agricultural product design terminology.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>data governance, metadata management, data lineage, data lake, ETL tools, cloud data services, AI‑powered automation</t>
+          <t>hardware product design, agri‑infrastructure, greenhouse systems, field research, SOP creation, QA/QC systems, mechanical engineering</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -4418,29 +4144,29 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Storable</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Account Opening</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -4454,19 +4180,19 @@
         <v>25</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit CRM experience.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as 'product strategy' and 'market research'.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>CRM, card payment processing, OKRs, A/B testing, customer behavior metrics</t>
+          <t>product strategy, market research, product backlog, key success metrics, AI native features, scalability</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -4489,24 +4215,24 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Electronic Arts (EA)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Knowledge Product Manager</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -4527,12 +4253,12 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key JD terms such as 'product strategy' and 'key success metrics'.</t>
+          <t>The JD requires 8+ years of product/knowledge management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several core knowledge‑management keywords.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>knowledge management strategy, taxonomy, metadata governance, serviceNow, confluence, operational knowledge assets, process definition, AI‑assisted support</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4550,29 +4276,29 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Storable</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Vice President) - Global Customer Platform</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -4593,12 +4319,12 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit "product strategy" language.</t>
+          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit CRM experience.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, market research, product backlog, key success metrics, operational management, change readiness</t>
+          <t>CRM, card payment processing, OKRs, A/B testing, customer behavior metrics</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -4616,7 +4342,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
@@ -4626,19 +4352,19 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>dsm-firmenich</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Manager D&amp;T Data+AI Product Manager - Sustainability</t>
+          <t>Product Manager (Vice President) - Global Customer Platform</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -4659,12 +4385,12 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key sustainability and data‑governance terminology.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit "product strategy" language.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>data governance, sustainability reporting, CSRD, EcoVadis, CDP, data catalog, AI/ML product lifecycle</t>
+          <t>product strategy, product vision, market research, product backlog, key success metrics, operational management, change readiness</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -4692,19 +4418,19 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Giggso</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Account Opening</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -4725,12 +4451,12 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core JD keywords such as "product strategy" and "AI native features".</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key data‑governance terminology.</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, discovery, roadmap, key success metrics, risk posture, reliability, AI native features, AI tools, NPS improvement</t>
+          <t>data governance, metadata management, data lineage, data lake, ETL tools, cloud data services, AI‑powered automation</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -4748,55 +4474,55 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>dsm-firmenich</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Data</t>
+          <t>Manager D&amp;T Data+AI Product Manager - Sustainability</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr"/>
       <c r="F31" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains several relevant keywords but misses many finance‑specific terms, lowering the ATS score, and the candidate's domain experience (travel SaaS, renewable energy) does not align well with a data‑focused product owner role in banking.</t>
+          <t>The JD requires 8+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key sustainability and data‑governance terminology.</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>KYC, AWS, Azure, risk and compliance, API design, product roadmap, OKRs</t>
+          <t>data governance, sustainability reporting, CSRD, EcoVadis, CDP, data catalog, AI/ML product lifecycle</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -4810,7 +4536,7 @@
         </is>
       </c>
       <c r="M31" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
@@ -4819,50 +4545,50 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Synechron</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Foreign Exchange</t>
+          <t>Technology Product Owner</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="3" t="inlineStr"/>
       <c r="F32" s="2" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume lacks several core FX and regulatory keywords, lowering the ATS score, and the candidate's domain experience (SaaS, travel, GenAI) does not align closely with the FX markets focus, reducing the fit score.</t>
+          <t>Hard rules pass (4 years experience matches the JD). The resume hits many ATS keywords (Jira, SQL, Agile, stakeholder management, SDLC) but lacks core risk‑banking terms, lowering the fit score.</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>FX markets, trade execution, regulatory compliance, risk management, downstream system integration, backlog prioritization</t>
+          <t>Credit Risk, Counterparty Grading, Limit Management, Probability of Default, Loss Given Default, Exposure at Default, Confluence, Investment Banking, Risk Metrics, Change Management</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -4880,29 +4606,29 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Qualys</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner, Data</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -4913,22 +4639,22 @@
       <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="3" t="inlineStr"/>
       <c r="F33" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G33" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G33" s="2" t="n">
-        <v>38</v>
-      </c>
       <c r="H33" s="2" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement), but it lacks many cybersecurity-specific keywords and domain experience, resulting in moderate ATS and low job fit scores; the biggest gap is missing risk and security terminology.</t>
+          <t>Hard rules are satisfied; the resume contains several relevant keywords but misses many finance‑specific terms, lowering the ATS score, and the candidate's domain experience (travel SaaS, renewable energy) does not align well with a data‑focused product owner role in banking.</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, CMDB, CSPM, vulnerability management, risk prioritization, cloud security, risk insights, remediation workflows, threat intelligence, compliance</t>
+          <t>KYC, AWS, Azure, risk and compliance, API design, product roadmap, OKRs</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -4951,50 +4677,50 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Sulzer</t>
+          <t>Synechron</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Product Owner / Business Analyst LeanIX</t>
+          <t>Product Owner - Foreign Exchange</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="3" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied, but the resume lacks most of the JD's core tools and platform terms, resulting in a low ATS match; the biggest keyword gap is the absence of any LeanIX/ServiceNow experience.</t>
+          <t>Hard rules are satisfied; the resume lacks several core FX and regulatory keywords, lowering the ATS score, and the candidate's domain experience (SaaS, travel, GenAI) does not align closely with the FX markets focus, reducing the fit score.</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>LeanIX, ServiceNow, Azure DevOps, API integration, IT portfolio governance, dashboard creation, metadata governance</t>
+          <t>FX markets, trade execution, regulatory compliance, risk management, downstream system integration, backlog prioritization</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -5012,7 +4738,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
@@ -5022,19 +4748,19 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager-Consultant</t>
+          <t>Global - Benefits Product Manager- SAP SuccessFactors Employee Central Benefits</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -5045,22 +4771,22 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many JD-specific technical keywords and the candidate is based in Bangalore while the role is in Pune, resulting in low ATS and fit scores; the most important keyword gap is the absence of any mention of IDE tooling (e.g., VS Code, IntelliJ) and language bindings (C++, Java, Python).</t>
+          <t>Hard rules are satisfied, but the resume lacks core HR and SAP SuccessFactors terminology, resulting in modest keyword coverage and a weak domain fit; the biggest gap is missing Benefits and SAP-specific keywords.</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>C++, Java, JavaScript, VBA, Python, VS Code, IntelliJ, SDK, API design governance, CMake, Maven, Gradle, npm</t>
+          <t>SAP SuccessFactors, Employee Central Benefits, Benefits configuration, Vendor integration, NPS improvement, Adoption KPIs, HR technology, Total Rewards</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -5078,55 +4804,55 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>Hempel A/S</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Finance Product Owner, PtP</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>The candidate has only 4 years of experience while the JD requires 10+ years (and explicitly mentions 5+ years), triggering hard rules that force both scores below 30; the resume also lacks key risk‑management terminology.</t>
+          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>CCAR, DFAST, retail credit risk, PD, LGD, EAD, risk modelling, SAFe 6.0 certification</t>
+          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -5144,29 +4870,29 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Sulzer</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Vice President - Product Manager-AI &amp; Digital Experience- Security Services</t>
+          <t>Product Owner / Business Analyst LeanIX</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -5177,22 +4903,22 @@
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as 'design thinking' and 'client segmentation'.</t>
+          <t>Hard rules are satisfied, but the resume lacks most of the JD's core tools and platform terms, resulting in a low ATS match; the biggest keyword gap is the absence of any LeanIX/ServiceNow experience.</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>design thinking, client segmentation, user persona development, OKRs, A/B testing, Snowflake, NPS improvement</t>
+          <t>LeanIX, ServiceNow, Azure DevOps, API integration, IT portfolio governance, dashboard creation, metadata governance</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -5210,7 +4936,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
@@ -5220,24 +4946,24 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Citi</t>
+          <t>Valeo</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>VP- Custody Product Manager -Data &amp; AI</t>
+          <t>Product Owner- Front Camera</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr"/>
@@ -5253,12 +4979,12 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>The job title includes 'VP', triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords. The resume lacks key Custody‑specific terms such as 'settlement' and 'asset servicing'.</t>
+          <t>The JD requires a minimum of 5+ years of front‑camera experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key automotive and ADAS terminology.</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>settlement, safekeeping, corporate actions, asset servicing, data product governance, AI‑powered workflow automation</t>
+          <t>ADAS, Front Camera, AEB, Traffic Sign Recognition, HIL testing, DOORS, ISO 26262, CAN-FD, FOTA</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -5276,7 +5002,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
@@ -5286,24 +5012,24 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Valeo</t>
+          <t>GlobalLogic</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Product Owner- Front Camera</t>
+          <t>Technical Product Owner IRC291187</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr"/>
@@ -5319,12 +5045,12 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>The JD requires a minimum of 5+ years of front‑camera experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key automotive and ADAS terminology.</t>
+          <t>Hard rule triggered: candidate has only 4 years experience while JD requires 6-8 years, so both scores are forced below 30; the resume also lacks key data platform terms.</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>ADAS, Front Camera, AEB, Traffic Sign Recognition, HIL testing, DOORS, ISO 26262, CAN-FD, FOTA</t>
+          <t>Data Lake, ETL, Data Warehouse, Snowflake, BI tool (Tableau), Data governance, metadata standards, API integration, advanced analytics</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -5342,17 +5068,17 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>
@@ -5408,7 +5134,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
@@ -5418,7 +5144,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-18
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pine Labs</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>AI Associate Product Manager</t>
+          <t>Product Owner - ATLAS Program (SAP Global Cloud Operations)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,26 +581,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Manager role, yielding strong ATS keyword coverage; the biggest gap is the lack of explicit mention of rapid AI prototyping frameworks like LLMs or A/B testing.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; the main gap is missing specific process frameworks like OKRs and RICE.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>LLMs, A/B testing, OKRs, RICE prioritization, experiment tracking, customer NPS improvement, Mixpanel, agent-based AI</t>
+          <t>OKRs, RICE prioritization, A/B testing, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -628,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Curefit</t>
+          <t>Aspire</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 2 - Operations Excellence</t>
+          <t>Product Manager - Local Payments</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -649,24 +647,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most JD keywords and meets location and experience criteria, yielding a high ATS score; however, the candidate lacks direct IoT and fitness‑center operations experience, lowering the fit score.</t>
+          <t>The resume meets the 4‑year minimum and location requirement, and contains many JD keywords, yielding a strong ATS score; however, the candidate lacks direct payments and fintech experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>IoT, vision-tech, real-time visibility, workflow automation, user research, OKRs, metrics, CCTV</t>
+          <t>payments, transaction management, risk management, regulatory compliance, A/B testing, OKRs, marketplace dynamics</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -720,19 +720,19 @@
         <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-5 year requirement and title level, yielding a solid ATS match, but lacks several finance‑specific product keywords and metrics.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, NPS improvement, MAU growth, Jobs-to-be-Done</t>
+          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,24 +750,24 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>WeRize</t>
+          <t>DigiCert</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -781,26 +781,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3-year minimum (has 4 years) and title seniority is acceptable, yielding a strong keyword match; the biggest gap is lack of fintech/financial‑product experience.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks domain-specific experience in DNS/cloud networking, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, MAU growth, financial product roadmap, unsecured consumer credit, social distribution platform, customer acquisition cost (CAC) reduction</t>
+          <t>AWS, Azure, GCP, DNS, MLOps, cloud-native, A/B testing, telemetry, inference pipelines</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>Pice®</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Credit Flow</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,24 +847,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -889,24 +889,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DigiCert</t>
+          <t>Jack &amp; Jill</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-II (40–50 LPA + Equity) at AI-native creative intelligence startup</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,24 +915,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks domain-specific experience in DNS/cloud networking, which lowers the fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement, so hard rules do not penalize the scores; the resume contains many JD keywords but lacks several core terms like LLM and marketing, leading to a solid ATS score but moderate job‑fit.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AWS, Azure, GCP, DNS, MLOps, cloud-native, A/B testing, telemetry, inference pipelines</t>
+          <t>LLM, agentic workflows, creative analysis, marketing, AdTech, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,55 +952,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Candescent</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SW product Manager III</t>
+          <t>Technical Product Manager - Python or SQL</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). It scores well on ATS keywords and title alignment but lacks several banking‑specific terms, lowering the fit.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap but missing key tools like Python and advanced Excel; fit score is limited by domain mismatch despite strong SaaS and GenAI experience.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>release planning, product roadmap, backlog grooming, digital banking, cloud‑based solutions, NPS improvement, OKRs, A/B testing</t>
+          <t>Python, advanced Excel, pivot tables, statistical analysis, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1016,55 +1018,55 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>DIAGEO India</t>
+          <t>Soho Square Solutions</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Owner</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many relevant keywords, but lacks several data‑asset specific terms from the JD, lowering the ATS score; the strongest keyword gap is data governance.</t>
+          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Data governance, Data quality, Data catalog, Snowflake, OKRs, A/B testing, NPS improvement</t>
+          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1078,33 +1080,33 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ve.ai - the intent company</t>
+          <t>Dr. Reddy's Laboratories</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Oncology</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1113,24 +1115,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F10" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains most required keywords and strong GenAI/SaaS experience, but lacks explicit mention of product roadmaps and machine learning.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS/GenAI) does not align with oncology/pharma, lowering the fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, machine learning, AI strategy, OKRs, A/B testing</t>
+          <t>oncology, pharmaceutical market analysis, clinical trial workflow, regulatory compliance, go-to-market strategy, KPIs such as NPS or market share growth, A/B testing</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,17 +1152,17 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1174,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1179,26 +1183,24 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, yielding a strong ATS match; the biggest gap is lack of HR‑specific terminology like OKRs and A/B testing.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, user feedback loops, product roadmap planning</t>
+          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1216,55 +1218,55 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Accurate Background</t>
+          <t>Fundtec</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager (IT Product)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>78</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>65</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>73</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume contains most required keywords and meets the experience level, yielding a strong ATS score; however, the candidate's domain (travel tech, renewable energy, FMCG) only partially aligns with background screening, lowering the fit score.</t>
+          <t>The resume meets the experience requirement (4 years) and title level, so hard rules do not penalize; it contains most JD keywords but lacks several tool and technology mentions, lowering the ATS score. The strongest keyword gap is the absence of "Trello"/"Confluence" and cloud/API related terms.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, NPS improvement, go-to-market, release notes, customer-facing collateral</t>
+          <t>Trello, Confluence, cloud technologies, API integration, DevOps, security compliance, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1278,38 +1280,38 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Allianz Technology</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Agile Product Owner_D2741</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1318,19 +1320,19 @@
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many core keywords, but lacks several JD-specific terms such as payments and compliance, leading to a moderate ATS score; the candidate's SaaS and travel‑tech background aligns reasonably well with the events platform domain.</t>
+          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>payments, risk compliance, regulatory requirements, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1344,11 +1346,11 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1358,45 +1360,45 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Digital Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap (Jira, SQL, Agile, stakeholder management) but missing key JD terms like OKRs and ROI. Fit score is lower because the candidate's domain (SaaS, travel, renewable energy) does not directly align with HSBC's banking digital products.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+          <t>OKRs, ROI, market research, user research, product backlog</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1410,7 +1412,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1419,608 +1421,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Dr. Reddy's Laboratories</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Oncology</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS/GenAI) does not align with oncology/pharma, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>oncology, pharmaceutical market analysis, clinical trial workflow, regulatory compliance, go-to-market strategy, KPIs such as NPS or market share growth, A/B testing</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TriNet</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>bp</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score; the biggest gap is the lack of explicit platform‑release and vendor management terminology.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>global platform, release readiness, vendor management, operational processes, OKRs, A/B testing, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>hackajob</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Tech Product Owner</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains many JD keywords and relevant experience, meeting the hard rules; the main gap is lack of explicit KYC/regulatory terminology.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>KYC, Regulatory compliance, Workflow automation, Risk management, API design</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Fundtec</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager (IT Product)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the experience requirement (4 years) and title level, so hard rules do not penalize; it contains most JD keywords but lacks several tool and technology mentions, lowering the ATS score. The strongest keyword gap is the absence of "Trello"/"Confluence" and cloud/API related terms.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Trello, Confluence, cloud technologies, API integration, DevOps, security compliance, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Capco</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>LEA Product Manager</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains many JD keywords and meets the experience level, so ATS score is high; however the candidate lacks direct experience in GenAI visualization and conversational analytics for financial services, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>visualization, conversational analytics, business intelligence (BI), A/B testing, OKRs, Snowflake, user adoption metrics, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Qualys</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules and scores high on keyword coverage and title alignment, but lacks cybersecurity domain experience required for the role, creating a notable fit gap.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Vulnerability Management, Risk Prioritization, Cloud Posture, ServiceNow integration, Compliance, Threat Intelligence</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>HSBC</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Manager</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap (Jira, SQL, Agile, stakeholder management) but missing key JD terms like OKRs and ROI. Fit score is lower because the candidate's domain (SaaS, travel, renewable energy) does not directly align with HSBC's banking digital products.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, ROI, market research, user research, product backlog</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Allianz Technology</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Agile Product Owner_D2741</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -2039,15 +1445,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2059,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2165,12 +1562,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Flexera</t>
+          <t>Columbia Sportswear Company</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Digital Product Owner (Emerging Brands)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2184,19 +1581,19 @@
         <v>62</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and the title is close enough, so hard rules do not penalize; however, the resume lacks many container‑cloud and FinOps keywords, lowering the ATS match and overall fit.</t>
+          <t>Hard rules pass (4 years experience matches no minimum &gt;4). ATS score is moderate due to good keyword overlap but missing core ecommerce tech terms. Fit score is limited by domain mismatch with ecommerce focus.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>containers, cloud computing, FinOps, cost optimization, hybrid IT, OKRs, A/B testing, NPS improvement</t>
+          <t>React, Salesforce Commerce Cloud, Amplience CMS, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth, Mixpanel</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2214,29 +1611,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GLOBELANCE</t>
+          <t>smallcase</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Acquisition &amp; Monetisation)</t>
+          <t>Product Manager 1- MF</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2257,12 +1654,12 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes hard rules, but the senior title and lack of direct acquisition/monetization keywords lower both scores; the most important missing keyword is 'A/B testing'.</t>
+          <t>The resume meets the 4‑year experience requirement and location, but lacks many fintech‑specific keywords, lowering the ATS score; the biggest gap is the absence of mutual‑fund/fintech terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, User acquisition, Monetization strategy, ARPU, Retention metrics, OKRs, Jobs-to-be-Done</t>
+          <t>Mutual Funds, Fintech, Mixpanel, Amplitude, Investor behavior, Roadmap, Pod ownership, Capital markets</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2280,29 +1677,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Recrew AI</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Inventory Purchasing and Positioning</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2313,22 +1710,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and title level, but lacks many JD-specific keywords and domain experience in accounting/tax, leading to a modest ATS score and moderate job fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap on Agile, Jira, stakeholder management but missing core inventory and supply‑chain terms. Fit score is lower because the candidate's SaaS/GenAI background does not align closely with Target's inventory purchasing and positioning domain.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>CPA, tax workflow, low-code prototyping, API integration, agentic architecture, retrieval approach, quality bar for AI output, async-first communication, Fintech, AI/ML</t>
+          <t>inventory management, capacity planning, supply chain analytics, data science collaboration, A/B testing, OKRs, Snowflake, Mixpanel, algorithmic decision‑making</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2351,24 +1748,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Ingram Micro</t>
+          <t>Recrew AI</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Assistant Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2377,26 +1774,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 1‑year minimum but lacks many vendor‑focused keywords, lowering the ATS score; the biggest gap is the absence of vendor management/contract negotiation terms.</t>
+          <t>The resume meets the 4-year experience requirement and title level, but lacks many JD-specific keywords and domain experience in accounting/tax, leading to a modest ATS score and moderate job fit.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>vendor management, contract negotiation, invoice reconciliation, marketing training, lifecycle solutions, cloud solutions, commerce platforms</t>
+          <t>CPA, tax workflow, low-code prototyping, API integration, agentic architecture, retrieval approach, quality bar for AI output, async-first communication, Fintech, AI/ML</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2419,50 +1814,50 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>Clari5 - A Perfios Company</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Wealth Management Product Manager</t>
+          <t>AML Product Manager – KYC, Transaction Monitoring, Analytics, Reporting</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is low due to limited overlap with wealth‑management specific keywords, while the most notable missing keyword is "advisor efficiency".</t>
+          <t>The JD expects 8-12 years of AML experience, but the candidate has only 4 years, triggering the hard rule that forces both scores below 30; the resume also lacks core AML keywords such as 'transaction monitoring' and 'FATF'.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>advisor efficiency, client‑facing digital platform, wealth management, financial advisor, client experience metrics, A/B testing, OKRs</t>
+          <t>transaction monitoring, AML detection frameworks, FATF guidelines, risk-based monitoring, CAMS certification, Actimize, SQL data modeling</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2480,7 +1875,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -2490,19 +1885,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro</t>
+          <t>ULTISOURCE</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - inverters &amp; Converters</t>
+          <t>Product Owner / Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2513,22 +1908,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume passes the hard rules but contains few power‑electronics keywords and limited domain relevance, resulting in low ATS and fit scores; the biggest gap is the absence of core product terms like AC‑DC converters.</t>
+          <t>Hard rules apply because the JD requires 6‑10 years experience, exceeding the candidate's 4 years, so both scores are forced below 30; the resume also lacks key fintech terminology such as "Digital Banking" and "Backlog Management".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AC‑DC converters, DC‑DC converters, EV chargers, inverters, energy storage systems, market sizing, competitive benchmarking, product roadmap</t>
+          <t>Digital Banking, User Story Creation, Backlog Management, Release Planning, Roadmap Acceleration, Financial Services domain, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2546,29 +1941,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Clari5 - A Perfios Company</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>AML Product Manager – KYC, Transaction Monitoring, Analytics, Reporting</t>
+          <t>Frimwide P&amp;A Innovation &amp; Transformation Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2582,19 +1977,19 @@
         <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD expects 8-12 years of AML experience, but the candidate has only 4 years, triggering the hard rule that forces both scores below 30; the resume also lacks core AML keywords such as 'transaction monitoring' and 'FATF'.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit financial analytics terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>transaction monitoring, AML detection frameworks, FATF guidelines, risk-based monitoring, CAMS certification, Actimize, SQL data modeling</t>
+          <t>financial forecasting, regulatory reporting, roadmap development, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2617,24 +2012,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Idyllic Services</t>
+          <t>Emergent</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2655,12 +2050,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 15+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30. The most important keyword gap is the lack of any cloud or banking domain terms such as AWS, Java, Spring Boot, or React.</t>
+          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key conversion and monetization terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>AWS, Java, Spring Boot, React, Banking domain, API integration patterns, DPIA/GDPR, Enterprise architecture</t>
+          <t>A/B testing, conversion funnel, LTV, churn reduction, growth experimentation, OKRs, Mixpanel, PLG, customer insight loop, pricing strategy</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2683,50 +2078,50 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Guidewire Software</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Release Engineering</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key release‑engineering terminology such as "CI/CD", "DevOps", and "release velocity".</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>CI/CD, DevOps, release velocity, KPIs, cloud hosting</t>
+          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2740,28 +2135,28 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Emergent</t>
+          <t>Talent Corner HR Services Pvt Ltd</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -2771,7 +2166,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -2780,19 +2175,19 @@
         <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key conversion and monetization terminology.</t>
+          <t>The JD requires 5+ years of product design experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any hardware or agricultural product design terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, conversion funnel, LTV, churn reduction, growth experimentation, OKRs, Mixpanel, PLG, customer insight loop, pricing strategy</t>
+          <t>hardware product design, agri‑infrastructure, greenhouse systems, field research, SOP creation, QA/QC systems, mechanical engineering</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2806,7 +2201,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -2820,24 +2215,24 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>nVent</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - API Services, Stakeholder Management</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
@@ -2853,12 +2248,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of experience but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "voice of the customer" and "product line strategy".</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key service‑product terms.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>voice of the customer (VOC), product line strategy, roadmap implementation, value proposition, networking and data center infrastructure</t>
+          <t>service roadmap, customer success, operational impact, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2872,59 +2267,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Saint-Gobain Group in India</t>
+          <t>Electronic Arts (EA)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER</t>
+          <t>Knowledge Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is low due to minimal keyword overlap with the polymer/film focus of the JD. The biggest keyword gap is the lack of any GTM or technical marketing terms.</t>
+          <t>The JD requires 8+ years of product/knowledge management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several core knowledge‑management keywords.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>GTM strategy, QFD, technical documentation, B2B sales cycle, marketing automation, product brochures</t>
+          <t>knowledge management strategy, taxonomy, metadata governance, serviceNow, confluence, operational knowledge assets, process definition, AI‑assisted support</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2938,33 +2333,33 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Penguin Ai</t>
+          <t>Advance Auto Parts India (India Innovation Center)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product owner - Payment Integrity</t>
+          <t>IT Product Manager (Workday Functional Consultant)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2975,22 +2370,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many generic product management keywords but lacks healthcare‑payment integrity specific terms, leading to moderate ATS score and lower fit score due to domain mismatch.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no &gt;4 year requirement). ATS score is low because the resume lacks core Workday/HRIS keywords and title alignment; the biggest gap is missing Workday-specific terminology.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>payment integrity, claims workflow, denials management, operational automation, AI/ML integration, roadmap planning, prior authorization</t>
+          <t>Workday, HRIS, Recruiting, Core Compensation, Business Process changes, System configuration, Implementation methodology</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3008,55 +2403,55 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Americas Securities settlements &amp; Confirmations</t>
+          <t>Product Owner, Data</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience matches the unspecified minimum). ATS score is low due to missing many finance‑specific keywords and limited title alignment; the biggest keyword gap is the lack of any securities‑settlements or DTCC terminology.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks several domain-specific terms (e.g., KYC, cards, risk, compliance) resulting in a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Securities settlements, DTCC, OKRs, UX testing, production stability, performance monitoring, financial regulatory compliance, risk management</t>
+          <t>KYC, risk and compliance, AWS or Azure, Python, API design, roadmap</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3070,59 +2465,59 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>AvenuesHR Consulting</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner – Virtual Accounts</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
+          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key virtual‑account and fintech terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>Virtual Accounts, cash management, treasury services, KYC/AML, payment platforms</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3136,747 +2531,21 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>hackajob</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Payments</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Talent Corner HR Services Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product design experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any hardware or agricultural product design terminology.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>hardware product design, agri‑infrastructure, greenhouse systems, field research, SOP creation, QA/QC systems, mechanical engineering</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>JPMorganChase</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Vice President - Product Manager - Machine Learning &amp; Intelligent Operations</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The JD explicitly requires 6+ years of AI/ML product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'machine learning'.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>machine learning, model governance, risk and compliance, AI strategy, product roadmap, customer contact reduction</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>hackajob</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - Account Opening</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as 'product strategy' and 'market research'.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>product strategy, market research, product backlog, key success metrics, AI native features, scalability</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>hackajob</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Vice President - Product Manager - Machine Learning &amp; Intelligent Operations</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 6+ years of technical product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'model governance' and 'risk compliance'.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>model governance, risk compliance, AI/ML product strategy, OKRs, A/B testing, customer contact reduction</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Giggso</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key data‑governance terminology.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>data governance, metadata management, data lineage, data lake, ETL tools, cloud data services, AI‑powered automation</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>hackajob</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner, Data</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks several domain-specific terms (e.g., KYC, cards, risk, compliance) resulting in a moderate ATS score and a lower fit due to domain mismatch.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>KYC, risk and compliance, AWS or Azure, Python, API design, roadmap</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Hempel A/S</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Finance Product Owner, PtP</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks finance/ERP terminology and the title does not align with Finance Product Owner, resulting in low keyword density and poor domain fit; the biggest gap is missing ERP/finance process keywords.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>ERP, Procure-to-Pay (PtP), SOP, process automation, finance transformation, change request management, training and coaching</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Sulzer</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner / Business Analyst LeanIX</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied, but the resume lacks most of the JD's core tools and platform terms, resulting in a low ATS match; the biggest keyword gap is the absence of any LeanIX/ServiceNow experience.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>LeanIX, ServiceNow, Azure DevOps, API integration, IT portfolio governance, dashboard creation, metadata governance</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>PTC</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Manager-Consultant</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>The resume lacks many JD-specific technical keywords and the candidate is based in Bangalore while the role is in Pune, resulting in low ATS and fit scores; the most important keyword gap is the absence of any mention of IDE tooling (e.g., VS Code, IntelliJ) and language bindings (C++, Java, Python).</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>C++, Java, JavaScript, VBA, Python, VS Code, IntelliJ, SDK, API design governance, CMake, Maven, Gradle, npm</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Valeo</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner- Front Camera</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires a minimum of 5+ years of front‑camera experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key automotive and ADAS terminology.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>ADAS, Front Camera, AEB, Traffic Sign Recognition, HIL testing, DOORS, ISO 26262, CAN-FD, FOTA</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -3897,17 +2566,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-19
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - ATLAS Program (SAP Global Cloud Operations)</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -583,22 +583,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a strong ATS score; the main gap is missing specific process frameworks like OKRs and RICE.</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, Snowflake, NPS improvement</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,29 +616,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Aspire</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Local Payments</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,26 +647,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year minimum and location requirement, and contains many JD keywords, yielding a strong ATS score; however, the candidate lacks direct payments and fintech experience, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains most of the core product management keywords, but lacks several JD‑specific terms such as market research and user testing, lowering the ATS score; domain mismatch with fintech reduces the fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>payments, transaction management, risk management, regulatory compliance, A/B testing, OKRs, marketplace dynamics</t>
+          <t>market research, user testing, A/B testing, OKRs, financial product decisioning, risk modeling, core metrics tracking, product analytics (e.g., Mixpanel), cross‑functional data science collaboration</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,19 +687,19 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>GoodScore</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -720,19 +718,19 @@
         <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many of the JD keywords, but lacks several core product‑management artifacts and analytics tools, lowering the ATS score; the biggest gap is the absence of explicit PRD/OKR/A‑B testing terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>Product Requirement Document (PRD), OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, customer insights, user research</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +748,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>DigiCert</t>
+          <t>GreedyGame</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,24 +779,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks domain-specific experience in DNS/cloud networking, which lowers the fit score.</t>
+          <t>The candidate meets the years and title requirements, but the resume lacks several B2C‑focused keywords (e.g., A/B testing, Python, Google Analytics) reducing the ATS score; overall domain and skill alignment is solid, giving a good fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>AWS, Azure, GCP, DNS, MLOps, cloud-native, A/B testing, telemetry, inference pipelines</t>
+          <t>A/B testing, Python, Google Analytics, Mixpanel, conversion rate optimization, retention metrics, competitor analysis, market analysis</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pice®</t>
+          <t>Revenera</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Credit Flow</t>
+          <t>Product Owner Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -847,26 +847,24 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
+          <t>The resume meets the basic hard rules and matches many core skills, but lacks several JD-specific terms such as software monetization and licensing, lowering the ATS score; the most important keyword gap is 'software monetization'.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
+          <t>software monetization, licensing, entitlement management, usage analytics, cloud, on-premises, product roadmap, OKRs, customer voice, release management</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -889,24 +887,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Jack &amp; Jill</t>
+          <t>DigiCert</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-II (40–50 LPA + Equity) at AI-native creative intelligence startup</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,26 +913,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, so hard rules do not penalize the scores; the resume contains many JD keywords but lacks several core terms like LLM and marketing, leading to a solid ATS score but moderate job‑fit.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks domain-specific experience in DNS/cloud networking, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>LLM, agentic workflows, creative analysis, marketing, AdTech, A/B testing, OKRs, NPS improvement</t>
+          <t>AWS, Azure, GCP, DNS, MLOps, cloud-native, A/B testing, telemetry, inference pipelines</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,55 +948,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Caterpillar Inc.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Python or SQL</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap but missing key tools like Python and advanced Excel; fit score is limited by domain mismatch despite strong SaaS and GenAI experience.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS, travel, FMCG) does not align closely with Caterpillar's mining technology focus, lowering the fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Python, advanced Excel, pivot tables, statistical analysis, A/B testing, OKRs</t>
+          <t>OKRs, RICE prioritization, A/B testing, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,55 +1014,57 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
+          <t>Jack &amp; Jill</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager-II (40–50 LPA + Equity) at AI-native creative intelligence startup</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+          <t>The candidate meets the 4‑year experience requirement, so hard rules do not penalize the scores; the resume contains many JD keywords but lacks several core terms like LLM and marketing, leading to a solid ATS score but moderate job‑fit.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+          <t>LLM, agentic workflows, creative analysis, marketing, AdTech, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1080,61 +1078,61 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dr. Reddy's Laboratories</t>
+          <t>Pice®</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Oncology</t>
+          <t>Product Manager - Credit Flow</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS/GenAI) does not align with oncology/pharma, lowering the fit score.</t>
+          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>oncology, pharmaceutical market analysis, clinical trial workflow, regulatory compliance, go-to-market strategy, KPIs such as NPS or market share growth, A/B testing</t>
+          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,33 +1146,33 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>Jade Global</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Technical Product Manager (TPM)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1183,24 +1181,26 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F11" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no &gt;5 year requirement) and contains many relevant keywords, but lacks several JD-specific terms and exact location match, leading to a solid ATS score but only moderate fit.</t>
+          <t>The candidate meets the 4‑year experience requirement and has strong keyword overlap (Jira, Agile, Figma, backlog, hypercare) but lacks ServiceNow‑specific terms, keeping the ATS score solid but not top tier; the biggest gap is the missing ServiceNow platform experience.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, NPS improvement, go-to-market strategy, customer segmentation, user satisfaction metrics</t>
+          <t>ServiceNow, ServiceNow Agile, Claude (AI‑assisted design tool), L1 and L2 solutioning, OKRs, incident triage, risk reporting</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1218,55 +1218,55 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Fundtec</t>
+          <t>Soho Square Solutions</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (IT Product)</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and title level, so hard rules do not penalize; it contains most JD keywords but lacks several tool and technology mentions, lowering the ATS score. The strongest keyword gap is the absence of "Trello"/"Confluence" and cloud/API related terms.</t>
+          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Trello, Confluence, cloud technologies, API integration, DevOps, security compliance, OKRs, A/B testing</t>
+          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1280,59 +1280,61 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Allianz Technology</t>
+          <t>Zeta</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Agile Product Owner_D2741</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
+          <t>The candidate meets the years requirement and title level, but the resume lacks many fintech‑specific terms from the JD, lowering both scores.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
+          <t>Card Management, Transaction Experience, Spend Insights, Risk Controls, SDK, mobile app, KPIs, product roadmap, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1346,87 +1348,421 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Dr. Reddy's Laboratories</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager</t>
+          <t>Product Manager - Oncology</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS/GenAI) does not align with oncology/pharma, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>oncology, pharmaceutical market analysis, clinical trial workflow, regulatory compliance, go-to-market strategy, KPIs such as NPS or market share growth, A/B testing</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>IFS</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Outbound Product Manager, Demo Architect - IFS Loops</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
           <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="2" t="n">
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume covers most core product and AI keywords but lacks demo‑environment and cloud‑infrastructure terms, lowering the ATS score. Overall fit is good given strong GenAI and SaaS experience.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>demo environment, cost optimization, cloud infrastructure (AWS/Azure/GCP), CI/CD pipelines, observability / monitoring</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Abacus Insights</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G16" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience vs 3 required) and contains many core keywords, but lacks several domain‑specific terms such as healthcare and cloud data platform, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>healthcare data, cloud data platform, data engineering, roadmap management, go-to-market strategy, story grooming, design reviews, sunset planning, decision workflows</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group - India</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap (Jira, SQL, Agile, stakeholder management) but missing key JD terms like OKRs and ROI. Fit score is lower because the candidate's domain (SaaS, travel, renewable energy) does not directly align with HSBC's banking digital products.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, ROI, market research, user research, product backlog</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and the title is comparable, yielding a decent ATS score, but it lacks many education‑specific keywords and domain experience, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>product backlog, product vision, education market, UK education sector, storytelling, technical liaison, OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Allianz Technology</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Agile Product Owner_D2741</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Zendesk</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3+ years requirement and has a relevant SaaS background, but the resume lacks many observability-specific keywords, lowering the ATS score; the biggest gap is missing terms like logging, tracing, and Grafana.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>observability, logging, tracing, Grafana, Prometheus, OpenTelemetry, runbooks</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -1445,6 +1781,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1456,7 +1797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1621,19 +1962,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>smallcase</t>
+          <t>Lokal</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 1- MF</t>
+          <t>Product Manager I/II</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1647,19 +1988,19 @@
         <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, but lacks many fintech‑specific keywords, lowering the ATS score; the biggest gap is the absence of mutual‑fund/fintech terminology.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is moderate due to limited overlap with the JD's sparse keyword set, while the fit score reflects some relevance in AI and SaaS but limited domain alignment with Lokal's local‑marketplace focus.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mutual Funds, Fintech, Mixpanel, Amplitude, Investor behavior, Roadmap, Pod ownership, Capital markets</t>
+          <t>local-language content, two-sided marketplace, user acquisition metrics, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1677,29 +2018,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>EnglishBhashi</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Inventory Purchasing and Positioning</t>
+          <t>Associate Product Manager(APM)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1710,22 +2051,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). ATS score is moderate due to good keyword overlap on Agile, Jira, stakeholder management but missing core inventory and supply‑chain terms. Fit score is lower because the candidate's SaaS/GenAI background does not align closely with Target's inventory purchasing and positioning domain.</t>
+          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>inventory management, capacity planning, supply chain analytics, data science collaboration, A/B testing, OKRs, Snowflake, Mixpanel, algorithmic decision‑making</t>
+          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1743,29 +2084,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Recrew AI</t>
+          <t>PW (PhysicsWallah)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1776,22 +2117,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and title level, but lacks many JD-specific keywords and domain experience in accounting/tax, leading to a modest ATS score and moderate job fit.</t>
+          <t>Hard rules pass (4 years meets the 2‑year minimum). ATS score is low because key JD terms like A/B testing, DAU/MAU, and engagement metrics are missing; fit score is moderate due to domain mismatch despite solid SaaS experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>CPA, tax workflow, low-code prototyping, API integration, agentic architecture, retrieval approach, quality bar for AI output, async-first communication, Fintech, AI/ML</t>
+          <t>A/B testing, DAU, MAU, engagement metrics, retention, habit formation, growth team collaboration, user behavior analysis</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1809,29 +2150,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Clari5 - A Perfios Company</t>
+          <t>MRI Software</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>AML Product Manager – KYC, Transaction Monitoring, Analytics, Reporting</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1852,12 +2193,12 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD expects 8-12 years of AML experience, but the candidate has only 4 years, triggering the hard rule that forces both scores below 30; the resume also lacks core AML keywords such as 'transaction monitoring' and 'FATF'.</t>
+          <t>The JD title includes 'Senior', triggering hard rule 3, so both scores must be below 30 regardless of experience or keyword overlap; the most important missing keyword is 'product pricing strategy'.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>transaction monitoring, AML detection frameworks, FATF guidelines, risk-based monitoring, CAMS certification, Actimize, SQL data modeling</t>
+          <t>product pricing strategy, OKRs, Jobs-to-be-Done, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1875,29 +2216,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ULTISOURCE</t>
+          <t>GE HealthCare</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner / Product Manager</t>
+          <t>Product Manager, IB Upgrade - South India</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1911,19 +2252,19 @@
         <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules apply because the JD requires 6‑10 years experience, exceeding the candidate's 4 years, so both scores are forced below 30; the resume also lacks key fintech terminology such as "Digital Banking" and "Backlog Management".</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key JD terms like 'Salesforce' and 'pricing strategy'.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Digital Banking, User Story Creation, Backlog Management, Release Planning, Roadmap Acceleration, Financial Services domain, OKRs, A/B testing, NPS improvement</t>
+          <t>Salesforce, pricing strategy, solution selling, KPI-driven performance management, medical imaging</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1941,29 +2282,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Tieto</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Frimwide P&amp;A Innovation &amp; Transformation Product Manager</t>
+          <t>Product Owner- 5G RAN- Tieto Tech Consulting (m/f/d)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1977,19 +2318,19 @@
         <v>25</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit financial analytics terminology.</t>
+          <t>The JD requires 8-14 years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks many core JD keywords such as '5G', 'RAN', and specific telecom terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>financial forecasting, regulatory reporting, roadmap development, OKRs, Snowflake</t>
+          <t>5G, RAN, telecom, network slicing, Lean portfolio management, OKRs, capacity planning</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2007,29 +2348,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Emergent</t>
+          <t>ULTISOURCE</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner / Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2050,12 +2391,12 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key conversion and monetization terminology.</t>
+          <t>Hard rules apply because the JD requires 6‑10 years experience, exceeding the candidate's 4 years, so both scores are forced below 30; the resume also lacks key fintech terminology such as "Digital Banking" and "Backlog Management".</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, conversion funnel, LTV, churn reduction, growth experimentation, OKRs, Mixpanel, PLG, customer insight loop, pricing strategy</t>
+          <t>Digital Banking, User Story Creation, Backlog Management, Release Planning, Roadmap Acceleration, Financial Services domain, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2073,29 +2414,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>YASH Technologies</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner Job</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2104,24 +2445,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several key JD terms such as "product strategy" and "key success metrics".</t>
+          <t>The JD explicitly requires 7+ years of experience, which violates the hard rule for a candidate with only 4 years, forcing both scores below 30; the biggest keyword gap is the lack of explicit mention of 'CSPO certification'.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product vision, key success metrics, market research, OKRs</t>
+          <t>CSCS/CSPO certification, Data Warehouse, Snowflake, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2139,29 +2482,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Talent Corner HR Services Pvt Ltd</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Vice President) - Global Customer Platform</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2175,19 +2518,19 @@
         <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product design experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any hardware or agricultural product design terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>hardware product design, agri‑infrastructure, greenhouse systems, field research, SOP creation, QA/QC systems, mechanical engineering</t>
+          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2205,7 +2548,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2215,7 +2558,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2614,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -2281,19 +2624,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Electronic Arts (EA)</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Knowledge Product Manager</t>
+          <t>Vice President - Product Manager - Machine Learning &amp; Intelligent Operations</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2314,12 +2657,12 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of product/knowledge management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks several core knowledge‑management keywords.</t>
+          <t>The JD requires 6+ years of technical product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'model governance' and 'risk compliance'.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>knowledge management strategy, taxonomy, metadata governance, serviceNow, confluence, operational knowledge assets, process definition, AI‑assisted support</t>
+          <t>model governance, risk compliance, AI/ML product strategy, OKRs, A/B testing, customer contact reduction</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2337,17 +2680,17 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -2403,7 +2746,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -2413,7 +2756,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2768,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Data</t>
+          <t>Product Owner- Technology</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2436,22 +2779,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>59</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks several domain-specific terms (e.g., KYC, cards, risk, compliance) resulting in a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>Hard rules are satisfied; however the resume lacks many core CLM and banking-specific terms (e.g., KYC, regulatory compliance) and does not mention Pune location, resulting in a modest ATS score and a moderate fit score.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>KYC, risk and compliance, AWS or Azure, Python, API design, roadmap</t>
+          <t>KYC, regulatory compliance, CLM (Contract Lifecycle Management), screening, API integration, risk &amp; control partnership, product roadmap, backlog refinement</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2474,50 +2817,50 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>AvenuesHR Consulting</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Virtual Accounts</t>
+          <t>Product Owner, Data</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key virtual‑account and fintech terminology.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks several domain-specific terms (e.g., KYC, cards, risk, compliance) resulting in a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Virtual Accounts, cash management, treasury services, KYC/AML, payment platforms</t>
+          <t>KYC, risk and compliance, AWS or Azure, Python, API design, roadmap</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2535,17 +2878,215 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Aumni</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'Confluence'.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, AI/ML platform experience, OKRs, A/B testing, Roadmap planning</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The most important keyword gap is the lack of any mention of migration to Java/Spring Boot stack.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, API development, migration planning, backward compatibility</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>AvenuesHR Consulting</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Domestic Payments -Product Owner</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The resume also lacks core payment‑domain keywords such as 'Virtual Accounts' and 'Real Time Payments'.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Virtual Accounts, Automated Clearing House, Real Time Payments, KYC/AML, cash management, treasury services, payment platform, reconciliation, liquidity optimization</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -2566,6 +3107,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-20
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Whatfix</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>AI Product Manager 2 : 19487</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -581,24 +581,26 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F2" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>85</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
+          <t>The candidate meets the 3‑year minimum and location requirement; the resume contains most core JD keywords but lacks several product‑specific terms, leading to a solid but not perfect ATS score. Strong GenAI and SaaS experience drives a high fit score.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
+          <t>ScreenSense, AI-native assistant, Product Analytics, Real-time guidance, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,19 +623,19 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Fam</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -652,19 +654,19 @@
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains most of the core product management keywords, but lacks several JD‑specific terms such as market research and user testing, lowering the ATS score; domain mismatch with fintech reduces the fit score.</t>
+          <t>The candidate meets the 4+ years requirement and has a closely related title, but several JD-specific tools and frameworks are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of Mixpanel or A/B testing.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>market research, user testing, A/B testing, OKRs, financial product decisioning, risk modeling, core metrics tracking, product analytics (e.g., Mixpanel), cross‑functional data science collaboration</t>
+          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -687,50 +689,52 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GoodScore</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Analyst (Product Owner, End to end product mgt, Stakeholder Management, Agile Execution, Jira, AI‑assisted Product Support) (3-5 years experience)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F4" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many of the JD keywords, but lacks several core product‑management artifacts and analytics tools, lowering the ATS score; the biggest gap is the absence of explicit PRD/OKR/A‑B testing terminology.</t>
+          <t>The candidate meets the 3‑year minimum and has a matching location and MBA, so no hard rule penalty; the resume covers most core JD keywords but lacks specific platform and process terms.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Product Requirement Document (PRD), OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, customer insights, user research</t>
+          <t>Icertis, Contract Lifecycle Management (CLM), sales enablement, backlog grooming, wiki documentation, AI‑assisted product support, OKRs</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,29 +752,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GreedyGame</t>
+          <t>Porter</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -780,25 +784,25 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and title requirements, but the resume lacks several B2C‑focused keywords (e.g., A/B testing, Python, Google Analytics) reducing the ATS score; overall domain and skill alignment is solid, giving a good fit score.</t>
+          <t>The candidate meets the 4-year experience requirement and has strong keyword overlap, but lacks several JD-specific terms like OKRs and A/B testing, which lowers the ATS score slightly.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Python, Google Analytics, Mixpanel, conversion rate optimization, retention metrics, competitor analysis, market analysis</t>
+          <t>OKRs, A/B testing, impact sizing, go-to-market planning, backlog management, metrics-driven monitoring</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -821,24 +825,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Revenera</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +853,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic hard rules and matches many core skills, but lacks several JD-specific terms such as software monetization and licensing, lowering the ATS score; the most important keyword gap is 'software monetization'.</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>software monetization, licensing, entitlement management, usage analytics, cloud, on-premises, product roadmap, OKRs, customer voice, release management</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,29 +886,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DigiCert</t>
+          <t>Stellantis</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Mid Product Manager(7-10 Years of experience in B2B consumer /software product)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,22 +919,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>69</v>
-      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks domain-specific experience in DNS/cloud networking, which lowers the fit score.</t>
+          <t>The resume meets the experience requirement (4 years) and contains many core keywords, but lacks several JD-specific terms like OKRs and metrics, leading to a solid but not top ATS score; the strongest keyword gap is the absence of OKRs.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AWS, Azure, GCP, DNS, MLOps, cloud-native, A/B testing, telemetry, inference pipelines</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization, Jobs-to-be-Done</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,34 +952,34 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Caterpillar Inc.</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -984,19 +988,19 @@
         <v>78</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS, travel, FMCG) does not align closely with Caterpillar's mining technology focus, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains most of the core product management keywords, but lacks several JD‑specific terms such as market research and user testing, lowering the ATS score; domain mismatch with fintech reduces the fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>OKRs, RICE prioritization, A/B testing, NPS improvement, Marketplace dynamics</t>
+          <t>market research, user testing, A/B testing, OKRs, financial product decisioning, risk modeling, core metrics tracking, product analytics (e.g., Mixpanel), cross‑functional data science collaboration</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,29 +1018,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Jack &amp; Jill</t>
+          <t>GoodScore</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-II (40–50 LPA + Equity) at AI-native creative intelligence startup</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,26 +1049,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, so hard rules do not penalize the scores; the resume contains many JD keywords but lacks several core terms like LLM and marketing, leading to a solid ATS score but moderate job‑fit.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many of the JD keywords, but lacks several core product‑management artifacts and analytics tools, lowering the ATS score; the biggest gap is the absence of explicit PRD/OKR/A‑B testing terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>LLM, agentic workflows, creative analysis, marketing, AdTech, A/B testing, OKRs, NPS improvement</t>
+          <t>Product Requirement Document (PRD), OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, customer insights, user research</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,29 +1084,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Pice®</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Credit Flow</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1113,26 +1115,24 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
+          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1150,57 +1150,57 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Jade Global</t>
+          <t>Parspec</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (TPM)</t>
+          <t>Product Manager (AI/ML)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has strong keyword overlap (Jira, Agile, Figma, backlog, hypercare) but lacks ServiceNow‑specific terms, keeping the ATS score solid but not top tier; the biggest gap is the missing ServiceNow platform experience.</t>
+          <t>The candidate meets the hard rules (4 years experience, appropriate title and location) but misses several JD-specific AI product keywords, lowering the ATS score; however, strong GenAI and SaaS experience gives a solid fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, ServiceNow Agile, Claude (AI‑assisted design tool), L1 and L2 solutioning, OKRs, incident triage, risk reporting</t>
+          <t>intelligent document ingestion, AI-driven product matching, classification, agentic workflows, PRD, AI/ML model evaluation, OKRs</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1223,50 +1223,50 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
+          <t>Hiver</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager II- Hybrid</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+          <t>The resume meets the hard‑rule experience requirement and contains many relevant keywords, but several core JD terms (e.g., Gmail integration, shared inbox, helpdesk, NPS) are missing, lowering the ATS score; overall domain and skill alignment is solid, yielding a good fit score.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+          <t>Gmail integration, shared inbox, helpdesk, customer satisfaction (NPS), A/B testing, OKRs, Mixpanel, Snowflake, roadmap management</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1289,52 +1289,52 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Zeta</t>
+          <t>GreedyGame</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and title level, but the resume lacks many fintech‑specific terms from the JD, lowering both scores.</t>
+          <t>The candidate meets the years and title requirements, but the resume lacks several B2C‑focused keywords (e.g., A/B testing, Python, Google Analytics) reducing the ATS score; overall domain and skill alignment is solid, giving a good fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Card Management, Transaction Experience, Spend Insights, Risk Controls, SDK, mobile app, KPIs, product roadmap, OKRs</t>
+          <t>A/B testing, Python, Google Analytics, Mixpanel, conversion rate optimization, retention metrics, competitor analysis, market analysis</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,11 +1348,11 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1362,47 +1362,45 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Dr. Reddy's Laboratories</t>
+          <t>Ralph Lauren</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Oncology</t>
+          <t>Associate Product Manager-1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but the candidate's domain (SaaS/GenAI) does not align with oncology/pharma, lowering the fit score.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement) and contains many relevant keywords, but misses several core data‑product terms, lowering the ATS score; the biggest gap is the lack of explicit KPI and dashboard experience.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>oncology, pharmaceutical market analysis, clinical trial workflow, regulatory compliance, go-to-market strategy, KPIs such as NPS or market share growth, A/B testing</t>
+          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1416,59 +1414,61 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>IFS</t>
+          <t>Propsoch</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Outbound Product Manager, Demo Architect - IFS Loops</t>
+          <t>Data &amp; AI Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F15" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume covers most core product and AI keywords but lacks demo‑environment and cloud‑infrastructure terms, lowering the ATS score. Overall fit is good given strong GenAI and SaaS experience.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several real‑estate‑specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>demo environment, cost optimization, cloud infrastructure (AWS/Azure/GCP), CI/CD pipelines, observability / monitoring</t>
+          <t>real estate data coverage, property scoring system, fair price calculator, AI‑powered extraction pipelines, research tools for buyer decisions, messy dataset handling, structured thinking, SQL advanced analytics</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1491,19 +1491,19 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Abacus Insights</t>
+          <t>Accenture in India</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -1524,19 +1524,19 @@
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience vs 3 required) and contains many core keywords, but lacks several domain‑specific terms such as healthcare and cloud data platform, lowering both scores.</t>
+          <t>The resume meets the 3‑year minimum and title level, but lacks several core JD terms (e.g., Personal Insurance, product backlog) resulting in a moderate ATS score; domain mismatch with insurance lowers the fit score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>healthcare data, cloud data platform, data engineering, roadmap management, go-to-market strategy, story grooming, design reviews, sunset planning, decision workflows</t>
+          <t>Personal Insurance, product backlog, roadmap, human‑centered design, feedback loops</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1550,38 +1550,38 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group - India</t>
+          <t>Ralph Lauren</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager-2</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1597,12 +1597,12 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title is comparable, yielding a decent ATS score, but it lacks many education‑specific keywords and domain experience, lowering the fit score.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, SQL, Power BI, Agile) but misses several JD‑specific terms like KPIs, dashboards, and data‑product metrics, lowering the ATS score. Domain fit is moderate; the candidate excels in SaaS and GenAI but lacks direct data‑product analytics experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>product backlog, product vision, education market, UK education sector, storytelling, technical liaison, OKRs, NPS improvement</t>
+          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1616,42 +1616,44 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Allianz Technology</t>
+          <t>Pice®</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Agile Product Owner_D2741</t>
+          <t>Product Manager - Credit Flow</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F18" s="2" t="n">
         <v>68</v>
       </c>
@@ -1663,12 +1665,12 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) and meets the 4‑year experience rule, but lacks location match and insurance‑specific terms, lowering the ATS score; the biggest keyword gap is the absence of insurance/policy management language.</t>
+          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>policy management, insurance domain, UPI planning, DORA implementation, vendor management, audit evidence gathering, backlog grooming, scrum ceremonies</t>
+          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1682,87 +1684,821 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Zendesk</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Technical Product Manager - Python or SQL</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap but missing key tools like Python and advanced Excel; fit score is limited by domain mismatch despite strong SaaS and GenAI experience.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Python, advanced Excel, pivot tables, statistical analysis, A/B testing, OKRs</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Jade Global</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager (TPM)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and has strong keyword overlap (Jira, Agile, Figma, backlog, hypercare) but lacks ServiceNow‑specific terms, keeping the ATS score solid but not top tier; the biggest gap is the missing ServiceNow platform experience.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>ServiceNow, ServiceNow Agile, Claude (AI‑assisted design tool), L1 and L2 solutioning, OKRs, incident triage, risk reporting</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Soho Square Solutions</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Opella</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner – Horizon</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title seniority, but lacks many JD‑specific terms such as backlog, roadmap, and data‑governance, resulting in a moderate ATS score; the biggest keyword gap is the absence of "backlog" and related Agile delivery language.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>backlog, roadmap, progressive web app (PWA), data governance, master data, market data, release quality metrics, advanced analytics, OKRs</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Zeta</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager I</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the years requirement and title level, but the resume lacks many fintech‑specific terms from the JD, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Card Management, Transaction Experience, Spend Insights, Risk Controls, SDK, mobile app, KPIs, product roadmap, OKRs</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>IFS</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Outbound Product Manager, Demo Architect - IFS Loops</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume covers most core product and AI keywords but lacks demo‑environment and cloud‑infrastructure terms, lowering the ATS score. Overall fit is good given strong GenAI and SaaS experience.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>demo environment, cost optimization, cloud infrastructure (AWS/Azure/GCP), CI/CD pipelines, observability / monitoring</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Abacus Insights</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience vs 3 required) and contains many core keywords, but lacks several domain‑specific terms such as healthcare and cloud data platform, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>healthcare data, cloud data platform, data engineering, roadmap management, go-to-market strategy, story grooming, design reviews, sunset planning, decision workflows</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ACI Worldwide</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G27" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="H27" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4+ years requirement and title level, but lacks key payments domain keywords (e.g., Visa, Mastercard) reducing both ATS and fit scores; the biggest keyword gap is the absence of payment/card network terminology.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Visa, Mastercard, transaction acquiring, payment processing, card network governance, payment platform, payment industry regulations, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Simplify Healthcare</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="G28" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years meets the 2-year minimum). The resume lacks several JD-specific terms like API, schema design, and release planning, lowering the ATS score; domain mismatch with healthcare reduces the fit score.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>API, schema design, data model, release planning, change management, healthcare benefit management, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group - India</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and the title is comparable, yielding a decent ATS score, but it lacks many education‑specific keywords and domain experience, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>product backlog, product vision, education market, UK education sector, storytelling, technical liaison, OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Zendesk</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H30" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>The candidate meets the 3+ years requirement and has a relevant SaaS background, but the resume lacks many observability-specific keywords, lowering the ATS score; the biggest gap is missing terms like logging, tracing, and Grafana.</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>observability, logging, tracing, Grafana, Prometheus, OpenTelemetry, runbooks</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -1786,6 +2522,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1797,7 +2544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1903,12 +2650,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Columbia Sportswear Company</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner (Emerging Brands)</t>
+          <t>Technical Product Manager, LLM/ML Domain</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1919,22 +2666,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches no minimum &gt;4). ATS score is moderate due to good keyword overlap but missing core ecommerce tech terms. Fit score is limited by domain mismatch with ecommerce focus.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>React, Salesforce Commerce Cloud, Amplience CMS, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth, Mixpanel</t>
+          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1952,29 +2699,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Lokal</t>
+          <t>McKinsey &amp; Company</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I/II</t>
+          <t>Product Manager II - Reach &amp; Engagement</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1985,22 +2732,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>55</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is moderate due to limited overlap with the JD's sparse keyword set, while the fit score reflects some relevance in AI and SaaS but limited domain alignment with Lokal's local‑marketplace focus.</t>
+          <t>The resume contains relevant product and AI experience but lacks many JD-specific terms (e.g., Drupal, intranet, citizen development), resulting in a moderate ATS score; overall fit is moderate due to domain differences.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>local-language content, two-sided marketplace, user acquisition metrics, NPS improvement, MAU growth</t>
+          <t>Drupal, microsite, internal intranet, citizen development, AI‑assisted development, prototype, user engagement metrics, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2023,24 +2770,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EnglishBhashi</t>
+          <t>Glomo</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(APM)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2051,22 +2798,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many fintech‑specific keywords (payments, AML, CFT, merchant sales) so ATS relevance is moderate; domain fit is acceptable but missing core payment industry experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
+          <t>cross‑border payments, payment systems, AML compliance, CFT compliance, fintech, merchant sales engagement, negotiation skills, regulatory compliance</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2089,24 +2836,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PW (PhysicsWallah)</t>
+          <t>Lokal</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-2</t>
+          <t>Product Manager I/II</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2117,22 +2864,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2‑year minimum). ATS score is low because key JD terms like A/B testing, DAU/MAU, and engagement metrics are missing; fit score is moderate due to domain mismatch despite solid SaaS experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is moderate due to limited overlap with the JD's sparse keyword set, while the fit score reflects some relevance in AI and SaaS but limited domain alignment with Lokal's local‑marketplace focus.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, DAU, MAU, engagement metrics, retention, habit formation, growth team collaboration, user behavior analysis</t>
+          <t>local-language content, two-sided marketplace, user acquisition metrics, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2150,29 +2897,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>MRI Software</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Technical Product Manager, Observability Domain</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2183,22 +2930,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD title includes 'Senior', triggering hard rule 3, so both scores must be below 30 regardless of experience or keyword overlap; the most important missing keyword is 'product pricing strategy'.</t>
+          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>product pricing strategy, OKRs, Jobs-to-be-Done, A/B testing, Mixpanel</t>
+          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2221,24 +2968,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GE HealthCare</t>
+          <t>Dayforce</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, IB Upgrade - South India</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2247,24 +2994,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key JD terms like 'Salesforce' and 'pricing strategy'.</t>
+          <t>Hard rules are satisfied (4 years meets the 3-year minimum). The resume lacks many JD-specific terms like Access Management and role‑based access, leading to a low ATS keyword match.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, pricing strategy, solution selling, KPI-driven performance management, medical imaging</t>
+          <t>Access Management, role‑based access, security compliance, roadmap planning, OKRs, A/B testing, customer onboarding metrics</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2287,24 +3036,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tieto</t>
+          <t>Tata Communications</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner- 5G RAN- Tieto Tech Consulting (m/f/d)</t>
+          <t>Product Manager (Deputy General Manager)- SMS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2315,22 +3064,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8-14 years of experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks many core JD keywords such as '5G', 'RAN', and specific telecom terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many core product keywords but lacks telecom-specific terms, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>5G, RAN, telecom, network slicing, Lean portfolio management, OKRs, capacity planning</t>
+          <t>SMS routing, A2P messaging, CPaaS platform, pricing models, vendor management, telecom regulations, delivery latency optimization</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2348,29 +3097,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ULTISOURCE</t>
+          <t>EnglishBhashi</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner / Product Manager</t>
+          <t>Associate Product Manager(APM)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2381,22 +3130,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules apply because the JD requires 6‑10 years experience, exceeding the candidate's 4 years, so both scores are forced below 30; the resume also lacks key fintech terminology such as "Digital Banking" and "Backlog Management".</t>
+          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Digital Banking, User Story Creation, Backlog Management, Release Planning, Roadmap Acceleration, Financial Services domain, OKRs, A/B testing, NPS improvement</t>
+          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2414,57 +3163,55 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>YASH Technologies</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner Job</t>
+          <t>FFC Banking Book Business Product Owner- Analyst</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 7+ years of experience, which violates the hard rule for a candidate with only 4 years, forcing both scores below 30; the biggest keyword gap is the lack of explicit mention of 'CSPO certification'.</t>
+          <t>The resume meets the hard‑rule years and location criteria, but it lacks many finance‑specific keywords and domain experience, resulting in a borderline ATS pass and limited fit.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>CSCS/CSPO certification, Data Warehouse, Snowflake, OKRs, A/B testing</t>
+          <t>cloud‑based big data architecture, data governance, data lineage, release management standards, financial risk analysis, Snowflake</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2478,59 +3225,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Lam Research</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Vice President) - Global Customer Platform</t>
+          <t>Product Manager 4</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
+          <t>Hard rules pass (4 years experience), but the resume lacks many semiconductor‑specific terms and senior product ownership language, resulting in low keyword overlap and poor domain fit.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>semiconductor, etch, manufacturability, Plan of Record, Product Option Architecture, supply chain, cost target, performance target</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2544,59 +3291,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>GlobalLogic</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - API Services, Stakeholder Management</t>
+          <t>Technical Product Owner IRC290693</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key service‑product terms.</t>
+          <t>Hard rules pass, but the resume lacks most of the JD's core technical keywords (iPaaS tools, API/REST, Postman, etc.) and the title does not directly match the Technical Product Owner role, resulting in low ATS and moderate fit scores.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>service roadmap, customer success, operational impact, OKRs, A/B testing, NPS improvement</t>
+          <t>Boomi, MuleSoft, Workato, Postman, RESTful APIs, microservices, JSON, XML, low-code platform, React</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2610,38 +3357,38 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Vice President - Product Manager - Machine Learning &amp; Intelligent Operations</t>
+          <t>Product Manager I/II</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -2650,19 +3397,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 6+ years of technical product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'model governance' and 'risk compliance'.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit “AI‑native enterprise talent platform” experience.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>model governance, risk compliance, AI/ML product strategy, OKRs, A/B testing, customer contact reduction</t>
+          <t>AI-native enterprise talent platform, agentic AI, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2676,59 +3423,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Advance Auto Parts India (India Innovation Center)</t>
+          <t>YASH Technologies Middle East</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>IT Product Manager (Workday Functional Consultant)</t>
+          <t>Contractor - Data Analyst(Data Product Owner) Job</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no &gt;4 year requirement). ATS score is low because the resume lacks core Workday/HRIS keywords and title alignment; the biggest gap is missing Workday-specific terminology.</t>
+          <t>The JD demands 7-9 years of experience while the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit accounting domain terms.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Workday, HRIS, Recruiting, Core Compensation, Business Process changes, System configuration, Implementation methodology</t>
+          <t>Accounting workflows, Reconciliations, Accounts Payable, Accounts Receivable, Financial reporting standards, SQL data profiling, Regulatory compliance</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2742,59 +3489,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner- Technology</t>
+          <t>Product Owner-Payments</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; however the resume lacks many core CLM and banking-specific terms (e.g., KYC, regulatory compliance) and does not mention Pune location, resulting in a modest ATS score and a moderate fit score.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any payments ISO messaging terms.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>KYC, regulatory compliance, CLM (Contract Lifecycle Management), screening, API integration, risk &amp; control partnership, product roadmap, backlog refinement</t>
+          <t>ISO 20022 messaging (pacs.008, pacs.009, pacs.004), SWIFT/FED/CHIPS/Target2/CHAPS, sanctions screening, funds control, payment platform migration</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2808,38 +3555,38 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Data</t>
+          <t>Technical Product Manager, Private Cloud Domain</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
@@ -2855,12 +3602,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and passes all hard rules, but lacks several domain-specific terms (e.g., KYC, cards, risk, compliance) resulting in a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>KYC, risk and compliance, AWS or Azure, Python, API design, roadmap</t>
+          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2874,59 +3621,59 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Aumni</t>
+          <t>Zenwork, Inc</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'Confluence'.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on SaaS and Agile tools but missing core payments/AP‑AR terms. The biggest fit gap is the lack of payments and AP/AR experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Confluence, AI/ML platform experience, OKRs, A/B testing, Roadmap planning</t>
+          <t>payments, AP/AR, API, tax automation, compliance, product roadmap, OKRs, U.S. market, payments platform</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2940,7 +3687,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -2949,19 +3696,19 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>Mondee</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2971,28 +3718,28 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The most important keyword gap is the lack of any mention of migration to Java/Spring Boot stack.</t>
+          <t>The JD requires 7‑9 years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "roadmap", "go‑to‑market" and "stakeholder presentations".</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, API development, migration planning, backward compatibility</t>
+          <t>roadmap, go-to-market strategy, stakeholder presentations, Confluence, OKRs</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3006,7 +3753,7 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
@@ -3015,29 +3762,29 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AvenuesHR Consulting</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Domestic Payments -Product Owner</t>
+          <t>Product Manager (Vice President) - Global Customer Platform</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
@@ -3046,47 +3793,643 @@
         <v>25</v>
       </c>
       <c r="G19" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>YASH Technologies</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner Job</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 7+ years of experience, which violates the hard rule for a candidate with only 4 years, forcing both scores below 30; the biggest keyword gap is the lack of explicit mention of 'CSPO certification'.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>CSCS/CSPO certification, Data Warehouse, Snowflake, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Optum India</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - API Services, Stakeholder Management</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 12+ years of product management experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The resume also lacks core payment‑domain keywords such as 'Virtual Accounts' and 'Real Time Payments'.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Virtual Accounts, Automated Clearing House, Real Time Payments, KYC/AML, cash management, treasury services, payment platform, reconciliation, liquidity optimization</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key service‑product terms.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>service roadmap, customer success, operational impact, OKRs, A/B testing, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Advance Auto Parts India (India Innovation Center)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>IT Product Manager (Workday Functional Consultant)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years experience, no senior title, no &gt;4 year requirement). ATS score is low because the resume lacks core Workday/HRIS keywords and title alignment; the biggest gap is missing Workday-specific terminology.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Workday, HRIS, Recruiting, Core Compensation, Business Process changes, System configuration, Implementation methodology</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>GCP Product Manager</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The resume lacks most cloud‑specific keywords and location match, resulting in a low ATS score; the biggest gap is the absence of GCP and landing‑zone experience.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Google Cloud Platform (GCP), Landing Zones, Regulated environment compliance, Risk and control management, Multi‑cloud (AWS, Azure) experience</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>HSBC</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Manager - Product Owner</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The resume lacks most payment‑specific terminology and the title is a level below the target role, resulting in a low ATS match; the biggest gap is the absence of core payments keywords.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Real time payments (RTP), ACH, Virtual Accounts, Cross Border Payments, NPCI, Payment product commercialization, Benefits tracking, Quality management reporting, Market research for payments</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>JPMorganChase</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Chase Travel</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "Lodging", "product roadmap", and "release management".</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Lodging product roadmap, release management, product backlog, OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Creospan Inc.</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner - Custody</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of Azure DevOps (ADO) or custody/asset servicing domain experience.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Azure DevOps (ADO), Custody, Asset Servicing, Securities Settlements, Corporate Actions, Trade Lifecycle, Reconciliation Processes, SWIFT messaging, CSPO / SAFe POPM certification</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Aumni</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'Confluence'.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, AI/ML platform experience, OKRs, A/B testing, Roadmap planning</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="P19" s="2" t="inlineStr">
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The most important keyword gap is the lack of any mention of migration to Java/Spring Boot stack.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, API development, migration planning, backward compatibility</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -3110,6 +4453,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-21
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,12 +567,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Whatfix</t>
+          <t>Pine Labs</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager 2 : 19487</t>
+          <t>AI Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -582,25 +582,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>85</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and location requirement; the resume contains most core JD keywords but lacks several product‑specific terms, leading to a solid but not perfect ATS score. Strong GenAI and SaaS experience drives a high fit score.</t>
+          <t>The candidate meets the 4-year experience requirement and the title aligns with the Associate Product Manager role, yielding strong ATS keyword coverage; the biggest gap is the lack of explicit mention of rapid AI prototyping frameworks like LLMs or A/B testing.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>ScreenSense, AI-native assistant, Product Analytics, Real-time guidance, A/B testing, OKRs, NPS improvement</t>
+          <t>LLMs, A/B testing, OKRs, RICE prioritization, experiment tracking, customer NPS improvement, Mixpanel, agent-based AI</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -623,24 +623,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Fam</t>
+          <t>Thomson Reuters</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -654,19 +654,19 @@
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4+ years requirement and has a closely related title, but several JD-specific tools and frameworks are missing, lowering the ATS score; the strongest keyword gap is the lack of any mention of Mixpanel or A/B testing.</t>
+          <t>The resume meets the 3+ year requirement and matches the Associate Product Manager title, but misses several JD-specific terms such as product roadmap and A/B testing, lowering the ATS score; overall domain and GenAI experience make the candidate a strong fit.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mixpanel, A/B testing, OKRs, RICE prioritization, NPS improvement, MAU growth</t>
+          <t>product roadmap, A/B testing, OKRs, NPS improvement, customer satisfaction metrics</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,29 +689,29 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>Whatfix</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Analyst (Product Owner, End to end product mgt, Stakeholder Management, Agile Execution, Jira, AI‑assisted Product Support) (3-5 years experience)</t>
+          <t>AI Product Manager 2 : 19487</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -722,19 +722,19 @@
         <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum and has a matching location and MBA, so no hard rule penalty; the resume covers most core JD keywords but lacks specific platform and process terms.</t>
+          <t>The candidate meets the 3‑year minimum and location requirement; the resume contains most core JD keywords but lacks several product‑specific terms, leading to a solid but not perfect ATS score. Strong GenAI and SaaS experience drives a high fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Icertis, Contract Lifecycle Management (CLM), sales enablement, backlog grooming, wiki documentation, AI‑assisted product support, OKRs</t>
+          <t>ScreenSense, AI-native assistant, Product Analytics, Real-time guidance, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -762,19 +762,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Porter</t>
+          <t>Building Ventures</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (AI/ML)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -784,25 +784,25 @@
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4-year experience requirement and has strong keyword overlap, but lacks several JD-specific terms like OKRs and A/B testing, which lowers the ATS score slightly.</t>
+          <t>The resume meets the years requirement and contains many relevant AI/GenAI and SaaS keywords, but lacks several JD-specific terms like intelligent document ingestion and AI-driven product matching.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, impact sizing, go-to-market planning, backlog management, metrics-driven monitoring</t>
+          <t>intelligent document ingestion, AI-driven product matching, agentic workflows, cross‑team dependencies, model capabilities</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -825,50 +825,52 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Navi</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Analyst (Product Owner, End to end product mgt, Stakeholder Management, Agile Execution, Jira, AI‑assisted Product Support) (3-5 years experience)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
+          <t>The candidate meets the 3‑year minimum and has a matching location and MBA, so no hard rule penalty; the resume covers most core JD keywords but lacks specific platform and process terms.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
+          <t>Icertis, Contract Lifecycle Management (CLM), sales enablement, backlog grooming, wiki documentation, AI‑assisted product support, OKRs</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -886,29 +888,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Stellantis</t>
+          <t>Porter</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Mid Product Manager(7-10 Years of experience in B2B consumer /software product)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -917,24 +919,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and contains many core keywords, but lacks several JD-specific terms like OKRs and metrics, leading to a solid but not top ATS score; the strongest keyword gap is the absence of OKRs.</t>
+          <t>The candidate meets the 4-year experience requirement and has strong keyword overlap, but lacks several JD-specific terms like OKRs and A/B testing, which lowers the ATS score slightly.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization, Jobs-to-be-Done</t>
+          <t>OKRs, A/B testing, impact sizing, go-to-market planning, backlog management, metrics-driven monitoring</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -962,7 +966,7 @@
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -974,7 +978,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -985,22 +989,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>68</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains most of the core product management keywords, but lacks several JD‑specific terms such as market research and user testing, lowering the ATS score; domain mismatch with fintech reduces the fit score.</t>
+          <t>The resume strongly matches the required keywords and title, meeting all hard rules; however, the candidate's domain experience is more in travel and enterprise SaaS than finance, creating a modest fit gap.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>market research, user testing, A/B testing, OKRs, financial product decisioning, risk modeling, core metrics tracking, product analytics (e.g., Mixpanel), cross‑functional data science collaboration</t>
+          <t>A/B testing, user testing, OKRs, NPS improvement, Mixpanel, metric definition and analysis</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1023,24 +1027,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GoodScore</t>
+          <t>Stellantis</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Mid Product Manager(7-10 Years of experience in B2B consumer /software product)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1054,19 +1058,19 @@
         <v>78</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and contains many of the JD keywords, but lacks several core product‑management artifacts and analytics tools, lowering the ATS score; the biggest gap is the absence of explicit PRD/OKR/A‑B testing terminology.</t>
+          <t>The resume meets the experience requirement (4 years) and contains many core keywords, but lacks several JD-specific terms like OKRs and metrics, leading to a solid but not top ATS score; the strongest keyword gap is the absence of OKRs.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Product Requirement Document (PRD), OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, customer insights, user research</t>
+          <t>OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, RICE prioritization, Jobs-to-be-Done</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1084,24 +1088,24 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HealthEdge</t>
+          <t>Navi</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1120,19 +1124,19 @@
         <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and contains most of the core product management keywords, but lacks several JD‑specific terms such as market research and user testing, lowering the ATS score; domain mismatch with fintech reduces the fit score.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
+          <t>market research, user testing, A/B testing, OKRs, financial product decisioning, risk modeling, core metrics tracking, product analytics (e.g., Mixpanel), cross‑functional data science collaboration</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1150,29 +1154,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Parspec</t>
+          <t>GoodScore</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (AI/ML)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1181,26 +1185,24 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the hard rules (4 years experience, appropriate title and location) but misses several JD-specific AI product keywords, lowering the ATS score; however, strong GenAI and SaaS experience gives a solid fit.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many of the JD keywords, but lacks several core product‑management artifacts and analytics tools, lowering the ATS score; the biggest gap is the absence of explicit PRD/OKR/A‑B testing terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>intelligent document ingestion, AI-driven product matching, classification, agentic workflows, PRD, AI/ML model evaluation, OKRs</t>
+          <t>Product Requirement Document (PRD), OKRs, A/B testing, Mixpanel, Snowflake, NPS improvement, MAU growth, customer insights, user research</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1218,29 +1220,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Hiver</t>
+          <t>Opus Global Services LLC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II- Hybrid</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1251,22 +1253,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard‑rule experience requirement and contains many relevant keywords, but several core JD terms (e.g., Gmail integration, shared inbox, helpdesk, NPS) are missing, lowering the ATS score; overall domain and skill alignment is solid, yielding a good fit score.</t>
+          <t>The resume meets the 2+ years requirement and has relevant GenAI and SaaS experience, but lacks several AI‑agent specific terms, keeping the ATS score moderate; the biggest keyword gap is the absence of NLP and AI‑agent terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Gmail integration, shared inbox, helpdesk, customer satisfaction (NPS), A/B testing, OKRs, Mixpanel, Snowflake, roadmap management</t>
+          <t>NLP, AI agent platform, prompt evaluation, A/B testing, growth metrics, user insights, iterative learning loops, modular architecture</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1289,24 +1291,24 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GreedyGame</t>
+          <t>HealthEdge</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1315,26 +1317,24 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H13" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="H13" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and title requirements, but the resume lacks several B2C‑focused keywords (e.g., A/B testing, Python, Google Analytics) reducing the ATS score; overall domain and skill alignment is solid, giving a good fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many JD keywords and matches location and education, yielding a solid ATS score, but the candidate's domain (travel/FMCG) does not align with healthcare claims, lowering the fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Python, Google Analytics, Mixpanel, conversion rate optimization, retention metrics, competitor analysis, market analysis</t>
+          <t>healthcare regulations, claims administration, AI-enabled tools, backlog prioritization, user-centered design, product roadmap planning</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1352,29 +1352,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Ralph Lauren</t>
+          <t>Parspec</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager-1</t>
+          <t>Product Manager (AI/ML)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1383,24 +1383,26 @@
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F14" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement) and contains many relevant keywords, but misses several core data‑product terms, lowering the ATS score; the biggest gap is the lack of explicit KPI and dashboard experience.</t>
+          <t>The candidate meets the hard rules (4 years experience, appropriate title and location) but misses several JD-specific AI product keywords, lowering the ATS score; however, strong GenAI and SaaS experience gives a solid fit.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing, OKRs, Snowflake</t>
+          <t>intelligent document ingestion, AI-driven product matching, classification, agentic workflows, PRD, AI/ML model evaluation, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1418,7 +1420,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1428,19 +1430,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Propsoch</t>
+          <t>GreedyGame</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Data &amp; AI Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1450,25 +1452,25 @@
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several real‑estate‑specific keywords and domain experience, lowering both scores.</t>
+          <t>The candidate meets the years and title requirements, but the resume lacks several B2C‑focused keywords (e.g., A/B testing, Python, Google Analytics) reducing the ATS score; overall domain and skill alignment is solid, giving a good fit score.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>real estate data coverage, property scoring system, fair price calculator, AI‑powered extraction pipelines, research tools for buyer decisions, messy dataset handling, structured thinking, SQL advanced analytics</t>
+          <t>A/B testing, Python, Google Analytics, Mixpanel, conversion rate optimization, retention metrics, competitor analysis, market analysis</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1486,29 +1488,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Accenture in India</t>
+          <t>Hiver</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager II- Hybrid</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1517,26 +1519,24 @@
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title level, but lacks several core JD terms (e.g., Personal Insurance, product backlog) resulting in a moderate ATS score; domain mismatch with insurance lowers the fit score.</t>
+          <t>The resume meets the hard‑rule experience requirement and contains many relevant keywords, but several core JD terms (e.g., Gmail integration, shared inbox, helpdesk, NPS) are missing, lowering the ATS score; overall domain and skill alignment is solid, yielding a good fit score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Personal Insurance, product backlog, roadmap, human‑centered design, feedback loops</t>
+          <t>Gmail integration, shared inbox, helpdesk, customer satisfaction (NPS), A/B testing, OKRs, Mixpanel, Snowflake, roadmap management</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1564,19 +1564,19 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Ralph Lauren</t>
+          <t>CoinSwitch</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager-2</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1585,24 +1585,26 @@
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F17" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, SQL, Power BI, Agile) but misses several JD‑specific terms like KPIs, dashboards, and data‑product metrics, lowering the ATS score. Domain fit is moderate; the candidate excels in SaaS and GenAI but lacks direct data‑product analytics experience.</t>
+          <t>The candidate meets the 4‑year experience requirement and title seniority rules, but the resume lacks several growth‑focused keywords from the JD, lowering the ATS score; the biggest gap is the absence of explicit growth‑experiment and conversion metrics terminology.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing</t>
+          <t>A/B testing, OKRs, Mixpanel, Snowflake, PLG, NPS improvement, conversion rate optimization, growth experiments, product funnel metrics</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1625,24 +1627,24 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Pice®</t>
+          <t>Revenera</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Credit Flow</t>
+          <t>Product Owner Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1651,26 +1653,24 @@
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
+          <t>The resume meets the basic hard rules and matches many core skills, but lacks several JD-specific terms such as software monetization and licensing, lowering the ATS score; the most important keyword gap is 'software monetization'.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
+          <t>software monetization, licensing, entitlement management, usage analytics, cloud, on-premises, product roadmap, OKRs, customer voice, release management</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1693,24 +1693,24 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>DigiCert</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager - Python or SQL</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1721,22 +1721,22 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap but missing key tools like Python and advanced Excel; fit score is limited by domain mismatch despite strong SaaS and GenAI experience.</t>
+          <t>The resume meets the 4-year experience requirement and contains many JD keywords, yielding a solid ATS score, but lacks domain-specific experience in DNS/cloud networking, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Python, advanced Excel, pivot tables, statistical analysis, A/B testing, OKRs</t>
+          <t>AWS, Azure, GCP, DNS, MLOps, cloud-native, A/B testing, telemetry, inference pipelines</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1754,57 +1754,55 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
           <t>2026-05-17</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Jade Global</t>
+          <t>TELUS Digital</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager (TPM)</t>
+          <t>Product Manager AI</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G20" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H20" s="2" t="n">
-        <v>74</v>
-      </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has strong keyword overlap (Jira, Agile, Figma, backlog, hypercare) but lacks ServiceNow‑specific terms, keeping the ATS score solid but not top tier; the biggest gap is the missing ServiceNow platform experience.</t>
+          <t>The resume meets the 4‑year experience requirement and contains many core keywords, but lacks several JD‑specific terms such as market research and NPS, lowering the ATS score; the strongest gap is the absence of explicit market/competitor analysis language.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, ServiceNow Agile, Claude (AI‑assisted design tool), L1 and L2 solutioning, OKRs, incident triage, risk reporting</t>
+          <t>market research, competitor analysis, customer interviews, NPS, adoption metrics, product roadmap, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1818,59 +1816,59 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many Azure‑specific keywords, lowering the ATS score; the biggest gap is the absence of Azure data‑service terms.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+          <t>Azure Cosmos DB, Azure Data Factory, Azure Synapse Analytics, Azure SQL DB, Azure Fabric, AI Copilot, OKRs, RICE prioritization, NPS improvement</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1884,7 +1882,7 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
@@ -1893,29 +1891,29 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Opella</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner – Horizon</t>
+          <t>Product Manager, Glean Protect (Security &amp; Governance)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1924,19 +1922,19 @@
         <v>68</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title seniority, but lacks many JD‑specific terms such as backlog, roadmap, and data‑governance, resulting in a moderate ATS score; the biggest keyword gap is the absence of "backlog" and related Agile delivery language.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but misses several core JD terms like LLM, security, and governance, lowering the ATS score. Domain and skill overlap are solid but not a perfect match for the security/governance focus.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>backlog, roadmap, progressive web app (PWA), data governance, master data, market data, release quality metrics, advanced analytics, OKRs</t>
+          <t>LLM, APIs, security governance, knowledge management, OKRs, A/B testing, enterprise search</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1950,7 +1948,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -1959,52 +1957,50 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Zeta</t>
+          <t>Ralph Lauren</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Associate Product Manager-1</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and title level, but the resume lacks many fintech‑specific terms from the JD, lowering both scores.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement) and contains many relevant keywords, but misses several core data‑product terms, lowering the ATS score; the biggest gap is the lack of explicit KPI and dashboard experience.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Card Management, Transaction Experience, Spend Insights, Risk Controls, SDK, mobile app, KPIs, product roadmap, OKRs</t>
+          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2018,59 +2014,61 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group</t>
+          <t>Propsoch</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Data &amp; AI Product Manager</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F24" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, but the resume lacks several real‑estate‑specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+          <t>real estate data coverage, property scoring system, fair price calculator, AI‑powered extraction pipelines, research tools for buyer decisions, messy dataset handling, structured thinking, SQL advanced analytics</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2084,59 +2082,59 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>IFS</t>
+          <t>Ralph Lauren</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Outbound Product Manager, Demo Architect - IFS Loops</t>
+          <t>Associate Product Manager-2</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume covers most core product and AI keywords but lacks demo‑environment and cloud‑infrastructure terms, lowering the ATS score. Overall fit is good given strong GenAI and SaaS experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title). The resume covers many core tools (Jira, SQL, Power BI, Agile) but misses several JD‑specific terms like KPIs, dashboards, and data‑product metrics, lowering the ATS score. Domain fit is moderate; the candidate excels in SaaS and GenAI but lacks direct data‑product analytics experience.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>demo environment, cost optimization, cloud infrastructure (AWS/Azure/GCP), CI/CD pipelines, observability / monitoring</t>
+          <t>KPIs, performance dashboards, data product strategy, adoption metrics, A/B testing</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2150,61 +2148,59 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Abacus Insights</t>
+          <t>Pice®</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - Credit Flow</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
         <v>68</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience vs 3 required) and contains many core keywords, but lacks several domain‑specific terms such as healthcare and cloud data platform, lowering both scores.</t>
+          <t>The candidate meets the 1‑year minimum (has 4 years) so hard rules do not penalize; however, key fintech/credit keywords are missing, lowering the ATS score. The biggest gap is lack of credit‑specific experience such as KYC and API integration.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>healthcare data, cloud data platform, data engineering, roadmap management, go-to-market strategy, story grooming, design reviews, sunset planning, decision workflows</t>
+          <t>API integration, KYC flows, lender rules, credit disbursal, Mixpanel, Confluence, Fintech payments</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2218,7 +2214,7 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
@@ -2227,50 +2223,50 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ACI Worldwide</t>
+          <t>Zynga</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager 2</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4+ years requirement and title level, but lacks key payments domain keywords (e.g., Visa, Mastercard) reducing both ATS and fit scores; the biggest keyword gap is the absence of payment/card network terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many JD keywords but lacks gaming‑specific terms, lowering the ATS score. The biggest gap is the absence of mobile gaming and player‑centric metrics.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Visa, Mastercard, transaction acquiring, payment processing, card network governance, payment platform, payment industry regulations, NPS improvement</t>
+          <t>mobile gaming, A/B testing, user acquisition, KPIs, OKRs, Mixpanel, player engagement metrics, live ops</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2284,7 +2280,7 @@
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
@@ -2293,52 +2289,50 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Simplify Healthcare</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager I/II - Platform</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2-year minimum). The resume lacks several JD-specific terms like API, schema design, and release planning, lowering the ATS score; domain mismatch with healthcare reduces the fit score.</t>
+          <t>The resume meets the 2+ year requirement and has no senior title, so hard rules pass; however, it lacks many JD-specific keywords such as Azure, AWS, and agentic AI, lowering the ATS score. The candidate's SaaS and GenAI experience aligns well with the role, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>API, schema design, data model, release planning, change management, healthcare benefit management, NPS improvement</t>
+          <t>Azure, AWS, agentic AI, IL4 compliance, talent acquisition market analysis, OKRs</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2352,7 +2346,7 @@
         </is>
       </c>
       <c r="M28" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
@@ -2361,50 +2355,50 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ParentPay Group - India</t>
+          <t>Groww</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title is comparable, yielding a decent ATS score, but it lacks many education‑specific keywords and domain experience, lowering the fit score.</t>
+          <t>Hard rules pass; title aligns but the JD's fintech and product‑strategy keywords are largely absent, lowering the ATS score. The biggest gap is the lack of fintech‑specific terminology.</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>product backlog, product vision, education market, UK education sector, storytelling, technical liaison, OKRs, NPS improvement</t>
+          <t>fintech, financial services, product strategy, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2418,87 +2412,889 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>TriNet</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 2‑year minimum and title alignment, yielding a strong ATS match; the biggest gap is lack of HR‑specific terminology like OKRs and A/B testing.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, NPS improvement, user feedback loops, product roadmap planning</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Jade Global</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager (TPM)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and has strong keyword overlap (Jira, Agile, Figma, backlog, hypercare) but lacks ServiceNow‑specific terms, keeping the ATS score solid but not top tier; the biggest gap is the missing ServiceNow platform experience.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>ServiceNow, ServiceNow Agile, Claude (AI‑assisted design tool), L1 and L2 solutioning, OKRs, incident triage, risk reporting</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Cendyn</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - AIDLC</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume covers many core product management terms but lacks several AI‑tool specific keywords, lowering the ATS score. The strongest gap is the absence of tool names like Claude or Microsoft Copilot.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Claude, Microsoft Copilot, product roadmap, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Capgemini</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>FBS Product Owner II</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the experience and seniority constraints and includes many core Agile and stakeholder keywords, but lacks several JD-specific terms, lowering the ATS score; the strongest gap is the absence of OKR/RICE prioritization language.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, RICE prioritization, A/B testing, NPS improvement, Program Increment (PI) planning, SAFe framework, Roadmap planning, Metrics-driven decision making</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Soho Square Solutions</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>The resume hits most ATS keywords (Agile, Jira, stakeholder management, user stories) but lacks core Salesforce terms, keeping the score below 80; the candidate’s domain (SaaS/GenAI) is strong but does not directly match the Salesforce CRM focus, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce, Sales Cloud, Service Cloud, Azure DevOps, backlog grooming, release planning, UAT coordination</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Zeta</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager I</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the years requirement and title level, but the resume lacks many fintech‑specific terms from the JD, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Card Management, Transaction Experience, Spend Insights, Risk Controls, SDK, mobile app, KPIs, product roadmap, OKRs</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Opella</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner – Horizon</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title seniority, but lacks many JD‑specific terms such as backlog, roadmap, and data‑governance, resulting in a moderate ATS score; the biggest keyword gap is the absence of "backlog" and related Agile delivery language.</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>backlog, roadmap, progressive web app (PWA), data governance, master data, market data, release quality metrics, advanced analytics, OKRs</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains many JD keywords and meets the 4‑year experience rule, but the candidate lacks direct education‑tech/payments domain experience, lowering the fit score; the most important missing keyword is 'OKRs'.</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, A/B testing, NPS improvement, customer feedback loops, competitive analysis, roadmap definition, market research</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Abacus Insights</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience vs 3 required) and contains many core keywords, but lacks several domain‑specific terms such as healthcare and cloud data platform, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>healthcare data, cloud data platform, data engineering, roadmap management, go-to-market strategy, story grooming, design reviews, sunset planning, decision workflows</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>ACI Worldwide</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4+ years requirement and title level, but lacks key payments domain keywords (e.g., Visa, Mastercard) reducing both ATS and fit scores; the biggest keyword gap is the absence of payment/card network terminology.</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Visa, Mastercard, transaction acquiring, payment processing, card network governance, payment platform, payment industry regulations, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Simplify Healthcare</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass (4 years meets the 2-year minimum). The resume lacks several JD-specific terms like API, schema design, and release planning, lowering the ATS score; domain mismatch with healthcare reduces the fit score.</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>API, schema design, data model, release planning, change management, healthcare benefit management, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>ParentPay Group - India</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and the title is comparable, yielding a decent ATS score, but it lacks many education‑specific keywords and domain experience, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>product backlog, product vision, education market, UK education sector, storytelling, technical liaison, OKRs, NPS improvement</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>Zendesk</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Technical Product Manager</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="2" t="n">
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H42" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>The candidate meets the 3+ years requirement and has a relevant SaaS background, but the resume lacks many observability-specific keywords, lowering the ATS score; the biggest gap is missing terms like logging, tracing, and Grafana.</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>observability, logging, tracing, Grafana, Prometheus, OpenTelemetry, runbooks</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="O42" s="2" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -2533,6 +3329,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2544,7 +3352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2650,12 +3458,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Societe Generale Global Solution Centre</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, LLM/ML Domain</t>
+          <t>Product Owner IT Asset Management - ServiceNow</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2676,12 +3484,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant Agile and stakeholder terms but misses several core ServiceNow/ITSM keywords, lowering the ATS score. The strongest gap is the lack of any mention of ServiceNow or IT Asset Management.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
+          <t>ServiceNow, ITSM, IT Asset Management, Scrum, backlog refinement, release planning, French, RTE, product owner, value chain optimization</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2704,24 +3512,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>McKinsey &amp; Company</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Reach &amp; Engagement</t>
+          <t>Technical Product Manager, Private Cloud Domain</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2732,22 +3540,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume contains relevant product and AI experience but lacks many JD-specific terms (e.g., Drupal, intranet, citizen development), resulting in a moderate ATS score; overall fit is moderate due to domain differences.</t>
+          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Drupal, microsite, internal intranet, citizen development, AI‑assisted development, prototype, user engagement metrics, NPS improvement, MAU growth</t>
+          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2765,17 +3573,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -2831,7 +3639,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -2841,7 +3649,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -2907,19 +3715,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Dayforce</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Observability Domain</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2928,24 +3736,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>Hard rules are satisfied (4 years meets the 3-year minimum). The resume lacks many JD-specific terms like Access Management and role‑based access, leading to a low ATS keyword match.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
+          <t>Access Management, role‑based access, security compliance, roadmap planning, OKRs, A/B testing, customer onboarding metrics</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2963,29 +3773,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dayforce</t>
+          <t>EnglishBhashi</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager(APM)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2994,26 +3804,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years meets the 3-year minimum). The resume lacks many JD-specific terms like Access Management and role‑based access, leading to a low ATS keyword match.</t>
+          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Access Management, role‑based access, security compliance, roadmap planning, OKRs, A/B testing, customer onboarding metrics</t>
+          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -3031,29 +3839,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tata Communications</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Deputy General Manager)- SMS</t>
+          <t>Product Manager, International Emerging Stores Payments</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3064,22 +3872,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>51</v>
-      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product keywords but lacks telecom-specific terms, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many payment‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>SMS routing, A2P messaging, CPaaS platform, pricing models, vendor management, telecom regulations, delivery latency optimization</t>
+          <t>payment processing, instant bank discount solution, payment gateway integration, financial services compliance, roadmap development, OKRs, market trends analysis, senior leadership presentations, cross‑functional alignment with Finance and Legal</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -3102,24 +3910,24 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>EnglishBhashi</t>
+          <t>Mewar Infotech Limited</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(APM)</t>
+          <t>AEM Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -3130,22 +3938,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
+          <t>The resume lacks core AEM and web development keywords and the title does not align with the Product Owner role, resulting in a low ATS score; the candidate's domain experience (GenAI, travel SaaS) only loosely matches the JD, giving a modest fit score.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
+          <t>Adobe Experience Manager (AEM), HTML, CSS, JavaScript, Scrum, backlog management, sprint planning, requirements gathering, stakeholder engagement, Certified Scrum Product Owner</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -3163,29 +3971,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Nokia</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>FFC Banking Book Business Product Owner- Analyst</t>
+          <t>ServiceNow Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3196,22 +4004,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard‑rule years and location criteria, but it lacks many finance‑specific keywords and domain experience, resulting in a borderline ATS pass and limited fit.</t>
+          <t>The resume lacks core ServiceNow and ITSM terminology required by the JD, resulting in a low ATS match; the candidate's SaaS and GenAI experience is relevant but does not align closely with the platform‑owner focus.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>cloud‑based big data architecture, data governance, data lineage, release management standards, financial risk analysis, Snowflake</t>
+          <t>ServiceNow, ITSM, ITOM, CSDM, CMDB, out‑of‑the‑box (OOTB) capabilities, platform governance, AIOps, workflow automation, demand prioritization</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3229,55 +4037,55 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Lam Research</t>
+          <t>Cognizant</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager 4</t>
+          <t>Product Owner (ISG)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience), but the resume lacks many semiconductor‑specific terms and senior product ownership language, resulting in low keyword overlap and poor domain fit.</t>
+          <t>Hard rules are satisfied, but the resume contains few of the fintech‑specific keywords (e.g., Swift, real‑time payments) required by the JD, leading to a low ATS score; domain mismatch reduces the fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>semiconductor, etch, manufacturability, Plan of Record, Product Option Architecture, supply chain, cost target, performance target</t>
+          <t>Swift Payment, real‑time payments, trade finance, cash management, financial compliance, payment messages, SWIFT standards, transaction monitoring</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -3295,17 +4103,17 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -3371,19 +4179,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Eightfold AI</t>
+          <t>PW (PhysicsWallah)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I/II</t>
+          <t>Product Manager-2</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3394,22 +4202,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit “AI‑native enterprise talent platform” experience.</t>
+          <t>Hard rules pass (4 years meets the 2‑year minimum). ATS score is low because key JD terms like A/B testing, DAU/MAU, and engagement metrics are missing; fit score is moderate due to domain mismatch despite solid SaaS experience.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>AI-native enterprise talent platform, agentic AI, OKRs, A/B testing, Snowflake</t>
+          <t>A/B testing, DAU, MAU, engagement metrics, retention, habit formation, growth team collaboration, user behavior analysis</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -3427,34 +4235,34 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>YASH Technologies Middle East</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Contractor - Data Analyst(Data Product Owner) Job</t>
+          <t>Product Manager I/II</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -3470,12 +4278,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD demands 7-9 years of experience while the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit accounting domain terms.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit “AI‑native enterprise talent platform” experience.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Accounting workflows, Reconciliations, Accounts Payable, Accounts Receivable, Financial reporting standards, SQL data profiling, Regulatory compliance</t>
+          <t>AI-native enterprise talent platform, agentic AI, OKRs, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3503,19 +4311,19 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>GE HealthCare</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner-Payments</t>
+          <t>Product Manager, IB Upgrade - South India</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3529,19 +4337,19 @@
         <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any payments ISO messaging terms.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key JD terms like 'Salesforce' and 'pricing strategy'.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>ISO 20022 messaging (pacs.008, pacs.009, pacs.004), SWIFT/FED/CHIPS/Target2/CHAPS, sanctions screening, funds control, payment platform migration</t>
+          <t>Salesforce, pricing strategy, solution selling, KPI-driven performance management, medical imaging</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -3559,55 +4367,55 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Agoda</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager, Private Cloud Domain</t>
+          <t>Product Owner-Payments</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume hits many core keywords (Jira, SQL, Agile, GenAI, RAG, stakeholder management) and the candidate has relevant travel‑tech experience, but it lacks location match and specific private‑cloud deployment terminology, lowering the ATS score; the overall domain fit is moderate.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any payments ISO messaging terms.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>private cloud, deployment orchestration, service reliability, SRE, cost optimization, production monitoring, OKRs</t>
+          <t>ISO 20022 messaging (pacs.008, pacs.009, pacs.004), SWIFT/FED/CHIPS/Target2/CHAPS, sanctions screening, funds control, payment platform migration</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3621,59 +4429,59 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Zenwork, Inc</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Vice President - Product Manager - Managed Solution</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>66</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on SaaS and Agile tools but missing core payments/AP‑AR terms. The biggest fit gap is the lack of payments and AP/AR experience.</t>
+          <t>The JD requires 10+ years of product management experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit AI/ML terminology such as "LLM" or "MLOps".</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>payments, AP/AR, API, tax automation, compliance, product roadmap, OKRs, U.S. market, payments platform</t>
+          <t>LLM, MLOps, prompt engineering, risk and compliance frameworks, executive storytelling, business case development</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3687,7 +4495,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -3696,19 +4504,19 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Mondee</t>
+          <t>Zenwork, Inc</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3724,22 +4532,22 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7‑9 years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "roadmap", "go‑to‑market" and "stakeholder presentations".</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on SaaS and Agile tools but missing core payments/AP‑AR terms. The biggest fit gap is the lack of payments and AP/AR experience.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>roadmap, go-to-market strategy, stakeholder presentations, Confluence, OKRs</t>
+          <t>payments, AP/AR, API, tax automation, compliance, product roadmap, OKRs, U.S. market, payments platform</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3757,29 +4565,29 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>EPAM Systems</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Vice President) - Global Customer Platform</t>
+          <t>Product Manager - User Stories</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3790,22 +4598,22 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
+          <t>The JD requires 10-15 years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of explicit "product roadmap" terminology.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
+          <t>product roadmap, product vision, INVEST user stories, release notes, OKRs</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3823,29 +4631,29 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>YASH Technologies</t>
+          <t>Mondee</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Owner Job</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3854,26 +4662,24 @@
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 7+ years of experience, which violates the hard rule for a candidate with only 4 years, forcing both scores below 30; the biggest keyword gap is the lack of explicit mention of 'CSPO certification'.</t>
+          <t>The JD requires 7‑9 years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "roadmap", "go‑to‑market" and "stakeholder presentations".</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>CSCS/CSPO certification, Data Warehouse, Snowflake, OKRs, A/B testing</t>
+          <t>roadmap, go-to-market strategy, stakeholder presentations, Confluence, OKRs</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3891,29 +4697,29 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - API Services, Stakeholder Management</t>
+          <t>Product Manager (Vice President) - Global Customer Platform</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3927,19 +4733,19 @@
         <v>25</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several key service‑product terms.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit 'product strategy' and 'roadmap' terminology.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>service roadmap, customer success, operational impact, OKRs, A/B testing, NPS improvement</t>
+          <t>product strategy, product roadmap, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3957,29 +4763,29 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Advance Auto Parts India (India Innovation Center)</t>
+          <t>DROGO DRONES</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>IT Product Manager (Workday Functional Consultant)</t>
+          <t>R&amp;D Product Manager – Tethered Drone Systems (UAV)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3990,22 +4796,22 @@
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no &gt;4 year requirement). ATS score is low because the resume lacks core Workday/HRIS keywords and title alignment; the biggest gap is missing Workday-specific terminology.</t>
+          <t>The JD explicitly requires 5+ years of UAV/drone experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks core drone‑specific keywords such as PX4, ArduPilot, and tethered systems.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Workday, HRIS, Recruiting, Core Compensation, Business Process changes, System configuration, Implementation methodology</t>
+          <t>PX4/ArduPilot, tethered drone systems, autonomous flight, payload integration, field testing</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -4023,29 +4829,29 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>GCP Product Manager</t>
+          <t>Technical Product Manager, LLM/ML Domain</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -4056,22 +4862,22 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks most cloud‑specific keywords and location match, resulting in a low ATS score; the biggest gap is the absence of GCP and landing‑zone experience.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords but lacks several JD-specific terms like ML platform and model deployment, leading to a moderate ATS score. The candidate's GenAI and SaaS experience aligns well with the role, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Google Cloud Platform (GCP), Landing Zones, Regulated environment compliance, Risk and control management, Multi‑cloud (AWS, Azure) experience</t>
+          <t>ML platform, LLM ops, model deployment, monitoring, scalability, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -4089,29 +4895,29 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HSBC</t>
+          <t>Agoda</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Manager - Product Owner</t>
+          <t>Technical Product Manager, Observability Domain</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -4122,22 +4928,22 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks most payment‑specific terminology and the title is a level below the target role, resulting in a low ATS match; the biggest gap is the absence of core payments keywords.</t>
+          <t>Hard rules are satisfied; the resume contains many core product management keywords but lacks observability‑specific terms, lowering the ATS score. The candidate's SaaS and GenAI experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Real time payments (RTP), ACH, Virtual Accounts, Cross Border Payments, NPCI, Payment product commercialization, Benefits tracking, Quality management reporting, Market research for payments</t>
+          <t>observability, telemetry, distributed tracing, anomaly detection, alerting, incident management, SRE collaboration</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -4155,29 +4961,29 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>HSBC</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Chase Travel</t>
+          <t>Manager - Product Owner</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -4188,22 +4994,22 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "Lodging", "product roadmap", and "release management".</t>
+          <t>The resume lacks most payment‑specific terminology and the title is a level below the target role, resulting in a low ATS match; the biggest gap is the absence of core payments keywords.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Lodging product roadmap, release management, product backlog, OKRs, NPS improvement</t>
+          <t>Real time payments (RTP), ACH, Virtual Accounts, Cross Border Payments, NPCI, Payment product commercialization, Benefits tracking, Quality management reporting, Market research for payments</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -4221,7 +5027,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -4231,45 +5037,45 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Creospan Inc.</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Custody</t>
+          <t>GCP Product Manager</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of Azure DevOps (ADO) or custody/asset servicing domain experience.</t>
+          <t>The resume lacks most cloud‑specific keywords and location match, resulting in a low ATS score; the biggest gap is the absence of GCP and landing‑zone experience.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Azure DevOps (ADO), Custody, Asset Servicing, Securities Settlements, Corporate Actions, Trade Lifecycle, Reconciliation Processes, SWIFT messaging, CSPO / SAFe POPM certification</t>
+          <t>Google Cloud Platform (GCP), Landing Zones, Regulated environment compliance, Risk and control management, Multi‑cloud (AWS, Azure) experience</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -4287,7 +5093,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -4297,19 +5103,19 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Aumni</t>
+          <t>Danfoss</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager Cybersecurity (m/f/d)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -4320,22 +5126,22 @@
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'Confluence'.</t>
+          <t>The resume lacks core cybersecurity keywords and regulatory standards required by the JD, and the candidate's location and domain do not align; the biggest gap is the absence of any cybersecurity or risk‑assessment terminology.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Confluence, AI/ML platform experience, OKRs, A/B testing, Roadmap planning</t>
+          <t>ISO 27001, IEC 62443, NIS2, threat analysis, risk assessment, cybersecurity, regulatory compliance, product security objectives</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4353,29 +5159,29 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Chase Travel</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -4386,22 +5192,22 @@
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The most important keyword gap is the lack of any mention of migration to Java/Spring Boot stack.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key terms like "Lodging", "product roadmap", and "release management".</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, API development, migration planning, backward compatibility</t>
+          <t>Lodging product roadmap, release management, product backlog, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -4419,17 +5225,215 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Creospan Inc.</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner - Custody</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the lack of any mention of Azure DevOps (ADO) or custody/asset servicing domain experience.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Azure DevOps (ADO), Custody, Asset Servicing, Securities Settlements, Corporate Actions, Trade Lifecycle, Reconciliation Processes, SWIFT messaging, CSPO / SAFe POPM certification</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Aumni</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important missing keyword is 'Confluence'.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, AI/ML platform experience, OKRs, A/B testing, Roadmap planning</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Persistent Systems</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 8+ years of experience, but the candidate has only 4 years, triggering a hard rule; therefore both scores are forced below 30. The most important keyword gap is the lack of any mention of migration to Java/Spring Boot stack.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, API development, migration planning, backward compatibility</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -4462,6 +5466,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-26
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,23 +567,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>peopleHum</t>
+          <t>Phigital Care</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
         <v>78</v>
       </c>
@@ -595,12 +593,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and includes most required keywords, but lacks explicit mentions of roadmap planning, PRDs, and structured customer interview processes.</t>
+          <t>The resume meets the hard rules and contains many relevant keywords, but lacks several cloud and analytics terms from the JD, resulting in a solid but not perfect ATS score; the strongest gap is missing explicit cloud platform experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>roadmap, PRD, customer interviews, OKRs, A/B testing</t>
+          <t>AWS, Azure, GCP, A/B testing, OKRs, NPS improvement, customer surveys, data product development</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -618,55 +616,57 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Solera Holdings, LLC.</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, but the resume lacks several JD‑specific terms such as demand management and usage analytics, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
+          <t>Demand Management, Quarterly planning, Usage analytics, User guides, Release notes</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -689,24 +689,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Zoca</t>
+          <t>Itron, Inc.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,22 +717,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI terms but misses several JD‑specific keywords and the title does not exactly match AI Product Manager.</t>
+          <t>The resume meets the 3+ years requirement and has no senior‑level title conflict; it covers most core keywords but lacks explicit roadmap/backlog and go‑to‑market language.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>AI agent development, ML model optimization, customer outcome metrics, roadmap planning (6‑12 month roadmap), A/B testing, OKRs, NPS improvement, voice AI</t>
+          <t>product roadmap, backlog prioritization, go‑to‑market strategy, product marketing collaboration, customer interviews / discovery</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -755,24 +755,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kobie</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Assisted Service</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,22 +783,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI keywords but lacks several marketplace‑specific terms, lowering the ATS score; the biggest gap is the absence of financial‑services and risk‑management language.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Financial Services, Risk Management, Trust &amp; Safety, AI‑powered decision flows, Customer Support tools, Marketplace dynamics, Two‑sided platform, A/B testing, OKRs</t>
+          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,57 +816,55 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TriNet</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and title alignment, yielding a strong ATS match; the biggest gap is lack of HR‑specific terminology like OKRs and A/B testing.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>OKRs, A/B testing, NPS improvement, user feedback loops, product roadmap planning</t>
+          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -880,28 +878,28 @@
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CoreTek Labs</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -911,13 +909,11 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>68</v>
       </c>
@@ -929,12 +925,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and has relevant GenAI and SaaS experience, but the resume lacks several core JD keywords (e.g., Confluence, A/B testing) and does not explicitly state Hyderabad location, lowering the ATS score.</t>
+          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Confluence, A/B testing, product analytics, NLP, LLMs, OKRs</t>
+          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,87 +944,623 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TekWissen India</t>
+          <t>Zoca</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>71</v>
       </c>
       <c r="H8" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI terms but misses several JD‑specific keywords and the title does not exactly match AI Product Manager.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>AI agent development, ML model optimization, customer outcome metrics, roadmap planning (6‑12 month roadmap), A/B testing, OKRs, NPS improvement, voice AI</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Puravankara Limited</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). The resume covers many Agile and Jira keywords but lacks fintech‑specific terms, lowering the ATS score; the biggest gap is missing credit‑card and OTP related keywords.</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>credit and debit card servicing, OTP authentication, OKRs, release readiness, Go/No‑Go, digital profile management, partner team coordination</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
+      <c r="H9" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title matches, but lacks several JD‑specific terms such as A/B testing and API integration, lowering the ATS score; the biggest keyword gap is the absence of any mention of A/B testing or API work.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>A/B testing, API integration, PRD (Product Requirements Document), product metrics tracking, risk / blocker identification, system workflow documentation, user engagement analysis</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Sabre</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Distribution Data Insights</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-24</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="F10" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks several core JD keywords such as APIs, data ingestion pipelines, and travel‑distribution terminology, lowering the ATS score. Domain experience is strong, especially in travel SaaS and data‑driven product work, yielding a solid fit score.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>APIs, data ingestion pipelines, distribution metrics, travel distribution channels, lodging content, agency partners, data quality metrics, search query analysis, booking data insights</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Golden Opportunities</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru East, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GHX India</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Eltropy</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager – AI &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Franklin Templeton India</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GENAI Product Manager</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core keywords but misses several AI‑product specific terms, lowering the ATS score; overall fit is strong due to GenAI and SaaS experience.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, OKRs, A/B testing, financial services, investment domain, user research, NPS improvement, risk management</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Owner</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title alignment, but lacks several domain‑specific terms from the JD such as PLM and railway product knowledge, leading to moderate ATS and fit scores.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Product Lifecycle Management (PLM), railway solution, legacy product architecture, non‑functional requirements, OKR framework</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>INTANGLES LAB PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several JD‑specific terms such as automobile/fleet domain and explicit acceptance testing language, lowering the ATS score.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>automobile domain, fleet management, definition of done, acceptance testing, release notes, industry trends monitoring</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -1041,6 +1573,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1052,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1209,7 +1749,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -1219,19 +1759,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Tata Communications</t>
+          <t>TOCUMULUS</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Deputy General Manager)- SMS</t>
+          <t>Product Owner / Business Analyst – Ecommerce &amp; Studio Production Platforms</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1242,22 +1782,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many core product keywords but lacks telecom-specific terms, leading to a moderate ATS score and a lower fit due to domain mismatch.</t>
+          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any ecommerce platform or DAM/PIM terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>SMS routing, A2P messaging, CPaaS platform, pricing models, vendor management, telecom regulations, delivery latency optimization</t>
+          <t>ecommerce platform, digital asset management (DAM), product information management (PIM), studio production workflow, omnichannel retail, creative operations, marketing technology integration</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1275,57 +1815,55 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>zenda</t>
+          <t>Sarvam</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager, Monetization &amp; Retention</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets the 2‑year minimum and no senior title). ATS score is low because key fintech/payment terms from the JD are missing, while the fit score is moderate due to transferable product skills but weak domain alignment.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of pricing, subscription, or billing expertise.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>payment gateway, transaction reconciliation, autopay configuration, KYC processes, MIS reporting</t>
+          <t>pricing strategy, subscription billing, metering, A/B testing, retention metrics, churn reduction, loyalty program, Razorpay, GST compliance</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1343,29 +1881,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EnglishBhashi</t>
+          <t>Everstage</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(APM)</t>
+          <t>Product Manager, Website</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1376,22 +1914,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
+          <t>The JD requires 5-7 years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any SEO or CRO specific terms.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
+          <t>SEO, CRO, A/B testing, Webflow, conversion rate optimization, structured data, site architecture, growth metrics, north-star metric</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1409,29 +1947,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>LSEG</t>
+          <t>frenzoft</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1442,22 +1980,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title), but contains few of the JD's specific financial‑data and multi‑cloud keywords, leading to a modest ATS score; the biggest gap is the lack of terms like Azure, Snowflake, and ETL pipelines.</t>
+          <t>The JD requires 10+ years of Salesforce product ownership experience, but the candidate has only 4 years, triggering a hard rule; consequently both scores are kept below 30. The most important keyword gap is the lack of any Salesforce‑related experience or terminology.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Azure, Snowflake, ETL pipelines, logical data model, financial market data, Refinitiv, multi‑cloud, data warehousing, licensing compliance</t>
+          <t>Salesforce Platform (Sales, Service, Experience, Marketing, Data Cloud), CRM product ownership, Backlog management, Risk &amp; dependency management, Multi‑cloud implementation</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1475,55 +2013,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Standard Chartered India</t>
+          <t>Experian</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume contains few of the JD's specific tools and terminology (e.g., Pega CDH, Adobe Campaign Manager), resulting in a low ATS score; the biggest keyword gap is the absence of any Pega or Adobe platform experience.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific terms such as AML, watchlist screening, and regulatory compliance, and the location does not match Hyderabad, resulting in moderate ATS and fit scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Pega Customer Decision Hub, Adobe Campaign Manager, Next Best Action (NBA) strategy, A/B testing, real‑time decisioning, event‑triggered campaigns, eligibility and suppression rules, predictive scoring, multivariate testing</t>
+          <t>AML, Watchlist Screening, Regulatory Compliance, False Positive Reduction, Data Provider Management, Risk Scoring, Identity Verification</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1537,59 +2075,59 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sitetracker</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD is for a Sr. Product Manager; the hard rule forces both scores below 30 despite the candidate meeting the 4‑year experience requirement. The resume lacks several senior‑level keywords such as "product positioning" and "business model".</t>
+          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>product positioning guide, business model development, OKRs, RICE prioritization, customer interview frameworks</t>
+          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1603,33 +2141,33 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Experian</t>
+          <t>Softobiz</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>TE-1434 Growth Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1640,22 +2178,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific terms such as AML, watchlist screening, and regulatory compliance, and the location does not match Hyderabad, resulting in moderate ATS and fit scores.</t>
+          <t>Hard rules pass, but the resume lacks many healthcare‑specific and conversion‑optimization keywords required for the intake role, resulting in a low ATS score; the biggest gap is the absence of telehealth/healthcare experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>AML, Watchlist Screening, Regulatory Compliance, False Positive Reduction, Data Provider Management, Risk Scoring, Identity Verification</t>
+          <t>telehealth, patient intake funnel, A/B testing, conversion rate optimization, Mixpanel, Snowflake, OKRs, unit economics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1673,17 +2211,17 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -1695,7 +2233,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
+          <t>GDD/EK - SAP PM &amp; Cross-Product Manager (m/f/d)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1706,22 +2244,22 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
+          <t>Hard rules pass, but the resume lacks many core SAP and tool keywords and the location/industry mismatch reduces both scores; the biggest gap is missing SAP-specific terms.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
+          <t>SAP PM, SAP S/4, SAP Fiori, Azure DevOps, Confluence, Kanban, Scrum</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1739,29 +2277,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>UST</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>GDB/A - Product Owner Orchestration (m/f/d)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1772,22 +2310,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as 'OpenText', 'Confluence', and 'Azure DevOps'.</t>
+          <t>The resume lacks most of the JD's core technical keywords (BPMN, Bizagi, .NET, Azure SQL, etc.) and the candidate is based in Bangalore while the role is in Hyderabad, resulting in a low ATS score; the biggest gap is the absence of BPM/automation platform experience.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>OpenText, Confluence, Azure DevOps, ServiceNow, microservices, CI/CD pipelines, enterprise content management, migration programs</t>
+          <t>BPMN 2.0, Bizagi (or Pegasystems/Appian), Node.js, C# / .NET, Azure SQL Database, ETL jobs, DevOps practices, Kanban methodology, SOAP services</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1805,29 +2343,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Speshally.nhs</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Salesforce Product Owner (10+ years)</t>
+          <t>GDE/DG - Product Manager/ S4 Hana AMS (m/f/d)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1838,22 +2376,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience while the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the resume also lacks key Salesforce and FMCG-specific terminology.</t>
+          <t>Hard rules pass, but the resume lacks SAP-specific keywords and experience, resulting in low ATS and fit scores; the most important gap is the absence of SAP S/4HANA and related technologies.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Salesforce B2B Commerce, Consumer Goods Cloud, Salesforce CRM, Marketing Automation, Order Taking</t>
+          <t>SAP S/4HANA, ABAP, BAPI, CDS, OData services, BTP, RAP, SAP FI/CO</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1876,50 +2414,50 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Worldline</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title level is appropriate, but the resume lacks many core payment‑product keywords and domain terms, lowering both scores.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, business case development, market analysis, pilot execution, roadmap prioritization, customer feedback loops, OKRs, A/B testing</t>
+          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1933,7 +2471,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -1942,24 +2480,24 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>YASH Technologies</t>
+          <t>Synechron</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Data - Product Manager Job</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1970,22 +2508,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit data‑analysis tools like Snowflake and data‑engineering terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and has no senior‑role conflict, but it lacks many trading‑specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Snowflake, Data engineering pipelines, OKRs, Data storytelling, Supply chain management</t>
+          <t>FX (foreign exchange), trading applications, KPIs, market trends analysis, product backlog prioritization, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2008,12 +2546,278 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Rockwell Automation</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager – ERP Finance &amp; AI Automation</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title level, but it lacks many finance‑specific ERP keywords required by the JD, resulting in a modest ATS score and a borderline fit.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Accounts Payable automation, Bank reconciliation, Journal entry automation, Cash‑flow prediction, ERP (Plex) finance, Supply chain procurement automation, AI strategy roadmap</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Tech Prescient</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager – IAM / IGA</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many IAM/IGA specific keywords and does not mention the required tools or location, lowering both scores; the biggest gap is the absence of identity‑management terminology.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Identity and Access Management, Identity Governance and Administration, SailPoint, Okta, PRD, Product Roadmap, Scrum</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Worldline</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title level is appropriate, but the resume lacks many core payment‑product keywords and domain terms, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>pricing strategy, business case development, market analysis, pilot execution, roadmap prioritization, customer feedback loops, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>YASH Technologies</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Data - Product Manager Job</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit data‑analysis tools like Snowflake and data‑engineering terminology.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Snowflake, Data engineering pipelines, OKRs, Data storytelling, Supply chain management</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -2032,6 +2836,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-27
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phigital Care</t>
+          <t>Itron, Inc.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -586,19 +586,19 @@
         <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and contains many relevant keywords, but lacks several cloud and analytics terms from the JD, resulting in a solid but not perfect ATS score; the strongest gap is missing explicit cloud platform experience.</t>
+          <t>The resume meets the 3+ years requirement and has no senior‑level title conflict; it covers most core keywords but lacks explicit roadmap/backlog and go‑to‑market language.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>AWS, Azure, GCP, A/B testing, OKRs, NPS improvement, customer surveys, data product development</t>
+          <t>product roadmap, backlog prioritization, go‑to‑market strategy, product marketing collaboration, customer interviews / discovery</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,14 +626,14 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Solera Holdings, LLC.</t>
+          <t>Kobie</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -643,30 +643,28 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban district, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, but the resume lacks several JD‑specific terms such as demand management and usage analytics, lowering the ATS score.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Demand Management, Quarterly planning, Usage analytics, User guides, Release notes</t>
+          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,24 +682,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Itron, Inc.</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -717,22 +715,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ years requirement and has no senior‑level title conflict; it covers most core keywords but lacks explicit roadmap/backlog and go‑to‑market language.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, backlog prioritization, go‑to‑market strategy, product marketing collaboration, customer interviews / discovery</t>
+          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,55 +748,55 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Kobie</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H5" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
+          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
+          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -821,50 +819,52 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>The Standard India</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Data Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
+          <t>Hard rules are satisfied (4 years meets the 2‑year minimum). The resume covers many core Agile and product management terms but lacks several data‑specific keywords from the JD, lowering the ATS score. The biggest gap is the absence of data‑product terminology like "PI Planning" and "story maps".</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
+          <t>PI Planning, story maps, non‑functional requirements, customer feedback loops, data governance, definition of done, data analytics, Snowflake</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,55 +882,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Scoutit</t>
+          <t>Zoca</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban district, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI terms but misses several JD‑specific keywords and the title does not exactly match AI Product Manager.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
+          <t>AI agent development, ML model optimization, customer outcome metrics, roadmap planning (6‑12 month roadmap), A/B testing, OKRs, NPS improvement, voice AI</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,55 +948,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Zoca</t>
+          <t>Golden Opportunities</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI terms but misses several JD‑specific keywords and the title does not exactly match AI Product Manager.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>AI agent development, ML model optimization, customer outcome metrics, roadmap planning (6‑12 month roadmap), A/B testing, OKRs, NPS improvement, voice AI</t>
+          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1019,52 +1019,52 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Puravankara Limited</t>
+          <t>GHX India</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title matches, but lacks several JD‑specific terms such as A/B testing and API integration, lowering the ATS score; the biggest keyword gap is the absence of any mention of A/B testing or API work.</t>
+          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, API integration, PRD (Product Requirements Document), product metrics tracking, risk / blocker identification, system workflow documentation, user engagement analysis</t>
+          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1078,76 +1078,76 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Sabre</t>
+          <t>GHX</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Distribution Data Insights</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior title triggers hard rules, but the resume lacks several core JD keywords such as APIs, data ingestion pipelines, and travel‑distribution terminology, lowering the ATS score. Domain experience is strong, especially in travel SaaS and data‑driven product work, yielding a solid fit score.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>APIs, data ingestion pipelines, distribution metrics, travel distribution channels, lodging content, agency partners, data quality metrics, search query analysis, booking data insights</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
           <t>nan</t>
@@ -1155,50 +1155,52 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Golden Opportunities</t>
+          <t>Eltropy</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
+          <t>Product Manager – AI &amp; Analytics</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
+          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1212,33 +1214,33 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GHX India</t>
+          <t>Franklin Templeton India</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>GENAI Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1247,26 +1249,24 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core keywords but misses several AI‑product specific terms, lowering the ATS score; overall fit is strong due to GenAI and SaaS experience.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
+          <t>product roadmap, OKRs, A/B testing, financial services, investment domain, user research, NPS improvement, risk management</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1284,57 +1284,55 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Eltropy</t>
+          <t>Modisoft Inc</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI &amp; Analytics</t>
+          <t>Product Manager, AI</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+          <t>The resume meets the experience requirement (4 years) and seniority constraints, and contains many of the required keywords, but lacks several AI‑specific terms such as roadmap and release notes.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+          <t>AI product roadmap, release notes, A/B testing, OKRs, customer NPS improvement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,7 +1346,7 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -1357,50 +1355,50 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Franklin Templeton India</t>
+          <t>Siemens</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>GENAI Product Manager</t>
+          <t>Associate Product Owner</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core keywords but misses several AI‑product specific terms, lowering the ATS score; overall fit is strong due to GenAI and SaaS experience.</t>
+          <t>The resume meets the 4‑year experience requirement and title alignment, but lacks several domain‑specific terms from the JD such as PLM and railway product knowledge, leading to moderate ATS and fit scores.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, financial services, investment domain, user research, NPS improvement, risk management</t>
+          <t>Product Lifecycle Management (PLM), railway solution, legacy product architecture, non‑functional requirements, OKR framework</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1414,11 +1412,11 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1428,45 +1426,45 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>INTANGLES LAB PRIVATE LIMITED</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H15" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title alignment, but lacks several domain‑specific terms from the JD such as PLM and railway product knowledge, leading to moderate ATS and fit scores.</t>
+          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several JD‑specific terms such as automobile/fleet domain and explicit acceptance testing language, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Product Lifecycle Management (PLM), railway solution, legacy product architecture, non‑functional requirements, OKR framework</t>
+          <t>automobile domain, fleet management, definition of done, acceptance testing, release notes, industry trends monitoring</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1494,45 +1492,45 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>INTANGLES LAB PRIVATE LIMITED</t>
+          <t>Principal Global Services</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several JD‑specific terms such as automobile/fleet domain and explicit acceptance testing language, lowering the ATS score.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant Agile and product management terms but lacks several data‑analytics specific keywords, lowering the ATS score. The biggest gap is the absence of data‑integration and governance terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>automobile domain, fleet management, definition of done, acceptance testing, release notes, industry trends monitoring</t>
+          <t>Data integration, Data governance, Business intelligence, Hub &amp; spoke operating model, OKRs, KPIs / product health metrics, Report creation, Enterprise Data Foundation</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1555,12 +1553,12 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1698,12 +1696,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Vedantu</t>
+          <t>Harness</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Growth</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1712,26 +1710,24 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic years requirement, but lacks many JD-specific keywords such as voice bot and LeadSquared, resulting in a low ATS score; the strongest gap is the missing conversational AI/voice bot experience.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks several core growth‑focused keywords from the JD, lowering the ATS score, while the candidate's SaaS and product experience gives a moderate fit for the growth role.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>LeadSquared, voice bot, conversational AI, CRM integration, real-time dashboards, intent design, LLM, bot automation</t>
+          <t>product‑led growth, growth funnel, A/B testing, conversion optimization, user acquisition, retention metrics, OKRs, PLG</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1754,24 +1750,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TOCUMULUS</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Owner / Business Analyst – Ecommerce &amp; Studio Production Platforms</t>
+          <t>Product Manager II - Corp Cards</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1782,22 +1778,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that caps both scores below 30; the biggest keyword gap is the lack of any ecommerce platform or DAM/PIM terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is low due to missing many JD‑specific AI and no‑code tool keywords; the biggest gap is the lack of Replit/Lovable/Cursor experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>ecommerce platform, digital asset management (DAM), product information management (PIM), studio production workflow, omnichannel retail, creative operations, marketing technology integration</t>
+          <t>Replit, Lovable, Cursor, no‑code/low‑code prototyping, agentic workflows, cross‑platform integration, compliance and risk governance, video‑coding stack</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1815,55 +1811,57 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Sarvam</t>
+          <t>Xoxoday</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Monetization &amp; Retention</t>
+          <t>Product Manager- Plum</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of pricing, subscription, or billing expertise.</t>
+          <t>The candidate meets the 2‑year minimum (4 years experience) and no senior title rule, but the resume lacks many JD‑specific keywords such as API, sales enablement, fintech, and market‑analysis terms, lowering the ATS score. The strongest gap is the absence of any API‑related experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, subscription billing, metering, A/B testing, retention metrics, churn reduction, loyalty program, Razorpay, GST compliance</t>
+          <t>API design and documentation, API contracts, sales enablement, fintech / payments, gift cards or rewards, market research, SWOT analysis, competitive analysis, business case development</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1886,24 +1884,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Everstage</t>
+          <t>Vedantu</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Website</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1912,24 +1910,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5-7 years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any SEO or CRO specific terms.</t>
+          <t>The resume meets the basic years requirement, but lacks many JD-specific keywords such as voice bot and LeadSquared, resulting in a low ATS score; the strongest gap is the missing conversational AI/voice bot experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>SEO, CRO, A/B testing, Webflow, conversion rate optimization, structured data, site architecture, growth metrics, north-star metric</t>
+          <t>LeadSquared, voice bot, conversational AI, CRM integration, real-time dashboards, intent design, LLM, bot automation</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1947,29 +1947,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>frenzoft</t>
+          <t>eGov Foundation</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - Digital Health (Public Health)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1980,22 +1980,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of Salesforce product ownership experience, but the candidate has only 4 years, triggering a hard rule; consequently both scores are kept below 30. The most important keyword gap is the lack of any Salesforce‑related experience or terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Salesforce Platform (Sales, Service, Experience, Marketing, Data Cloud), CRM product ownership, Backlog management, Risk &amp; dependency management, Multi‑cloud implementation</t>
+          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2018,19 +2018,19 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Experian</t>
+          <t>Career Crafterz</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2040,28 +2040,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific terms such as AML, watchlist screening, and regulatory compliance, and the location does not match Hyderabad, resulting in moderate ATS and fit scores.</t>
+          <t>Hard rules pass (4 years meets 2+ year requirement and title is not senior), but the resume lacks many fintech‑specific keywords such as A/B testing, attach rate, conversion rate, credit underwriting, and risk metrics, leading to low ATS and fit scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AML, Watchlist Screening, Regulatory Compliance, False Positive Reduction, Data Provider Management, Risk Scoring, Identity Verification</t>
+          <t>A/B testing, attach rate, conversion rate, credit underwriting, risk metrics, default rate, Excel, consumer lending, market &amp; competitor analysis</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2075,59 +2075,61 @@
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>TELUS Digital AI Data Solutions</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
+          <t>Product Manager - Robotics</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
+          <t>The resume meets the 2‑year minimum and has no senior‑level title, but it lacks most robotics and physical‑AI specific keywords, resulting in a low ATS score; the biggest gap is the absence of any robotics or data‑collection platform terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
+          <t>robotics, physical AI, data collection platform, sensor data integration, hardware operations</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2141,7 +2143,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -2150,50 +2152,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Softobiz</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>TE-1434 Growth Product Manager</t>
+          <t>Vice President, Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many healthcare‑specific and conversion‑optimization keywords required for the intake role, resulting in a low ATS score; the biggest gap is the absence of telehealth/healthcare experience.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of "LLM" or "large language model" experience.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>telehealth, patient intake funnel, A/B testing, conversion rate optimization, Mixpanel, Snowflake, OKRs, unit economics</t>
+          <t>large language model (LLM), conversational design, A/B testing, OKRs, adoption metrics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2207,59 +2209,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>KredX</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>GDD/EK - SAP PM &amp; Cross-Product Manager (m/f/d)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core SAP and tool keywords and the location/industry mismatch reduces both scores; the biggest gap is missing SAP-specific terms.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of 'customer acquisition' or related metrics.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>SAP PM, SAP S/4, SAP Fiori, Azure DevOps, Confluence, Kanban, Scrum</t>
+          <t>customer acquisition, product placement, messaging, roadmap development, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2273,7 +2275,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2282,50 +2284,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>Sarvam</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>GDB/A - Product Owner Orchestration (m/f/d)</t>
+          <t>Product Manager, Monetization &amp; Retention</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks most of the JD's core technical keywords (BPMN, Bizagi, .NET, Azure SQL, etc.) and the candidate is based in Bangalore while the role is in Hyderabad, resulting in a low ATS score; the biggest gap is the absence of BPM/automation platform experience.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of pricing, subscription, or billing expertise.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>BPMN 2.0, Bizagi (or Pegasystems/Appian), Node.js, C# / .NET, Azure SQL Database, ETL jobs, DevOps practices, Kanban methodology, SOAP services</t>
+          <t>pricing strategy, subscription billing, metering, A/B testing, retention metrics, churn reduction, loyalty program, Razorpay, GST compliance</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2339,11 +2341,11 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2353,45 +2355,45 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>GDE/DG - Product Manager/ S4 Hana AMS (m/f/d)</t>
+          <t>Product Manager - Fraud Rule Platforms</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP-specific keywords and experience, resulting in low ATS and fit scores; the most important gap is the absence of SAP S/4HANA and related technologies.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit fraud‑related terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, ABAP, BAPI, CDS, OData services, BTP, RAP, SAP FI/CO</t>
+          <t>fraud detection, risk management, rule engine, fraud analytics, regulatory compliance</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2405,7 +2407,7 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -2414,29 +2416,29 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Sarvam</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
+          <t>Product Manager, Growth</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -2452,12 +2454,12 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any growth‑focused metrics or tools such as A/B testing, attribution, or CAC.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
+          <t>A/B testing, CAC (Customer Acquisition Cost), Attribution modeling, Growth analytics (e.g., Mixpanel, Amplitude), Referral/virality mechanics</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2471,59 +2473,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Synechron</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and has no senior‑role conflict, but it lacks many trading‑specific keywords and domain experience, lowering both scores.</t>
+          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>FX (foreign exchange), trading applications, KPIs, market trends analysis, product backlog prioritization, OKRs</t>
+          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2537,59 +2539,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Rockwell Automation</t>
+          <t>Softobiz</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – ERP Finance &amp; AI Automation</t>
+          <t>TE-1434 Growth Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but it lacks many finance‑specific ERP keywords required by the JD, resulting in a modest ATS score and a borderline fit.</t>
+          <t>Hard rules pass, but the resume lacks many healthcare‑specific and conversion‑optimization keywords required for the intake role, resulting in a low ATS score; the biggest gap is the absence of telehealth/healthcare experience.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Accounts Payable automation, Bank reconciliation, Journal entry automation, Cash‑flow prediction, ERP (Plex) finance, Supply chain procurement automation, AI strategy roadmap</t>
+          <t>telehealth, patient intake funnel, A/B testing, conversion rate optimization, Mixpanel, Snowflake, OKRs, unit economics</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2603,11 +2605,11 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -2617,47 +2619,45 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Tech Prescient</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – IAM / IGA</t>
+          <t>GDD/EK - SAP PM &amp; Cross-Product Manager (m/f/d)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many IAM/IGA specific keywords and does not mention the required tools or location, lowering both scores; the biggest gap is the absence of identity‑management terminology.</t>
+          <t>Hard rules pass, but the resume lacks many core SAP and tool keywords and the location/industry mismatch reduces both scores; the biggest gap is missing SAP-specific terms.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Identity and Access Management, Identity Governance and Administration, SailPoint, Okta, PRD, Product Roadmap, Scrum</t>
+          <t>SAP PM, SAP S/4, SAP Fiori, Azure DevOps, Confluence, Kanban, Scrum</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2671,11 +2671,11 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -2685,45 +2685,45 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Worldline</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>GDB/A - Product Owner Orchestration (m/f/d)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title level is appropriate, but the resume lacks many core payment‑product keywords and domain terms, lowering both scores.</t>
+          <t>The resume lacks most of the JD's core technical keywords (BPMN, Bizagi, .NET, Azure SQL, etc.) and the candidate is based in Bangalore while the role is in Hyderabad, resulting in a low ATS score; the biggest gap is the absence of BPM/automation platform experience.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, business case development, market analysis, pilot execution, roadmap prioritization, customer feedback loops, OKRs, A/B testing</t>
+          <t>BPMN 2.0, Bizagi (or Pegasystems/Appian), Node.js, C# / .NET, Azure SQL Database, ETL jobs, DevOps practices, Kanban methodology, SOAP services</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2737,87 +2737,549 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>YASH Technologies</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Data - Product Manager Job</t>
+          <t>GDE/DG - Product Manager/ S4 Hana AMS (m/f/d)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks SAP-specific keywords and experience, resulting in low ATS and fit scores; the most important gap is the absence of SAP S/4HANA and related technologies.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>SAP S/4HANA, ABAP, BAPI, CDS, OData services, BTP, RAP, SAP FI/CO</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G19" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>frenzoft</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 10+ years of Salesforce product ownership experience, but the candidate has only 4 years, triggering a hard rule; consequently both scores are kept below 30. The most important keyword gap is the lack of any Salesforce‑related experience or terminology.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce Platform (Sales, Service, Experience, Marketing, Data Cloud), CRM product ownership, Backlog management, Risk &amp; dependency management, Multi‑cloud implementation</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Synechron</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and has no senior‑role conflict, but it lacks many trading‑specific keywords and domain experience, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>FX (foreign exchange), trading applications, KPIs, market trends analysis, product backlog prioritization, OKRs</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Rockwell Automation</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager – ERP Finance &amp; AI Automation</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the 4‑year experience requirement and title level, but it lacks many finance‑specific ERP keywords required by the JD, resulting in a modest ATS score and a borderline fit.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Accounts Payable automation, Bank reconciliation, Journal entry automation, Cash‑flow prediction, ERP (Plex) finance, Supply chain procurement automation, AI strategy roadmap</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Worldline</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title level is appropriate, but the resume lacks many core payment‑product keywords and domain terms, lowering both scores.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>pricing strategy, business case development, market analysis, pilot execution, roadmap prioritization, customer feedback loops, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>YASH Technologies</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Data - Product Manager Job</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G24" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit data‑analysis tools like Snowflake and data‑engineering terminology.</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Snowflake, Data engineering pipelines, OKRs, Data storytelling, Supply chain management</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>hackajob</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Manager -VP</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The JD title includes 'VP', triggering hard rule 3, so both scores must be below 30 regardless of experience; the most important keyword gap is the absence of explicit 'OKRs' and 'AI Banking Companion' terminology.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, AI Banking Companion, customer journey mapping, risk compliance, regulatory compliance</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -2840,6 +3302,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-28
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Itron, Inc.</t>
+          <t>Phigital Care</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -586,19 +586,19 @@
         <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ years requirement and has no senior‑level title conflict; it covers most core keywords but lacks explicit roadmap/backlog and go‑to‑market language.</t>
+          <t>The resume meets the hard rules and contains many relevant keywords, but lacks several cloud and analytics terms from the JD, resulting in a solid but not perfect ATS score; the strongest gap is missing explicit cloud platform experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, backlog prioritization, go‑to‑market strategy, product marketing collaboration, customer interviews / discovery</t>
+          <t>AWS, Azure, GCP, A/B testing, OKRs, NPS improvement, customer surveys, data product development</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -626,14 +626,14 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kobie</t>
+          <t>Solera Holdings, LLC.</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -643,28 +643,30 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, but the resume lacks several JD‑specific terms such as demand management and usage analytics, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
+          <t>Demand Management, Quarterly planning, Usage analytics, User guides, Release notes</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -687,19 +689,19 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Itron, Inc.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -715,22 +717,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant keywords and matches the location and education, but it misses several JD‑specific terms like LLM and API. The strongest gap is the lack of explicit AI‑assistant / agentic terminology.</t>
+          <t>The resume meets the 3+ years requirement and has no senior‑level title conflict; it covers most core keywords but lacks explicit roadmap/backlog and go‑to‑market language.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>LLM, API integration, Enterprise Graph, AI Assistant, agentic capabilities, OKRs, A/B testing, Mixpanel, Snowflake</t>
+          <t>product roadmap, backlog prioritization, go‑to‑market strategy, product marketing collaboration, customer interviews / discovery</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -748,55 +750,57 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Scoutit</t>
+          <t>Leucine - AI for Pharma</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban district, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns, but lacks key tech keywords (React, Node.js, vibe‑coding, B.Tech, explicit PRD) which lowers the ATS score; overall fit is solid on SaaS and GenAI but pharma domain is only tangential.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
+          <t>React, Node.js, vibe‑coding, B.Tech, PRD</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -819,52 +823,50 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>The Standard India</t>
+          <t>Kobie</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Data Product Owner</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years meets the 2‑year minimum). The resume covers many core Agile and product management terms but lacks several data‑specific keywords from the JD, lowering the ATS score. The biggest gap is the absence of data‑product terminology like "PI Planning" and "story maps".</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>PI Planning, story maps, non‑functional requirements, customer feedback loops, data governance, definition of done, data analytics, Snowflake</t>
+          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,29 +884,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Zoca</t>
+          <t>Signzy</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,22 +917,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume contains many relevant product and AI terms but misses several JD‑specific keywords and the title does not exactly match AI Product Manager.</t>
+          <t>Hard rules pass (4 years experience matches the non‑specified minimum). The resume covers many relevant skills but misses several core JD terms like product strategy and pricing plans, lowering the ATS score; overall domain and experience alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>AI agent development, ML model optimization, customer outcome metrics, roadmap planning (6‑12 month roadmap), A/B testing, OKRs, NPS improvement, voice AI</t>
+          <t>product strategy, pricing plans, target segment, partnerships, quality assurance testing, distribution partners, campaign strategies, original research, structured thinking</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -948,55 +950,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Golden Opportunities</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
+          <t>Product Manager - TST - MANAGER</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several JD-specific keywords like Scrum and Java, lowering the ATS score; overall domain and experience alignment is strong, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
+          <t>Scrum, Java or .Net, ReactJS, budget management, client relationship building, product roadmap, vision and strategy definition, OKRs</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,57 +1016,55 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GHX India</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
+          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
+          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1078,101 +1078,99 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GHX</t>
+          <t>Golden Opportunities</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Eltropy</t>
+          <t>GHX India</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI &amp; Analytics</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1182,25 +1180,25 @@
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H11" s="2" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1228,19 +1226,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Franklin Templeton India</t>
+          <t>GHX</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>GENAI Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1249,24 +1247,26 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core keywords but misses several AI‑product specific terms, lowering the ATS score; overall fit is strong due to GenAI and SaaS experience.</t>
+          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, financial services, investment domain, user research, NPS improvement, risk management</t>
+          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1284,55 +1284,57 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Modisoft Inc</t>
+          <t>Eltropy</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AI</t>
+          <t>Product Manager – AI &amp; Analytics</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F13" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and seniority constraints, and contains many of the required keywords, but lacks several AI‑specific terms such as roadmap and release notes.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>AI product roadmap, release notes, A/B testing, OKRs, customer NPS improvement</t>
+          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1346,59 +1348,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Siemens</t>
+          <t>Franklin Templeton India</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Owner</t>
+          <t>GENAI Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H14" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title alignment, but lacks several domain‑specific terms from the JD such as PLM and railway product knowledge, leading to moderate ATS and fit scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core keywords but misses several AI‑product specific terms, lowering the ATS score; overall fit is strong due to GenAI and SaaS experience.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Product Lifecycle Management (PLM), railway solution, legacy product architecture, non‑functional requirements, OKR framework</t>
+          <t>product roadmap, OKRs, A/B testing, financial services, investment domain, user research, NPS improvement, risk management</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1412,7 +1414,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1426,24 +1428,24 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>INTANGLES LAB PRIVATE LIMITED</t>
+          <t>Tachyon Technologies</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -1452,19 +1454,19 @@
         <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several JD‑specific terms such as automobile/fleet domain and explicit acceptance testing language, lowering the ATS score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management keywords but lacks several recruiting‑specific terms, lowering the ATS score; the biggest gap is the absence of recruiting‑domain keywords like candidate matching.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>automobile domain, fleet management, definition of done, acceptance testing, release notes, industry trends monitoring</t>
+          <t>candidate matching, recruiter agents, job intake automation, sourcing agents, screening agents, interview workflow automation, release notes, AI/ML integration, ATS integration</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1478,33 +1480,33 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Principal Global Services</t>
+          <t>Modisoft Inc</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager I</t>
+          <t>Product Manager, AI</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1515,22 +1517,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant Agile and product management terms but lacks several data‑analytics specific keywords, lowering the ATS score. The biggest gap is the absence of data‑integration and governance terminology.</t>
+          <t>The resume meets the experience requirement (4 years) and seniority constraints, and contains many of the required keywords, but lacks several AI‑specific terms such as roadmap and release notes.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Data integration, Data governance, Business intelligence, Hub &amp; spoke operating model, OKRs, KPIs / product health metrics, Report creation, Enterprise Data Foundation</t>
+          <t>AI product roadmap, release notes, A/B testing, OKRs, customer NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,7 +1550,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1558,7 +1560,139 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>INTANGLES LAB PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pune City, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several JD‑specific terms such as automobile/fleet domain and explicit acceptance testing language, lowering the ATS score.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>automobile domain, fleet management, definition of done, acceptance testing, release notes, industry trends monitoring</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Principal Global Services</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager I</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; the resume contains many relevant Agile and product management terms but lacks several data‑analytics specific keywords, lowering the ATS score. The biggest gap is the absence of data‑integration and governance terminology.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Data integration, Data governance, Business intelligence, Hub &amp; spoke operating model, OKRs, KPIs / product health metrics, Report creation, Enterprise Data Foundation</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
           <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -1579,6 +1713,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1590,7 +1726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1755,7 +1891,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1903,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Corp Cards</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1778,22 +1914,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>55</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is low due to missing many JD‑specific AI and no‑code tool keywords; the biggest gap is the lack of Replit/Lovable/Cursor experience.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Replit, Lovable, Cursor, no‑code/low‑code prototyping, agentic workflows, cross‑platform integration, compliance and risk governance, video‑coding stack</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1811,57 +1947,55 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Xoxoday</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Plum</t>
+          <t>Product Manager II - Corp Cards</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (4 years experience) and no senior title rule, but the resume lacks many JD‑specific keywords such as API, sales enablement, fintech, and market‑analysis terms, lowering the ATS score. The strongest gap is the absence of any API‑related experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title). ATS score is low due to missing many JD‑specific AI and no‑code tool keywords; the biggest gap is the lack of Replit/Lovable/Cursor experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>API design and documentation, API contracts, sales enablement, fintech / payments, gift cards or rewards, market research, SWOT analysis, competitive analysis, business case development</t>
+          <t>Replit, Lovable, Cursor, no‑code/low‑code prototyping, agentic workflows, cross‑platform integration, compliance and risk governance, video‑coding stack</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1879,7 +2013,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -1889,47 +2023,47 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Vedantu</t>
+          <t>Xoxoday</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager- Plum</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic years requirement, but lacks many JD-specific keywords such as voice bot and LeadSquared, resulting in a low ATS score; the strongest gap is the missing conversational AI/voice bot experience.</t>
+          <t>The candidate meets the 2‑year minimum (4 years experience) and no senior title rule, but the resume lacks many JD‑specific keywords such as API, sales enablement, fintech, and market‑analysis terms, lowering the ATS score. The strongest gap is the absence of any API‑related experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>LeadSquared, voice bot, conversational AI, CRM integration, real-time dashboards, intent design, LLM, bot automation</t>
+          <t>API design and documentation, API contracts, sales enablement, fintech / payments, gift cards or rewards, market research, SWOT analysis, competitive analysis, business case development</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1947,17 +2081,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2147,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -2023,14 +2157,14 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Career Crafterz</t>
+          <t>Aptita</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2040,28 +2174,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets 2+ year requirement and title is not senior), but the resume lacks many fintech‑specific keywords such as A/B testing, attach rate, conversion rate, credit underwriting, and risk metrics, leading to low ATS and fit scores.</t>
+          <t>The resume meets the 4‑year experience requirement and location, but lacks many JD‑specific keywords (e.g., Confluence, API, microservices), resulting in a low ATS score; the candidate’s SaaS and enterprise background is relevant but the banking/financial domain is a mismatch.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, attach rate, conversion rate, credit underwriting, risk metrics, default rate, Excel, consumer lending, market &amp; competitor analysis</t>
+          <t>Confluence, API, microservices, CI/CD, financial compliance</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2084,52 +2218,50 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TELUS Digital AI Data Solutions</t>
+          <t>Career Crafterz</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Robotics</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and has no senior‑level title, but it lacks most robotics and physical‑AI specific keywords, resulting in a low ATS score; the biggest gap is the absence of any robotics or data‑collection platform terminology.</t>
+          <t>Hard rules pass (4 years meets 2+ year requirement and title is not senior), but the resume lacks many fintech‑specific keywords such as A/B testing, attach rate, conversion rate, credit underwriting, and risk metrics, leading to low ATS and fit scores.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>robotics, physical AI, data collection platform, sensor data integration, hardware operations</t>
+          <t>A/B testing, attach rate, conversion rate, credit underwriting, risk metrics, default rate, Excel, consumer lending, market &amp; competitor analysis</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2147,7 +2279,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -2157,19 +2289,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>TELUS Digital AI Data Solutions</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Vice President, Product Manager</t>
+          <t>Product Manager - Robotics</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2178,24 +2310,26 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of "LLM" or "large language model" experience.</t>
+          <t>The resume meets the 2‑year minimum and has no senior‑level title, but it lacks most robotics and physical‑AI specific keywords, resulting in a low ATS score; the biggest gap is the absence of any robotics or data‑collection platform terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>large language model (LLM), conversational design, A/B testing, OKRs, adoption metrics</t>
+          <t>robotics, physical AI, data collection platform, sensor data integration, hardware operations</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2213,7 +2347,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -2223,19 +2357,19 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>KredX</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager- Data and Quality- Associate</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2244,24 +2378,26 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of 'customer acquisition' or related metrics.</t>
+          <t>The candidate meets the years and location requirements, but the resume lacks most of the specific platform and tool keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of ACES/NGP and related data‑platform tools.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>customer acquisition, product placement, messaging, roadmap development, OKRs, A/B testing, NPS improvement</t>
+          <t>ACES, NGP, QlikSense, Business Objects, Alteryx, Snowflake, change management, defect management, release management, data warehouse</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2284,24 +2420,24 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Sarvam</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Monetization &amp; Retention</t>
+          <t>Vice President, Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2322,12 +2458,12 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of pricing, subscription, or billing expertise.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of "LLM" or "large language model" experience.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, subscription billing, metering, A/B testing, retention metrics, churn reduction, loyalty program, Razorpay, GST compliance</t>
+          <t>large language model (LLM), conversational design, A/B testing, OKRs, adoption metrics</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2350,24 +2486,24 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Sarvam</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Fraud Rule Platforms</t>
+          <t>Product Manager, Monetization &amp; Retention</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2378,22 +2514,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit fraud‑related terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of pricing, subscription, or billing expertise.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, risk management, rule engine, fraud analytics, regulatory compliance</t>
+          <t>pricing strategy, subscription billing, metering, A/B testing, retention metrics, churn reduction, loyalty program, Razorpay, GST compliance</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2411,29 +2547,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Sarvam</t>
+          <t>The IT Firm</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Growth</t>
+          <t>Techno-Functional Consultant/Product Manager - CLM Platform</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2447,19 +2583,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any growth‑focused metrics or tools such as A/B testing, attribution, or CAC.</t>
+          <t>The JD explicitly requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any CLM platform names (e.g., Icertis, Conga).</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CAC (Customer Acquisition Cost), Attribution modeling, Growth analytics (e.g., Mixpanel, Amplitude), Referral/virality mechanics</t>
+          <t>Icertis, Conga, SirionLabs, Ironclad, Oracle CLM, REST API integrations, DocuSign, AI/LLM contract summarization, OCR/document intelligence</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2477,55 +2613,55 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
+          <t>Product Manager - Fraud Rule Platforms</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit fraud‑related terminology.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
+          <t>fraud detection, risk management, rule engine, fraud analytics, regulatory compliance</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2539,59 +2675,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Softobiz</t>
+          <t>Mojro</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>TE-1434 Growth Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many healthcare‑specific and conversion‑optimization keywords required for the intake role, resulting in a low ATS score; the biggest gap is the absence of telehealth/healthcare experience.</t>
+          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key logistics and supply‑chain terminology such as "digital twin" and "logistics optimization".</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>telehealth, patient intake funnel, A/B testing, conversion rate optimization, Mixpanel, Snowflake, OKRs, unit economics</t>
+          <t>digital twin, logistics optimization, supply chain analytics, OKRs, RICE prioritization, customer journey mapping, NPS improvement, A/B testing</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2605,59 +2741,59 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>Wayfair</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>GDD/EK - SAP PM &amp; Cross-Product Manager (m/f/d)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core SAP and tool keywords and the location/industry mismatch reduces both scores; the biggest gap is missing SAP-specific terms.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any supply‑chain or fulfillment terminology.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>SAP PM, SAP S/4, SAP Fiori, Azure DevOps, Confluence, Kanban, Scrum</t>
+          <t>Supply chain, Fulfillment, Inventory management, Warehouse operations, LLM‑powered experiences, Roadmap prioritization, Scalable architecture, Operational leaders</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2671,59 +2807,59 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>Sarvam</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GDB/A - Product Owner Orchestration (m/f/d)</t>
+          <t>Product Manager, Growth</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks most of the JD's core technical keywords (BPMN, Bizagi, .NET, Azure SQL, etc.) and the candidate is based in Bangalore while the role is in Hyderabad, resulting in a low ATS score; the biggest gap is the absence of BPM/automation platform experience.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any growth‑focused metrics or tools such as A/B testing, attribution, or CAC.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>BPMN 2.0, Bizagi (or Pegasystems/Appian), Node.js, C# / .NET, Azure SQL Database, ETL jobs, DevOps practices, Kanban methodology, SOAP services</t>
+          <t>A/B testing, CAC (Customer Acquisition Cost), Attribution modeling, Growth analytics (e.g., Mixpanel, Amplitude), Referral/virality mechanics</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2737,7 +2873,7 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
@@ -2746,50 +2882,50 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>GDE/DG - Product Manager/ S4 Hana AMS (m/f/d)</t>
+          <t>Product Manager - Payments</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP-specific keywords and experience, resulting in low ATS and fit scores; the most important gap is the absence of SAP S/4HANA and related technologies.</t>
+          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, ABAP, BAPI, CDS, OData services, BTP, RAP, SAP FI/CO</t>
+          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2803,33 +2939,33 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
+          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2840,22 +2976,22 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
+          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
+          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2878,24 +3014,24 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>frenzoft</t>
+          <t>BASF</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>GDE/DG - Product Manager/ S4 Hana AMS (m/f/d)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2906,22 +3042,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of Salesforce product ownership experience, but the candidate has only 4 years, triggering a hard rule; consequently both scores are kept below 30. The most important keyword gap is the lack of any Salesforce‑related experience or terminology.</t>
+          <t>Hard rules pass, but the resume lacks SAP-specific keywords and experience, resulting in low ATS and fit scores; the most important gap is the absence of SAP S/4HANA and related technologies.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Salesforce Platform (Sales, Service, Experience, Marketing, Data Cloud), CRM product ownership, Backlog management, Risk &amp; dependency management, Multi‑cloud implementation</t>
+          <t>SAP S/4HANA, ABAP, BAPI, CDS, OData services, BTP, RAP, SAP FI/CO</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2939,55 +3075,55 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Synechron</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>L55 - Product Manager II</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and has no senior‑role conflict, but it lacks many trading‑specific keywords and domain experience, lowering both scores.</t>
+          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit KPI/OKR or profit‑and‑loss responsibility language.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>FX (foreign exchange), trading applications, KPIs, market trends analysis, product backlog prioritization, OKRs</t>
+          <t>profit and loss ownership, KPIs, OKRs, market research, competitive analysis, user research, roadmap, product vision</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3001,59 +3137,59 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Rockwell Automation</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – ERP Finance &amp; AI Automation</t>
+          <t>L50 - Product Manager I</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but it lacks many finance‑specific ERP keywords required by the JD, resulting in a modest ATS score and a borderline fit.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit profit &amp; loss ownership terminology.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Accounts Payable automation, Bank reconciliation, Journal entry automation, Cash‑flow prediction, ERP (Plex) finance, Supply chain procurement automation, AI strategy roadmap</t>
+          <t>profit and loss ownership, KPIs, OKRs, market research, user research, competitive analysis, roadmap, product vision</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3067,59 +3203,59 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Worldline</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title level is appropriate, but the resume lacks many core payment‑product keywords and domain terms, lowering both scores.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, business case development, market analysis, pilot execution, roadmap prioritization, customer feedback loops, OKRs, A/B testing</t>
+          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -3133,33 +3269,33 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>YASH Technologies</t>
+          <t>Synechron</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Data - Product Manager Job</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3170,22 +3306,22 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of explicit data‑analysis tools like Snowflake and data‑engineering terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and has no senior‑role conflict, but it lacks many trading‑specific keywords and domain experience, lowering both scores.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Snowflake, Data engineering pipelines, OKRs, Data storytelling, Supply chain management</t>
+          <t>FX (foreign exchange), trading applications, KPIs, market trends analysis, product backlog prioritization, OKRs</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -3203,29 +3339,29 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Rockwell Automation</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager -VP</t>
+          <t>Product Manager – ERP Finance &amp; AI Automation</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3236,22 +3372,22 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The JD title includes 'VP', triggering hard rule 3, so both scores must be below 30 regardless of experience; the most important keyword gap is the absence of explicit 'OKRs' and 'AI Banking Companion' terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but it lacks many finance‑specific ERP keywords required by the JD, resulting in a modest ATS score and a borderline fit.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>OKRs, AI Banking Companion, customer journey mapping, risk compliance, regulatory compliance</t>
+          <t>Accounts Payable automation, Bank reconciliation, Journal entry automation, Cash‑flow prediction, ERP (Plex) finance, Supply chain procurement automation, AI strategy roadmap</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -3269,17 +3405,215 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>upEducators</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager - II</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass, but the resume lacks many education‑specific keywords and domain experience, resulting in moderate ATS and fit scores; the biggest gap is missing education‑focused product terminology.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>product roadmap, KPIs, market research, competitive analysis, educational technology</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Owner</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains many relevant product management terms but misses several core JD keywords (e.g., technical debt, KTLO, incident management) and the location does not match Pune, lowering the ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably with the role.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>technical debt, KTLO, regulatory change, platform optimisation, incident management, operational resilience, governance standards, architecture standards, security standards, market research</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Innova ESI</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Technical Product Manager (AI &amp; Healthcare)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>The JD requires 6+ years of experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. Additionally, key terms like OKRs and API testing are missing.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>OKRs, API testing, SQL hands‑on, product backlog refinement, budget monitoring, market and technology insights</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -3309,6 +3643,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-29
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,17 +567,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phigital Care</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -586,19 +586,19 @@
         <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules and contains many relevant keywords, but lacks several cloud and analytics terms from the JD, resulting in a solid but not perfect ATS score; the strongest gap is missing explicit cloud platform experience.</t>
+          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>AWS, Azure, GCP, A/B testing, OKRs, NPS improvement, customer surveys, data product development</t>
+          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,57 +616,57 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Solera Holdings, LLC.</t>
+          <t>Leucine - AI for Pharma</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban district, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, but the resume lacks several JD‑specific terms such as demand management and usage analytics, lowering the ATS score.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title aligns, but lacks key tech keywords (React, Node.js, vibe‑coding, B.Tech, explicit PRD) which lowers the ATS score; overall fit is solid on SaaS and GenAI but pharma domain is only tangential.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Demand Management, Quarterly planning, Usage analytics, User guides, Release notes</t>
+          <t>React, Node.js, vibe‑coding, B.Tech, PRD</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,24 +684,24 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Itron, Inc.</t>
+          <t>Signzy</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -717,22 +717,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>75</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3+ years requirement and has no senior‑level title conflict; it covers most core keywords but lacks explicit roadmap/backlog and go‑to‑market language.</t>
+          <t>Hard rules pass (4 years experience matches the non‑specified minimum). The resume covers many relevant skills but misses several core JD terms like product strategy and pricing plans, lowering the ATS score; overall domain and experience alignment is strong, yielding a solid fit score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, backlog prioritization, go‑to‑market strategy, product marketing collaboration, customer interviews / discovery</t>
+          <t>product strategy, pricing plans, target segment, partnerships, quality assurance testing, distribution partners, campaign strategies, original research, structured thinking</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Leucine - AI for Pharma</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager - TST - MANAGER</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,26 +781,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>70</v>
-      </c>
       <c r="H5" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns, but lacks key tech keywords (React, Node.js, vibe‑coding, B.Tech, explicit PRD) which lowers the ATS score; overall fit is solid on SaaS and GenAI but pharma domain is only tangential.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several JD-specific keywords like Scrum and Java, lowering the ATS score; overall domain and experience alignment is strong, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>React, Node.js, vibe‑coding, B.Tech, PRD</t>
+          <t>Scrum, Java or .Net, ReactJS, budget management, client relationship building, product roadmap, vision and strategy definition, OKRs</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,7 +816,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -828,19 +826,19 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Kobie</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -851,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume contains many JD keywords but lacks explicit mentions of roadmap planning, product backlog management, and loyalty-specific metrics, lowering the ATS score slightly; overall strong SaaS and GenAI experience drives a solid fit score.</t>
+          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>roadmap planning, product backlog, OKRs, release management, customer loyalty, NPS improvement, A/B testing, Snowflake</t>
+          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -884,24 +882,24 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Signzy</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -911,7 +909,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -927,12 +925,12 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches the non‑specified minimum). The resume covers many relevant skills but misses several core JD terms like product strategy and pricing plans, lowering the ATS score; overall domain and experience alignment is strong, yielding a solid fit score.</t>
+          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>product strategy, pricing plans, target segment, partnerships, quality assurance testing, distribution partners, campaign strategies, original research, structured thinking</t>
+          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -955,24 +953,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>Eightfold AI</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - TST - MANAGER</t>
+          <t>Product Manager II - Talent Management</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -983,22 +981,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>72</v>
-      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several JD-specific keywords like Scrum and Java, lowering the ATS score; overall domain and experience alignment is strong, giving a solid fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core PM keywords but lacks several talent‑management specific terms, leading to a solid but not outstanding ATS score. The biggest gap is domain‑specific language around talent acquisition and Azure/AWS infrastructure.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Scrum, Java or .Net, ReactJS, budget management, client relationship building, product roadmap, vision and strategy definition, OKRs</t>
+          <t>Azure, AWS, IL4 compliance, agentic AI, talent acquisition, market landscape analysis, product roadmap development, OKRs, customer adoption metrics, NPS improvement</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1016,24 +1014,24 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Scoutit</t>
+          <t>Tekion Corp</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1043,28 +1041,30 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban district, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F9" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H9" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>72</v>
-      </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, so hard rules pass. The resume contains many SaaS and Agile keywords but misses several retail‑dealership specific terms, lowering the ATS score. The biggest gap is the lack of explicit "roadmap" and "dealer pain points" language.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
+          <t>roadmap, dealer pain points, go-to-market, reporting, AI‑powered automation, customer empathy, NPS improvement, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1087,50 +1087,52 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Golden Opportunities</t>
+          <t>Binocs.co</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Healthcare - GO/JC/3075/2026</t>
+          <t>Binocs - AI Product Manager - FinTech Domain</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>1</v>
+      </c>
       <c r="F10" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>65</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>61</v>
-      </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap (Jira, Agile, GenAI, RAG, SaaS) but missing key terms like OKRs, roadmap, portfolio, ROI. Fit score is lower because the candidate's domain (travel, FMCG, renewable) does not match the healthcare focus of the role.</t>
+          <t>The resume meets the hard rules but lacks several fintech‑specific keywords and domain experience, lowering both scores; the biggest gap is the absence of explicit market research and competitor analysis experience.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>OKRs, roadmap, portfolio management, ROI, CBA, stakeholder feedback loops, cross‑domain initiatives, financial investment management</t>
+          <t>Fintech, Market research, Customer insights, Competitor analysis, Product specifications, OKRs</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,85 +1150,83 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GHX India</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - Tech</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many generic product management keywords but lacks shipping/logistics specific terms, lowering the ATS score; the biggest gap is missing carrier integration and shipping logistics terminology.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>carrier integration, label generation, shipping logistics, e-commerce marketplace, tracking and billing, compliance, scalability, partner integration, fulfillment</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement and aligns well with the Product Owner role, showing strong keyword overlap; the main gap is missing explicit mentions of technical debt and OKR processes.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>technical debt, security, OKRs, roadmap planning, platform scalability, A/B testing, backlog grooming</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -1294,19 +1294,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Eltropy</t>
+          <t>Tachyon Technologies</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager – AI &amp; Analytics</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1315,26 +1315,24 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and title seniority is appropriate, yielding a strong keyword match but some gaps in specific analytics/BI terms.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management keywords but lacks several recruiting‑specific terms, lowering the ATS score; the biggest gap is the absence of recruiting‑domain keywords like candidate matching.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Executive dashboards, KPI frameworks, real-time data pipelines, AI-powered natural language querying, OKRs</t>
+          <t>candidate matching, recruiter agents, job intake automation, sourcing agents, screening agents, interview workflow automation, release notes, AI/ML integration, ATS integration</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1352,29 +1350,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Franklin Templeton India</t>
+          <t>BIG4</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>GENAI Product Manager</t>
+          <t>Business Analyst\Product Owner (4-7 years Early joiner Preferred)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1385,22 +1383,22 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core keywords but misses several AI‑product specific terms, lowering the ATS score; overall fit is strong due to GenAI and SaaS experience.</t>
+          <t>The resume meets the 4-year experience requirement and contains many relevant keywords, but lacks several JD-specific terms and does not clearly indicate Hyderabad location, lowering the ATS score; the strongest keyword gap is the absence of "Roadmap" and related planning terms.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>product roadmap, OKRs, A/B testing, financial services, investment domain, user research, NPS improvement, risk management</t>
+          <t>Roadmap, Risk Management, Incident Management, User Acceptance Testing (UAT), Customer Centricity, Release Notes, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1418,29 +1416,29 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Tachyon Technologies</t>
+          <t>Hitachi Digital Services</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-63827</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1451,22 +1449,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management keywords but lacks several recruiting‑specific terms, lowering the ATS score; the biggest gap is the absence of recruiting‑domain keywords like candidate matching.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>candidate matching, recruiter agents, job intake automation, sourcing agents, screening agents, interview workflow automation, release notes, AI/ML integration, ATS integration</t>
+          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1489,12 +1487,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -1560,24 +1558,24 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>INTANGLES LAB PRIVATE LIMITED</t>
+          <t>Modisoft Inc</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Pune City, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -1586,19 +1584,19 @@
         <v>68</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and seniority constraints, but the resume lacks several JD‑specific terms such as automobile/fleet domain and explicit acceptance testing language, lowering the ATS score.</t>
+          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however, key JD terms like retail/restaurant focus, roadmap, and release notes are missing, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>automobile domain, fleet management, definition of done, acceptance testing, release notes, industry trends monitoring</t>
+          <t>Retail, Restaurant, product roadmap, release notes, A/B testing, OKRs, customer NPS, AI product strategy</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1616,17 +1614,17 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1690,73 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>EXL</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Manager-Product Development-Technology/Digital Product Owner</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -1715,6 +1779,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1726,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1832,12 +1897,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Harness</t>
+          <t>GreedyGame</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Growth</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1848,22 +1913,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>65</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title). The resume lacks several core growth‑focused keywords from the JD, lowering the ATS score, while the candidate's SaaS and product experience gives a moderate fit for the growth role.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many JD‑specific tools and mobile‑app domain terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>product‑led growth, growth funnel, A/B testing, conversion optimization, user acquisition, retention metrics, OKRs, PLG</t>
+          <t>Firebase Metrics, Google Analytics, BigQuery, Looker Studio, Rewarded/Incentive Mobile Apps, Mobile App User Journey, A/B testing, MAU growth</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1881,17 +1946,17 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -1947,7 +2012,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -1957,45 +2022,47 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Xoxoday</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Corp Cards</t>
+          <t>Product Manager- Plum</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F4" s="2" t="n">
         <v>45</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title). ATS score is low due to missing many JD‑specific AI and no‑code tool keywords; the biggest gap is the lack of Replit/Lovable/Cursor experience.</t>
+          <t>The candidate meets the 2‑year minimum (4 years experience) and no senior title rule, but the resume lacks many JD‑specific keywords such as API, sales enablement, fintech, and market‑analysis terms, lowering the ATS score. The strongest gap is the absence of any API‑related experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Replit, Lovable, Cursor, no‑code/low‑code prototyping, agentic workflows, cross‑platform integration, compliance and risk governance, video‑coding stack</t>
+          <t>API design and documentation, API contracts, sales enablement, fintech / payments, gift cards or rewards, market research, SWOT analysis, competitive analysis, business case development</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2013,7 +2080,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -2023,47 +2090,45 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Xoxoday</t>
+          <t>eGov Foundation</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Plum</t>
+          <t>Product Manager - Digital Health (Public Health)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>62</v>
-      </c>
       <c r="H5" s="2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (4 years experience) and no senior title rule, but the resume lacks many JD‑specific keywords such as API, sales enablement, fintech, and market‑analysis terms, lowering the ATS score. The strongest gap is the absence of any API‑related experience.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>API design and documentation, API contracts, sales enablement, fintech / payments, gift cards or rewards, market research, SWOT analysis, competitive analysis, business case development</t>
+          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2081,29 +2146,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>eGov Foundation</t>
+          <t>EnglishBhashi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Digital Health (Public Health)</t>
+          <t>Associate Product Manager(APM)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2114,22 +2179,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
+          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
+          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2147,24 +2212,24 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Aptita</t>
+          <t>Career Crafterz</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2174,28 +2239,28 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, but lacks many JD‑specific keywords (e.g., Confluence, API, microservices), resulting in a low ATS score; the candidate’s SaaS and enterprise background is relevant but the banking/financial domain is a mismatch.</t>
+          <t>Hard rules pass (4 years meets 2+ year requirement and title is not senior), but the resume lacks many fintech‑specific keywords such as A/B testing, attach rate, conversion rate, credit underwriting, and risk metrics, leading to low ATS and fit scores.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Confluence, API, microservices, CI/CD, financial compliance</t>
+          <t>A/B testing, attach rate, conversion rate, credit underwriting, risk metrics, default rate, Excel, consumer lending, market &amp; competitor analysis</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2213,24 +2278,24 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Career Crafterz</t>
+          <t>Xurrent</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -2240,28 +2305,30 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets 2+ year requirement and title is not senior), but the resume lacks many fintech‑specific keywords such as A/B testing, attach rate, conversion rate, credit underwriting, and risk metrics, leading to low ATS and fit scores.</t>
+          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most ITAM‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of network‑discovery tool names.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, attach rate, conversion rate, credit underwriting, risk metrics, default rate, Excel, consumer lending, market &amp; competitor analysis</t>
+          <t>inTune, Lansweeper, Jamf, LogicMonitor, SNMP, WMI, SSH, SOC 2, ISO certification, KPI‑driven release cycle</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2279,17 +2346,17 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2357,47 +2424,45 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>QpiAI</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Data and Quality- Associate</t>
+          <t>Product manager Quantum computers</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and location requirements, but the resume lacks most of the specific platform and tool keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of ACES/NGP and related data‑platform tools.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any quantum computing or hardware terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>ACES, NGP, QlikSense, Business Objects, Alteryx, Snowflake, change management, defect management, release management, data warehouse</t>
+          <t>quantum computing, qubit fidelity, hardware roadmap, QCaaS, technical marketing collateral</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2415,29 +2480,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Vice President, Product Manager</t>
+          <t>Product Manager - Fraud Rule Platforms</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2458,12 +2523,12 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of "LLM" or "large language model" experience.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the absence of fraud‑specific terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>large language model (LLM), conversational design, A/B testing, OKRs, adoption metrics</t>
+          <t>fraud detection, risk management, rule engine, fraud rule lifecycle, data governance, A/B testing, OKRs, Snowflake</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2481,29 +2546,29 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Sarvam</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Monetization &amp; Retention</t>
+          <t>L55 - Product Manager II</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2524,12 +2589,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of pricing, subscription, or billing expertise.</t>
+          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit KPI/OKR or profit‑and‑loss responsibility language.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>pricing strategy, subscription billing, metering, A/B testing, retention metrics, churn reduction, loyalty program, Razorpay, GST compliance</t>
+          <t>profit and loss ownership, KPIs, OKRs, market research, competitive analysis, user research, roadmap, product vision</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2547,29 +2612,29 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>The IT Firm</t>
+          <t>KredX</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Techno-Functional Consultant/Product Manager - CLM Platform</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2580,22 +2645,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any CLM platform names (e.g., Icertis, Conga).</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of 'customer acquisition' or related metrics.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Icertis, Conga, SirionLabs, Ironclad, Oracle CLM, REST API integrations, DocuSign, AI/LLM contract summarization, OCR/document intelligence</t>
+          <t>customer acquisition, product placement, messaging, roadmap development, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2613,17 +2678,17 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2754,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2745,7 +2810,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -2755,7 +2820,7 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2876,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -2821,45 +2886,45 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Sarvam</t>
+          <t>Olympus Corporation</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Growth</t>
+          <t>Supply Chain Solutions Product Owner</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any growth‑focused metrics or tools such as A/B testing, attribution, or CAC.</t>
+          <t>Hard rules pass, but the resume lacks many supply chain‑specific terms (SAP, o9, UAT, training/adoption) and only partially matches the JD keywords, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, CAC (Customer Acquisition Cost), Attribution modeling, Growth analytics (e.g., Mixpanel, Amplitude), Referral/virality mechanics</t>
+          <t>SAP S/4, o9, UAT, training and adoption, roadmap</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2873,38 +2938,38 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>L50 - Product Manager I</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
@@ -2913,19 +2978,19 @@
         <v>25</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit profit &amp; loss ownership terminology.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
+          <t>profit and loss ownership, KPIs, OKRs, market research, user research, competitive analysis, roadmap, product vision</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2939,59 +3004,59 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>Barclays</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>GDE/A - Product Manager SAP Authorization (m/f/d)</t>
+          <t>Digital Product Owner</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP and several JD-specific terms, reducing keyword density; the candidate's SaaS/GenAI background only partially aligns with the SAP‑focused role.</t>
+          <t>The resume contains many relevant product management terms but misses several core JD keywords (e.g., technical debt, KTLO, incident management) and the location does not match Pune, lowering the ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably with the role.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>SAP, Business Informatics, Application Project Management, OKRs, RICE prioritization, Customer Orientation, Conflict Management</t>
+          <t>technical debt, KTLO, regulatory change, platform optimisation, incident management, operational resilience, governance standards, architecture standards, security standards, market research</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3005,59 +3070,59 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BASF</t>
+          <t>Aumni</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>GDE/DG - Product Manager/ S4 Hana AMS (m/f/d)</t>
+          <t>Product Owner - Roadmap &amp;amp; Strategy</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks SAP-specific keywords and experience, resulting in low ATS and fit scores; the most important gap is the absence of SAP S/4HANA and related technologies.</t>
+          <t>Candidate has only 4 years experience while the JD explicitly requires 5+ years, triggering a hard rule that caps both scores below 30; also the resume lacks several core JD keywords such as Confluence and roadmap planning.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4HANA, ABAP, BAPI, CDS, OData services, BTP, RAP, SAP FI/CO</t>
+          <t>Confluence, AI/ML platforms, roadmap planning, product strategy, OKRs, RICE prioritization, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3071,59 +3136,59 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>L55 - Product Manager II</t>
+          <t>Digital Product Manager -VP</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit KPI/OKR or profit‑and‑loss responsibility language.</t>
+          <t>The JD title includes 'VP', triggering hard rule 3, so both scores must be below 30 regardless of experience; the most important keyword gap is the absence of explicit 'OKRs' and 'AI Banking Companion' terminology.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>profit and loss ownership, KPIs, OKRs, market research, competitive analysis, user research, roadmap, product vision</t>
+          <t>OKRs, AI Banking Companion, customer journey mapping, risk compliance, regulatory compliance</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3137,38 +3202,38 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Virtusa</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>L50 - Product Manager I</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -3177,19 +3242,19 @@
         <v>25</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit profit &amp; loss ownership terminology.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>profit and loss ownership, KPIs, OKRs, market research, user research, competitive analysis, roadmap, product vision</t>
+          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3203,7 +3268,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -3212,408 +3277,12 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager, Global AR Process Excellence &amp; Automation, Global Accounts Receivable</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'process simplification' which is central to the role.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>process simplification, AI‑first automation, human‑in‑the‑loop, global accounts receivable, metric tracking (cycle time reduction, automation rate)</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="P23" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Synechron</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and has no senior‑role conflict, but it lacks many trading‑specific keywords and domain experience, lowering both scores.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>FX (foreign exchange), trading applications, KPIs, market trends analysis, product backlog prioritization, OKRs</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Rockwell Automation</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager – ERP Finance &amp; AI Automation</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but it lacks many finance‑specific ERP keywords required by the JD, resulting in a modest ATS score and a borderline fit.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Accounts Payable automation, Bank reconciliation, Journal entry automation, Cash‑flow prediction, ERP (Plex) finance, Supply chain procurement automation, AI strategy roadmap</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>upEducators</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager - II</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many education‑specific keywords and domain experience, resulting in moderate ATS and fit scores; the biggest gap is missing education‑focused product terminology.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>product roadmap, KPIs, market research, competitive analysis, educational technology</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Barclays</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Owner</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains many relevant product management terms but misses several core JD keywords (e.g., technical debt, KTLO, incident management) and the location does not match Pune, lowering the ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably with the role.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>technical debt, KTLO, regulatory change, platform optimisation, incident management, operational resilience, governance standards, architecture standards, security standards, market research</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Innova ESI</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Technical Product Manager (AI &amp; Healthcare)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H28" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 6+ years of experience; the candidate has only 4 years, triggering a hard rule that forces both scores below 30. Additionally, key terms like OKRs and API testing are missing.</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>OKRs, API testing, SQL hands‑on, product backlog refinement, budget monitoring, market and technology insights</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
     </row>
@@ -3640,12 +3309,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-30
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -760,19 +760,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - TST - MANAGER</t>
+          <t>Product Manager - Personalization &amp; Data Platforms</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,24 +781,26 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management terms but misses several JD-specific keywords like Scrum and Java, lowering the ATS score; overall domain and experience alignment is strong, giving a solid fit score.</t>
+          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Scrum, Java or .Net, ReactJS, budget management, client relationship building, product roadmap, vision and strategy definition, OKRs</t>
+          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +818,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Amazon Business India</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +851,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
+          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
+          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -892,45 +894,47 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Scoutit</t>
+          <t>Peoplebox.ai</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager (APM)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the years requirement and title level, but the resume lacks many exact JD keywords such as product discovery and success metrics, lowering the ATS score; overall domain and experience align well, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
+          <t>Product Discovery, customer interviews, data analysis, competitive research, success metrics, product roadmap, AI tools, prototypes, mockups</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -953,24 +957,24 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Eightfold AI</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Talent Management</t>
+          <t>Product Manager - Tech</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -981,22 +985,22 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume covers many core PM keywords but lacks several talent‑management specific terms, leading to a solid but not outstanding ATS score. The biggest gap is domain‑specific language around talent acquisition and Azure/AWS infrastructure.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many generic product management keywords but lacks shipping/logistics specific terms, lowering the ATS score; the biggest gap is missing carrier integration and shipping logistics terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Azure, AWS, IL4 compliance, agentic AI, talent acquisition, market landscape analysis, product roadmap development, OKRs, customer adoption metrics, NPS improvement</t>
+          <t>carrier integration, label generation, shipping logistics, e-commerce marketplace, tracking and billing, compliance, scalability, partner integration, fulfillment</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1014,7 +1018,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1024,19 +1028,19 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Tekion Corp</t>
+          <t>Kroll</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1045,26 +1049,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3‑year minimum (has 4 years) and no senior‑level title conflict, so hard rules pass. The resume contains many SaaS and Agile keywords but misses several retail‑dealership specific terms, lowering the ATS score. The biggest gap is the lack of explicit "roadmap" and "dealer pain points" language.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>roadmap, dealer pain points, go-to-market, reporting, AI‑powered automation, customer empathy, NPS improvement, OKRs, RICE prioritization</t>
+          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1082,57 +1084,57 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Binocs.co</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Binocs - AI Product Manager - FinTech Domain</t>
+          <t>Product Owner — General</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules but lacks several fintech‑specific keywords and domain experience, lowering both scores; the biggest gap is the absence of explicit market research and competitor analysis experience.</t>
+          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Fintech, Market research, Customer insights, Competitor analysis, Product specifications, OKRs</t>
+          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1146,59 +1148,61 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Tech</t>
+          <t>Product Owner (Tax)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F11" s="2" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many generic product management keywords but lacks shipping/logistics specific terms, lowering the ATS score; the biggest gap is missing carrier integration and shipping logistics terminology.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>carrier integration, label generation, shipping logistics, e-commerce marketplace, tracking and billing, compliance, scalability, partner integration, fulfillment</t>
+          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1212,7 +1216,7 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1221,24 +1225,24 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GHX</t>
+          <t>Hitachi Digital Services</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager-63827</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1247,26 +1251,24 @@
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and aligns well with the Product Owner role, yielding strong keyword coverage; the biggest gap is the absence of explicit platform‑scalability and technical‑debt terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>technical debt, platform scalability, security considerations, OKRs, RICE prioritization, A/B testing, roadmap planning, release management</t>
+          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1284,34 +1286,34 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Tachyon Technologies</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>PRODUCT MANAGER L2</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -1320,19 +1322,19 @@
         <v>68</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume covers many core product management keywords but lacks several recruiting‑specific terms, lowering the ATS score; the biggest gap is the absence of recruiting‑domain keywords like candidate matching.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the resume lacks several JD‑specific terms such as RFP, DevOps, and user acceptance testing, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>candidate matching, recruiter agents, job intake automation, sourcing agents, screening agents, interview workflow automation, release notes, AI/ML integration, ATS integration</t>
+          <t>RFP coordination, pre‑sales team collaboration, DevOps integration, user acceptance testing, impact analysis, product vision and roadmap</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1346,59 +1348,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BIG4</t>
+          <t>Modisoft Inc</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Business Analyst\Product Owner (4-7 years Early joiner Preferred)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4-year experience requirement and contains many relevant keywords, but lacks several JD-specific terms and does not clearly indicate Hyderabad location, lowering the ATS score; the strongest keyword gap is the absence of "Roadmap" and related planning terms.</t>
+          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however, key JD terms like retail/restaurant focus, roadmap, and release notes are missing, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Roadmap, Risk Management, Incident Management, User Acceptance Testing (UAT), Customer Centricity, Release Notes, OKRs</t>
+          <t>Retail, Restaurant, product roadmap, release notes, A/B testing, OKRs, customer NPS, AI product strategy</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1412,59 +1414,59 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-63827</t>
+          <t>Digital Product Owner</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+          <t>No hard rule violations; the resume covers many Agile and Jira terms but misses several JD-specific technical backlog concepts, lowering the ATS score. The main keyword gap is the absence of terms like "technical debt" and "regulatory change".</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+          <t>technical debt, KTLO, regulatory change, platform optimisation, risk and controls</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1478,7 +1480,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1487,24 +1489,24 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Modisoft Inc</t>
+          <t>EXL</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, AI</t>
+          <t>Manager-Product Development-Technology/Digital Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1515,22 +1517,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the experience requirement (4 years) and seniority constraints, and contains many of the required keywords, but lacks several AI‑specific terms such as roadmap and release notes.</t>
+          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>AI product roadmap, release notes, A/B testing, OKRs, customer NPS improvement</t>
+          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,215 +1550,17 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Modisoft Inc</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however, key JD terms like retail/restaurant focus, roadmap, and release notes are missing, lowering the ATS score.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Retail, Restaurant, product roadmap, release notes, A/B testing, OKRs, customer NPS, AI product strategy</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Principal Global Services</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager I</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many relevant Agile and product management terms but lacks several data‑analytics specific keywords, lowering the ATS score. The biggest gap is the absence of data‑integration and governance terminology.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Data integration, Data governance, Business intelligence, Hub &amp; spoke operating model, OKRs, KPIs / product health metrics, Report creation, Enterprise Data Foundation</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>EXL</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Manager-Product Development-Technology/Digital Product Owner</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -1777,9 +1581,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1791,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1897,12 +1698,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GreedyGame</t>
+          <t>Capco</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Azure Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1913,22 +1714,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>57</v>
-      </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many JD‑specific tools and mobile‑app domain terms, lowering both scores.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume misses core Azure/cloud keywords, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate job fit.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Firebase Metrics, Google Analytics, BigQuery, Looker Studio, Rewarded/Incentive Mobile Apps, Mobile App User Journey, A/B testing, MAU growth</t>
+          <t>Azure, Microsoft Azure, Cloud services, Azure DevOps, OKRs, A/B testing, Snowflake, NPS improvement, RICE prioritization</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1946,29 +1747,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Tesco Bengaluru</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1982,19 +1783,19 @@
         <v>55</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core payment and checkout keywords from the JD, lowering the ATS score; the biggest gap is the absence of any payments/API experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
+          <t>Online Payments API, OKRs, checkout, basket building, payment methods (card, digital wallets, gift cards, BNPL), authorisation success metrics, settlement process, omnichannel platform</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2017,24 +1818,24 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Xoxoday</t>
+          <t>NTT DATA, Inc.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Plum</t>
+          <t>Product Owner - ServiceNow HRSD AI</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2043,26 +1844,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>62</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 2‑year minimum (4 years experience) and no senior title rule, but the resume lacks many JD‑specific keywords such as API, sales enablement, fintech, and market‑analysis terms, lowering the ATS score. The strongest gap is the absence of any API‑related experience.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific terms (ServiceNow, SAFe, HR, PI planning, ART) resulting in a low ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>API design and documentation, API contracts, sales enablement, fintech / payments, gift cards or rewards, market research, SWOT analysis, competitive analysis, business case development</t>
+          <t>ServiceNow, Now Assist, SAFe, PI planning, Agile Release Train (ART), HR service delivery, ROI analysis, OKRs</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2080,29 +1879,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>eGov Foundation</t>
+          <t>EnglishBhashi</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Digital Health (Public Health)</t>
+          <t>Associate Product Manager(APM)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2113,22 +1912,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H5" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is moderate due to good keyword overlap on product management tools but missing health‑specific terms; fit score is lower because the candidate's domain experience is SaaS/travel rather than digital public health.</t>
+          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>public health, digital public infrastructure, open‑source platform, OKRs, A/B testing, NPS improvement</t>
+          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2146,29 +1945,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EnglishBhashi</t>
+          <t>Nykaa</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(APM)</t>
+          <t>Product Manager II - Personalisation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2179,22 +1978,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>55</v>
-      </c>
       <c r="H6" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
+          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2212,24 +2011,24 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Career Crafterz</t>
+          <t>Xurrent</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2239,28 +2038,30 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years meets 2+ year requirement and title is not senior), but the resume lacks many fintech‑specific keywords such as A/B testing, attach rate, conversion rate, credit underwriting, and risk metrics, leading to low ATS and fit scores.</t>
+          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most ITAM‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of network‑discovery tool names.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, attach rate, conversion rate, credit underwriting, risk metrics, default rate, Excel, consumer lending, market &amp; competitor analysis</t>
+          <t>inTune, Lansweeper, Jamf, LogicMonitor, SNMP, WMI, SSH, SOC 2, ISO certification, KPI‑driven release cycle</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2278,24 +2079,24 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Xurrent</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -2305,30 +2106,28 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most ITAM‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of network‑discovery tool names.</t>
+          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>inTune, Lansweeper, Jamf, LogicMonitor, SNMP, WMI, SSH, SOC 2, ISO certification, KPI‑driven release cycle</t>
+          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2351,52 +2150,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TELUS Digital AI Data Solutions</t>
+          <t>Infineon Technologies</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Robotics</t>
+          <t>Product Owner Hardware Web Experience</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2‑year minimum and has no senior‑level title, but it lacks most robotics and physical‑AI specific keywords, resulting in a low ATS score; the biggest gap is the absence of any robotics or data‑collection platform terminology.</t>
+          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many core hardware/web keywords from the JD, resulting in a low ATS match and poor domain fit.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>robotics, physical AI, data collection platform, sensor data integration, hardware operations</t>
+          <t>A/B testing, Evaluation Board Finder, hardware/web product ownership, CX reports / customer experience analytics, board and kit management</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2419,50 +2216,52 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>QpiAI</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product manager Quantum computers</t>
+          <t>Product Manager- Data and Quality- Associate</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the biggest keyword gap is the lack of any quantum computing or hardware terminology.</t>
+          <t>The candidate meets the years and location requirements, but the resume lacks most of the specific platform and tool keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of ACES/NGP and related data‑platform tools.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>quantum computing, qubit fidelity, hardware roadmap, QCaaS, technical marketing collateral</t>
+          <t>ACES, NGP, QlikSense, Business Objects, Alteryx, Snowflake, change management, defect management, release management, data warehouse</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2480,29 +2279,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Ctruh</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Fraud Rule Platforms</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2523,12 +2322,12 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the absence of fraud‑specific terminology.</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of LLMs, diffusion models, or computer vision.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, risk management, rule engine, fraud rule lifecycle, data governance, A/B testing, OKRs, Snowflake</t>
+          <t>LLMs, diffusion models, computer vision, Python prototyping, OpenAI API integration</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2546,17 +2345,17 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -2622,19 +2421,19 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>KredX</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>L50 - Product Manager I</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2645,22 +2444,22 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of 'customer acquisition' or related metrics.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit profit &amp; loss ownership terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>customer acquisition, product placement, messaging, roadmap development, OKRs, A/B testing, NPS improvement</t>
+          <t>profit and loss ownership, KPIs, OKRs, market research, user research, competitive analysis, roadmap, product vision</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2678,29 +2477,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>The IT Firm</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Fraud Rule Platforms</t>
+          <t>Technical/Functional CLM Consultant/Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2714,19 +2513,19 @@
         <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit fraud‑related terminology.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core CLM and AI/LLM keywords.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, risk management, rule engine, fraud analytics, regulatory compliance</t>
+          <t>Icertis, Conga, REST API integrations, AWS / Azure / GCP, OCR &amp; Document Intelligence, Vector Search / RAG Architecture, Contract Summarization, Clause Extraction, Risk Scoring, Enterprise CLM workflow automation</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2744,29 +2543,29 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Mojro</t>
+          <t>Luxoft</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner - Cash Management (Small and medium enterprises)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2787,12 +2586,12 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key logistics and supply‑chain terminology such as "digital twin" and "logistics optimization".</t>
+          <t>The JD requires 12+ years total experience (well above the candidate's 4 years), triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any banking or cash‑management specific terms.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>digital twin, logistics optimization, supply chain analytics, OKRs, RICE prioritization, customer journey mapping, NPS improvement, A/B testing</t>
+          <t>SME cash management, mobile banking, payment &amp; collections, regulatory framework, OKRs, self‑serve capabilities, omnichannel strategy, user onboarding for banking</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2810,17 +2609,17 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -2886,45 +2685,45 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Olympus Corporation</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Solutions Product Owner</t>
+          <t>Product Manager - Payments</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many supply chain‑specific terms (SAP, o9, UAT, training/adoption) and only partially matches the JD keywords, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4, o9, UAT, training and adoption, roadmap</t>
+          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2938,33 +2737,33 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>L50 - Product Manager I</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2975,22 +2774,22 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit profit &amp; loss ownership terminology.</t>
+          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>profit and loss ownership, KPIs, OKRs, market research, user research, competitive analysis, roadmap, product vision</t>
+          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3008,55 +2807,55 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>Keyloop</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>45</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>65</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>53</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management terms but misses several core JD keywords (e.g., technical debt, KTLO, incident management) and the location does not match Pune, lowering the ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably with the role.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>technical debt, KTLO, regulatory change, platform optimisation, incident management, operational resilience, governance standards, architecture standards, security standards, market research</t>
+          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3070,59 +2869,59 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Aumni</t>
+          <t>Olympus Corporation</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Roadmap &amp;amp; Strategy</t>
+          <t>Supply Chain Solutions Product Owner</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Candidate has only 4 years experience while the JD explicitly requires 5+ years, triggering a hard rule that caps both scores below 30; also the resume lacks several core JD keywords such as Confluence and roadmap planning.</t>
+          <t>Hard rules pass, but the resume lacks many supply chain‑specific terms (SAP, o9, UAT, training/adoption) and only partially matches the JD keywords, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Confluence, AI/ML platforms, roadmap planning, product strategy, OKRs, RICE prioritization, NPS improvement, A/B testing, Snowflake</t>
+          <t>SAP S/4, o9, UAT, training and adoption, roadmap</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3136,11 +2935,11 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -3150,45 +2949,45 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Manager -VP</t>
+          <t>Product Owner - Specialist Manager, Project - Hyderabad</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD title includes 'VP', triggering hard rule 3, so both scores must be below 30 regardless of experience; the most important keyword gap is the absence of explicit 'OKRs' and 'AI Banking Companion' terminology.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "change management" and "operational metrics".</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>OKRs, AI Banking Companion, customer journey mapping, risk compliance, regulatory compliance</t>
+          <t>change management, operational metrics, release readiness, defect resolution, standard operating procedures, risk indicators, roadmap planning, governance</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3202,38 +3001,38 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -3249,40 +3048,372 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Sonata Software</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager (E-Commerce)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Pune District, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules are satisfied; however the resume lacks many JD-specific terms (e.g., POS, inventory management, circular economy) and does not show Pune location, resulting in a modest ATS score. The candidate’s GenAI and SaaS experience aligns reasonably with the role, giving a moderate fit score.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Point-of-Sale, inventory management, circular economy, field service management, pricing optimisation, CRM, fleet management, demand forecasting, OKRs</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Digital Product Owner</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>The resume contains many relevant product management terms but misses several core JD keywords (e.g., technical debt, KTLO, incident management) and the location does not match Pune, lowering the ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably with the role.</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>technical debt, KTLO, regulatory change, platform optimisation, incident management, operational resilience, governance standards, architecture standards, security standards, market research</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Unbox Robotics</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>The resume lacks core hardware and robotics keywords required by the JD and does not demonstrate experience with EVT/DVT/PVT cycles, resulting in a low ATS score; the biggest gap is the absence of any hardware product development terminology.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>EVT, DVT, PVT, NPI, robotics, industrial automation, IoT hardware, hardware roadmap, supply chain coordination, embedded control units</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Aumni</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner - Roadmap &amp;amp; Strategy</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Candidate has only 4 years experience while the JD explicitly requires 5+ years, triggering a hard rule that caps both scores below 30; also the resume lacks several core JD keywords such as Confluence and roadmap planning.</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Confluence, AI/ML platforms, roadmap planning, product strategy, OKRs, RICE prioritization, NPS improvement, A/B testing, Snowflake</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Virtusa</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Product Owner</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
           <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
         </is>
       </c>
     </row>
@@ -3309,6 +3440,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-05-31
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -626,19 +626,19 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Leucine - AI for Pharma</t>
+          <t>MiQ</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,26 +647,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title aligns, but lacks key tech keywords (React, Node.js, vibe‑coding, B.Tech, explicit PRD) which lowers the ATS score; overall fit is solid on SaaS and GenAI but pharma domain is only tangential.</t>
+          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>React, Node.js, vibe‑coding, B.Tech, PRD</t>
+          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +682,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Signzy</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Personalization &amp; Data Platforms</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -715,24 +713,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience matches the non‑specified minimum). The resume covers many relevant skills but misses several core JD terms like product strategy and pricing plans, lowering the ATS score; overall domain and experience alignment is strong, yielding a solid fit score.</t>
+          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>product strategy, pricing plans, target segment, partnerships, quality assurance testing, distribution partners, campaign strategies, original research, structured thinking</t>
+          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,29 +750,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>Hinge Health</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Personalization &amp; Data Platforms</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -781,26 +781,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
+          <t>The candidate meets the 3+ years requirement and has a relevant title, so hard rules do not penalize. The resume covers many core keywords (Jira, Agile, SQL, Power BI, GenAI) but misses several JD‑specific terms such as RBAC, audit logging, and algorithmic matching, limiting the ATS score.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
+          <t>RBAC, audit logging, algorithmic matching, capacity management, microservices architecture, OKRs, KPIs, roadmap</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -818,17 +816,17 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -884,7 +882,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -894,19 +892,19 @@
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Peoplebox.ai</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (APM)</t>
+          <t>Product Manager -Growth</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -915,26 +913,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and title level, but the resume lacks many exact JD keywords such as product discovery and success metrics, lowering the ATS score; overall domain and experience align well, giving a solid fit score.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, stakeholder management, SaaS, data‑driven) but lacks growth‑specific terms, lowering the ATS score. The biggest keyword gap is the absence of explicit growth‑experiment language such as "A/B testing".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Product Discovery, customer interviews, data analysis, competitive research, success metrics, product roadmap, AI tools, prototypes, mockups</t>
+          <t>A/B testing, Mixpanel, Snowflake, OKRs, Referral program, Loyalty program, Personalized notifications, Cohort analysis</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -952,29 +948,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Peoplebox.ai</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Tech</t>
+          <t>Associate Product Manager (APM)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -983,24 +979,26 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F8" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many generic product management keywords but lacks shipping/logistics specific terms, lowering the ATS score; the biggest gap is missing carrier integration and shipping logistics terminology.</t>
+          <t>The candidate meets the years requirement and title level, but the resume lacks many exact JD keywords such as product discovery and success metrics, lowering the ATS score; overall domain and experience align well, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>carrier integration, label generation, shipping logistics, e-commerce marketplace, tracking and billing, compliance, scalability, partner integration, fulfillment</t>
+          <t>Product Discovery, customer interviews, data analysis, competitive research, success metrics, product roadmap, AI tools, prototypes, mockups</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,29 +1016,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kroll</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager - Tech</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1051,22 +1049,22 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H9" s="2" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many generic product management keywords but lacks shipping/logistics specific terms, lowering the ATS score; the biggest gap is missing carrier integration and shipping logistics terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
+          <t>carrier integration, label generation, shipping logistics, e-commerce marketplace, tracking and billing, compliance, scalability, partner integration, fulfillment</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1089,52 +1087,50 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Kroll</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner — General</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
+          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
+          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,21 +1144,21 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1170,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (Tax)</t>
+          <t>Product Owner — General</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1184,25 +1180,25 @@
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>69</v>
-      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
+          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
+          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1220,7 +1216,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1230,19 +1226,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services</t>
+          <t>Merck Life Science</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-63827</t>
+          <t>Global Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1253,22 +1249,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1286,55 +1282,57 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER L2</t>
+          <t>Product Owner (Tax)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F13" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the resume lacks several JD‑specific terms such as RFP, DevOps, and user acceptance testing, lowering the ATS score.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>RFP coordination, pre‑sales team collaboration, DevOps integration, user acceptance testing, impact analysis, product vision and roadmap</t>
+          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1348,59 +1346,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Modisoft Inc</t>
+          <t>Hitachi Digital Services</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-63827</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however, key JD terms like retail/restaurant focus, roadmap, and release notes are missing, lowering the ATS score.</t>
+          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Retail, Restaurant, product roadmap, release notes, A/B testing, OKRs, customer NPS, AI product strategy</t>
+          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1414,7 +1412,7 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1423,24 +1421,24 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>hackajob</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner</t>
+          <t>Associate Product Manager | Pune</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1451,22 +1449,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>No hard rule violations; the resume covers many Agile and Jira terms but misses several JD-specific technical backlog concepts, lowering the ATS score. The main keyword gap is the absence of terms like "technical debt" and "regulatory change".</t>
+          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>technical debt, KTLO, regulatory change, platform optimisation, risk and controls</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1489,24 +1487,24 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>EXL</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Manager-Product Development-Technology/Digital Product Owner</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1517,22 +1515,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
+          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
+          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1550,17 +1548,413 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Wipro</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT MANAGER L2</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the resume lacks several JD‑specific terms such as RFP, DevOps, and user acceptance testing, lowering the ATS score.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>RFP coordination, pre‑sales team collaboration, DevOps integration, user acceptance testing, impact analysis, product vision and roadmap</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PerkinElmer</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Software Product Manager (GTM Strategy)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) giving a strong ATS score, but lacks domain-specific scientific software experience, lowering the fit score.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>go-to-market strategy, customer migration, adoption metrics, NPS improvement, OKRs</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>House Of Edtech</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager — Learning &amp; EdTech</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the experience requirement (4 years vs 2-3 years needed) and title alignment, but lacks several JD-specific tools and mobile platform keywords, lowering the ATS score; the biggest gap is the absence of analytics tools like Amplitude or Mixpanel.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Amplitude, Mixpanel, Google Analytics, iOS, Android, A/B testing, OKRs</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Modisoft Inc</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Product Manager</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however, key JD terms like retail/restaurant focus, roadmap, and release notes are missing, lowering the ATS score.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Retail, Restaurant, product roadmap, release notes, A/B testing, OKRs, customer NPS, AI product strategy</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>EXL</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Manager-Product Development-Technology/Digital Product Owner</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>House Of Edtech</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager — Consumer &amp; Streaming</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Pune Division, Maharashtra, India</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>The resume meets the years requirement and title level, but lacks several consumer‑streaming specific keywords, lowering the ATS score; the biggest gap is the absence of product analytics tools like Mixpanel/Amplitude.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Mixpanel, Amplitude, Firebase, product roadmap, PRD, backlog grooming, user research, usability testing, NPS improvement, MAU growth</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Linkedin</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -1581,6 +1975,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1698,12 +2098,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Capco</t>
+          <t>Endava</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Azure Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1714,22 +2114,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>58</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no 5+ year requirement). The resume misses core Azure/cloud keywords, lowering the ATS score, while the candidate's SaaS and GenAI background gives a moderate job fit.</t>
+          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Azure, Microsoft Azure, Cloud services, Azure DevOps, OKRs, A/B testing, Snowflake, NPS improvement, RICE prioritization</t>
+          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1747,24 +2147,24 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Tesco Bengaluru</t>
+          <t>GreedyGame</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1780,22 +2180,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>55</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>60</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>57</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core payment and checkout keywords from the JD, lowering the ATS score; the biggest gap is the absence of any payments/API experience.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks many JD‑specific tools and mobile‑app domain terms, lowering both scores.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, basket building, payment methods (card, digital wallets, gift cards, BNPL), authorisation success metrics, settlement process, omnichannel platform</t>
+          <t>Firebase Metrics, Google Analytics, BigQuery, Looker Studio, Rewarded/Incentive Mobile Apps, Mobile App User Journey, A/B testing, MAU growth</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1813,55 +2213,55 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>NTT DATA, Inc.</t>
+          <t>Tesco Bengaluru</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - ServiceNow HRSD AI</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific terms (ServiceNow, SAFe, HR, PI planning, ART) resulting in a low ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a moderate job‑fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core payment and checkout keywords from the JD, lowering the ATS score; the biggest gap is the absence of any payments/API experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, Now Assist, SAFe, PI planning, Agile Release Train (ART), HR service delivery, ROI analysis, OKRs</t>
+          <t>Online Payments API, OKRs, checkout, basket building, payment methods (card, digital wallets, gift cards, BNPL), authorisation success metrics, settlement process, omnichannel platform</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1889,19 +2289,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>EnglishBhashi</t>
+          <t>Razorpay</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager(APM)</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1912,22 +2312,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>55</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, matching title, location), but lacks many JD-specific tools and user‑research keywords, lowering the ATS score; the domain mismatch (EdTech vs SaaS/Travel) reduces the fit score.</t>
+          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Amplitude, Mixpanel, Firebase, Microsoft Clarity, CleverTap, MoEngage, WebEngage, push notifications, in‑app messaging, gamification</t>
+          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1945,55 +2345,55 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Nykaa</t>
+          <t>NTT DATA, Inc.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Personalisation</t>
+          <t>Product Owner - ServiceNow HRSD AI</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific terms (ServiceNow, SAFe, HR, PI planning, ART) resulting in a low ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a moderate job‑fit.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
+          <t>ServiceNow, Now Assist, SAFe, PI planning, Agile Release Train (ART), HR service delivery, ROI analysis, OKRs</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2011,57 +2411,55 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Xurrent</t>
+          <t>Nykaa</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager II - Personalisation</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most ITAM‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of network‑discovery tool names.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>inTune, Lansweeper, Jamf, LogicMonitor, SNMP, WMI, SSH, SOC 2, ISO certification, KPI‑driven release cycle</t>
+          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2079,55 +2477,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>TE Connectivity</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>PRODUCT MANAGER INDIA ( Panel &amp; Relay Solutions)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
+          <t>The resume lacks many core JD keywords such as go‑to‑market strategy, pricing support, and portfolio P&amp;L, resulting in a low ATS match; also the candidate's SaaS/GenAI background does not align well with the industrial panel &amp; relay hardware domain.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
+          <t>go to market strategy, pricing support, portfolio P&amp;L, competitive analysis, market segmentation, voice of customer, product lifecycle management, 5‑year strategic growth plan, channel strategy, sales enablement training</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2145,55 +2543,57 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Infineon Technologies</t>
+          <t>Xurrent</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner Hardware Web Experience</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bangalore Urban, Karnataka, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F9" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement, but the resume lacks many core hardware/web keywords from the JD, resulting in a low ATS match and poor domain fit.</t>
+          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most ITAM‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of network‑discovery tool names.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Evaluation Board Finder, hardware/web product ownership, CX reports / customer experience analytics, board and kit management</t>
+          <t>inTune, Lansweeper, Jamf, LogicMonitor, SNMP, WMI, SSH, SOC 2, ISO certification, KPI‑driven release cycle</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2211,29 +2611,29 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager- Data and Quality- Associate</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2242,26 +2642,24 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years and location requirements, but the resume lacks most of the specific platform and tool keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of ACES/NGP and related data‑platform tools.</t>
+          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>ACES, NGP, QlikSense, Business Objects, Alteryx, Snowflake, change management, defect management, release management, data warehouse</t>
+          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2279,29 +2677,29 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Ctruh</t>
+          <t>Luxoft</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>AI Product Manager</t>
+          <t>Product Owner - Cash Management (Small and medium enterprises)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2312,22 +2710,22 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of LLMs, diffusion models, or computer vision.</t>
+          <t>The JD requires 12+ years total experience (well above the candidate's 4 years), triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any banking or cash‑management specific terms.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>LLMs, diffusion models, computer vision, Python prototyping, OpenAI API integration</t>
+          <t>SME cash management, mobile banking, payment &amp; collections, regulatory framework, OKRs, self‑serve capabilities, omnichannel strategy, user onboarding for banking</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2345,7 +2743,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -2355,19 +2753,19 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Luxoft</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>L55 - Product Manager II</t>
+          <t>Product Owner - SME Cash Management</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2378,22 +2776,22 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit KPI/OKR or profit‑and‑loss responsibility language.</t>
+          <t>The JD requires 12+ years of experience (and 8+ years as a Product Owner), which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks many core banking and SME cash‑management keywords.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>profit and loss ownership, KPIs, OKRs, market research, competitive analysis, user research, roadmap, product vision</t>
+          <t>SME cash management, mobile banking, web banking, OKRs, regulatory framework, payments &amp; collections, self‑serve capabilities (e‑statements, account management), omnichannel strategy</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2411,34 +2809,34 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>American Express Global Business Travel</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>L50 - Product Manager I</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bengaluru East, Karnataka, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
@@ -2447,19 +2845,19 @@
         <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that caps both scores below 30; the most important keyword gap is the absence of explicit profit &amp; loss ownership terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like "WordPress" and "API integrations".</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>profit and loss ownership, KPIs, OKRs, market research, user research, competitive analysis, roadmap, product vision</t>
+          <t>WordPress, API integrations, content management system, website performance monitoring, vendor management</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2477,29 +2875,29 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>The IT Firm</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Technical/Functional CLM Consultant/Product Manager</t>
+          <t>Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2513,19 +2911,19 @@
         <v>25</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core CLM and AI/LLM keywords.</t>
+          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Icertis, Conga, REST API integrations, AWS / Azure / GCP, OCR &amp; Document Intelligence, Vector Search / RAG Architecture, Contract Summarization, Clause Extraction, Risk Scoring, Enterprise CLM workflow automation</t>
+          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2543,55 +2941,55 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Luxoft</t>
+          <t>Optum India</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Cash Management (Small and medium enterprises)</t>
+          <t>Technical Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years total experience (well above the candidate's 4 years), triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any banking or cash‑management specific terms.</t>
+          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>SME cash management, mobile banking, payment &amp; collections, regulatory framework, OKRs, self‑serve capabilities, omnichannel strategy, user onboarding for banking</t>
+          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2605,28 +3003,28 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Wayfair</t>
+          <t>Keyloop</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -2636,28 +3034,28 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any supply‑chain or fulfillment terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Supply chain, Fulfillment, Inventory management, Warehouse operations, LLM‑powered experiences, Roadmap prioritization, Scalable architecture, Operational leaders</t>
+          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -2671,59 +3069,59 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Payments</t>
+          <t>Product Manager (Materials Program)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several core payment‑domain keywords.</t>
+          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>payment integrations, API management, transaction flow optimization, regulatory compliance, payment success rate, A/B testing, OKRs</t>
+          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2737,33 +3135,33 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Olympus Corporation</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Supply Chain Solutions Product Owner</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -2777,19 +3175,19 @@
         <v>55</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
+          <t>Hard rules pass, but the resume lacks many supply chain‑specific terms (SAP, o9, UAT, training/adoption) and only partially matches the JD keywords, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
+          <t>SAP S/4, o9, UAT, training and adoption, roadmap</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2807,29 +3205,29 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Keyloop</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner - Specialist Manager, Project - Hyderabad</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2840,22 +3238,22 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "change management" and "operational metrics".</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
+          <t>change management, operational metrics, release readiness, defect resolution, standard operating procedures, risk indicators, roadmap planning, governance</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2873,29 +3271,29 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Olympus Corporation</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Solutions Product Owner</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2906,22 +3304,22 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many supply chain‑specific terms (SAP, o9, UAT, training/adoption) and only partially matches the JD keywords, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4, o9, UAT, training and adoption, roadmap</t>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -2944,50 +3342,50 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Specialist Manager, Project - Hyderabad</t>
+          <t>Product Manager (E-Commerce)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "change management" and "operational metrics".</t>
+          <t>Hard rules are satisfied; however the resume lacks many JD-specific terms (e.g., POS, inventory management, circular economy) and does not show Pune location, resulting in a modest ATS score. The candidate’s GenAI and SaaS experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>change management, operational metrics, release readiness, defect resolution, standard operating procedures, risk indicators, roadmap planning, governance</t>
+          <t>Point-of-Sale, inventory management, circular economy, field service management, pricing optimisation, CRM, fleet management, demand forecasting, OKRs</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3001,11 +3399,11 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -3015,45 +3413,45 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Xplor Technologies</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Product Owner, Billing &amp; Settlement</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3067,7 +3465,7 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -3076,50 +3474,52 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>Unbox Robotics</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (E-Commerce)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Pune District, Maharashtra, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F23" s="2" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; however the resume lacks many JD-specific terms (e.g., POS, inventory management, circular economy) and does not show Pune location, resulting in a modest ATS score. The candidate’s GenAI and SaaS experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>The resume lacks core hardware and robotics keywords required by the JD and does not demonstrate experience with EVT/DVT/PVT cycles, resulting in a low ATS score; the biggest gap is the absence of any hardware product development terminology.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Point-of-Sale, inventory management, circular economy, field service management, pricing optimisation, CRM, fleet management, demand forecasting, OKRs</t>
+          <t>EVT, DVT, PVT, NPI, robotics, industrial automation, IoT hardware, hardware roadmap, supply chain coordination, embedded control units</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -3137,7 +3537,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -3147,19 +3547,19 @@
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Barclays</t>
+          <t>Aumni</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Digital Product Owner</t>
+          <t>Product Owner - Roadmap &amp;amp; Strategy</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3170,22 +3570,22 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management terms but misses several core JD keywords (e.g., technical debt, KTLO, incident management) and the location does not match Pune, lowering the ATS score; however, the candidate's SaaS and GenAI experience aligns reasonably with the role.</t>
+          <t>Candidate has only 4 years experience while the JD explicitly requires 5+ years, triggering a hard rule that caps both scores below 30; also the resume lacks several core JD keywords such as Confluence and roadmap planning.</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>technical debt, KTLO, regulatory change, platform optimisation, incident management, operational resilience, governance standards, architecture standards, security standards, market research</t>
+          <t>Confluence, AI/ML platforms, roadmap planning, product strategy, OKRs, RICE prioritization, NPS improvement, A/B testing, Snowflake</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -3203,29 +3603,29 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Unbox Robotics</t>
+          <t>Virtusa</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -3234,26 +3634,24 @@
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core hardware and robotics keywords required by the JD and does not demonstrate experience with EVT/DVT/PVT cycles, resulting in a low ATS score; the biggest gap is the absence of any hardware product development terminology.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>EVT, DVT, PVT, NPI, robotics, industrial automation, IoT hardware, hardware roadmap, supply chain coordination, embedded control units</t>
+          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -3271,29 +3669,29 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Aumni</t>
+          <t>Sibros</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Roadmap &amp;amp; Strategy</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3307,19 +3705,19 @@
         <v>25</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Candidate has only 4 years experience while the JD explicitly requires 5+ years, triggering a hard rule that caps both scores below 30; also the resume lacks several core JD keywords such as Confluence and roadmap planning.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Confluence, AI/ML platforms, roadmap planning, product strategy, OKRs, RICE prioritization, NPS improvement, A/B testing, Snowflake</t>
+          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -3337,55 +3735,57 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>Azuga, Inc.</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager – Connected Hardware &amp; Telematics (HW / FW / IoT)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Bagalur, Karnataka, India</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F27" s="2" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
+          <t>The candidate meets the 3‑year minimum experience, but the resume lacks most hardware/IoT keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of telematics and firmware terminology.</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
+          <t>OBD‑II, J1939, CAN protocol, OTA firmware upgrade, BLE beacon, LTE Cat M1, FCC certification, telematics vendor management</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -3399,7 +3799,7 @@
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
@@ -3408,12 +3808,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: daily job scan 2026-06-01
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,38 +567,38 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>85</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and the title aligns, so hard rules do not penalize; it contains many JD keywords but lacks a few core terms like data ingestion and governance.</t>
+          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>data ingestion, data governance, self‑service platform, usability studies, market analysis, metrics tracking, A/B testing</t>
+          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -616,29 +616,29 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MiQ</t>
+          <t>MakeMyTrip</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Personalization &amp; Data Platforms</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,24 +647,26 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F3" s="2" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ year requirement and includes many JD keywords, yielding a strong ATS score; however, the candidate's domain (SaaS/GenAI) does not closely match MiQ's ad‑tech/programmatic focus, creating a moderate fit gap.</t>
+          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>programmatic, advertising technology, A/B testing, OKRs, Mixpanel, Snowflake</t>
+          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -682,7 +684,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -692,19 +694,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>Hinge Health</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Personalization &amp; Data Platforms</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -713,26 +715,24 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
+          <t>The candidate meets the 3+ years requirement and has a relevant title, so hard rules do not penalize. The resume covers many core keywords (Jira, Agile, SQL, Power BI, GenAI) but misses several JD‑specific terms such as RBAC, audit logging, and algorithmic matching, limiting the ATS score.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
+          <t>RBAC, audit logging, algorithmic matching, capacity management, microservices architecture, OKRs, KPIs, roadmap</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -755,24 +755,24 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hinge Health</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager, Amazon Business India</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -783,22 +783,22 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>69</v>
-      </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and has a relevant title, so hard rules do not penalize. The resume covers many core keywords (Jira, Agile, SQL, Power BI, GenAI) but misses several JD‑specific terms such as RBAC, audit logging, and algorithmic matching, limiting the ATS score.</t>
+          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>RBAC, audit logging, algorithmic matching, capacity management, microservices architecture, OKRs, KPIs, roadmap</t>
+          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -821,24 +821,24 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Axi</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Business India</t>
+          <t>Product Manager -Growth</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -849,22 +849,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, stakeholder management, SaaS, data‑driven) but lacks growth‑specific terms, lowering the ATS score. The biggest keyword gap is the absence of explicit growth‑experiment language such as "A/B testing".</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
+          <t>A/B testing, Mixpanel, Snowflake, OKRs, Referral program, Loyalty program, Personalized notifications, Cohort analysis</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -887,24 +887,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Peoplebox.ai</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Growth</t>
+          <t>Associate Product Manager (APM)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -913,24 +913,26 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F7" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="H7" s="2" t="n">
-        <v>66</v>
-      </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, stakeholder management, SaaS, data‑driven) but lacks growth‑specific terms, lowering the ATS score. The biggest keyword gap is the absence of explicit growth‑experiment language such as "A/B testing".</t>
+          <t>The candidate meets the years requirement and title level, but the resume lacks many exact JD keywords such as product discovery and success metrics, lowering the ATS score; overall domain and experience align well, giving a solid fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Snowflake, OKRs, Referral program, Loyalty program, Personalized notifications, Cohort analysis</t>
+          <t>Product Discovery, customer interviews, data analysis, competitive research, success metrics, product roadmap, AI tools, prototypes, mockups</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -953,29 +955,29 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Peoplebox.ai</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (APM)</t>
+          <t>Product Owner — General</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -983,22 +985,22 @@
         <v>2</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="G8" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="H8" s="2" t="n">
-        <v>64</v>
-      </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and title level, but the resume lacks many exact JD keywords such as product discovery and success metrics, lowering the ATS score; overall domain and experience align well, giving a solid fit score.</t>
+          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Product Discovery, customer interviews, data analysis, competitive research, success metrics, product roadmap, AI tools, prototypes, mockups</t>
+          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1012,7 +1014,7 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1021,50 +1023,50 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Merck Life Science</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Tech</t>
+          <t>Global Product Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title requirement). The resume contains many generic product management keywords but lacks shipping/logistics specific terms, lowering the ATS score; the biggest gap is missing carrier integration and shipping logistics terminology.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>carrier integration, label generation, shipping logistics, e-commerce marketplace, tracking and billing, compliance, scalability, partner integration, fulfillment</t>
+          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1078,59 +1080,61 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Kroll</t>
+          <t>InvoiceCloud, Inc.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Owner (Tax)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F10" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>68</v>
-      </c>
       <c r="H10" s="2" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and seniority constraints, but it lacks many JD‑specific terms such as roadmap, backlog, data governance, and KPI metrics, lowering the ATS score; the strongest keyword gap is the absence of any mention of a product roadmap or backlog.</t>
+          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>roadmap, backlog, data governance, BI/Reporting, KPIs, success metrics, release discipline</t>
+          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1144,61 +1148,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner — General</t>
+          <t>Associate Product Manager | Pune</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
+          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1212,11 +1214,11 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1226,45 +1228,45 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Merck Life Science</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Global Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
+          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
+          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1278,11 +1280,11 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1292,47 +1294,45 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>PerkinElmer</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (Tax)</t>
+          <t>Software Product Manager (GTM Strategy)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) giving a strong ATS score, but lacks domain-specific scientific software experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
+          <t>go-to-market strategy, customer migration, adoption metrics, NPS improvement, OKRs</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1346,59 +1346,59 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Hitachi Digital Services</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-63827</t>
+          <t>PRODUCT MANAGER L2</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title, no 5+ year requirement). ATS score is solid due to strong keyword overlap (Jira, Agile, SaaS, GenAI, RAG, Power BI, SQL, stakeholder management). Fit score is lower because the candidate's domain (SaaS, travel, FMCG) does not align well with the MES/Digital Manufacturing focus of the role.</t>
+          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the resume lacks several JD‑specific terms such as RFP, DevOps, and user acceptance testing, lowering the ATS score.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>MES, IIoT, Industry 4.0, Lean, Operational Excellence, Roadmap, OKRs</t>
+          <t>RFP coordination, pre‑sales team collaboration, DevOps integration, user acceptance testing, impact analysis, product vision and roadmap</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1412,33 +1412,33 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>House Of Edtech</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager | Pune</t>
+          <t>Associate Product Manager — Learning &amp; EdTech</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1449,22 +1449,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
+          <t>The candidate meets the experience requirement (4 years vs 2-3 years needed) and title alignment, but lacks several JD-specific tools and mobile platform keywords, lowering the ATS score; the biggest gap is the absence of analytics tools like Amplitude or Mixpanel.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
+          <t>Amplitude, Mixpanel, Google Analytics, iOS, Android, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1482,29 +1482,29 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>hackajob</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Digital Product Owner</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1515,22 +1515,22 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
+          <t>No hard rule violations; the resume covers many Agile and Jira terms but misses several JD-specific technical backlog concepts, lowering the ATS score. The main keyword gap is the absence of terms like "technical debt" and "regulatory change".</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
+          <t>technical debt, KTLO, regulatory change, platform optimisation, risk and controls</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1548,29 +1548,29 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Wipro</t>
+          <t>House Of Edtech</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER L2</t>
+          <t>Associate Product Manager — Consumer &amp; Streaming</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1581,22 +1581,22 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the resume lacks several JD‑specific terms such as RFP, DevOps, and user acceptance testing, lowering the ATS score.</t>
+          <t>The resume meets the years requirement and title level, but lacks several consumer‑streaming specific keywords, lowering the ATS score; the biggest gap is the absence of product analytics tools like Mixpanel/Amplitude.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>RFP coordination, pre‑sales team collaboration, DevOps integration, user acceptance testing, impact analysis, product vision and roadmap</t>
+          <t>Mixpanel, Amplitude, Firebase, product roadmap, PRD, backlog grooming, user research, usability testing, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1619,342 +1619,12 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>PerkinElmer</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Software Product Manager (GTM Strategy)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) giving a strong ATS score, but lacks domain-specific scientific software experience, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>go-to-market strategy, customer migration, adoption metrics, NPS improvement, OKRs</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>House Of Edtech</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager — Learning &amp; EdTech</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the experience requirement (4 years vs 2-3 years needed) and title alignment, but lacks several JD-specific tools and mobile platform keywords, lowering the ATS score; the biggest gap is the absence of analytics tools like Amplitude or Mixpanel.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Amplitude, Mixpanel, Google Analytics, iOS, Android, A/B testing, OKRs</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Modisoft Inc</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3+ years requirement (4 years) and has no senior title, so hard rules pass; however, key JD terms like retail/restaurant focus, roadmap, and release notes are missing, lowering the ATS score.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Retail, Restaurant, product roadmap, release notes, A/B testing, OKRs, customer NPS, AI product strategy</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>EXL</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Manager-Product Development-Technology/Digital Product Owner</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass; the resume contains many JD keywords and relevant tools, but the candidate's domain (travel tech, SaaS, GenAI) does not align with the FNOL/insurance focus of the role, creating the biggest gap.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>FNON, Insurance claims, Service Level Agreement, Transaction monitoring, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>House Of Edtech</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager — Consumer &amp; Streaming</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the years requirement and title level, but lacks several consumer‑streaming specific keywords, lowering the ATS score; the biggest gap is the absence of product analytics tools like Mixpanel/Amplitude.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Mixpanel, Amplitude, Firebase, product roadmap, PRD, backlog grooming, user research, usability testing, NPS improvement, MAU growth</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -1976,11 +1646,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1992,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2098,12 +1763,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Endava</t>
+          <t>Abnormal AI</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager II</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2114,22 +1779,22 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
+          <t>The resume meets the hard rules but contains only partial keyword overlap with the JD, especially missing core integration and API lifecycle terms, leading to a moderate ATS score; the candidate's SaaS and GenAI background aligns reasonably with the role, giving a decent fit score.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
+          <t>REST API, SIEM integration, SOAR integration, API lifecycle management, token management, versioning, schema governance, MCP server, notifications, product configuration</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2152,24 +1817,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GreedyGame</t>
+          <t>Endava</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2180,22 +1845,22 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>57</v>
-      </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks many JD‑specific tools and mobile‑app domain terms, lowering both scores.</t>
+          <t>The resume meets the 4‑year experience requirement and location, so hard rules pass; however, key FinTech and fraud‑detection terms are missing, lowering the ATS keyword density. The biggest gap is the lack of fraud‑detection / regulatory experience.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Firebase Metrics, Google Analytics, BigQuery, Looker Studio, Rewarded/Incentive Mobile Apps, Mobile App User Journey, A/B testing, MAU growth</t>
+          <t>fraud detection, financial crime, real-time fraud prevention, regulatory compliance, risk management, ROI analysis, non-functional requirements, user journey mapping</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2213,17 +1878,17 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -2289,19 +1954,19 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Razorpay</t>
+          <t>Booking Holdings (NASDAQ: BKNG)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2310,7 +1975,9 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F5" s="2" t="n">
         <v>55</v>
       </c>
@@ -2322,12 +1989,12 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many fintech‑specific keywords and domain experience, leading to moderate ATS and fit scores; the biggest gap is the absence of payment‑processing terminology.</t>
+          <t>The candidate meets the 4‑year requirement, but the resume lacks many FinTech/payment‑specific keywords and direct experience, resulting in moderate ATS and fit scores; the biggest gap is missing payment‑domain terminology.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>payments processing, fraud detection, automated reconciliation, payroll automation, checkout experience, risk intelligence, OKRs, A/B testing, Mixpanel</t>
+          <t>Payment Service Provider (PSP), Alternative Payment Methods (APM), FinTech, Payment gateway integration, Conversion rate optimization, KPI tracking, A/B testing, OKRs, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2350,50 +2017,50 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NTT DATA, Inc.</t>
+          <t>Nykaa</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - ServiceNow HRSD AI</t>
+          <t>Product Manager II - Personalisation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>54</v>
-      </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific terms (ServiceNow, SAFe, HR, PI planning, ART) resulting in a low ATS score; however, the candidate's GenAI and enterprise SaaS experience gives a moderate job‑fit.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>ServiceNow, Now Assist, SAFe, PI planning, Agile Release Train (ART), HR service delivery, ROI analysis, OKRs</t>
+          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2416,24 +2083,24 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Nykaa</t>
+          <t>Tesco Technology</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Personalisation</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2444,22 +2111,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
+          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
+          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2482,50 +2149,50 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TE Connectivity</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PRODUCT MANAGER INDIA ( Panel &amp; Relay Solutions)</t>
+          <t>Product Manager - HashiCorp Boundary</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks many core JD keywords such as go‑to‑market strategy, pricing support, and portfolio P&amp;L, resulting in a low ATS match; also the candidate's SaaS/GenAI background does not align well with the industrial panel &amp; relay hardware domain.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'Privileged Access Management'.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>go to market strategy, pricing support, portfolio P&amp;L, competitive analysis, market segmentation, voice of customer, product lifecycle management, 5‑year strategic growth plan, channel strategy, sales enablement training</t>
+          <t>Privileged Access Management, session recording, secrets management, PKI, threat monitoring</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2543,29 +2210,29 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Xurrent</t>
+          <t>Virtusa</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2574,26 +2241,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title), but the resume lacks most ITAM‑specific keywords and domain experience, resulting in low ATS and fit scores; the biggest gap is the absence of network‑discovery tool names.</t>
+          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>inTune, Lansweeper, Jamf, LogicMonitor, SNMP, WMI, SSH, SOC 2, ISO certification, KPI‑driven release cycle</t>
+          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2611,55 +2276,55 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>40</v>
-      </c>
       <c r="H10" s="2" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2673,59 +2338,59 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Luxoft</t>
+          <t>Keyloop</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Cash Management (Small and medium enterprises)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years total experience (well above the candidate's 4 years), triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any banking or cash‑management specific terms.</t>
+          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>SME cash management, mobile banking, payment &amp; collections, regulatory framework, OKRs, self‑serve capabilities, omnichannel strategy, user onboarding for banking</t>
+          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2739,59 +2404,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Luxoft</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - SME Cash Management</t>
+          <t>Product Manager (Materials Program)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 12+ years of experience (and 8+ years as a Product Owner), which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks many core banking and SME cash‑management keywords.</t>
+          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SME cash management, mobile banking, web banking, OKRs, regulatory framework, payments &amp; collections, self‑serve capabilities (e‑statements, account management), omnichannel strategy</t>
+          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2805,59 +2470,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>American Express Global Business Travel</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Owner - Specialist Manager, Project - Hyderabad</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru East, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like "WordPress" and "API integrations".</t>
+          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "change management" and "operational metrics".</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>WordPress, API integrations, content management system, website performance monitoring, vendor management</t>
+          <t>change management, operational metrics, release readiness, defect resolution, standard operating procedures, risk indicators, roadmap planning, governance</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2871,38 +2536,38 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Vice President</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -2918,12 +2583,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2937,21 +2602,21 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2633,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -3003,7 +2668,7 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -3017,45 +2682,45 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Keyloop</t>
+          <t>Sonata Software</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager (E-Commerce)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>Hard rules are satisfied; however the resume lacks many JD-specific terms (e.g., POS, inventory management, circular economy) and does not show Pune location, resulting in a modest ATS score. The candidate’s GenAI and SaaS experience aligns reasonably with the role, giving a moderate fit score.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
+          <t>Point-of-Sale, inventory management, circular economy, field service management, pricing optimisation, CRM, fleet management, demand forecasting, OKRs</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -3069,7 +2734,7 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -3078,29 +2743,29 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>Xplor Technologies</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Materials Program)</t>
+          <t>Product Owner, Billing &amp; Settlement</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
@@ -3116,12 +2781,12 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
+          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
+          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -3135,59 +2800,59 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Olympus Corporation</t>
+          <t>Cybage Software</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Supply Chain Solutions Product Owner</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune City, Maharashtra, India</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>45</v>
-      </c>
       <c r="H18" s="2" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many supply chain‑specific terms (SAP, o9, UAT, training/adoption) and only partially matches the JD keywords, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>Hard rules pass, but the resume lacks many JD-specific keywords (e.g., HTML graphics, studio automation) and does not show location alignment, resulting in a low ATS score; domain mismatch lowers the fit score.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>SAP S/4, o9, UAT, training and adoption, roadmap</t>
+          <t>HTML graphics, studio automation, product vision, roadmap, KPIs, A/B testing, OKRs, data‑driven metrics, product experimentation</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -3201,59 +2866,61 @@
         </is>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Unbox Robotics</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Specialist Manager, Project - Hyderabad</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F19" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "change management" and "operational metrics".</t>
+          <t>The resume lacks core hardware and robotics keywords required by the JD and does not demonstrate experience with EVT/DVT/PVT cycles, resulting in a low ATS score; the biggest gap is the absence of any hardware product development terminology.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>change management, operational metrics, release readiness, defect resolution, standard operating procedures, risk indicators, roadmap planning, governance</t>
+          <t>EVT, DVT, PVT, NPI, robotics, industrial automation, IoT hardware, hardware roadmap, supply chain coordination, embedded control units</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -3267,7 +2934,7 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
@@ -3281,45 +2948,45 @@
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Nasdaq</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>Product Manager Specialist</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>The resume meets the 4-year experience requirement, but lacks many domain-specific keywords and regulatory expertise required for the Nasdaq role, resulting in low ATS and fit scores; the biggest gap is the absence of regulatory reporting and Chartered Accountant credentials.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>Chartered Accountant, Regulatory reporting, Basel, Financial statements, Functional Specification Document, ControllerView, AxiomSL, Banking products, APAC regulatory frameworks</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -3333,33 +3000,33 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Sonata Software</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (E-Commerce)</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3370,22 +3037,22 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; however the resume lacks many JD-specific terms (e.g., POS, inventory management, circular economy) and does not show Pune location, resulting in a modest ATS score. The candidate’s GenAI and SaaS experience aligns reasonably with the role, giving a moderate fit score.</t>
+          <t>The JD requires 6+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any hyperscaler or AI service stack mentions (e.g., Azure, AWS, OpenAI).</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Point-of-Sale, inventory management, circular economy, field service management, pricing optimisation, CRM, fleet management, demand forecasting, OKRs</t>
+          <t>Azure, AWS, Google Cloud, OpenAI, Responsible AI, AI service stack, hyperscaler ecosystem, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -3403,55 +3070,55 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Xplor Technologies</t>
+          <t>Seventh Contact Hiring Solutions</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Product Owner, Billing &amp; Settlement</t>
+          <t>Product Manager II (Front end Architecture Exp) with US based product company- Remote.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Pune Division, Maharashtra, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule so both scores are forced below 30; the most important keyword gap is the lack of explicit front‑end architecture experience.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
+          <t>front‑end architecture, reusable component library, widget‑based product design, OKRs, A/B testing, customer NPS improvement</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -3474,19 +3141,19 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Unbox Robotics</t>
+          <t>Sibros</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -3500,26 +3167,24 @@
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>The resume lacks core hardware and robotics keywords required by the JD and does not demonstrate experience with EVT/DVT/PVT cycles, resulting in a low ATS score; the biggest gap is the absence of any hardware product development terminology.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>EVT, DVT, PVT, NPI, robotics, industrial automation, IoT hardware, hardware roadmap, supply chain coordination, embedded control units</t>
+          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -3537,283 +3202,17 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Aumni</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner - Roadmap &amp;amp; Strategy</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>Candidate has only 4 years experience while the JD explicitly requires 5+ years, triggering a hard rule that caps both scores below 30; also the resume lacks several core JD keywords such as Confluence and roadmap planning.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>Confluence, AI/ML platforms, roadmap planning, product strategy, OKRs, RICE prioritization, NPS improvement, A/B testing, Snowflake</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Virtusa</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Sibros</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Azuga, Inc.</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager – Connected Hardware &amp; Telematics (HW / FW / IoT)</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Bagalur, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 3‑year minimum experience, but the resume lacks most hardware/IoT keywords required for the role, resulting in a low ATS score; the biggest gap is the absence of telematics and firmware terminology.</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>OBD‑II, J1939, CAN protocol, OTA firmware upgrade, BLE beacon, LTE Cat M1, FCC certification, telematics vendor management</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="N27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -3841,10 +3240,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: daily job scan 2026-06-02
</commit_message>
<xml_diff>
--- a/output/jobs_master.xlsx
+++ b/output/jobs_master.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scoutit</t>
+          <t>Lumber</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -577,28 +577,30 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban district, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="F2" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
+          <t>The candidate meets the 2‑year minimum and has a relevant Associate Product Manager title, but the resume lacks several exact JD keywords such as Confluence, Trello, and explicit API/integration experience.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
+          <t>Confluence, Trello, API integrations, product roadmap, competitor research</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -621,24 +623,24 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MakeMyTrip</t>
+          <t>Curefit</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - Personalization &amp; Data Platforms</t>
+          <t>Product Manager 2 - Operations Excellence</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -647,26 +649,24 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year minimum and has strong keyword overlap, but lacks several JD‑specific terms such as A/B testing and real‑time personalization, lowering the ATS score; the biggest gap is missing explicit personalization/MarTech experience.</t>
+          <t>The resume hits most JD keywords and meets location and experience criteria, yielding a high ATS score; however, the candidate lacks direct IoT and fitness‑center operations experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, real-time personalization, MarTech, data platform, OKRs, experimentation framework, customer lifecycle metrics</t>
+          <t>IoT, vision-tech, real-time visibility, workflow automation, user research, OKRs, metrics, CCTV</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -684,29 +684,29 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Hinge Health</t>
+          <t>Pocket FM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -717,22 +717,22 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 3+ years requirement and has a relevant title, so hard rules do not penalize. The resume covers many core keywords (Jira, Agile, SQL, Power BI, GenAI) but misses several JD‑specific terms such as RBAC, audit logging, and algorithmic matching, limiting the ATS score.</t>
+          <t>The resume meets the experience requirement (4 years vs 1-2 years needed) and title alignment, yielding a solid ATS score; the most important keyword gap is the lack of explicit mention of subscription and loyalty program experience.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>RBAC, audit logging, algorithmic matching, capacity management, microservices architecture, OKRs, KPIs, roadmap</t>
+          <t>Subscription, Loyalty Programs, Pricing strategy, Offers, A/B testing, OKRs, NPS improvement</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -750,55 +750,55 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Scoutit</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager, Amazon Business India</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore Urban district, India</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>78</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2+ years requirement and location, and contains many relevant keywords, but lacks several JD-specific terms and the title is one level below the target, lowering the ATS score; the strongest keyword gap is the absence of 'approval workflows'.</t>
+          <t>The candidate meets the experience requirement and has a relevant title, but the resume lacks several JD-specific keywords such as helpdesk and conversion metrics, lowering the ATS score; overall domain and skill alignment are strong.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>approval workflows, GST compliance, spend analytics, multi-user accounts, OKRs, A/B testing</t>
+          <t>helpdesk solutions, customer success management, A/B testing, OKRs, conversion rate optimization</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -816,29 +816,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Axi</t>
+          <t>Aspire</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager -Growth</t>
+          <t>Product Manager - Local Payments</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -847,24 +847,26 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="F6" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>64</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, stakeholder management, SaaS, data‑driven) but lacks growth‑specific terms, lowering the ATS score. The biggest keyword gap is the absence of explicit growth‑experiment language such as "A/B testing".</t>
+          <t>The resume meets the 4‑year minimum and location requirement, and contains many JD keywords, yielding a strong ATS score; however, the candidate lacks direct payments and fintech experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Mixpanel, Snowflake, OKRs, Referral program, Loyalty program, Personalized notifications, Cohort analysis</t>
+          <t>payments, transaction management, risk management, regulatory compliance, A/B testing, OKRs, marketplace dynamics</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -882,29 +884,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Peoplebox.ai</t>
+          <t>Meesho</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager (APM)</t>
+          <t>Product Manager I</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -913,26 +915,24 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>78</v>
-      </c>
       <c r="H7" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the years requirement and title level, but the resume lacks many exact JD keywords such as product discovery and success metrics, lowering the ATS score; overall domain and experience align well, giving a solid fit score.</t>
+          <t>The resume meets the 4-year experience requirement and passes all hard rules; it contains many JD keywords but lacks FinTech and lending-specific terms, which lowers the fit score.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Product Discovery, customer interviews, data analysis, competitive research, success metrics, product roadmap, AI tools, prototypes, mockups</t>
+          <t>lending APIs, bank integration, BNPL, conversion funnel metrics, A/B testing, OKRs</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -950,29 +950,29 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Merck Life Science</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Owner — General</t>
+          <t>Global Product Manager</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -981,26 +981,24 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 2-year minimum and title seniority rules, yielding a strong ATS match due to many exact keywords; the biggest gap is lack of fintech-specific terms like account management and data synchronization.</t>
+          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>account management, data synchronization, consumer payment experience, customer onboarding, rapid prototyping, OKRs, A/B testing, Mixpanel</t>
+          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1018,7 +1016,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1028,45 +1026,45 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Merck Life Science</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Global Product Manager</t>
+          <t>Associate Product Manager | Pune</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 4‑year experience requirement and title level, but lacks several JD‑specific keywords such as supply‑disruption communication and lifecycle analysis, lowering the ATS score; the strongest gap is the absence of explicit product‑line management terminology.</t>
+          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>supply disruption communication, product lifecycle analysis, risk mitigation, investment planning deliverables, customer change notification process, portfolio analysis</t>
+          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1080,7 +1078,7 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1094,47 +1092,45 @@
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>InvoiceCloud, Inc.</t>
+          <t>Cornerstone OnDemand</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Owner (Tax)</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
         <v>78</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the 3‑year minimum and title seniority rules, yielding solid keyword coverage but limited fintech tax domain experience, which lowers the fit score; the biggest gap is lack of tax‑specific terminology.</t>
+          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>tax bill presentment, municipal tax integration, installment payment workflows, regulatory compliance, digital adoption metrics, OKRs, A/B testing</t>
+          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1148,11 +1144,11 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1162,19 +1158,19 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cornerstone OnDemand</t>
+          <t>PerkinElmer</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Associate Product Manager | Pune</t>
+          <t>Software Product Manager (GTM Strategy)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1188,19 +1184,19 @@
         <v>78</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>The resume aligns well with the 0-2 year requirement and the Associate Product Manager title, yielding strong keyword coverage; the biggest gap is the lack of explicit mention of product analytics tools and prioritization frameworks.</t>
+          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) giving a strong ATS score, but lacks domain-specific scientific software experience, lowering the fit score.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, OKRs, Mixpanel, NPS improvement, RICE prioritization, customer interviews, product analytics</t>
+          <t>go-to-market strategy, customer migration, adoption metrics, NPS improvement, OKRs</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1223,408 +1219,12 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Cornerstone OnDemand</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>The resume contains most high‑impact keywords and the title matches exactly, yielding a strong ATS score; the candidate's SaaS and GenAI experience aligns well with the role, giving a high fit score. The main keyword gap is the lack of explicit mention of user research/roadmap planning.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>user research, customer feedback, roadmap planning, Scrum, OKRs, metrics tracking, NPS improvement</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>PerkinElmer</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Software Product Manager (GTM Strategy)</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the hard rules (4 years experience, no senior title requirement). It contains many JD keywords (Jira, Agile, SQL, Power BI, GenAI, RAG) giving a strong ATS score, but lacks domain-specific scientific software experience, lowering the fit score.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>go-to-market strategy, customer migration, adoption metrics, NPS improvement, OKRs</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Wipro</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>PRODUCT MANAGER L2</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the 4‑year experience requirement and the title is appropriate, but the resume lacks several JD‑specific terms such as RFP, DevOps, and user acceptance testing, lowering the ATS score.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>RFP coordination, pre‑sales team collaboration, DevOps integration, user acceptance testing, impact analysis, product vision and roadmap</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>House Of Edtech</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager — Learning &amp; EdTech</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>The candidate meets the experience requirement (4 years vs 2-3 years needed) and title alignment, but lacks several JD-specific tools and mobile platform keywords, lowering the ATS score; the biggest gap is the absence of analytics tools like Amplitude or Mixpanel.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Amplitude, Mixpanel, Google Analytics, iOS, Android, A/B testing, OKRs</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>hackajob</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Digital Product Owner</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>No hard rule violations; the resume covers many Agile and Jira terms but misses several JD-specific technical backlog concepts, lowering the ATS score. The main keyword gap is the absence of terms like "technical debt" and "regulatory change".</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>technical debt, KTLO, regulatory change, platform optimisation, risk and controls</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>House Of Edtech</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Associate Product Manager — Consumer &amp; Streaming</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the years requirement and title level, but lacks several consumer‑streaming specific keywords, lowering the ATS score; the biggest gap is the absence of product analytics tools like Mixpanel/Amplitude.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Mixpanel, Amplitude, Firebase, product roadmap, PRD, backlog grooming, user research, usability testing, NPS improvement, MAU growth</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -1640,12 +1240,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1657,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1763,12 +1357,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Abnormal AI</t>
+          <t>Urban Company</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II</t>
+          <t>Associate Product Manager</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1789,12 +1383,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the hard rules but contains only partial keyword overlap with the JD, especially missing core integration and API lifecycle terms, leading to a moderate ATS score; the candidate's SaaS and GenAI background aligns reasonably with the role, giving a decent fit score.</t>
+          <t>Hard rules are satisfied (4 years experience, no senior title requirement). ATS score is moderate due to limited overlap with JD-specific terminology, while the fit score reflects decent domain relevance but missing many partner‑empowerment concepts.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>REST API, SIEM integration, SOAR integration, API lifecycle management, token management, versioning, schema governance, MCP server, notifications, product configuration</t>
+          <t>partner empowerment, micro‑entrepreneur platform, market access, standardization (SOPs, pricing, delivery tracking), training &amp; upskilling programs, financing and insurance products, two‑sided marketplace dynamics, NPS improvement, MAU growth</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1817,12 +1411,12 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1472,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -1888,19 +1482,19 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tesco Bengaluru</t>
+          <t>Slikk</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - Supply / Warehouse</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1909,24 +1503,26 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="F4" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>60</v>
-      </c>
       <c r="H4" s="2" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass (4 years experience, no senior title requirement). The resume lacks many core payment and checkout keywords from the JD, lowering the ATS score; the biggest gap is the absence of any payments/API experience.</t>
+          <t>The resume meets the 3‑year minimum and location/education criteria, but lacks many warehouse and supply‑chain specific terms, resulting in a modest ATS score; the biggest gap is the absence of WMS/OMS and inventory‑visibility keywords.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, basket building, payment methods (card, digital wallets, gift cards, BNPL), authorisation success metrics, settlement process, omnichannel platform</t>
+          <t>Warehouse Management System (WMS), Order Management System (OMS), inventory visibility, real-time inventory tracking, inbound/outbound logistics, pick and pack workflow, supply chain optimization, operational dashboards for warehouse, SQL analytics for inventory</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1944,29 +1540,29 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Booking Holdings (NASDAQ: BKNG)</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager - HashiCorp Boundary</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1975,26 +1571,24 @@
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>The candidate meets the 4‑year requirement, but the resume lacks many FinTech/payment‑specific keywords and direct experience, resulting in moderate ATS and fit scores; the biggest gap is missing payment‑domain terminology.</t>
+          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'Privileged Access Management'.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Payment Service Provider (PSP), Alternative Payment Methods (APM), FinTech, Payment gateway integration, Conversion rate optimization, KPI tracking, A/B testing, OKRs, Marketplace dynamics</t>
+          <t>Privileged Access Management, session recording, secrets management, PKI, threat monitoring</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2012,29 +1606,29 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Nykaa</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Manager II - Personalisation</t>
+          <t>Product Manager - Vice President</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2045,22 +1639,22 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied (4 years experience, no senior title, no &gt;4 year requirement). ATS score is moderate due to good keyword overlap on Jira, SQL, Agile but missing key personalization and ML terms; fit score is lower because the candidate's domain (B2B SaaS, travel, FMCG) does not align closely with Nykaa's beauty/fashion personalization focus.</t>
+          <t>The job title includes VP, triggering hard rule 3, so both scores must be below 30 regardless of experience or keywords; the resume lacks several core JD terms such as "customer service operations" and "CRM platform".</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A/B testing, Recommendation engine, Personalization, Machine learning collaboration, API integration, Data Science partnership, OKRs, NPS improvement, MAU growth</t>
+          <t>CRM platform, customer service operations, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2078,29 +1672,29 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tesco Technology</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager-Tech III, Finance Automation</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2111,22 +1705,22 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass, but the resume lacks many core payment and checkout keywords from the JD, resulting in low ATS and fit scores; the biggest gap is the absence of payment‑related terminology.</t>
+          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Online Payments API, OKRs, checkout, digital wallets, gift card payments, Buy now pay later, basket building, payment authorization metrics, omnichannel platform</t>
+          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2144,55 +1738,55 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Product Manager - HashiCorp Boundary</t>
+          <t>Product Manager (Reference Standards)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 5+ years of product management experience, but the candidate has only 4+ years, triggering a hard rule that forces both scores below 30; the resume also lacks the keyword 'Privileged Access Management'.</t>
+          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Privileged Access Management, session recording, secrets management, PKI, threat monitoring</t>
+          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2206,59 +1800,59 @@
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Virtusa</t>
+          <t>US Pharmacopeia</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Product Manager (Materials Program)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Bangalore Urban, Karnataka, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks key terms like 'investment banking' and 'payment systems'.</t>
+          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>investment banking, payment systems, data product, digital adoption platform (specific tool name), Python or Java development</t>
+          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2272,59 +1866,59 @@
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>Xplor Technologies</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Reference Standards)</t>
+          <t>Product Owner, Billing &amp; Settlement</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>45</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>The resume contains many relevant product management keywords and tools, giving a moderate ATS score, but the candidate's domain (SaaS/GenAI) does not align with the pharma reference‑standards focus, lowering the fit score; the most important missing keyword is "reference standards".</t>
+          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>reference standards, small molecules, forecasting, financial modeling, regulatory compliance, portfolio management, OKRs, RICE prioritization</t>
+          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -2338,7 +1932,7 @@
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -2347,50 +1941,50 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Keyloop</t>
+          <t>Nasdaq</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Product Manager Specialist</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune Division, Maharashtra, India</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Hard rules are satisfied; the resume contains many relevant product management keywords but lacks automotive finance and ERP-specific terms, leading to a moderate ATS score and a lower fit score due to domain mismatch.</t>
+          <t>The resume meets the 4-year experience requirement, but lacks many domain-specific keywords and regulatory expertise required for the Nasdaq role, resulting in low ATS and fit scores; the biggest gap is the absence of regulatory reporting and Chartered Accountant credentials.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>SAP, Oracle, ERP integrations, predictive analytics, A/B testing, OKRs, NPS improvement, Marketplace dynamics</t>
+          <t>Chartered Accountant, Regulatory reporting, Basel, Financial statements, Functional Specification Document, ControllerView, AxiomSL, Banking products, APAC regulatory frameworks</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2404,59 +1998,59 @@
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>US Pharmacopeia</t>
+          <t>FPL Technologies</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Product Manager (Materials Program)</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>The resume meets the basic experience requirement (4 years) and passes all hard rules, but lacks many pharma‑specific keywords and domain experience, lowering the fit score; the biggest keyword gap is the absence of pharmaceutical reference material terminology.</t>
+          <t>The JD requires 5+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of explicit fintech or financial‑wellness domain terms.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Pharmaceutical analytical impurities, Certified Reference Materials, Regulatory compliance, Portfolio management, Quality standards, Scientific stakeholder engagement, OKRs, Snowflake, NPS improvement</t>
+          <t>financial wellness, fintech, consumer banking, AI/ML model productization, API‑driven onboarding, user segmentation, growth metrics (MAU, NPS), risk and compliance</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2470,59 +2064,59 @@
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Seventh Contact Hiring Solutions</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Product Owner - Specialist Manager, Project - Hyderabad</t>
+          <t>Product Manager II (Widget /reusable Ui Component Exp) with US based product company- Remote.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 10+ years of experience, which exceeds the candidate's 4 years, triggering a hard rule that forces both scores below 30; the resume also lacks several core JD keywords such as "change management" and "operational metrics".</t>
+          <t>The JD explicitly requires 5+ years of product management experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any mention of reusable UI component or widget architecture.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>change management, operational metrics, release readiness, defect resolution, standard operating procedures, risk indicators, roadmap planning, governance</t>
+          <t>reusable UI components, widget-based front‑end architecture, OKRs, A/B testing, NPS improvement</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2536,38 +2130,38 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>HCLTech</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Product Manager-Tech III, Finance Automation</t>
+          <t>AI Product Manager</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Pune District, Maharashtra, India</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -2583,12 +2177,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>The JD requires 7+ years of experience; the candidate has only 4 years, triggering a hard rule so both scores are forced below 30. The resume also lacks several key JD terms such as "press release" and "non‑functional requirements".</t>
+          <t>The JD requires 6+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any hyperscaler or AI service stack mentions (e.g., Azure, AWS, OpenAI).</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>press release, FAQs, non‑functional requirements, OKRs, A/B testing</t>
+          <t>Azure, AWS, Google Cloud, OpenAI, Responsible AI, AI service stack, hyperscaler ecosystem, OKRs, A/B testing</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -2602,33 +2196,33 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Optum India</t>
+          <t>Sibros</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Technical Product Manager</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -2639,22 +2233,22 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Hard rules pass; the resume contains many core keywords but lacks Rally, Aha! and design system terms, and the location does not match Pune, leading to a moderate ATS score. Fit is decent due to strong SaaS and GenAI experience, though the domain differs from health tech.</t>
+          <t>The JD requires 5+ years of experience; the candidate has only 4 years, triggering a hard rule that caps both scores below 30. The resume also lacks several key JD terms such as A/B testing and telemetry.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Rally, Aha!, design systems, component libraries, OKRs</t>
+          <t>A/B testing, telemetry, fleet intelligence, predictive maintenance, OKRs, Mixpanel</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -2672,547 +2266,17 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Sonata Software</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager (E-Commerce)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; however the resume lacks many JD-specific terms (e.g., POS, inventory management, circular economy) and does not show Pune location, resulting in a modest ATS score. The candidate’s GenAI and SaaS experience aligns reasonably with the role, giving a moderate fit score.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Point-of-Sale, inventory management, circular economy, field service management, pricing optimisation, CRM, fleet management, demand forecasting, OKRs</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Xplor Technologies</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Product Owner, Billing &amp; Settlement</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules are satisfied; the resume contains many Agile and product management terms but lacks core billing/settlement keywords and payment domain experience, leading to moderate ATS and lower fit scores.</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>billing, settlement, reconciliation, ledger, pricing models, revenue recognition, financial reporting, payment processing, compliance</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Cybage Software</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Pune City, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Hard rules pass, but the resume lacks many JD-specific keywords (e.g., HTML graphics, studio automation) and does not show location alignment, resulting in a low ATS score; domain mismatch lowers the fit score.</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>HTML graphics, studio automation, product vision, roadmap, KPIs, A/B testing, OKRs, data‑driven metrics, product experimentation</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Unbox Robotics</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>The resume lacks core hardware and robotics keywords required by the JD and does not demonstrate experience with EVT/DVT/PVT cycles, resulting in a low ATS score; the biggest gap is the absence of any hardware product development terminology.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>EVT, DVT, PVT, NPI, robotics, industrial automation, IoT hardware, hardware roadmap, supply chain coordination, embedded control units</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Nasdaq</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Product Manager Specialist</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Pune Division, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>The resume meets the 4-year experience requirement, but lacks many domain-specific keywords and regulatory expertise required for the Nasdaq role, resulting in low ATS and fit scores; the biggest gap is the absence of regulatory reporting and Chartered Accountant credentials.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Chartered Accountant, Regulatory reporting, Basel, Financial statements, Functional Specification Document, ControllerView, AxiomSL, Banking products, APAC regulatory frameworks</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>HCLTech</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>AI Product Manager</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Pune District, Maharashtra, India</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>The JD requires 6+ years of experience, but the candidate has only 4 years, triggering a hard rule that forces both scores below 30; the most important keyword gap is the lack of any hyperscaler or AI service stack mentions (e.g., Azure, AWS, OpenAI).</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Azure, AWS, Google Cloud, OpenAI, Responsible AI, AI service stack, hyperscaler ecosystem, OKRs, A/B testing</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Linkedin</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
- 